<commit_message>
Fill 'nowy format' sheet from Podsumowanie and remove empty rows
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3QuwGR9tgiXrdWSSrWcuu
</commit_message>
<xml_diff>
--- a/Wniosek_o_platnosc_str26-34.xlsx
+++ b/Wniosek_o_platnosc_str26-34.xlsx
@@ -5,13 +5,17 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Podsumowanie" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Kontrola" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Uwagi" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="nowy format" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'nowy format'!$A$2:$G$43</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -22,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="113">
   <si>
     <t xml:space="preserve">Wniosek o płatność – PODSUMOWANIE (PDF str. 27–34)</t>
   </si>
@@ -346,6 +350,21 @@
   </si>
   <si>
     <t xml:space="preserve">W nazwach zadań usunięto zdublowaną numerację (PDF: 'Zadanie 1. 1. …').</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wydatki narastająco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wydatki w projekcie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wydatki ogółem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wydatki kwalifikowane</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dofinansowanie</t>
   </si>
 </sst>
 </file>
@@ -383,14 +402,14 @@
       <b val="true"/>
       <sz val="12"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <i val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -398,7 +417,7 @@
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -406,34 +425,34 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="11"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -506,7 +525,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -587,6 +606,18 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -596,11 +627,50 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF1F3864"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9E1F2"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -666,6 +736,10 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -849,7 +923,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H162"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="16"/>
@@ -859,7 +933,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -869,7 +943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -895,7 +969,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>10</v>
       </c>
@@ -1695,7 +1769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
         <v>23</v>
       </c>
@@ -2335,7 +2409,7 @@
         <v>-0</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="9" t="s">
         <v>31</v>
       </c>
@@ -2575,7 +2649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="s">
         <v>34</v>
       </c>
@@ -4263,7 +4337,7 @@
         <v>-0</v>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="9" t="s">
         <v>56</v>
       </c>
@@ -5086,7 +5160,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G85"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
@@ -5097,7 +5171,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>66</v>
       </c>
@@ -7388,7 +7462,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
@@ -7410,7 +7484,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
         <v>91</v>
       </c>
@@ -7418,7 +7492,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
         <v>93</v>
       </c>
@@ -7426,7 +7500,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
         <v>95</v>
       </c>
@@ -7434,7 +7508,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
         <v>97</v>
       </c>
@@ -7442,7 +7516,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
         <v>55</v>
       </c>
@@ -7450,7 +7524,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
         <v>100</v>
       </c>
@@ -7491,4 +7565,1262 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="true">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G57"/>
+  <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="71.67"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="F2" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="G2" s="21" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="22" t="n">
+        <f aca="false">Podsumowanie!D5</f>
+        <v>807424.87</v>
+      </c>
+      <c r="C3" s="22" t="n">
+        <f aca="false">Podsumowanie!D6</f>
+        <v>807424.87</v>
+      </c>
+      <c r="D3" s="22" t="n">
+        <f aca="false">Podsumowanie!D7</f>
+        <v>645939.9</v>
+      </c>
+      <c r="E3" s="22" t="n">
+        <f aca="false">Podsumowanie!E5</f>
+        <v>868383.93</v>
+      </c>
+      <c r="F3" s="22" t="n">
+        <f aca="false">Podsumowanie!E6</f>
+        <v>868383.93</v>
+      </c>
+      <c r="G3" s="22" t="n">
+        <f aca="false">Podsumowanie!E7</f>
+        <v>694707.14</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="22" t="n">
+        <f aca="false">Podsumowanie!D8</f>
+        <v>277000</v>
+      </c>
+      <c r="C4" s="22" t="n">
+        <f aca="false">Podsumowanie!D9</f>
+        <v>277000</v>
+      </c>
+      <c r="D4" s="22" t="n">
+        <f aca="false">Podsumowanie!D10</f>
+        <v>221600</v>
+      </c>
+      <c r="E4" s="22" t="n">
+        <f aca="false">Podsumowanie!E8</f>
+        <v>277000</v>
+      </c>
+      <c r="F4" s="22" t="n">
+        <f aca="false">Podsumowanie!E9</f>
+        <v>277000</v>
+      </c>
+      <c r="G4" s="22" t="n">
+        <f aca="false">Podsumowanie!E10</f>
+        <v>221600</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="22" t="n">
+        <f aca="false">Podsumowanie!D11</f>
+        <v>94300</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <f aca="false">Podsumowanie!D12</f>
+        <v>94300</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <f aca="false">Podsumowanie!D13</f>
+        <v>75440</v>
+      </c>
+      <c r="E5" s="22" t="n">
+        <f aca="false">Podsumowanie!E11</f>
+        <v>94300</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <f aca="false">Podsumowanie!E12</f>
+        <v>94300</v>
+      </c>
+      <c r="G5" s="22" t="n">
+        <f aca="false">Podsumowanie!E13</f>
+        <v>75440</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="22" t="n">
+        <f aca="false">Podsumowanie!D14</f>
+        <v>121994.98</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <f aca="false">Podsumowanie!D15</f>
+        <v>121994.98</v>
+      </c>
+      <c r="D6" s="22" t="n">
+        <f aca="false">Podsumowanie!D16</f>
+        <v>97595.98</v>
+      </c>
+      <c r="E6" s="22" t="n">
+        <f aca="false">Podsumowanie!E14</f>
+        <v>135550</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <f aca="false">Podsumowanie!E15</f>
+        <v>135550</v>
+      </c>
+      <c r="G6" s="22" t="n">
+        <f aca="false">Podsumowanie!E16</f>
+        <v>108440</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="22" t="n">
+        <f aca="false">Podsumowanie!D17</f>
+        <v>50828.54</v>
+      </c>
+      <c r="C7" s="22" t="n">
+        <f aca="false">Podsumowanie!D18</f>
+        <v>50828.54</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <f aca="false">Podsumowanie!D19</f>
+        <v>40662.83</v>
+      </c>
+      <c r="E7" s="22" t="n">
+        <f aca="false">Podsumowanie!E17</f>
+        <v>51562.5</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <f aca="false">Podsumowanie!E18</f>
+        <v>51562.5</v>
+      </c>
+      <c r="G7" s="22" t="n">
+        <f aca="false">Podsumowanie!E19</f>
+        <v>41250</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="22" t="n">
+        <f aca="false">Podsumowanie!D20</f>
+        <v>34550.27</v>
+      </c>
+      <c r="C8" s="22" t="n">
+        <f aca="false">Podsumowanie!D21</f>
+        <v>34550.27</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <f aca="false">Podsumowanie!D22</f>
+        <v>27640.23</v>
+      </c>
+      <c r="E8" s="22" t="n">
+        <f aca="false">Podsumowanie!E20</f>
+        <v>37200</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <f aca="false">Podsumowanie!E21</f>
+        <v>37200</v>
+      </c>
+      <c r="G8" s="22" t="n">
+        <f aca="false">Podsumowanie!E22</f>
+        <v>29760</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="22" t="n">
+        <f aca="false">Podsumowanie!D23</f>
+        <v>24600</v>
+      </c>
+      <c r="C9" s="22" t="n">
+        <f aca="false">Podsumowanie!D24</f>
+        <v>24600</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <f aca="false">Podsumowanie!D25</f>
+        <v>19680</v>
+      </c>
+      <c r="E9" s="22" t="n">
+        <f aca="false">Podsumowanie!E23</f>
+        <v>67325</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <f aca="false">Podsumowanie!E24</f>
+        <v>67325</v>
+      </c>
+      <c r="G9" s="22" t="n">
+        <f aca="false">Podsumowanie!E25</f>
+        <v>53860</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="22" t="n">
+        <f aca="false">Podsumowanie!D26</f>
+        <v>103125</v>
+      </c>
+      <c r="C10" s="22" t="n">
+        <f aca="false">Podsumowanie!D27</f>
+        <v>103125</v>
+      </c>
+      <c r="D10" s="22" t="n">
+        <f aca="false">Podsumowanie!D28</f>
+        <v>82500</v>
+      </c>
+      <c r="E10" s="22" t="n">
+        <f aca="false">Podsumowanie!E26</f>
+        <v>103125</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <f aca="false">Podsumowanie!E27</f>
+        <v>103125</v>
+      </c>
+      <c r="G10" s="22" t="n">
+        <f aca="false">Podsumowanie!E28</f>
+        <v>82500</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="22" t="n">
+        <f aca="false">Podsumowanie!D29</f>
+        <v>2276.08</v>
+      </c>
+      <c r="C11" s="22" t="n">
+        <f aca="false">Podsumowanie!D30</f>
+        <v>2276.08</v>
+      </c>
+      <c r="D11" s="22" t="n">
+        <f aca="false">Podsumowanie!D31</f>
+        <v>1820.86</v>
+      </c>
+      <c r="E11" s="22" t="n">
+        <f aca="false">Podsumowanie!E29</f>
+        <v>3571.43</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <f aca="false">Podsumowanie!E30</f>
+        <v>3571.43</v>
+      </c>
+      <c r="G11" s="22" t="n">
+        <f aca="false">Podsumowanie!E31</f>
+        <v>2857.14</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="22" t="n">
+        <f aca="false">Podsumowanie!D32</f>
+        <v>98750</v>
+      </c>
+      <c r="C12" s="22" t="n">
+        <f aca="false">Podsumowanie!D33</f>
+        <v>98750</v>
+      </c>
+      <c r="D12" s="22" t="n">
+        <f aca="false">Podsumowanie!D34</f>
+        <v>79000</v>
+      </c>
+      <c r="E12" s="22" t="n">
+        <f aca="false">Podsumowanie!E32</f>
+        <v>98750</v>
+      </c>
+      <c r="F12" s="22" t="n">
+        <f aca="false">Podsumowanie!E33</f>
+        <v>98750</v>
+      </c>
+      <c r="G12" s="22" t="n">
+        <f aca="false">Podsumowanie!E34</f>
+        <v>79000</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="22" t="n">
+        <f aca="false">Podsumowanie!D35</f>
+        <v>1008769.29</v>
+      </c>
+      <c r="C13" s="22" t="n">
+        <f aca="false">Podsumowanie!D36</f>
+        <v>842569.29</v>
+      </c>
+      <c r="D13" s="22" t="n">
+        <f aca="false">Podsumowanie!D37</f>
+        <v>674055.43</v>
+      </c>
+      <c r="E13" s="22" t="n">
+        <f aca="false">Podsumowanie!E35</f>
+        <v>1226935.71</v>
+      </c>
+      <c r="F13" s="22" t="n">
+        <f aca="false">Podsumowanie!E36</f>
+        <v>1203935.71</v>
+      </c>
+      <c r="G13" s="22" t="n">
+        <f aca="false">Podsumowanie!E37</f>
+        <v>963148.56</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="22" t="n">
+        <f aca="false">Podsumowanie!D38</f>
+        <v>332400</v>
+      </c>
+      <c r="C14" s="22" t="n">
+        <f aca="false">Podsumowanie!D39</f>
+        <v>166200</v>
+      </c>
+      <c r="D14" s="22" t="n">
+        <f aca="false">Podsumowanie!D40</f>
+        <v>132960</v>
+      </c>
+      <c r="E14" s="22" t="n">
+        <f aca="false">Podsumowanie!E38</f>
+        <v>332400</v>
+      </c>
+      <c r="F14" s="22" t="n">
+        <f aca="false">Podsumowanie!E39</f>
+        <v>332400</v>
+      </c>
+      <c r="G14" s="22" t="n">
+        <f aca="false">Podsumowanie!E40</f>
+        <v>265920</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="22" t="n">
+        <f aca="false">Podsumowanie!D41</f>
+        <v>113168.16</v>
+      </c>
+      <c r="C15" s="22" t="n">
+        <f aca="false">Podsumowanie!D42</f>
+        <v>113168.16</v>
+      </c>
+      <c r="D15" s="22" t="n">
+        <f aca="false">Podsumowanie!D43</f>
+        <v>90534.53</v>
+      </c>
+      <c r="E15" s="22" t="n">
+        <f aca="false">Podsumowanie!E41</f>
+        <v>113160</v>
+      </c>
+      <c r="F15" s="22" t="n">
+        <f aca="false">Podsumowanie!E42</f>
+        <v>113160</v>
+      </c>
+      <c r="G15" s="22" t="n">
+        <f aca="false">Podsumowanie!E43</f>
+        <v>90528</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="22" t="n">
+        <f aca="false">Podsumowanie!D44</f>
+        <v>121024.78</v>
+      </c>
+      <c r="C16" s="22" t="n">
+        <f aca="false">Podsumowanie!D45</f>
+        <v>121024.78</v>
+      </c>
+      <c r="D16" s="22" t="n">
+        <f aca="false">Podsumowanie!D46</f>
+        <v>96819.8</v>
+      </c>
+      <c r="E16" s="22" t="n">
+        <f aca="false">Podsumowanie!E44</f>
+        <v>162660</v>
+      </c>
+      <c r="F16" s="22" t="n">
+        <f aca="false">Podsumowanie!E45</f>
+        <v>162660</v>
+      </c>
+      <c r="G16" s="22" t="n">
+        <f aca="false">Podsumowanie!E46</f>
+        <v>130128</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="22" t="n">
+        <f aca="false">Podsumowanie!D47</f>
+        <v>123750</v>
+      </c>
+      <c r="C17" s="22" t="n">
+        <f aca="false">Podsumowanie!D48</f>
+        <v>123750</v>
+      </c>
+      <c r="D17" s="22" t="n">
+        <f aca="false">Podsumowanie!D49</f>
+        <v>99000</v>
+      </c>
+      <c r="E17" s="22" t="n">
+        <f aca="false">Podsumowanie!E47</f>
+        <v>123750</v>
+      </c>
+      <c r="F17" s="22" t="n">
+        <f aca="false">Podsumowanie!E48</f>
+        <v>123750</v>
+      </c>
+      <c r="G17" s="22" t="n">
+        <f aca="false">Podsumowanie!E49</f>
+        <v>99000</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" s="22" t="n">
+        <f aca="false">Podsumowanie!D50</f>
+        <v>44388.77</v>
+      </c>
+      <c r="C18" s="22" t="n">
+        <f aca="false">Podsumowanie!D51</f>
+        <v>44388.77</v>
+      </c>
+      <c r="D18" s="22" t="n">
+        <f aca="false">Podsumowanie!D52</f>
+        <v>35511.02</v>
+      </c>
+      <c r="E18" s="22" t="n">
+        <f aca="false">Podsumowanie!E50</f>
+        <v>44640</v>
+      </c>
+      <c r="F18" s="22" t="n">
+        <f aca="false">Podsumowanie!E51</f>
+        <v>44640</v>
+      </c>
+      <c r="G18" s="22" t="n">
+        <f aca="false">Podsumowanie!E52</f>
+        <v>35712</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="22" t="n">
+        <f aca="false">Podsumowanie!D53</f>
+        <v>123750</v>
+      </c>
+      <c r="C19" s="22" t="n">
+        <f aca="false">Podsumowanie!D54</f>
+        <v>123750</v>
+      </c>
+      <c r="D19" s="22" t="n">
+        <f aca="false">Podsumowanie!D55</f>
+        <v>99000</v>
+      </c>
+      <c r="E19" s="22" t="n">
+        <f aca="false">Podsumowanie!E53</f>
+        <v>123750</v>
+      </c>
+      <c r="F19" s="22" t="n">
+        <f aca="false">Podsumowanie!E54</f>
+        <v>123750</v>
+      </c>
+      <c r="G19" s="22" t="n">
+        <f aca="false">Podsumowanie!E55</f>
+        <v>99000</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" s="22" t="n">
+        <f aca="false">Podsumowanie!D56</f>
+        <v>29517.79</v>
+      </c>
+      <c r="C20" s="22" t="n">
+        <f aca="false">Podsumowanie!D57</f>
+        <v>29517.79</v>
+      </c>
+      <c r="D20" s="22" t="n">
+        <f aca="false">Podsumowanie!D58</f>
+        <v>23614.23</v>
+      </c>
+      <c r="E20" s="22" t="n">
+        <f aca="false">Podsumowanie!E56</f>
+        <v>80790</v>
+      </c>
+      <c r="F20" s="22" t="n">
+        <f aca="false">Podsumowanie!E57</f>
+        <v>80790</v>
+      </c>
+      <c r="G20" s="22" t="n">
+        <f aca="false">Podsumowanie!E58</f>
+        <v>64632</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21" s="22" t="n">
+        <f aca="false">Podsumowanie!D59</f>
+        <v>0</v>
+      </c>
+      <c r="C21" s="22" t="n">
+        <f aca="false">Podsumowanie!D60</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="22" t="n">
+        <f aca="false">Podsumowanie!D61</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="22" t="n">
+        <f aca="false">Podsumowanie!E59</f>
+        <v>123000</v>
+      </c>
+      <c r="F21" s="22" t="n">
+        <f aca="false">Podsumowanie!E60</f>
+        <v>100000</v>
+      </c>
+      <c r="G21" s="22" t="n">
+        <f aca="false">Podsumowanie!E61</f>
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="22" t="n">
+        <f aca="false">Podsumowanie!D62</f>
+        <v>2276.08</v>
+      </c>
+      <c r="C22" s="22" t="n">
+        <f aca="false">Podsumowanie!D63</f>
+        <v>2276.08</v>
+      </c>
+      <c r="D22" s="22" t="n">
+        <f aca="false">Podsumowanie!D64</f>
+        <v>1820.88</v>
+      </c>
+      <c r="E22" s="22" t="n">
+        <f aca="false">Podsumowanie!E62</f>
+        <v>4285.71</v>
+      </c>
+      <c r="F22" s="22" t="n">
+        <f aca="false">Podsumowanie!E63</f>
+        <v>4285.71</v>
+      </c>
+      <c r="G22" s="22" t="n">
+        <f aca="false">Podsumowanie!E64</f>
+        <v>3428.56</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="22" t="n">
+        <f aca="false">Podsumowanie!D65</f>
+        <v>118493.71</v>
+      </c>
+      <c r="C23" s="22" t="n">
+        <f aca="false">Podsumowanie!D66</f>
+        <v>118493.71</v>
+      </c>
+      <c r="D23" s="22" t="n">
+        <f aca="false">Podsumowanie!D67</f>
+        <v>94794.97</v>
+      </c>
+      <c r="E23" s="22" t="n">
+        <f aca="false">Podsumowanie!E65</f>
+        <v>118500</v>
+      </c>
+      <c r="F23" s="22" t="n">
+        <f aca="false">Podsumowanie!E66</f>
+        <v>118500</v>
+      </c>
+      <c r="G23" s="22" t="n">
+        <f aca="false">Podsumowanie!E67</f>
+        <v>94800</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="22" t="n">
+        <f aca="false">Podsumowanie!D68</f>
+        <v>0</v>
+      </c>
+      <c r="C24" s="22" t="n">
+        <f aca="false">Podsumowanie!D69</f>
+        <v>0</v>
+      </c>
+      <c r="D24" s="22" t="n">
+        <f aca="false">Podsumowanie!D70</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="22" t="n">
+        <f aca="false">Podsumowanie!E68</f>
+        <v>1103935.71</v>
+      </c>
+      <c r="F24" s="22" t="n">
+        <f aca="false">Podsumowanie!E69</f>
+        <v>1103935.71</v>
+      </c>
+      <c r="G24" s="22" t="n">
+        <f aca="false">Podsumowanie!E70</f>
+        <v>883148.56</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" s="22" t="n">
+        <f aca="false">Podsumowanie!D71</f>
+        <v>0</v>
+      </c>
+      <c r="C25" s="22" t="n">
+        <f aca="false">Podsumowanie!D72</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="22" t="n">
+        <f aca="false">Podsumowanie!D73</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="22" t="n">
+        <f aca="false">Podsumowanie!E71</f>
+        <v>332400</v>
+      </c>
+      <c r="F25" s="22" t="n">
+        <f aca="false">Podsumowanie!E72</f>
+        <v>332400</v>
+      </c>
+      <c r="G25" s="22" t="n">
+        <f aca="false">Podsumowanie!E73</f>
+        <v>265920</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" s="22" t="n">
+        <f aca="false">Podsumowanie!D74</f>
+        <v>0</v>
+      </c>
+      <c r="C26" s="22" t="n">
+        <f aca="false">Podsumowanie!D75</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="22" t="n">
+        <f aca="false">Podsumowanie!D76</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="22" t="n">
+        <f aca="false">Podsumowanie!E74</f>
+        <v>113160</v>
+      </c>
+      <c r="F26" s="22" t="n">
+        <f aca="false">Podsumowanie!E75</f>
+        <v>113160</v>
+      </c>
+      <c r="G26" s="22" t="n">
+        <f aca="false">Podsumowanie!E76</f>
+        <v>90528</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" s="22" t="n">
+        <f aca="false">Podsumowanie!D77</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="22" t="n">
+        <f aca="false">Podsumowanie!D78</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="22" t="n">
+        <f aca="false">Podsumowanie!D79</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="22" t="n">
+        <f aca="false">Podsumowanie!E77</f>
+        <v>162660</v>
+      </c>
+      <c r="F27" s="22" t="n">
+        <f aca="false">Podsumowanie!E78</f>
+        <v>162660</v>
+      </c>
+      <c r="G27" s="22" t="n">
+        <f aca="false">Podsumowanie!E79</f>
+        <v>130128</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B28" s="22" t="n">
+        <f aca="false">Podsumowanie!D80</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="22" t="n">
+        <f aca="false">Podsumowanie!D81</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="22" t="n">
+        <f aca="false">Podsumowanie!D82</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="22" t="n">
+        <f aca="false">Podsumowanie!E80</f>
+        <v>123750</v>
+      </c>
+      <c r="F28" s="22" t="n">
+        <f aca="false">Podsumowanie!E81</f>
+        <v>123750</v>
+      </c>
+      <c r="G28" s="22" t="n">
+        <f aca="false">Podsumowanie!E82</f>
+        <v>99000</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B29" s="22" t="n">
+        <f aca="false">Podsumowanie!D83</f>
+        <v>0</v>
+      </c>
+      <c r="C29" s="22" t="n">
+        <f aca="false">Podsumowanie!D84</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="22" t="n">
+        <f aca="false">Podsumowanie!D85</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="22" t="n">
+        <f aca="false">Podsumowanie!E83</f>
+        <v>44640</v>
+      </c>
+      <c r="F29" s="22" t="n">
+        <f aca="false">Podsumowanie!E84</f>
+        <v>44640</v>
+      </c>
+      <c r="G29" s="22" t="n">
+        <f aca="false">Podsumowanie!E85</f>
+        <v>35712</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B30" s="22" t="n">
+        <f aca="false">Podsumowanie!D86</f>
+        <v>0</v>
+      </c>
+      <c r="C30" s="22" t="n">
+        <f aca="false">Podsumowanie!D87</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="22" t="n">
+        <f aca="false">Podsumowanie!D88</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="22" t="n">
+        <f aca="false">Podsumowanie!E86</f>
+        <v>123750</v>
+      </c>
+      <c r="F30" s="22" t="n">
+        <f aca="false">Podsumowanie!E87</f>
+        <v>123750</v>
+      </c>
+      <c r="G30" s="22" t="n">
+        <f aca="false">Podsumowanie!E88</f>
+        <v>99000</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B31" s="22" t="n">
+        <f aca="false">Podsumowanie!D89</f>
+        <v>0</v>
+      </c>
+      <c r="C31" s="22" t="n">
+        <f aca="false">Podsumowanie!D90</f>
+        <v>0</v>
+      </c>
+      <c r="D31" s="22" t="n">
+        <f aca="false">Podsumowanie!D91</f>
+        <v>0</v>
+      </c>
+      <c r="E31" s="22" t="n">
+        <f aca="false">Podsumowanie!E89</f>
+        <v>80790</v>
+      </c>
+      <c r="F31" s="22" t="n">
+        <f aca="false">Podsumowanie!E90</f>
+        <v>80790</v>
+      </c>
+      <c r="G31" s="22" t="n">
+        <f aca="false">Podsumowanie!E91</f>
+        <v>64632</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" s="22" t="n">
+        <f aca="false">Podsumowanie!D92</f>
+        <v>0</v>
+      </c>
+      <c r="C32" s="22" t="n">
+        <f aca="false">Podsumowanie!D93</f>
+        <v>0</v>
+      </c>
+      <c r="D32" s="22" t="n">
+        <f aca="false">Podsumowanie!D94</f>
+        <v>0</v>
+      </c>
+      <c r="E32" s="22" t="n">
+        <f aca="false">Podsumowanie!E92</f>
+        <v>4285.71</v>
+      </c>
+      <c r="F32" s="22" t="n">
+        <f aca="false">Podsumowanie!E93</f>
+        <v>4285.71</v>
+      </c>
+      <c r="G32" s="22" t="n">
+        <f aca="false">Podsumowanie!E94</f>
+        <v>3428.56</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B33" s="22" t="n">
+        <f aca="false">Podsumowanie!D95</f>
+        <v>0</v>
+      </c>
+      <c r="C33" s="22" t="n">
+        <f aca="false">Podsumowanie!D96</f>
+        <v>0</v>
+      </c>
+      <c r="D33" s="22" t="n">
+        <f aca="false">Podsumowanie!D97</f>
+        <v>0</v>
+      </c>
+      <c r="E33" s="22" t="n">
+        <f aca="false">Podsumowanie!E95</f>
+        <v>118500</v>
+      </c>
+      <c r="F33" s="22" t="n">
+        <f aca="false">Podsumowanie!E96</f>
+        <v>118500</v>
+      </c>
+      <c r="G33" s="22" t="n">
+        <f aca="false">Podsumowanie!E97</f>
+        <v>94800</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B34" s="22" t="n">
+        <f aca="false">Podsumowanie!D98</f>
+        <v>0</v>
+      </c>
+      <c r="C34" s="22" t="n">
+        <f aca="false">Podsumowanie!D99</f>
+        <v>0</v>
+      </c>
+      <c r="D34" s="22" t="n">
+        <f aca="false">Podsumowanie!D100</f>
+        <v>0</v>
+      </c>
+      <c r="E34" s="22" t="n">
+        <f aca="false">Podsumowanie!E98</f>
+        <v>698237.14</v>
+      </c>
+      <c r="F34" s="22" t="n">
+        <f aca="false">Podsumowanie!E99</f>
+        <v>698237.14</v>
+      </c>
+      <c r="G34" s="22" t="n">
+        <f aca="false">Podsumowanie!E100</f>
+        <v>418942.28</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B35" s="22" t="n">
+        <f aca="false">Podsumowanie!D101</f>
+        <v>0</v>
+      </c>
+      <c r="C35" s="22" t="n">
+        <f aca="false">Podsumowanie!D102</f>
+        <v>0</v>
+      </c>
+      <c r="D35" s="22" t="n">
+        <f aca="false">Podsumowanie!D103</f>
+        <v>0</v>
+      </c>
+      <c r="E35" s="22" t="n">
+        <f aca="false">Podsumowanie!E101</f>
+        <v>221600</v>
+      </c>
+      <c r="F35" s="22" t="n">
+        <f aca="false">Podsumowanie!E102</f>
+        <v>221600</v>
+      </c>
+      <c r="G35" s="22" t="n">
+        <f aca="false">Podsumowanie!E103</f>
+        <v>132960</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B36" s="22" t="n">
+        <f aca="false">Podsumowanie!D104</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="22" t="n">
+        <f aca="false">Podsumowanie!D105</f>
+        <v>0</v>
+      </c>
+      <c r="D36" s="22" t="n">
+        <f aca="false">Podsumowanie!D106</f>
+        <v>0</v>
+      </c>
+      <c r="E36" s="22" t="n">
+        <f aca="false">Podsumowanie!E104</f>
+        <v>37720</v>
+      </c>
+      <c r="F36" s="22" t="n">
+        <f aca="false">Podsumowanie!E105</f>
+        <v>37720</v>
+      </c>
+      <c r="G36" s="22" t="n">
+        <f aca="false">Podsumowanie!E106</f>
+        <v>22632</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B37" s="22" t="n">
+        <f aca="false">Podsumowanie!D107</f>
+        <v>0</v>
+      </c>
+      <c r="C37" s="22" t="n">
+        <f aca="false">Podsumowanie!D108</f>
+        <v>0</v>
+      </c>
+      <c r="D37" s="22" t="n">
+        <f aca="false">Podsumowanie!D109</f>
+        <v>0</v>
+      </c>
+      <c r="E37" s="22" t="n">
+        <f aca="false">Podsumowanie!E107</f>
+        <v>108440</v>
+      </c>
+      <c r="F37" s="22" t="n">
+        <f aca="false">Podsumowanie!E108</f>
+        <v>108440</v>
+      </c>
+      <c r="G37" s="22" t="n">
+        <f aca="false">Podsumowanie!E109</f>
+        <v>65064</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B38" s="22" t="n">
+        <f aca="false">Podsumowanie!D110</f>
+        <v>0</v>
+      </c>
+      <c r="C38" s="22" t="n">
+        <f aca="false">Podsumowanie!D111</f>
+        <v>0</v>
+      </c>
+      <c r="D38" s="22" t="n">
+        <f aca="false">Podsumowanie!D112</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="22" t="n">
+        <f aca="false">Podsumowanie!E110</f>
+        <v>82500</v>
+      </c>
+      <c r="F38" s="22" t="n">
+        <f aca="false">Podsumowanie!E111</f>
+        <v>82500</v>
+      </c>
+      <c r="G38" s="22" t="n">
+        <f aca="false">Podsumowanie!E112</f>
+        <v>49500</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B39" s="22" t="n">
+        <f aca="false">Podsumowanie!D113</f>
+        <v>0</v>
+      </c>
+      <c r="C39" s="22" t="n">
+        <f aca="false">Podsumowanie!D114</f>
+        <v>0</v>
+      </c>
+      <c r="D39" s="22" t="n">
+        <f aca="false">Podsumowanie!D115</f>
+        <v>0</v>
+      </c>
+      <c r="E39" s="22" t="n">
+        <f aca="false">Podsumowanie!E113</f>
+        <v>29760</v>
+      </c>
+      <c r="F39" s="22" t="n">
+        <f aca="false">Podsumowanie!E114</f>
+        <v>29760</v>
+      </c>
+      <c r="G39" s="22" t="n">
+        <f aca="false">Podsumowanie!E115</f>
+        <v>17856</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B40" s="22" t="n">
+        <f aca="false">Podsumowanie!D116</f>
+        <v>0</v>
+      </c>
+      <c r="C40" s="22" t="n">
+        <f aca="false">Podsumowanie!D117</f>
+        <v>0</v>
+      </c>
+      <c r="D40" s="22" t="n">
+        <f aca="false">Podsumowanie!D118</f>
+        <v>0</v>
+      </c>
+      <c r="E40" s="22" t="n">
+        <f aca="false">Podsumowanie!E116</f>
+        <v>82500</v>
+      </c>
+      <c r="F40" s="22" t="n">
+        <f aca="false">Podsumowanie!E117</f>
+        <v>82500</v>
+      </c>
+      <c r="G40" s="22" t="n">
+        <f aca="false">Podsumowanie!E118</f>
+        <v>49500</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B41" s="22" t="n">
+        <f aca="false">Podsumowanie!D119</f>
+        <v>0</v>
+      </c>
+      <c r="C41" s="22" t="n">
+        <f aca="false">Podsumowanie!D120</f>
+        <v>0</v>
+      </c>
+      <c r="D41" s="22" t="n">
+        <f aca="false">Podsumowanie!D121</f>
+        <v>0</v>
+      </c>
+      <c r="E41" s="22" t="n">
+        <f aca="false">Podsumowanie!E119</f>
+        <v>2857.14</v>
+      </c>
+      <c r="F41" s="22" t="n">
+        <f aca="false">Podsumowanie!E120</f>
+        <v>2857.14</v>
+      </c>
+      <c r="G41" s="22" t="n">
+        <f aca="false">Podsumowanie!E121</f>
+        <v>1714.28</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B42" s="22" t="n">
+        <f aca="false">Podsumowanie!D122</f>
+        <v>0</v>
+      </c>
+      <c r="C42" s="22" t="n">
+        <f aca="false">Podsumowanie!D123</f>
+        <v>0</v>
+      </c>
+      <c r="D42" s="22" t="n">
+        <f aca="false">Podsumowanie!D124</f>
+        <v>0</v>
+      </c>
+      <c r="E42" s="22" t="n">
+        <f aca="false">Podsumowanie!E122</f>
+        <v>79000</v>
+      </c>
+      <c r="F42" s="22" t="n">
+        <f aca="false">Podsumowanie!E123</f>
+        <v>79000</v>
+      </c>
+      <c r="G42" s="22" t="n">
+        <f aca="false">Podsumowanie!E124</f>
+        <v>47400</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B43" s="22" t="n">
+        <f aca="false">Podsumowanie!D125</f>
+        <v>0</v>
+      </c>
+      <c r="C43" s="22" t="n">
+        <f aca="false">Podsumowanie!D126</f>
+        <v>0</v>
+      </c>
+      <c r="D43" s="22" t="n">
+        <f aca="false">Podsumowanie!D127</f>
+        <v>0</v>
+      </c>
+      <c r="E43" s="22" t="n">
+        <f aca="false">Podsumowanie!E125</f>
+        <v>53860</v>
+      </c>
+      <c r="F43" s="22" t="n">
+        <f aca="false">Podsumowanie!E126</f>
+        <v>53860</v>
+      </c>
+      <c r="G43" s="22" t="n">
+        <f aca="false">Podsumowanie!E127</f>
+        <v>32316</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <autoFilter ref="A2:G43">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+  </autoFilter>
+  <mergeCells count="2">
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="E1:G1"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Compute licence dofinansowanie (G21) as 80% of remaining amount; adjust Z3 correction
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3QuwGR9tgiXrdWSSrWcuu
</commit_message>
<xml_diff>
--- a/Wniosek_o_platnosc_str26-34.xlsx
+++ b/Wniosek_o_platnosc_str26-34.xlsx
@@ -489,7 +489,7 @@
     <t xml:space="preserve">Licencje: mnożnik ogółem / kwalifikowalne (VAT 23%)</t>
   </si>
   <si>
-    <t xml:space="preserve">Licencje: dofinansowanie reszty (zł) – przyjęto 0</t>
+    <t xml:space="preserve">Licencje: dofinansowanie reszty = reszta kwalifikowalna × intensywność Z2</t>
   </si>
   <si>
     <t xml:space="preserve">CEL: wydatki kwalifikowalne razem (budżet pierwotny)</t>
@@ -579,7 +579,7 @@
     <t xml:space="preserve">3. Z1 i Z2 w nowym budżecie = wydatki narastająco (ogółem, kwalifikowalne, dofinansowanie) per pozycja. Poz. 2.1 (Ekspert AI, Z2): przyjęto 332 400 zł kwalifikowalnych / 265 920 zł dofinansowania (PARP wstrzymał wypłatę, budżet nie jest tracony).</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Licencje (Z2): wykonanie 0, więc całość uwalnia środki. Na licencjach zostaje tylko reszta, która domyka sumę kwalifikowalnych do celu (C14); dofinansowanie tej reszty = C9 (0 zł).</t>
+    <t xml:space="preserve">4. Licencje (Z2): wykonanie 0, więc całość uwalnia środki. Na licencjach zostaje tylko reszta, która domyka sumę kwalifikowalnych do celu (C14); dofinansowanie tej reszty = reszta × 80% (C9); nadwyżkę dofinansowania koryguje się w Z3 (punkt 11).</t>
   </si>
   <si>
     <t xml:space="preserve">5. Z3 i Z4 = prognoza: stawka × etat × miesiące (arkusz „plan etatów”). Z3 nie jest przycinane.</t>
@@ -1270,11 +1270,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -12086,14 +12086,15 @@
         <v>152</v>
       </c>
       <c r="C9" s="44" t="n">
-        <v>0</v>
+        <f aca="false">ROUND(C14*C5,2)</f>
+        <v>3393.53</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="41" t="s">
         <v>153</v>
       </c>
-      <c r="C10" s="44" t="n">
+      <c r="C10" s="45" t="n">
         <v>4843115.61</v>
       </c>
     </row>
@@ -12101,7 +12102,7 @@
       <c r="A11" s="41" t="s">
         <v>154</v>
       </c>
-      <c r="C11" s="44" t="n">
+      <c r="C11" s="45" t="n">
         <v>3699933.17</v>
       </c>
     </row>
@@ -12109,7 +12110,7 @@
       <c r="A12" s="41" t="s">
         <v>155</v>
       </c>
-      <c r="C12" s="45" t="n">
+      <c r="C12" s="44" t="n">
         <f aca="false">Podsumowanie!E146</f>
         <v>3874492.49</v>
       </c>
@@ -12118,7 +12119,7 @@
       <c r="A13" s="41" t="s">
         <v>156</v>
       </c>
-      <c r="C13" s="45" t="n">
+      <c r="C13" s="44" t="n">
         <f aca="false">Podsumowanie!E147</f>
         <v>2959946.54</v>
       </c>
@@ -12136,7 +12137,7 @@
       <c r="A15" s="41" t="s">
         <v>158</v>
       </c>
-      <c r="C15" s="45" t="n">
+      <c r="C15" s="44" t="n">
         <f aca="false">'nowy format 2'!F24</f>
         <v>1389999.28</v>
       </c>
@@ -12145,7 +12146,7 @@
       <c r="A16" s="41" t="s">
         <v>159</v>
       </c>
-      <c r="C16" s="45" t="n">
+      <c r="C16" s="44" t="n">
         <f aca="false">C15*C6</f>
         <v>1111999.424</v>
       </c>
@@ -12154,18 +12155,18 @@
       <c r="A17" s="41" t="s">
         <v>160</v>
       </c>
-      <c r="C17" s="45" t="n">
+      <c r="C17" s="44" t="n">
         <f aca="false">'nowy format 2'!G4+'nowy format 2'!G5+'nowy format 2'!G6+'nowy format 2'!G7+'nowy format 2'!G8+'nowy format 2'!G9+'nowy format 2'!G10+'nowy format 2'!G11+'nowy format 2'!G12+'nowy format 2'!G14+'nowy format 2'!G15+'nowy format 2'!G16+'nowy format 2'!G17+'nowy format 2'!G18+'nowy format 2'!G19+'nowy format 2'!G20+'nowy format 2'!G21+'nowy format 2'!G22+'nowy format 2'!G23+'nowy format 2'!F34*C7</f>
-        <v>1851389.614</v>
+        <v>1854783.144</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="41" t="s">
         <v>161</v>
       </c>
-      <c r="C18" s="45" t="n">
+      <c r="C18" s="44" t="n">
         <f aca="false">C16+C17-C13</f>
-        <v>3442.49799999967</v>
+        <v>6836.02799999993</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12174,14 +12175,14 @@
       </c>
       <c r="C19" s="47" t="n">
         <f aca="false">C18/C15</f>
-        <v>0.00247661854903959</v>
+        <v>0.00491800830285317</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
         <v>163</v>
       </c>
-      <c r="C20" s="45" t="n">
+      <c r="C20" s="44" t="n">
         <f aca="false">zmiana!C9*('plan etatów'!E7-'plan etatów'!D7+1)</f>
         <v>34180</v>
       </c>
@@ -12190,7 +12191,7 @@
       <c r="A21" s="41" t="s">
         <v>164</v>
       </c>
-      <c r="C21" s="45" t="n">
+      <c r="C21" s="44" t="n">
         <f aca="false">C14-C20</f>
         <v>-29938.09</v>
       </c>
@@ -38362,7 +38363,7 @@
       </c>
       <c r="C166" s="49" t="n">
         <f aca="false">SUM(D166:Z166)</f>
-        <v>0</v>
+        <v>3393.53</v>
       </c>
       <c r="D166" s="49" t="n">
         <f aca="false">IF(D$4='plan etatów'!$E$5,założenia!$C$9,0)</f>
@@ -38406,7 +38407,7 @@
       </c>
       <c r="N166" s="49" t="n">
         <f aca="false">IF(N$4='plan etatów'!$E$5,założenia!$C$9,0)</f>
-        <v>0</v>
+        <v>3393.53</v>
       </c>
       <c r="O166" s="49" t="n">
         <f aca="false">IF(O$4='plan etatów'!$E$5,założenia!$C$9,0)</f>
@@ -38674,7 +38675,7 @@
       </c>
       <c r="C169" s="49" t="n">
         <f aca="false">SUM(D169:Z169)</f>
-        <v>353462.362659066</v>
+        <v>352380.338720176</v>
       </c>
       <c r="D169" s="49" t="n">
         <f aca="false">D75*(założenia!$C$6-założenia!$C$19)</f>
@@ -38722,35 +38723,35 @@
       </c>
       <c r="O169" s="49" t="n">
         <f aca="false">O75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44182.7953323832</v>
+        <v>44047.5423400219</v>
       </c>
       <c r="P169" s="49" t="n">
         <f aca="false">P75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44182.7953323832</v>
+        <v>44047.5423400219</v>
       </c>
       <c r="Q169" s="49" t="n">
         <f aca="false">Q75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44182.7953323832</v>
+        <v>44047.5423400219</v>
       </c>
       <c r="R169" s="49" t="n">
         <f aca="false">R75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44182.7953323832</v>
+        <v>44047.5423400219</v>
       </c>
       <c r="S169" s="49" t="n">
         <f aca="false">S75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44182.7953323832</v>
+        <v>44047.5423400219</v>
       </c>
       <c r="T169" s="49" t="n">
         <f aca="false">T75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44182.7953323832</v>
+        <v>44047.5423400219</v>
       </c>
       <c r="U169" s="49" t="n">
         <f aca="false">U75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44182.7953323832</v>
+        <v>44047.5423400219</v>
       </c>
       <c r="V169" s="49" t="n">
         <f aca="false">V75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44182.7953323832</v>
+        <v>44047.5423400219</v>
       </c>
       <c r="W169" s="49" t="n">
         <f aca="false">W75*(założenia!$C$6-założenia!$C$19)</f>
@@ -38778,7 +38779,7 @@
       </c>
       <c r="C170" s="49" t="n">
         <f aca="false">SUM(D170:Z170)</f>
-        <v>120330.327793321</v>
+        <v>119961.970907266</v>
       </c>
       <c r="D170" s="49" t="n">
         <f aca="false">D76*(założenia!$C$6-założenia!$C$19)</f>
@@ -38826,35 +38827,35 @@
       </c>
       <c r="O170" s="49" t="n">
         <f aca="false">O76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15041.2909741651</v>
+        <v>14995.2463634082</v>
       </c>
       <c r="P170" s="49" t="n">
         <f aca="false">P76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15041.2909741651</v>
+        <v>14995.2463634082</v>
       </c>
       <c r="Q170" s="49" t="n">
         <f aca="false">Q76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15041.2909741651</v>
+        <v>14995.2463634082</v>
       </c>
       <c r="R170" s="49" t="n">
         <f aca="false">R76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15041.2909741651</v>
+        <v>14995.2463634082</v>
       </c>
       <c r="S170" s="49" t="n">
         <f aca="false">S76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15041.2909741651</v>
+        <v>14995.2463634082</v>
       </c>
       <c r="T170" s="49" t="n">
         <f aca="false">T76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15041.2909741651</v>
+        <v>14995.2463634082</v>
       </c>
       <c r="U170" s="49" t="n">
         <f aca="false">U76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15041.2909741651</v>
+        <v>14995.2463634082</v>
       </c>
       <c r="V170" s="49" t="n">
         <f aca="false">V76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15041.2909741651</v>
+        <v>14995.2463634082</v>
       </c>
       <c r="W170" s="49" t="n">
         <f aca="false">W76*(założenia!$C$6-założenia!$C$19)</f>
@@ -38882,7 +38883,7 @@
       </c>
       <c r="C171" s="49" t="n">
         <f aca="false">SUM(D171:Z171)</f>
-        <v>162156.441533517</v>
+        <v>161660.045961822</v>
       </c>
       <c r="D171" s="49" t="n">
         <f aca="false">D77*(założenia!$C$6-założenia!$C$19)</f>
@@ -38930,35 +38931,35 @@
       </c>
       <c r="O171" s="49" t="n">
         <f aca="false">O77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16215.6441533517</v>
+        <v>16166.0045961822</v>
       </c>
       <c r="P171" s="49" t="n">
         <f aca="false">P77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16215.6441533517</v>
+        <v>16166.0045961822</v>
       </c>
       <c r="Q171" s="49" t="n">
         <f aca="false">Q77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>21620.8588711355</v>
+        <v>21554.6727949097</v>
       </c>
       <c r="R171" s="49" t="n">
         <f aca="false">R77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>21620.8588711355</v>
+        <v>21554.6727949097</v>
       </c>
       <c r="S171" s="49" t="n">
         <f aca="false">S77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>21620.8588711355</v>
+        <v>21554.6727949097</v>
       </c>
       <c r="T171" s="49" t="n">
         <f aca="false">T77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>21620.8588711355</v>
+        <v>21554.6727949097</v>
       </c>
       <c r="U171" s="49" t="n">
         <f aca="false">U77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>21620.8588711355</v>
+        <v>21554.6727949097</v>
       </c>
       <c r="V171" s="49" t="n">
         <f aca="false">V77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>21620.8588711355</v>
+        <v>21554.6727949097</v>
       </c>
       <c r="W171" s="49" t="n">
         <f aca="false">W77*(założenia!$C$6-założenia!$C$19)</f>
@@ -38986,7 +38987,7 @@
       </c>
       <c r="C172" s="49" t="n">
         <f aca="false">SUM(D172:Z172)</f>
-        <v>131591.357939408</v>
+        <v>131188.528630029</v>
       </c>
       <c r="D172" s="49" t="n">
         <f aca="false">D78*(założenia!$C$6-założenia!$C$19)</f>
@@ -39034,35 +39035,35 @@
       </c>
       <c r="O172" s="49" t="n">
         <f aca="false">O78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="P172" s="49" t="n">
         <f aca="false">P78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="Q172" s="49" t="n">
         <f aca="false">Q78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="R172" s="49" t="n">
         <f aca="false">R78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="S172" s="49" t="n">
         <f aca="false">S78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="T172" s="49" t="n">
         <f aca="false">T78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="U172" s="49" t="n">
         <f aca="false">U78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="V172" s="49" t="n">
         <f aca="false">V78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="W172" s="49" t="n">
         <f aca="false">W78*(założenia!$C$6-założenia!$C$19)</f>
@@ -39090,7 +39091,7 @@
       </c>
       <c r="C173" s="49" t="n">
         <f aca="false">SUM(D173:Z173)</f>
-        <v>47468.5916639612</v>
+        <v>47323.2801458142</v>
       </c>
       <c r="D173" s="49" t="n">
         <f aca="false">D79*(założenia!$C$6-założenia!$C$19)</f>
@@ -39138,35 +39139,35 @@
       </c>
       <c r="O173" s="49" t="n">
         <f aca="false">O79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5933.57395799515</v>
+        <v>5915.41001822677</v>
       </c>
       <c r="P173" s="49" t="n">
         <f aca="false">P79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5933.57395799515</v>
+        <v>5915.41001822677</v>
       </c>
       <c r="Q173" s="49" t="n">
         <f aca="false">Q79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5933.57395799515</v>
+        <v>5915.41001822677</v>
       </c>
       <c r="R173" s="49" t="n">
         <f aca="false">R79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5933.57395799515</v>
+        <v>5915.41001822677</v>
       </c>
       <c r="S173" s="49" t="n">
         <f aca="false">S79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5933.57395799515</v>
+        <v>5915.41001822677</v>
       </c>
       <c r="T173" s="49" t="n">
         <f aca="false">T79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5933.57395799515</v>
+        <v>5915.41001822677</v>
       </c>
       <c r="U173" s="49" t="n">
         <f aca="false">U79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5933.57395799515</v>
+        <v>5915.41001822677</v>
       </c>
       <c r="V173" s="49" t="n">
         <f aca="false">V79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5933.57395799515</v>
+        <v>5915.41001822677</v>
       </c>
       <c r="W173" s="49" t="n">
         <f aca="false">W79*(założenia!$C$6-założenia!$C$19)</f>
@@ -39194,7 +39195,7 @@
       </c>
       <c r="C174" s="49" t="n">
         <f aca="false">SUM(D174:Z174)</f>
-        <v>131591.357939408</v>
+        <v>131188.528630029</v>
       </c>
       <c r="D174" s="49" t="n">
         <f aca="false">D80*(założenia!$C$6-założenia!$C$19)</f>
@@ -39242,35 +39243,35 @@
       </c>
       <c r="O174" s="49" t="n">
         <f aca="false">O80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="P174" s="49" t="n">
         <f aca="false">P80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="Q174" s="49" t="n">
         <f aca="false">Q80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="R174" s="49" t="n">
         <f aca="false">R80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="S174" s="49" t="n">
         <f aca="false">S80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="T174" s="49" t="n">
         <f aca="false">T80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="U174" s="49" t="n">
         <f aca="false">U80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="V174" s="49" t="n">
         <f aca="false">V80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16448.9197424261</v>
+        <v>16398.5660787537</v>
       </c>
       <c r="W174" s="49" t="n">
         <f aca="false">W80*(założenia!$C$6-założenia!$C$19)</f>
@@ -39298,7 +39299,7 @@
       </c>
       <c r="C175" s="49" t="n">
         <f aca="false">SUM(D175:Z175)</f>
-        <v>31390.5202939098</v>
+        <v>31294.4271931997</v>
       </c>
       <c r="D175" s="49" t="n">
         <f aca="false">D81*(założenia!$C$6-założenia!$C$19)</f>
@@ -39346,35 +39347,35 @@
       </c>
       <c r="O175" s="49" t="n">
         <f aca="false">O81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3923.81503673873</v>
+        <v>3911.80339914996</v>
       </c>
       <c r="P175" s="49" t="n">
         <f aca="false">P81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3923.81503673873</v>
+        <v>3911.80339914996</v>
       </c>
       <c r="Q175" s="49" t="n">
         <f aca="false">Q81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3923.81503673873</v>
+        <v>3911.80339914996</v>
       </c>
       <c r="R175" s="49" t="n">
         <f aca="false">R81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3923.81503673873</v>
+        <v>3911.80339914996</v>
       </c>
       <c r="S175" s="49" t="n">
         <f aca="false">S81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3923.81503673873</v>
+        <v>3911.80339914996</v>
       </c>
       <c r="T175" s="49" t="n">
         <f aca="false">T81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3923.81503673873</v>
+        <v>3911.80339914996</v>
       </c>
       <c r="U175" s="49" t="n">
         <f aca="false">U81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3923.81503673873</v>
+        <v>3911.80339914996</v>
       </c>
       <c r="V175" s="49" t="n">
         <f aca="false">V81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3923.81503673873</v>
+        <v>3911.80339914996</v>
       </c>
       <c r="W175" s="49" t="n">
         <f aca="false">W81*(założenia!$C$6-założenia!$C$19)</f>
@@ -39402,7 +39403,7 @@
       </c>
       <c r="C176" s="49" t="n">
         <f aca="false">SUM(D176:Z176)</f>
-        <v>4557.27190815759</v>
+        <v>4543.32112351517</v>
       </c>
       <c r="D176" s="49" t="n">
         <f aca="false">D82*(założenia!$C$6-założenia!$C$19)</f>
@@ -39450,35 +39451,35 @@
       </c>
       <c r="O176" s="49" t="n">
         <f aca="false">O82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>569.658988519699</v>
+        <v>567.915140439397</v>
       </c>
       <c r="P176" s="49" t="n">
         <f aca="false">P82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>569.658988519699</v>
+        <v>567.915140439397</v>
       </c>
       <c r="Q176" s="49" t="n">
         <f aca="false">Q82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>569.658988519699</v>
+        <v>567.915140439397</v>
       </c>
       <c r="R176" s="49" t="n">
         <f aca="false">R82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>569.658988519699</v>
+        <v>567.915140439397</v>
       </c>
       <c r="S176" s="49" t="n">
         <f aca="false">S82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>569.658988519699</v>
+        <v>567.915140439397</v>
       </c>
       <c r="T176" s="49" t="n">
         <f aca="false">T82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>569.658988519699</v>
+        <v>567.915140439397</v>
       </c>
       <c r="U176" s="49" t="n">
         <f aca="false">U82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>569.658988519699</v>
+        <v>567.915140439397</v>
       </c>
       <c r="V176" s="49" t="n">
         <f aca="false">V82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>569.658988519699</v>
+        <v>567.915140439397</v>
       </c>
       <c r="W176" s="49" t="n">
         <f aca="false">W82*(założenia!$C$6-założenia!$C$19)</f>
@@ -39506,7 +39507,7 @@
       </c>
       <c r="C177" s="49" t="n">
         <f aca="false">SUM(D177:Z177)</f>
-        <v>126008.694269252</v>
+        <v>125622.954688149</v>
       </c>
       <c r="D177" s="49" t="n">
         <f aca="false">D83*(założenia!$C$6-założenia!$C$19)</f>
@@ -39554,35 +39555,35 @@
       </c>
       <c r="O177" s="49" t="n">
         <f aca="false">O83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15751.0867836565</v>
+        <v>15702.8693360187</v>
       </c>
       <c r="P177" s="49" t="n">
         <f aca="false">P83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15751.0867836565</v>
+        <v>15702.8693360187</v>
       </c>
       <c r="Q177" s="49" t="n">
         <f aca="false">Q83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15751.0867836565</v>
+        <v>15702.8693360187</v>
       </c>
       <c r="R177" s="49" t="n">
         <f aca="false">R83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15751.0867836565</v>
+        <v>15702.8693360187</v>
       </c>
       <c r="S177" s="49" t="n">
         <f aca="false">S83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15751.0867836565</v>
+        <v>15702.8693360187</v>
       </c>
       <c r="T177" s="49" t="n">
         <f aca="false">T83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15751.0867836565</v>
+        <v>15702.8693360187</v>
       </c>
       <c r="U177" s="49" t="n">
         <f aca="false">U83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15751.0867836565</v>
+        <v>15702.8693360187</v>
       </c>
       <c r="V177" s="49" t="n">
         <f aca="false">V83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15751.0867836565</v>
+        <v>15702.8693360187</v>
       </c>
       <c r="W177" s="49" t="n">
         <f aca="false">W83*(założenia!$C$6-założenia!$C$19)</f>
@@ -40650,7 +40651,7 @@
       </c>
       <c r="C188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,C$150:C$186)</f>
-        <v>807015.43</v>
+        <v>810408.96</v>
       </c>
       <c r="D188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,D$150:D$186)</f>
@@ -40694,7 +40695,7 @@
       </c>
       <c r="N188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,N$150:N$186)</f>
-        <v>134502.571666667</v>
+        <v>137896.101666667</v>
       </c>
       <c r="O188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,O$150:O$186)</f>
@@ -40754,7 +40755,7 @@
       </c>
       <c r="C189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,C$150:C$186)</f>
-        <v>1108556.926</v>
+        <v>1105163.396</v>
       </c>
       <c r="D189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,D$150:D$186)</f>
@@ -40802,35 +40803,35 @@
       </c>
       <c r="O189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,O$150:O$186)</f>
-        <v>134515.704711662</v>
+        <v>134103.923350954</v>
       </c>
       <c r="P189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,P$150:P$186)</f>
-        <v>134515.704711662</v>
+        <v>134103.923350954</v>
       </c>
       <c r="Q189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,Q$150:Q$186)</f>
-        <v>139920.919429446</v>
+        <v>139492.591549682</v>
       </c>
       <c r="R189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,R$150:R$186)</f>
-        <v>139920.919429446</v>
+        <v>139492.591549682</v>
       </c>
       <c r="S189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,S$150:S$186)</f>
-        <v>139920.919429446</v>
+        <v>139492.591549682</v>
       </c>
       <c r="T189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,T$150:T$186)</f>
-        <v>139920.919429446</v>
+        <v>139492.591549682</v>
       </c>
       <c r="U189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,U$150:U$186)</f>
-        <v>139920.919429446</v>
+        <v>139492.591549682</v>
       </c>
       <c r="V189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,V$150:V$186)</f>
-        <v>139920.919429446</v>
+        <v>139492.591549682</v>
       </c>
       <c r="W189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,W$150:W$186)</f>
@@ -41004,39 +41005,39 @@
       </c>
       <c r="N191" s="63" t="n">
         <f aca="false">SUM(N187:N190)</f>
-        <v>134502.571666667</v>
+        <v>137896.101666667</v>
       </c>
       <c r="O191" s="63" t="n">
         <f aca="false">SUM(O187:O190)</f>
-        <v>134515.704711662</v>
+        <v>134103.923350954</v>
       </c>
       <c r="P191" s="63" t="n">
         <f aca="false">SUM(P187:P190)</f>
-        <v>134515.704711662</v>
+        <v>134103.923350954</v>
       </c>
       <c r="Q191" s="63" t="n">
         <f aca="false">SUM(Q187:Q190)</f>
-        <v>139920.919429446</v>
+        <v>139492.591549682</v>
       </c>
       <c r="R191" s="63" t="n">
         <f aca="false">SUM(R187:R190)</f>
-        <v>139920.919429446</v>
+        <v>139492.591549682</v>
       </c>
       <c r="S191" s="63" t="n">
         <f aca="false">SUM(S187:S190)</f>
-        <v>139920.919429446</v>
+        <v>139492.591549682</v>
       </c>
       <c r="T191" s="63" t="n">
         <f aca="false">SUM(T187:T190)</f>
-        <v>139920.919429446</v>
+        <v>139492.591549682</v>
       </c>
       <c r="U191" s="63" t="n">
         <f aca="false">SUM(U187:U190)</f>
-        <v>139920.919429446</v>
+        <v>139492.591549682</v>
       </c>
       <c r="V191" s="63" t="n">
         <f aca="false">SUM(V187:V190)</f>
-        <v>139920.919429446</v>
+        <v>139492.591549682</v>
       </c>
       <c r="W191" s="63" t="n">
         <f aca="false">SUM(W187:W190)</f>
@@ -41208,39 +41209,39 @@
       </c>
       <c r="N193" s="63" t="n">
         <f aca="false">N191+N192</f>
-        <v>167423.422359367</v>
+        <v>170816.952359367</v>
       </c>
       <c r="O193" s="63" t="n">
         <f aca="false">O191+O192</f>
-        <v>166729.257064791</v>
+        <v>166317.475704083</v>
       </c>
       <c r="P193" s="63" t="n">
         <f aca="false">P191+P192</f>
-        <v>166729.257064791</v>
+        <v>166317.475704083</v>
       </c>
       <c r="Q193" s="63" t="n">
         <f aca="false">Q191+Q192</f>
-        <v>173428.901809644</v>
+        <v>173000.57392988</v>
       </c>
       <c r="R193" s="63" t="n">
         <f aca="false">R191+R192</f>
-        <v>173428.901809644</v>
+        <v>173000.57392988</v>
       </c>
       <c r="S193" s="63" t="n">
         <f aca="false">S191+S192</f>
-        <v>173428.901809644</v>
+        <v>173000.57392988</v>
       </c>
       <c r="T193" s="63" t="n">
         <f aca="false">T191+T192</f>
-        <v>173428.901809644</v>
+        <v>173000.57392988</v>
       </c>
       <c r="U193" s="63" t="n">
         <f aca="false">U191+U192</f>
-        <v>173428.901809644</v>
+        <v>173000.57392988</v>
       </c>
       <c r="V193" s="63" t="n">
         <f aca="false">V191+V192</f>
-        <v>173428.901809644</v>
+        <v>173000.57392988</v>
       </c>
       <c r="W193" s="63" t="n">
         <f aca="false">W191+W192</f>
@@ -41307,35 +41308,35 @@
       </c>
       <c r="N194" s="63" t="n">
         <f aca="false">M194+N193</f>
-        <v>1800639.15314555</v>
+        <v>1804032.68314555</v>
       </c>
       <c r="O194" s="63" t="n">
         <f aca="false">N194+O193</f>
-        <v>1967368.41021034</v>
+        <v>1970350.15884963</v>
       </c>
       <c r="P194" s="63" t="n">
         <f aca="false">O194+P193</f>
-        <v>2134097.66727513</v>
+        <v>2136667.63455372</v>
       </c>
       <c r="Q194" s="63" t="n">
         <f aca="false">P194+Q193</f>
-        <v>2307526.56908478</v>
+        <v>2309668.2084836</v>
       </c>
       <c r="R194" s="63" t="n">
         <f aca="false">Q194+R193</f>
-        <v>2480955.47089442</v>
+        <v>2482668.78241348</v>
       </c>
       <c r="S194" s="63" t="n">
         <f aca="false">R194+S193</f>
-        <v>2654384.37270407</v>
+        <v>2655669.35634336</v>
       </c>
       <c r="T194" s="63" t="n">
         <f aca="false">S194+T193</f>
-        <v>2827813.27451371</v>
+        <v>2828669.93027324</v>
       </c>
       <c r="U194" s="63" t="n">
         <f aca="false">T194+U193</f>
-        <v>3001242.17632335</v>
+        <v>3001670.50420312</v>
       </c>
       <c r="V194" s="63" t="n">
         <f aca="false">U194+V193</f>
@@ -42073,7 +42074,7 @@
       </c>
       <c r="G13" s="71" t="n">
         <f aca="false">SUM(G14:G23)</f>
-        <v>807015.43</v>
+        <v>810408.96</v>
       </c>
       <c r="H13" s="63"/>
       <c r="I13" s="71" t="n">
@@ -42098,7 +42099,7 @@
       </c>
       <c r="N13" s="71" t="n">
         <f aca="false">G13-K13</f>
-        <v>-156133.13</v>
+        <v>-152739.6</v>
       </c>
       <c r="O13" s="40"/>
       <c r="P13" s="70" t="str">
@@ -42545,7 +42546,7 @@
       </c>
       <c r="G21" s="74" t="n">
         <f aca="false">założenia!$C$9</f>
-        <v>0</v>
+        <v>3393.53</v>
       </c>
       <c r="H21" s="49"/>
       <c r="I21" s="73" t="n">
@@ -42570,7 +42571,7 @@
       </c>
       <c r="N21" s="73" t="n">
         <f aca="false">G21-K21</f>
-        <v>-80000</v>
+        <v>-76606.47</v>
       </c>
       <c r="O21" s="41"/>
       <c r="P21" s="72" t="str">
@@ -42722,7 +42723,7 @@
       </c>
       <c r="G24" s="71" t="n">
         <f aca="false">SUM(G25:G33)</f>
-        <v>1108556.93</v>
+        <v>1105163.4</v>
       </c>
       <c r="H24" s="63"/>
       <c r="I24" s="71" t="n">
@@ -42747,7 +42748,7 @@
       </c>
       <c r="N24" s="71" t="n">
         <f aca="false">G24-K24</f>
-        <v>225408.37</v>
+        <v>222014.84</v>
       </c>
       <c r="O24" s="40"/>
       <c r="P24" s="70" t="str">
@@ -42781,7 +42782,7 @@
       </c>
       <c r="G25" s="74" t="n">
         <f aca="false">ROUND(założenia!$C$13-(G4+G5+G6+G7+G8+G9+G10+G11+G12+G14+G15+G16+G17+G18+G19+G20+G21+G22+G23+G26+G27+G28+G29+G30+G31+G32+G33+G35+G36+G37+G38+G39+G40+G41+G42+G43),2)</f>
-        <v>353462.37</v>
+        <v>352380.34</v>
       </c>
       <c r="H25" s="49"/>
       <c r="I25" s="73" t="n">
@@ -42806,7 +42807,7 @@
       </c>
       <c r="N25" s="73" t="n">
         <f aca="false">G25-K25</f>
-        <v>87542.37</v>
+        <v>86460.34</v>
       </c>
       <c r="O25" s="41"/>
       <c r="P25" s="72" t="str">
@@ -42843,7 +42844,7 @@
       </c>
       <c r="G26" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$170,2)</f>
-        <v>120330.33</v>
+        <v>119961.97</v>
       </c>
       <c r="H26" s="49"/>
       <c r="I26" s="73" t="n">
@@ -42868,7 +42869,7 @@
       </c>
       <c r="N26" s="73" t="n">
         <f aca="false">G26-K26</f>
-        <v>29802.33</v>
+        <v>29433.97</v>
       </c>
       <c r="O26" s="41"/>
       <c r="P26" s="72" t="str">
@@ -42902,7 +42903,7 @@
       </c>
       <c r="G27" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$171,2)</f>
-        <v>162156.44</v>
+        <v>161660.05</v>
       </c>
       <c r="H27" s="49"/>
       <c r="I27" s="73" t="n">
@@ -42927,7 +42928,7 @@
       </c>
       <c r="N27" s="73" t="n">
         <f aca="false">G27-K27</f>
-        <v>32028.44</v>
+        <v>31532.05</v>
       </c>
       <c r="O27" s="41"/>
       <c r="P27" s="72" t="str">
@@ -42961,7 +42962,7 @@
       </c>
       <c r="G28" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$172,2)</f>
-        <v>131591.36</v>
+        <v>131188.53</v>
       </c>
       <c r="H28" s="49"/>
       <c r="I28" s="73" t="n">
@@ -42986,7 +42987,7 @@
       </c>
       <c r="N28" s="73" t="n">
         <f aca="false">G28-K28</f>
-        <v>32591.36</v>
+        <v>32188.53</v>
       </c>
       <c r="O28" s="41"/>
       <c r="P28" s="72" t="str">
@@ -43020,7 +43021,7 @@
       </c>
       <c r="G29" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$173,2)</f>
-        <v>47468.59</v>
+        <v>47323.28</v>
       </c>
       <c r="H29" s="49"/>
       <c r="I29" s="73" t="n">
@@ -43045,7 +43046,7 @@
       </c>
       <c r="N29" s="73" t="n">
         <f aca="false">G29-K29</f>
-        <v>11756.59</v>
+        <v>11611.28</v>
       </c>
       <c r="O29" s="41"/>
       <c r="P29" s="72" t="str">
@@ -43079,7 +43080,7 @@
       </c>
       <c r="G30" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$174,2)</f>
-        <v>131591.36</v>
+        <v>131188.53</v>
       </c>
       <c r="H30" s="49"/>
       <c r="I30" s="73" t="n">
@@ -43104,7 +43105,7 @@
       </c>
       <c r="N30" s="73" t="n">
         <f aca="false">G30-K30</f>
-        <v>32591.36</v>
+        <v>32188.53</v>
       </c>
       <c r="O30" s="41"/>
       <c r="P30" s="72" t="str">
@@ -43138,7 +43139,7 @@
       </c>
       <c r="G31" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$175,2)</f>
-        <v>31390.52</v>
+        <v>31294.43</v>
       </c>
       <c r="H31" s="49"/>
       <c r="I31" s="73" t="n">
@@ -43163,7 +43164,7 @@
       </c>
       <c r="N31" s="73" t="n">
         <f aca="false">G31-K31</f>
-        <v>-33241.48</v>
+        <v>-33337.57</v>
       </c>
       <c r="O31" s="41"/>
       <c r="P31" s="72" t="str">
@@ -43197,7 +43198,7 @@
       </c>
       <c r="G32" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$176,2)</f>
-        <v>4557.27</v>
+        <v>4543.32</v>
       </c>
       <c r="H32" s="49"/>
       <c r="I32" s="73" t="n">
@@ -43222,7 +43223,7 @@
       </c>
       <c r="N32" s="73" t="n">
         <f aca="false">G32-K32</f>
-        <v>1128.71</v>
+        <v>1114.76</v>
       </c>
       <c r="O32" s="41"/>
       <c r="P32" s="72" t="str">
@@ -43256,7 +43257,7 @@
       </c>
       <c r="G33" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$177,2)</f>
-        <v>126008.69</v>
+        <v>125622.95</v>
       </c>
       <c r="H33" s="49"/>
       <c r="I33" s="73" t="n">
@@ -43281,7 +43282,7 @@
       </c>
       <c r="N33" s="73" t="n">
         <f aca="false">G33-K33</f>
-        <v>31208.69</v>
+        <v>30822.95</v>
       </c>
       <c r="O33" s="41"/>
       <c r="P33" s="72" t="str">

</xml_diff>

<commit_message>
Z3 dofinansowanie at 80%, excess absorbed in Z4; poz. 2.9 per plan
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3QuwGR9tgiXrdWSSrWcuu
</commit_message>
<xml_diff>
--- a/Wniosek_o_platnosc_str26-34.xlsx
+++ b/Wniosek_o_platnosc_str26-34.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1118" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1119" uniqueCount="267">
   <si>
     <t xml:space="preserve">Wniosek o płatność – PODSUMOWANIE (PDF str. 27–34)</t>
   </si>
@@ -507,19 +507,19 @@
     <t xml:space="preserve">Pozostaje na licencjach – kwalifikowalne (cel − wszystkie pozostałe pozycje)</t>
   </si>
   <si>
-    <t xml:space="preserve">Z3 – kwalifikowalne razem (prognoza)</t>
+    <t xml:space="preserve">Z4 – kwalifikowalne razem (prognoza)</t>
   </si>
   <si>
-    <t xml:space="preserve">Z3 – dofinansowanie przy pełnej intensywności (Z3 × intensywność)</t>
+    <t xml:space="preserve">Z3 – dofinansowanie przy pełnej intensywności (Z3 × 80%)</t>
   </si>
   <si>
-    <t xml:space="preserve">Dofinansowanie pozostałe: Z1+Z2 (wykonanie, z licencją) + Z4 (kwal. × intensywność)</t>
+    <t xml:space="preserve">Dofinansowanie pozostałe: Z1+Z2 (wykonanie, poz. 2.9 wg planu, z licencją) + Z4 przy pełnej intensywności</t>
   </si>
   <si>
-    <t xml:space="preserve">Korekta dofinansowania w Z3 potrzebna, by suma nie wzrosła (zł)</t>
+    <t xml:space="preserve">Nadwyżka dofinansowania ponad cel (do obniżenia w Z4), zł</t>
   </si>
   <si>
-    <t xml:space="preserve">Korekta intensywności Z3 (o ile obniżamy 80%)</t>
+    <t xml:space="preserve">Obniżenie intensywności Z4 (60% minus ta wartość)</t>
   </si>
   <si>
     <t xml:space="preserve">TEST: koszt wakatu grafika w Z4 (stawka × miesiące Z4), gdyby został</t>
@@ -552,7 +552,7 @@
     <t xml:space="preserve">Dofinansowanie razem = cel</t>
   </si>
   <si>
-    <t xml:space="preserve">Z1 i Z2 w nowym budżecie = wydatki narastająco (suma różnic)</t>
+    <t xml:space="preserve">Z1 i Z2 w nowym budżecie = wydatki narastająco, bez poz. 2.9 i licencji (suma różnic)</t>
   </si>
   <si>
     <t xml:space="preserve">Suma miesięcy „będzie” (K) = nowy format 2 (koszty bezpośrednie)</t>
@@ -576,7 +576,7 @@
     <t xml:space="preserve">2. Cel: wydatki kwalifikowalne razem 4 843 115,61 zł i dofinansowanie razem 3 699 933,17 zł bez zmian vs budżet pierwotny. Wartość ogółem może się zmienić (VAT licencji).</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Z1 i Z2 w nowym budżecie = wydatki narastająco (ogółem, kwalifikowalne, dofinansowanie) per pozycja. Poz. 2.1 (Ekspert AI, Z2): przyjęto 332 400 zł kwalifikowalnych / 265 920 zł dofinansowania (PARP wstrzymał wypłatę, budżet nie jest tracony).</t>
+    <t xml:space="preserve">3. Z1 i Z2 w nowym budżecie = wydatki narastająco (ogółem, kwalifikowalne, dofinansowanie) per pozycja, z wyjątkiem poz. 2.9 (amortyzacja laptopów w Z2) – bez zmian wg planu: 4 285,71 zł. Poz. 2.1 (Ekspert AI, Z2): przyjęto 332 400 zł kwalifikowalnych / 265 920 zł dofinansowania (PARP wstrzymał wypłatę, budżet nie jest tracony).</t>
   </si>
   <si>
     <t xml:space="preserve">4. Licencje (Z2): wykonanie 0, więc całość uwalnia środki. Na licencjach zostaje tylko reszta, która domyka sumę kwalifikowalnych do celu (C14); dofinansowanie tej reszty = reszta × 80% (C9); nadwyżkę dofinansowania koryguje się w Z3 (punkt 11).</t>
@@ -600,10 +600,13 @@
     <t xml:space="preserve">10. Amortyzacja laptopów: 714,29 zł/mies.; wydłużenie Z3 do 8 m-cy zwiększa amortyzację Z3 (5 714,29 zł). Z4 bez zmian.</t>
   </si>
   <si>
-    <t xml:space="preserve">11. Dofinansowanie: intensywność 80% w Z1–Z3 i 60% w Z4 (jak w PDF). Ponieważ środki z wakatu w Z4 (60%) trafiają do Z3 (80%), suma dofinansowania wzrosłaby – dlatego dofinansowanie Z3 obniżono o kwotę z C18 (równomiernie, ułamek C19), aby suma dofinansowania nie zmieniła się. Własny wkład w Z3 rośnie o tę kwotę.</t>
+    <t xml:space="preserve">11. Dofinansowanie: Z3 dokładnie 80% kosztów kwalifikowalnych (poz. 3.1–3.9), Z1 i Z2 jak wykonanie. Suma dofinansowania nie może przekroczyć 3 699 933,17 zł, a środki z wakatu w Z4 (60%) trafiają do Z3 (80%), więc nadwyżkę z C18 odjęto od dofinansowania Z4 (równomiernie, intensywność Z4 spada o C19). Własny wkład w Z4 rośnie o tę kwotę. Alternatywa: obniżyć dofinansowanie w innym miejscu (np. koszty pośrednie).</t>
   </si>
   <si>
     <t xml:space="preserve">12. Koszty pośrednie: 25% kwalifikowalnych kosztów bezpośrednich – bez zmian, bo suma bezpośrednich bez zmian.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14. Daty zadań (PDF): Z1 2025-10-01 – 2026-02-28, Z2 2026-03-01 – 2026-08-31, Z3 2026-09-01 – 2027-04-30, Z4 2027-05-01 – 2027-08-31 (poprawione).</t>
   </si>
   <si>
     <t xml:space="preserve">13. Miesięczne dane dla Z1 i Z2 to rozkład wykonania proporcjonalnie do planu etatów (brak miesięcznych danych rzeczywistych); reszta na licencjach wpisana w ostatnim miesiącu Z2 (m 11).</t>
@@ -12023,7 +12026,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="80"/>
@@ -12087,7 +12090,7 @@
       </c>
       <c r="C9" s="44" t="n">
         <f aca="false">ROUND(C14*C5,2)</f>
-        <v>3393.53</v>
+        <v>1785.82</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12130,7 +12133,7 @@
       </c>
       <c r="C14" s="46" t="n">
         <f aca="false">ROUND(C12-('nowy format 2'!F4+'nowy format 2'!F5+'nowy format 2'!F6+'nowy format 2'!F7+'nowy format 2'!F8+'nowy format 2'!F9+'nowy format 2'!F10+'nowy format 2'!F11+'nowy format 2'!F12+'nowy format 2'!F14+'nowy format 2'!F15+'nowy format 2'!F16+'nowy format 2'!F17+'nowy format 2'!F18+'nowy format 2'!F19+'nowy format 2'!F20+'nowy format 2'!F22+'nowy format 2'!F23+'nowy format 2'!F25+'nowy format 2'!F26+'nowy format 2'!F27+'nowy format 2'!F28+'nowy format 2'!F29+'nowy format 2'!F30+'nowy format 2'!F31+'nowy format 2'!F32+'nowy format 2'!F33+'nowy format 2'!F35+'nowy format 2'!F36+'nowy format 2'!F37+'nowy format 2'!F38+'nowy format 2'!F39+'nowy format 2'!F40+'nowy format 2'!F41+'nowy format 2'!F42+'nowy format 2'!F43),2)</f>
-        <v>4241.91</v>
+        <v>2232.28</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12138,8 +12141,8 @@
         <v>158</v>
       </c>
       <c r="C15" s="44" t="n">
-        <f aca="false">'nowy format 2'!F24</f>
-        <v>1389999.28</v>
+        <f aca="false">'nowy format 2'!F34</f>
+        <v>664057.14</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12147,7 +12150,7 @@
         <v>159</v>
       </c>
       <c r="C16" s="44" t="n">
-        <f aca="false">C15*C6</f>
+        <f aca="false">'nowy format 2'!F24*C6</f>
         <v>1111999.424</v>
       </c>
     </row>
@@ -12156,8 +12159,8 @@
         <v>160</v>
       </c>
       <c r="C17" s="44" t="n">
-        <f aca="false">'nowy format 2'!G4+'nowy format 2'!G5+'nowy format 2'!G6+'nowy format 2'!G7+'nowy format 2'!G8+'nowy format 2'!G9+'nowy format 2'!G10+'nowy format 2'!G11+'nowy format 2'!G12+'nowy format 2'!G14+'nowy format 2'!G15+'nowy format 2'!G16+'nowy format 2'!G17+'nowy format 2'!G18+'nowy format 2'!G19+'nowy format 2'!G20+'nowy format 2'!G21+'nowy format 2'!G22+'nowy format 2'!G23+'nowy format 2'!F34*C7</f>
-        <v>1854783.144</v>
+        <f aca="false">'nowy format 2'!G4+'nowy format 2'!G5+'nowy format 2'!G6+'nowy format 2'!G7+'nowy format 2'!G8+'nowy format 2'!G9+'nowy format 2'!G10+'nowy format 2'!G11+'nowy format 2'!G12+'nowy format 2'!G14+'nowy format 2'!G15+'nowy format 2'!G16+'nowy format 2'!G17+'nowy format 2'!G18+'nowy format 2'!G19+'nowy format 2'!G20+'nowy format 2'!G21+'nowy format 2'!G22+'nowy format 2'!G23+C15*C7</f>
+        <v>1854783.114</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12166,7 +12169,7 @@
       </c>
       <c r="C18" s="44" t="n">
         <f aca="false">C16+C17-C13</f>
-        <v>6836.02799999993</v>
+        <v>6835.99800000014</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12175,7 +12178,7 @@
       </c>
       <c r="C19" s="47" t="n">
         <f aca="false">C18/C15</f>
-        <v>0.00491800830285317</v>
+        <v>0.0102942918436208</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12193,7 +12196,7 @@
       </c>
       <c r="C21" s="44" t="n">
         <f aca="false">C14-C20</f>
-        <v>-29938.09</v>
+        <v>-31947.72</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12269,7 +12272,7 @@
         <v>173</v>
       </c>
       <c r="C27" s="49" t="n">
-        <f aca="false">ABS('nowy format 2'!E4-'nowy format 2'!B4)+ABS('nowy format 2'!F4-'nowy format 2'!C4)+ABS('nowy format 2'!G4-'nowy format 2'!D4)+ABS('nowy format 2'!E5-'nowy format 2'!B5)+ABS('nowy format 2'!F5-'nowy format 2'!C5)+ABS('nowy format 2'!G5-'nowy format 2'!D5)+ABS('nowy format 2'!E6-'nowy format 2'!B6)+ABS('nowy format 2'!F6-'nowy format 2'!C6)+ABS('nowy format 2'!G6-'nowy format 2'!D6)+ABS('nowy format 2'!E7-'nowy format 2'!B7)+ABS('nowy format 2'!F7-'nowy format 2'!C7)+ABS('nowy format 2'!G7-'nowy format 2'!D7)+ABS('nowy format 2'!E8-'nowy format 2'!B8)+ABS('nowy format 2'!F8-'nowy format 2'!C8)+ABS('nowy format 2'!G8-'nowy format 2'!D8)+ABS('nowy format 2'!E9-'nowy format 2'!B9)+ABS('nowy format 2'!F9-'nowy format 2'!C9)+ABS('nowy format 2'!G9-'nowy format 2'!D9)+ABS('nowy format 2'!E10-'nowy format 2'!B10)+ABS('nowy format 2'!F10-'nowy format 2'!C10)+ABS('nowy format 2'!G10-'nowy format 2'!D10)+ABS('nowy format 2'!E11-'nowy format 2'!B11)+ABS('nowy format 2'!F11-'nowy format 2'!C11)+ABS('nowy format 2'!G11-'nowy format 2'!D11)+ABS('nowy format 2'!E12-'nowy format 2'!B12)+ABS('nowy format 2'!F12-'nowy format 2'!C12)+ABS('nowy format 2'!G12-'nowy format 2'!D12)+ABS('nowy format 2'!E14-'nowy format 2'!B14)+ABS('nowy format 2'!F14-'nowy format 2'!C14)+ABS('nowy format 2'!G14-'nowy format 2'!D14)+ABS('nowy format 2'!E15-'nowy format 2'!B15)+ABS('nowy format 2'!F15-'nowy format 2'!C15)+ABS('nowy format 2'!G15-'nowy format 2'!D15)+ABS('nowy format 2'!E16-'nowy format 2'!B16)+ABS('nowy format 2'!F16-'nowy format 2'!C16)+ABS('nowy format 2'!G16-'nowy format 2'!D16)+ABS('nowy format 2'!E17-'nowy format 2'!B17)+ABS('nowy format 2'!F17-'nowy format 2'!C17)+ABS('nowy format 2'!G17-'nowy format 2'!D17)+ABS('nowy format 2'!E18-'nowy format 2'!B18)+ABS('nowy format 2'!F18-'nowy format 2'!C18)+ABS('nowy format 2'!G18-'nowy format 2'!D18)+ABS('nowy format 2'!E19-'nowy format 2'!B19)+ABS('nowy format 2'!F19-'nowy format 2'!C19)+ABS('nowy format 2'!G19-'nowy format 2'!D19)+ABS('nowy format 2'!E20-'nowy format 2'!B20)+ABS('nowy format 2'!F20-'nowy format 2'!C20)+ABS('nowy format 2'!G20-'nowy format 2'!D20)+ABS('nowy format 2'!E22-'nowy format 2'!B22)+ABS('nowy format 2'!F22-'nowy format 2'!C22)+ABS('nowy format 2'!G22-'nowy format 2'!D22)+ABS('nowy format 2'!E23-'nowy format 2'!B23)+ABS('nowy format 2'!F23-'nowy format 2'!C23)+ABS('nowy format 2'!G23-'nowy format 2'!D23)</f>
+        <f aca="false">ABS('nowy format 2'!E4-'nowy format 2'!B4)+ABS('nowy format 2'!F4-'nowy format 2'!C4)+ABS('nowy format 2'!G4-'nowy format 2'!D4)+ABS('nowy format 2'!E5-'nowy format 2'!B5)+ABS('nowy format 2'!F5-'nowy format 2'!C5)+ABS('nowy format 2'!G5-'nowy format 2'!D5)+ABS('nowy format 2'!E6-'nowy format 2'!B6)+ABS('nowy format 2'!F6-'nowy format 2'!C6)+ABS('nowy format 2'!G6-'nowy format 2'!D6)+ABS('nowy format 2'!E7-'nowy format 2'!B7)+ABS('nowy format 2'!F7-'nowy format 2'!C7)+ABS('nowy format 2'!G7-'nowy format 2'!D7)+ABS('nowy format 2'!E8-'nowy format 2'!B8)+ABS('nowy format 2'!F8-'nowy format 2'!C8)+ABS('nowy format 2'!G8-'nowy format 2'!D8)+ABS('nowy format 2'!E9-'nowy format 2'!B9)+ABS('nowy format 2'!F9-'nowy format 2'!C9)+ABS('nowy format 2'!G9-'nowy format 2'!D9)+ABS('nowy format 2'!E10-'nowy format 2'!B10)+ABS('nowy format 2'!F10-'nowy format 2'!C10)+ABS('nowy format 2'!G10-'nowy format 2'!D10)+ABS('nowy format 2'!E11-'nowy format 2'!B11)+ABS('nowy format 2'!F11-'nowy format 2'!C11)+ABS('nowy format 2'!G11-'nowy format 2'!D11)+ABS('nowy format 2'!E12-'nowy format 2'!B12)+ABS('nowy format 2'!F12-'nowy format 2'!C12)+ABS('nowy format 2'!G12-'nowy format 2'!D12)+ABS('nowy format 2'!E14-'nowy format 2'!B14)+ABS('nowy format 2'!F14-'nowy format 2'!C14)+ABS('nowy format 2'!G14-'nowy format 2'!D14)+ABS('nowy format 2'!E15-'nowy format 2'!B15)+ABS('nowy format 2'!F15-'nowy format 2'!C15)+ABS('nowy format 2'!G15-'nowy format 2'!D15)+ABS('nowy format 2'!E16-'nowy format 2'!B16)+ABS('nowy format 2'!F16-'nowy format 2'!C16)+ABS('nowy format 2'!G16-'nowy format 2'!D16)+ABS('nowy format 2'!E17-'nowy format 2'!B17)+ABS('nowy format 2'!F17-'nowy format 2'!C17)+ABS('nowy format 2'!G17-'nowy format 2'!D17)+ABS('nowy format 2'!E18-'nowy format 2'!B18)+ABS('nowy format 2'!F18-'nowy format 2'!C18)+ABS('nowy format 2'!G18-'nowy format 2'!D18)+ABS('nowy format 2'!E19-'nowy format 2'!B19)+ABS('nowy format 2'!F19-'nowy format 2'!C19)+ABS('nowy format 2'!G19-'nowy format 2'!D19)+ABS('nowy format 2'!E20-'nowy format 2'!B20)+ABS('nowy format 2'!F20-'nowy format 2'!C20)+ABS('nowy format 2'!G20-'nowy format 2'!D20)+ABS('nowy format 2'!E23-'nowy format 2'!B23)+ABS('nowy format 2'!F23-'nowy format 2'!C23)+ABS('nowy format 2'!G23-'nowy format 2'!D23)</f>
         <v>0</v>
       </c>
       <c r="D27" s="49"/>
@@ -12486,8 +12489,18 @@
       <c r="E46" s="50"/>
       <c r="F46" s="50"/>
     </row>
+    <row r="47" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="50" t="s">
+        <v>192</v>
+      </c>
+      <c r="B47" s="50"/>
+      <c r="C47" s="50"/>
+      <c r="D47" s="50"/>
+      <c r="E47" s="50"/>
+      <c r="F47" s="50"/>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A34:F34"/>
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="A36:F36"/>
@@ -12501,6 +12514,7 @@
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A45:F45"/>
     <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A47:F47"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -12529,37 +12543,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="51" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="40" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B3" s="40" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C3" s="40" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D3" s="40" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E3" s="40" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F3" s="40" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="41" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B4" s="52" t="n">
         <v>1</v>
@@ -12574,12 +12588,12 @@
         <v>5</v>
       </c>
       <c r="F4" s="41" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="41" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B5" s="52" t="n">
         <v>6</v>
@@ -12594,12 +12608,12 @@
         <v>11</v>
       </c>
       <c r="F5" s="41" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="41" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B6" s="52" t="n">
         <v>12</v>
@@ -12614,12 +12628,12 @@
         <v>19</v>
       </c>
       <c r="F6" s="41" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="41" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B7" s="52" t="n">
         <v>18</v>
@@ -12634,23 +12648,23 @@
         <v>23</v>
       </c>
       <c r="F7" s="41" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="40" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="53" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B10" s="53" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C10" s="53" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D10" s="53" t="n">
         <v>1</v>
@@ -12722,12 +12736,12 @@
         <v>23</v>
       </c>
       <c r="AA10" s="53" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="41" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B11" s="54" t="n">
         <v>27700</v>
@@ -13189,7 +13203,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="41" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B17" s="54" t="n">
         <v>19750</v>
@@ -13343,7 +13357,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="41" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B19" s="54" t="n">
         <f aca="false">ROUND(4285.71/6,4)</f>
@@ -13421,18 +13435,18 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="40" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="53" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B23" s="53" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C23" s="53" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D23" s="53" t="n">
         <v>1</v>
@@ -13504,12 +13518,12 @@
         <v>23</v>
       </c>
       <c r="AA23" s="53" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="41" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B24" s="54" t="n">
         <v>27700</v>
@@ -13661,7 +13675,7 @@
         <v>0.5</v>
       </c>
       <c r="AB25" s="55" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13741,7 +13755,7 @@
         <v>2</v>
       </c>
       <c r="AB26" s="55" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13821,7 +13835,7 @@
         <v>1</v>
       </c>
       <c r="AB27" s="55" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13980,7 +13994,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="41" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B30" s="54" t="n">
         <v>19750</v>
@@ -14134,7 +14148,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="41" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B32" s="54" t="n">
         <f aca="false">ROUND(4285.71/6,4)</f>
@@ -14210,23 +14224,23 @@
         <v>1</v>
       </c>
       <c r="AB32" s="55" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="40" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="53" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B36" s="53" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C36" s="53" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D36" s="53" t="n">
         <v>1</v>
@@ -14298,7 +14312,7 @@
         <v>23</v>
       </c>
       <c r="AA36" s="53" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18128,18 +18142,18 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="40" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="53" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B77" s="53" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C77" s="53" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D77" s="53" t="n">
         <v>1</v>
@@ -18211,7 +18225,7 @@
         <v>23</v>
       </c>
       <c r="AA77" s="53" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22066,17 +22080,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="39" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="51" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="58" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B3" s="59"/>
       <c r="C3" s="59"/>
@@ -22175,13 +22189,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="58" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B4" s="59" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C4" s="59" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D4" s="59" t="n">
         <v>1</v>
@@ -22255,7 +22269,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="58" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B5" s="59"/>
       <c r="C5" s="59"/>
@@ -22354,7 +22368,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="58" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B6" s="59"/>
       <c r="C6" s="59"/>
@@ -22481,7 +22495,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="60" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B8" s="61"/>
       <c r="C8" s="62"/>
@@ -26359,7 +26373,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="40" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B46" s="40" t="n">
         <v>1</v>
@@ -26463,7 +26477,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="40" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B47" s="40" t="n">
         <v>2</v>
@@ -26567,7 +26581,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="40" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B48" s="40" t="n">
         <v>3</v>
@@ -26671,7 +26685,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="40" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B49" s="40" t="n">
         <v>4</v>
@@ -26877,7 +26891,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="40" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B51" s="40"/>
       <c r="C51" s="63" t="n">
@@ -26979,7 +26993,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="40" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B52" s="40"/>
       <c r="C52" s="63" t="n">
@@ -27081,7 +27095,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="40" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B53" s="40"/>
       <c r="C53" s="63"/>
@@ -27208,7 +27222,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="64" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B55" s="65"/>
       <c r="C55" s="66"/>
@@ -28909,7 +28923,7 @@
       </c>
       <c r="C72" s="49" t="n">
         <f aca="false">SUM(D72:Z72)</f>
-        <v>4241.91</v>
+        <v>2232.28</v>
       </c>
       <c r="D72" s="49" t="n">
         <f aca="false">IF(D$4='plan etatów'!$E$5,założenia!$C$14,0)</f>
@@ -28953,7 +28967,7 @@
       </c>
       <c r="N72" s="49" t="n">
         <f aca="false">IF(N$4='plan etatów'!$E$5,założenia!$C$14,0)</f>
-        <v>4241.91</v>
+        <v>2232.28</v>
       </c>
       <c r="O72" s="49" t="n">
         <f aca="false">IF(O$4='plan etatów'!$E$5,założenia!$C$14,0)</f>
@@ -29013,98 +29027,98 @@
       </c>
       <c r="C73" s="49" t="n">
         <f aca="false">SUM(D73:Z73)</f>
-        <v>2276.08</v>
+        <v>4285.71</v>
       </c>
       <c r="D73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!D95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!D95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="E73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!E95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!E95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="F73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!F95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!F95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="G73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!G95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!G95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="H73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!H95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!H95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="I73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!I95/'plan etatów'!$AA$95)</f>
-        <v>379.346666666667</v>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!I95/'plan etatów'!$AA$95)</f>
+        <v>714.285</v>
       </c>
       <c r="J73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!J95/'plan etatów'!$AA$95)</f>
-        <v>379.346666666667</v>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!J95/'plan etatów'!$AA$95)</f>
+        <v>714.285</v>
       </c>
       <c r="K73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!K95/'plan etatów'!$AA$95)</f>
-        <v>379.346666666667</v>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!K95/'plan etatów'!$AA$95)</f>
+        <v>714.285</v>
       </c>
       <c r="L73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!L95/'plan etatów'!$AA$95)</f>
-        <v>379.346666666667</v>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!L95/'plan etatów'!$AA$95)</f>
+        <v>714.285</v>
       </c>
       <c r="M73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!M95/'plan etatów'!$AA$95)</f>
-        <v>379.346666666667</v>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!M95/'plan etatów'!$AA$95)</f>
+        <v>714.285</v>
       </c>
       <c r="N73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!N95/'plan etatów'!$AA$95)</f>
-        <v>379.346666666667</v>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!N95/'plan etatów'!$AA$95)</f>
+        <v>714.285</v>
       </c>
       <c r="O73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!O95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!O95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="P73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!P95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!P95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="Q73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!Q95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!Q95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="R73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!R95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!R95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="S73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!S95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!S95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="T73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!T95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!T95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="U73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!U95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!U95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="V73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!V95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!V95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="W73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!W95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!W95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="X73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!X95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!X95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="Y73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!Y95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!Y95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="Z73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$C$22*'plan etatów'!Z95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!Z95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
     </row>
@@ -31086,7 +31100,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="40" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B93" s="40" t="n">
         <v>1</v>
@@ -31190,7 +31204,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="40" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B94" s="40" t="n">
         <v>2</v>
@@ -31221,27 +31235,27 @@
       </c>
       <c r="I94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,I$56:I$92)</f>
-        <v>168128.215</v>
+        <v>168463.153333333</v>
       </c>
       <c r="J94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,J$56:J$92)</f>
-        <v>168128.215</v>
+        <v>168463.153333333</v>
       </c>
       <c r="K94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,K$56:K$92)</f>
-        <v>168128.215</v>
+        <v>168463.153333333</v>
       </c>
       <c r="L94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,L$56:L$92)</f>
-        <v>168128.215</v>
+        <v>168463.153333333</v>
       </c>
       <c r="M94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,M$56:M$92)</f>
-        <v>168128.215</v>
+        <v>168463.153333333</v>
       </c>
       <c r="N94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,N$56:N$92)</f>
-        <v>172370.125</v>
+        <v>170695.433333333</v>
       </c>
       <c r="O94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,O$56:O$92)</f>
@@ -31294,7 +31308,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="40" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B95" s="40" t="n">
         <v>3</v>
@@ -31398,7 +31412,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="40" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B96" s="40" t="n">
         <v>4</v>
@@ -31531,27 +31545,27 @@
       </c>
       <c r="I97" s="63" t="n">
         <f aca="false">SUM(I93:I96)</f>
-        <v>168128.215</v>
+        <v>168463.153333333</v>
       </c>
       <c r="J97" s="63" t="n">
         <f aca="false">SUM(J93:J96)</f>
-        <v>168128.215</v>
+        <v>168463.153333333</v>
       </c>
       <c r="K97" s="63" t="n">
         <f aca="false">SUM(K93:K96)</f>
-        <v>168128.215</v>
+        <v>168463.153333333</v>
       </c>
       <c r="L97" s="63" t="n">
         <f aca="false">SUM(L93:L96)</f>
-        <v>168128.215</v>
+        <v>168463.153333333</v>
       </c>
       <c r="M97" s="63" t="n">
         <f aca="false">SUM(M93:M96)</f>
-        <v>168128.215</v>
+        <v>168463.153333333</v>
       </c>
       <c r="N97" s="63" t="n">
         <f aca="false">SUM(N93:N96)</f>
-        <v>172370.125</v>
+        <v>170695.433333333</v>
       </c>
       <c r="O97" s="63" t="n">
         <f aca="false">SUM(O93:O96)</f>
@@ -31604,7 +31618,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="40" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B98" s="40"/>
       <c r="C98" s="63" t="n">
@@ -31633,27 +31647,27 @@
       </c>
       <c r="I98" s="63" t="n">
         <f aca="false">0.25*I97</f>
-        <v>42032.05375</v>
+        <v>42115.7883333333</v>
       </c>
       <c r="J98" s="63" t="n">
         <f aca="false">0.25*J97</f>
-        <v>42032.05375</v>
+        <v>42115.7883333333</v>
       </c>
       <c r="K98" s="63" t="n">
         <f aca="false">0.25*K97</f>
-        <v>42032.05375</v>
+        <v>42115.7883333333</v>
       </c>
       <c r="L98" s="63" t="n">
         <f aca="false">0.25*L97</f>
-        <v>42032.05375</v>
+        <v>42115.7883333333</v>
       </c>
       <c r="M98" s="63" t="n">
         <f aca="false">0.25*M97</f>
-        <v>42032.05375</v>
+        <v>42115.7883333333</v>
       </c>
       <c r="N98" s="63" t="n">
         <f aca="false">0.25*N97</f>
-        <v>43092.53125</v>
+        <v>42673.8583333333</v>
       </c>
       <c r="O98" s="63" t="n">
         <f aca="false">0.25*O97</f>
@@ -31706,7 +31720,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="40" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B99" s="40"/>
       <c r="C99" s="63" t="n">
@@ -31735,27 +31749,27 @@
       </c>
       <c r="I99" s="63" t="n">
         <f aca="false">I97+I98</f>
-        <v>210160.26875</v>
+        <v>210578.941666667</v>
       </c>
       <c r="J99" s="63" t="n">
         <f aca="false">J97+J98</f>
-        <v>210160.26875</v>
+        <v>210578.941666667</v>
       </c>
       <c r="K99" s="63" t="n">
         <f aca="false">K97+K98</f>
-        <v>210160.26875</v>
+        <v>210578.941666667</v>
       </c>
       <c r="L99" s="63" t="n">
         <f aca="false">L97+L98</f>
-        <v>210160.26875</v>
+        <v>210578.941666667</v>
       </c>
       <c r="M99" s="63" t="n">
         <f aca="false">M97+M98</f>
-        <v>210160.26875</v>
+        <v>210578.941666667</v>
       </c>
       <c r="N99" s="63" t="n">
         <f aca="false">N97+N98</f>
-        <v>215462.65625</v>
+        <v>213369.291666667</v>
       </c>
       <c r="O99" s="63" t="n">
         <f aca="false">O97+O98</f>
@@ -31808,7 +31822,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="40" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B100" s="40"/>
       <c r="C100" s="63"/>
@@ -31834,23 +31848,23 @@
       </c>
       <c r="I100" s="63" t="n">
         <f aca="false">H100+I99</f>
-        <v>1219441.35625</v>
+        <v>1219860.02916667</v>
       </c>
       <c r="J100" s="63" t="n">
         <f aca="false">I100+J99</f>
-        <v>1429601.625</v>
+        <v>1430438.97083333</v>
       </c>
       <c r="K100" s="63" t="n">
         <f aca="false">J100+K99</f>
-        <v>1639761.89375</v>
+        <v>1641017.9125</v>
       </c>
       <c r="L100" s="63" t="n">
         <f aca="false">K100+L99</f>
-        <v>1849922.1625</v>
+        <v>1851596.85416667</v>
       </c>
       <c r="M100" s="63" t="n">
         <f aca="false">L100+M99</f>
-        <v>2060082.43125</v>
+        <v>2062175.79583333</v>
       </c>
       <c r="N100" s="63" t="n">
         <f aca="false">M100+N99</f>
@@ -31935,7 +31949,7 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="60" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B102" s="61"/>
       <c r="C102" s="62"/>
@@ -35813,7 +35827,7 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="40" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B140" s="40" t="n">
         <v>1</v>
@@ -35917,7 +35931,7 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="40" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B141" s="40" t="n">
         <v>2</v>
@@ -36021,7 +36035,7 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="40" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B142" s="40" t="n">
         <v>3</v>
@@ -36125,7 +36139,7 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="40" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B143" s="40" t="n">
         <v>4</v>
@@ -36331,7 +36345,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="40" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B145" s="40"/>
       <c r="C145" s="63" t="n">
@@ -36433,7 +36447,7 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="40" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B146" s="40"/>
       <c r="C146" s="63" t="n">
@@ -36535,7 +36549,7 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="40" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B147" s="40"/>
       <c r="C147" s="63"/>
@@ -36662,7 +36676,7 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="64" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B149" s="65"/>
       <c r="C149" s="66"/>
@@ -38363,7 +38377,7 @@
       </c>
       <c r="C166" s="49" t="n">
         <f aca="false">SUM(D166:Z166)</f>
-        <v>3393.53</v>
+        <v>1785.82</v>
       </c>
       <c r="D166" s="49" t="n">
         <f aca="false">IF(D$4='plan etatów'!$E$5,założenia!$C$9,0)</f>
@@ -38407,7 +38421,7 @@
       </c>
       <c r="N166" s="49" t="n">
         <f aca="false">IF(N$4='plan etatów'!$E$5,założenia!$C$9,0)</f>
-        <v>3393.53</v>
+        <v>1785.82</v>
       </c>
       <c r="O166" s="49" t="n">
         <f aca="false">IF(O$4='plan etatów'!$E$5,założenia!$C$9,0)</f>
@@ -38467,98 +38481,98 @@
       </c>
       <c r="C167" s="49" t="n">
         <f aca="false">SUM(D167:Z167)</f>
-        <v>1820.88</v>
+        <v>3428.56</v>
       </c>
       <c r="D167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!D95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!D95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="E167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!E95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!E95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="F167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!F95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!F95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="G167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!G95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!G95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="H167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!H95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!H95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="I167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!I95/'plan etatów'!$AA$95)</f>
-        <v>303.48</v>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!I95/'plan etatów'!$AA$95)</f>
+        <v>571.426666666667</v>
       </c>
       <c r="J167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!J95/'plan etatów'!$AA$95)</f>
-        <v>303.48</v>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!J95/'plan etatów'!$AA$95)</f>
+        <v>571.426666666667</v>
       </c>
       <c r="K167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!K95/'plan etatów'!$AA$95)</f>
-        <v>303.48</v>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!K95/'plan etatów'!$AA$95)</f>
+        <v>571.426666666667</v>
       </c>
       <c r="L167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!L95/'plan etatów'!$AA$95)</f>
-        <v>303.48</v>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!L95/'plan etatów'!$AA$95)</f>
+        <v>571.426666666667</v>
       </c>
       <c r="M167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!M95/'plan etatów'!$AA$95)</f>
-        <v>303.48</v>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!M95/'plan etatów'!$AA$95)</f>
+        <v>571.426666666667</v>
       </c>
       <c r="N167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!N95/'plan etatów'!$AA$95)</f>
-        <v>303.48</v>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!N95/'plan etatów'!$AA$95)</f>
+        <v>571.426666666667</v>
       </c>
       <c r="O167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!O95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!O95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="P167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!P95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!P95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="Q167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!Q95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!Q95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="R167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!R95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!R95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="S167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!S95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!S95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="T167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!T95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!T95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="U167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!U95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!U95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="V167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!V95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!V95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="W167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!W95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!W95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="X167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!X95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!X95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="Y167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!Y95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!Y95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
       <c r="Z167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$D$22*'plan etatów'!Z95/'plan etatów'!$AA$95)</f>
+        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!Z95/'plan etatów'!$AA$95)</f>
         <v>0</v>
       </c>
     </row>
@@ -38675,98 +38689,98 @@
       </c>
       <c r="C169" s="49" t="n">
         <f aca="false">SUM(D169:Z169)</f>
-        <v>352380.338720176</v>
+        <v>354560</v>
       </c>
       <c r="D169" s="49" t="n">
-        <f aca="false">D75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">D75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="E169" s="49" t="n">
-        <f aca="false">E75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">E75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="F169" s="49" t="n">
-        <f aca="false">F75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">F75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="G169" s="49" t="n">
-        <f aca="false">G75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">G75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="H169" s="49" t="n">
-        <f aca="false">H75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">H75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="I169" s="49" t="n">
-        <f aca="false">I75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">I75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="J169" s="49" t="n">
-        <f aca="false">J75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">J75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="K169" s="49" t="n">
-        <f aca="false">K75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">K75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="L169" s="49" t="n">
-        <f aca="false">L75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">L75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="M169" s="49" t="n">
-        <f aca="false">M75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">M75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="N169" s="49" t="n">
-        <f aca="false">N75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">N75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="O169" s="49" t="n">
-        <f aca="false">O75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44047.5423400219</v>
+        <f aca="false">O75*założenia!$C$6</f>
+        <v>44320</v>
       </c>
       <c r="P169" s="49" t="n">
-        <f aca="false">P75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44047.5423400219</v>
+        <f aca="false">P75*założenia!$C$6</f>
+        <v>44320</v>
       </c>
       <c r="Q169" s="49" t="n">
-        <f aca="false">Q75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44047.5423400219</v>
+        <f aca="false">Q75*założenia!$C$6</f>
+        <v>44320</v>
       </c>
       <c r="R169" s="49" t="n">
-        <f aca="false">R75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44047.5423400219</v>
+        <f aca="false">R75*założenia!$C$6</f>
+        <v>44320</v>
       </c>
       <c r="S169" s="49" t="n">
-        <f aca="false">S75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44047.5423400219</v>
+        <f aca="false">S75*założenia!$C$6</f>
+        <v>44320</v>
       </c>
       <c r="T169" s="49" t="n">
-        <f aca="false">T75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44047.5423400219</v>
+        <f aca="false">T75*założenia!$C$6</f>
+        <v>44320</v>
       </c>
       <c r="U169" s="49" t="n">
-        <f aca="false">U75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44047.5423400219</v>
+        <f aca="false">U75*założenia!$C$6</f>
+        <v>44320</v>
       </c>
       <c r="V169" s="49" t="n">
-        <f aca="false">V75*(założenia!$C$6-założenia!$C$19)</f>
-        <v>44047.5423400219</v>
+        <f aca="false">V75*założenia!$C$6</f>
+        <v>44320</v>
       </c>
       <c r="W169" s="49" t="n">
-        <f aca="false">W75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">W75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="X169" s="49" t="n">
-        <f aca="false">X75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">X75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Y169" s="49" t="n">
-        <f aca="false">Y75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Y75*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Z169" s="49" t="n">
-        <f aca="false">Z75*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Z75*założenia!$C$6</f>
         <v>0</v>
       </c>
     </row>
@@ -38779,98 +38793,98 @@
       </c>
       <c r="C170" s="49" t="n">
         <f aca="false">SUM(D170:Z170)</f>
-        <v>119961.970907266</v>
+        <v>120704</v>
       </c>
       <c r="D170" s="49" t="n">
-        <f aca="false">D76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">D76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="E170" s="49" t="n">
-        <f aca="false">E76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">E76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="F170" s="49" t="n">
-        <f aca="false">F76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">F76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="G170" s="49" t="n">
-        <f aca="false">G76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">G76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="H170" s="49" t="n">
-        <f aca="false">H76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">H76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="I170" s="49" t="n">
-        <f aca="false">I76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">I76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="J170" s="49" t="n">
-        <f aca="false">J76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">J76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="K170" s="49" t="n">
-        <f aca="false">K76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">K76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="L170" s="49" t="n">
-        <f aca="false">L76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">L76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="M170" s="49" t="n">
-        <f aca="false">M76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">M76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="N170" s="49" t="n">
-        <f aca="false">N76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">N76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="O170" s="49" t="n">
-        <f aca="false">O76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>14995.2463634082</v>
+        <f aca="false">O76*założenia!$C$6</f>
+        <v>15088</v>
       </c>
       <c r="P170" s="49" t="n">
-        <f aca="false">P76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>14995.2463634082</v>
+        <f aca="false">P76*założenia!$C$6</f>
+        <v>15088</v>
       </c>
       <c r="Q170" s="49" t="n">
-        <f aca="false">Q76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>14995.2463634082</v>
+        <f aca="false">Q76*założenia!$C$6</f>
+        <v>15088</v>
       </c>
       <c r="R170" s="49" t="n">
-        <f aca="false">R76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>14995.2463634082</v>
+        <f aca="false">R76*założenia!$C$6</f>
+        <v>15088</v>
       </c>
       <c r="S170" s="49" t="n">
-        <f aca="false">S76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>14995.2463634082</v>
+        <f aca="false">S76*założenia!$C$6</f>
+        <v>15088</v>
       </c>
       <c r="T170" s="49" t="n">
-        <f aca="false">T76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>14995.2463634082</v>
+        <f aca="false">T76*założenia!$C$6</f>
+        <v>15088</v>
       </c>
       <c r="U170" s="49" t="n">
-        <f aca="false">U76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>14995.2463634082</v>
+        <f aca="false">U76*założenia!$C$6</f>
+        <v>15088</v>
       </c>
       <c r="V170" s="49" t="n">
-        <f aca="false">V76*(założenia!$C$6-założenia!$C$19)</f>
-        <v>14995.2463634082</v>
+        <f aca="false">V76*założenia!$C$6</f>
+        <v>15088</v>
       </c>
       <c r="W170" s="49" t="n">
-        <f aca="false">W76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">W76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="X170" s="49" t="n">
-        <f aca="false">X76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">X76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Y170" s="49" t="n">
-        <f aca="false">Y76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Y76*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Z170" s="49" t="n">
-        <f aca="false">Z76*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Z76*założenia!$C$6</f>
         <v>0</v>
       </c>
     </row>
@@ -38883,98 +38897,98 @@
       </c>
       <c r="C171" s="49" t="n">
         <f aca="false">SUM(D171:Z171)</f>
-        <v>161660.045961822</v>
+        <v>162660</v>
       </c>
       <c r="D171" s="49" t="n">
-        <f aca="false">D77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">D77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="E171" s="49" t="n">
-        <f aca="false">E77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">E77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="F171" s="49" t="n">
-        <f aca="false">F77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">F77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="G171" s="49" t="n">
-        <f aca="false">G77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">G77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="H171" s="49" t="n">
-        <f aca="false">H77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">H77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="I171" s="49" t="n">
-        <f aca="false">I77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">I77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="J171" s="49" t="n">
-        <f aca="false">J77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">J77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="K171" s="49" t="n">
-        <f aca="false">K77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">K77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="L171" s="49" t="n">
-        <f aca="false">L77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">L77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="M171" s="49" t="n">
-        <f aca="false">M77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">M77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="N171" s="49" t="n">
-        <f aca="false">N77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">N77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="O171" s="49" t="n">
-        <f aca="false">O77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16166.0045961822</v>
+        <f aca="false">O77*założenia!$C$6</f>
+        <v>16266</v>
       </c>
       <c r="P171" s="49" t="n">
-        <f aca="false">P77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16166.0045961822</v>
+        <f aca="false">P77*założenia!$C$6</f>
+        <v>16266</v>
       </c>
       <c r="Q171" s="49" t="n">
-        <f aca="false">Q77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>21554.6727949097</v>
+        <f aca="false">Q77*założenia!$C$6</f>
+        <v>21688</v>
       </c>
       <c r="R171" s="49" t="n">
-        <f aca="false">R77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>21554.6727949097</v>
+        <f aca="false">R77*założenia!$C$6</f>
+        <v>21688</v>
       </c>
       <c r="S171" s="49" t="n">
-        <f aca="false">S77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>21554.6727949097</v>
+        <f aca="false">S77*założenia!$C$6</f>
+        <v>21688</v>
       </c>
       <c r="T171" s="49" t="n">
-        <f aca="false">T77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>21554.6727949097</v>
+        <f aca="false">T77*założenia!$C$6</f>
+        <v>21688</v>
       </c>
       <c r="U171" s="49" t="n">
-        <f aca="false">U77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>21554.6727949097</v>
+        <f aca="false">U77*założenia!$C$6</f>
+        <v>21688</v>
       </c>
       <c r="V171" s="49" t="n">
-        <f aca="false">V77*(założenia!$C$6-założenia!$C$19)</f>
-        <v>21554.6727949097</v>
+        <f aca="false">V77*założenia!$C$6</f>
+        <v>21688</v>
       </c>
       <c r="W171" s="49" t="n">
-        <f aca="false">W77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">W77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="X171" s="49" t="n">
-        <f aca="false">X77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">X77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Y171" s="49" t="n">
-        <f aca="false">Y77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Y77*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Z171" s="49" t="n">
-        <f aca="false">Z77*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Z77*założenia!$C$6</f>
         <v>0</v>
       </c>
     </row>
@@ -38987,98 +39001,98 @@
       </c>
       <c r="C172" s="49" t="n">
         <f aca="false">SUM(D172:Z172)</f>
-        <v>131188.528630029</v>
+        <v>132000</v>
       </c>
       <c r="D172" s="49" t="n">
-        <f aca="false">D78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">D78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="E172" s="49" t="n">
-        <f aca="false">E78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">E78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="F172" s="49" t="n">
-        <f aca="false">F78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">F78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="G172" s="49" t="n">
-        <f aca="false">G78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">G78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="H172" s="49" t="n">
-        <f aca="false">H78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">H78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="I172" s="49" t="n">
-        <f aca="false">I78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">I78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="J172" s="49" t="n">
-        <f aca="false">J78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">J78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="K172" s="49" t="n">
-        <f aca="false">K78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">K78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="L172" s="49" t="n">
-        <f aca="false">L78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">L78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="M172" s="49" t="n">
-        <f aca="false">M78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">M78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="N172" s="49" t="n">
-        <f aca="false">N78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">N78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="O172" s="49" t="n">
-        <f aca="false">O78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">O78*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="P172" s="49" t="n">
-        <f aca="false">P78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">P78*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="Q172" s="49" t="n">
-        <f aca="false">Q78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">Q78*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="R172" s="49" t="n">
-        <f aca="false">R78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">R78*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="S172" s="49" t="n">
-        <f aca="false">S78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">S78*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="T172" s="49" t="n">
-        <f aca="false">T78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">T78*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="U172" s="49" t="n">
-        <f aca="false">U78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">U78*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="V172" s="49" t="n">
-        <f aca="false">V78*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">V78*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="W172" s="49" t="n">
-        <f aca="false">W78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">W78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="X172" s="49" t="n">
-        <f aca="false">X78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">X78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Y172" s="49" t="n">
-        <f aca="false">Y78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Y78*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Z172" s="49" t="n">
-        <f aca="false">Z78*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Z78*założenia!$C$6</f>
         <v>0</v>
       </c>
     </row>
@@ -39091,98 +39105,98 @@
       </c>
       <c r="C173" s="49" t="n">
         <f aca="false">SUM(D173:Z173)</f>
-        <v>47323.2801458142</v>
+        <v>47616</v>
       </c>
       <c r="D173" s="49" t="n">
-        <f aca="false">D79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">D79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="E173" s="49" t="n">
-        <f aca="false">E79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">E79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="F173" s="49" t="n">
-        <f aca="false">F79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">F79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="G173" s="49" t="n">
-        <f aca="false">G79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">G79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="H173" s="49" t="n">
-        <f aca="false">H79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">H79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="I173" s="49" t="n">
-        <f aca="false">I79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">I79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="J173" s="49" t="n">
-        <f aca="false">J79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">J79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="K173" s="49" t="n">
-        <f aca="false">K79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">K79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="L173" s="49" t="n">
-        <f aca="false">L79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">L79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="M173" s="49" t="n">
-        <f aca="false">M79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">M79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="N173" s="49" t="n">
-        <f aca="false">N79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">N79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="O173" s="49" t="n">
-        <f aca="false">O79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5915.41001822677</v>
+        <f aca="false">O79*założenia!$C$6</f>
+        <v>5952</v>
       </c>
       <c r="P173" s="49" t="n">
-        <f aca="false">P79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5915.41001822677</v>
+        <f aca="false">P79*założenia!$C$6</f>
+        <v>5952</v>
       </c>
       <c r="Q173" s="49" t="n">
-        <f aca="false">Q79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5915.41001822677</v>
+        <f aca="false">Q79*założenia!$C$6</f>
+        <v>5952</v>
       </c>
       <c r="R173" s="49" t="n">
-        <f aca="false">R79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5915.41001822677</v>
+        <f aca="false">R79*założenia!$C$6</f>
+        <v>5952</v>
       </c>
       <c r="S173" s="49" t="n">
-        <f aca="false">S79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5915.41001822677</v>
+        <f aca="false">S79*założenia!$C$6</f>
+        <v>5952</v>
       </c>
       <c r="T173" s="49" t="n">
-        <f aca="false">T79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5915.41001822677</v>
+        <f aca="false">T79*założenia!$C$6</f>
+        <v>5952</v>
       </c>
       <c r="U173" s="49" t="n">
-        <f aca="false">U79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5915.41001822677</v>
+        <f aca="false">U79*założenia!$C$6</f>
+        <v>5952</v>
       </c>
       <c r="V173" s="49" t="n">
-        <f aca="false">V79*(założenia!$C$6-założenia!$C$19)</f>
-        <v>5915.41001822677</v>
+        <f aca="false">V79*założenia!$C$6</f>
+        <v>5952</v>
       </c>
       <c r="W173" s="49" t="n">
-        <f aca="false">W79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">W79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="X173" s="49" t="n">
-        <f aca="false">X79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">X79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Y173" s="49" t="n">
-        <f aca="false">Y79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Y79*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Z173" s="49" t="n">
-        <f aca="false">Z79*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Z79*założenia!$C$6</f>
         <v>0</v>
       </c>
     </row>
@@ -39195,98 +39209,98 @@
       </c>
       <c r="C174" s="49" t="n">
         <f aca="false">SUM(D174:Z174)</f>
-        <v>131188.528630029</v>
+        <v>132000</v>
       </c>
       <c r="D174" s="49" t="n">
-        <f aca="false">D80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">D80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="E174" s="49" t="n">
-        <f aca="false">E80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">E80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="F174" s="49" t="n">
-        <f aca="false">F80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">F80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="G174" s="49" t="n">
-        <f aca="false">G80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">G80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="H174" s="49" t="n">
-        <f aca="false">H80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">H80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="I174" s="49" t="n">
-        <f aca="false">I80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">I80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="J174" s="49" t="n">
-        <f aca="false">J80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">J80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="K174" s="49" t="n">
-        <f aca="false">K80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">K80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="L174" s="49" t="n">
-        <f aca="false">L80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">L80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="M174" s="49" t="n">
-        <f aca="false">M80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">M80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="N174" s="49" t="n">
-        <f aca="false">N80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">N80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="O174" s="49" t="n">
-        <f aca="false">O80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">O80*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="P174" s="49" t="n">
-        <f aca="false">P80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">P80*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="Q174" s="49" t="n">
-        <f aca="false">Q80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">Q80*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="R174" s="49" t="n">
-        <f aca="false">R80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">R80*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="S174" s="49" t="n">
-        <f aca="false">S80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">S80*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="T174" s="49" t="n">
-        <f aca="false">T80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">T80*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="U174" s="49" t="n">
-        <f aca="false">U80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">U80*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="V174" s="49" t="n">
-        <f aca="false">V80*(założenia!$C$6-założenia!$C$19)</f>
-        <v>16398.5660787537</v>
+        <f aca="false">V80*założenia!$C$6</f>
+        <v>16500</v>
       </c>
       <c r="W174" s="49" t="n">
-        <f aca="false">W80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">W80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="X174" s="49" t="n">
-        <f aca="false">X80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">X80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Y174" s="49" t="n">
-        <f aca="false">Y80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Y80*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Z174" s="49" t="n">
-        <f aca="false">Z80*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Z80*założenia!$C$6</f>
         <v>0</v>
       </c>
     </row>
@@ -39299,98 +39313,98 @@
       </c>
       <c r="C175" s="49" t="n">
         <f aca="false">SUM(D175:Z175)</f>
-        <v>31294.4271931997</v>
+        <v>31488</v>
       </c>
       <c r="D175" s="49" t="n">
-        <f aca="false">D81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">D81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="E175" s="49" t="n">
-        <f aca="false">E81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">E81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="F175" s="49" t="n">
-        <f aca="false">F81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">F81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="G175" s="49" t="n">
-        <f aca="false">G81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">G81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="H175" s="49" t="n">
-        <f aca="false">H81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">H81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="I175" s="49" t="n">
-        <f aca="false">I81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">I81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="J175" s="49" t="n">
-        <f aca="false">J81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">J81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="K175" s="49" t="n">
-        <f aca="false">K81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">K81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="L175" s="49" t="n">
-        <f aca="false">L81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">L81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="M175" s="49" t="n">
-        <f aca="false">M81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">M81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="N175" s="49" t="n">
-        <f aca="false">N81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">N81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="O175" s="49" t="n">
-        <f aca="false">O81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3911.80339914996</v>
+        <f aca="false">O81*założenia!$C$6</f>
+        <v>3936</v>
       </c>
       <c r="P175" s="49" t="n">
-        <f aca="false">P81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3911.80339914996</v>
+        <f aca="false">P81*założenia!$C$6</f>
+        <v>3936</v>
       </c>
       <c r="Q175" s="49" t="n">
-        <f aca="false">Q81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3911.80339914996</v>
+        <f aca="false">Q81*założenia!$C$6</f>
+        <v>3936</v>
       </c>
       <c r="R175" s="49" t="n">
-        <f aca="false">R81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3911.80339914996</v>
+        <f aca="false">R81*założenia!$C$6</f>
+        <v>3936</v>
       </c>
       <c r="S175" s="49" t="n">
-        <f aca="false">S81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3911.80339914996</v>
+        <f aca="false">S81*założenia!$C$6</f>
+        <v>3936</v>
       </c>
       <c r="T175" s="49" t="n">
-        <f aca="false">T81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3911.80339914996</v>
+        <f aca="false">T81*założenia!$C$6</f>
+        <v>3936</v>
       </c>
       <c r="U175" s="49" t="n">
-        <f aca="false">U81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3911.80339914996</v>
+        <f aca="false">U81*założenia!$C$6</f>
+        <v>3936</v>
       </c>
       <c r="V175" s="49" t="n">
-        <f aca="false">V81*(założenia!$C$6-założenia!$C$19)</f>
-        <v>3911.80339914996</v>
+        <f aca="false">V81*założenia!$C$6</f>
+        <v>3936</v>
       </c>
       <c r="W175" s="49" t="n">
-        <f aca="false">W81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">W81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="X175" s="49" t="n">
-        <f aca="false">X81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">X81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Y175" s="49" t="n">
-        <f aca="false">Y81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Y81*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Z175" s="49" t="n">
-        <f aca="false">Z81*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Z81*założenia!$C$6</f>
         <v>0</v>
       </c>
     </row>
@@ -39403,98 +39417,98 @@
       </c>
       <c r="C176" s="49" t="n">
         <f aca="false">SUM(D176:Z176)</f>
-        <v>4543.32112351517</v>
+        <v>4571.424</v>
       </c>
       <c r="D176" s="49" t="n">
-        <f aca="false">D82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">D82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="E176" s="49" t="n">
-        <f aca="false">E82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">E82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="F176" s="49" t="n">
-        <f aca="false">F82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">F82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="G176" s="49" t="n">
-        <f aca="false">G82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">G82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="H176" s="49" t="n">
-        <f aca="false">H82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">H82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="I176" s="49" t="n">
-        <f aca="false">I82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">I82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="J176" s="49" t="n">
-        <f aca="false">J82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">J82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="K176" s="49" t="n">
-        <f aca="false">K82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">K82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="L176" s="49" t="n">
-        <f aca="false">L82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">L82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="M176" s="49" t="n">
-        <f aca="false">M82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">M82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="N176" s="49" t="n">
-        <f aca="false">N82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">N82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="O176" s="49" t="n">
-        <f aca="false">O82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>567.915140439397</v>
+        <f aca="false">O82*założenia!$C$6</f>
+        <v>571.428</v>
       </c>
       <c r="P176" s="49" t="n">
-        <f aca="false">P82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>567.915140439397</v>
+        <f aca="false">P82*założenia!$C$6</f>
+        <v>571.428</v>
       </c>
       <c r="Q176" s="49" t="n">
-        <f aca="false">Q82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>567.915140439397</v>
+        <f aca="false">Q82*założenia!$C$6</f>
+        <v>571.428</v>
       </c>
       <c r="R176" s="49" t="n">
-        <f aca="false">R82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>567.915140439397</v>
+        <f aca="false">R82*założenia!$C$6</f>
+        <v>571.428</v>
       </c>
       <c r="S176" s="49" t="n">
-        <f aca="false">S82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>567.915140439397</v>
+        <f aca="false">S82*założenia!$C$6</f>
+        <v>571.428</v>
       </c>
       <c r="T176" s="49" t="n">
-        <f aca="false">T82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>567.915140439397</v>
+        <f aca="false">T82*założenia!$C$6</f>
+        <v>571.428</v>
       </c>
       <c r="U176" s="49" t="n">
-        <f aca="false">U82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>567.915140439397</v>
+        <f aca="false">U82*założenia!$C$6</f>
+        <v>571.428</v>
       </c>
       <c r="V176" s="49" t="n">
-        <f aca="false">V82*(założenia!$C$6-założenia!$C$19)</f>
-        <v>567.915140439397</v>
+        <f aca="false">V82*założenia!$C$6</f>
+        <v>571.428</v>
       </c>
       <c r="W176" s="49" t="n">
-        <f aca="false">W82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">W82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="X176" s="49" t="n">
-        <f aca="false">X82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">X82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Y176" s="49" t="n">
-        <f aca="false">Y82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Y82*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Z176" s="49" t="n">
-        <f aca="false">Z82*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Z82*założenia!$C$6</f>
         <v>0</v>
       </c>
     </row>
@@ -39507,98 +39521,98 @@
       </c>
       <c r="C177" s="49" t="n">
         <f aca="false">SUM(D177:Z177)</f>
-        <v>125622.954688149</v>
+        <v>126400</v>
       </c>
       <c r="D177" s="49" t="n">
-        <f aca="false">D83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">D83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="E177" s="49" t="n">
-        <f aca="false">E83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">E83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="F177" s="49" t="n">
-        <f aca="false">F83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">F83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="G177" s="49" t="n">
-        <f aca="false">G83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">G83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="H177" s="49" t="n">
-        <f aca="false">H83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">H83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="I177" s="49" t="n">
-        <f aca="false">I83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">I83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="J177" s="49" t="n">
-        <f aca="false">J83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">J83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="K177" s="49" t="n">
-        <f aca="false">K83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">K83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="L177" s="49" t="n">
-        <f aca="false">L83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">L83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="M177" s="49" t="n">
-        <f aca="false">M83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">M83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="N177" s="49" t="n">
-        <f aca="false">N83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">N83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="O177" s="49" t="n">
-        <f aca="false">O83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15702.8693360187</v>
+        <f aca="false">O83*założenia!$C$6</f>
+        <v>15800</v>
       </c>
       <c r="P177" s="49" t="n">
-        <f aca="false">P83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15702.8693360187</v>
+        <f aca="false">P83*założenia!$C$6</f>
+        <v>15800</v>
       </c>
       <c r="Q177" s="49" t="n">
-        <f aca="false">Q83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15702.8693360187</v>
+        <f aca="false">Q83*założenia!$C$6</f>
+        <v>15800</v>
       </c>
       <c r="R177" s="49" t="n">
-        <f aca="false">R83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15702.8693360187</v>
+        <f aca="false">R83*założenia!$C$6</f>
+        <v>15800</v>
       </c>
       <c r="S177" s="49" t="n">
-        <f aca="false">S83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15702.8693360187</v>
+        <f aca="false">S83*założenia!$C$6</f>
+        <v>15800</v>
       </c>
       <c r="T177" s="49" t="n">
-        <f aca="false">T83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15702.8693360187</v>
+        <f aca="false">T83*założenia!$C$6</f>
+        <v>15800</v>
       </c>
       <c r="U177" s="49" t="n">
-        <f aca="false">U83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15702.8693360187</v>
+        <f aca="false">U83*założenia!$C$6</f>
+        <v>15800</v>
       </c>
       <c r="V177" s="49" t="n">
-        <f aca="false">V83*(założenia!$C$6-założenia!$C$19)</f>
-        <v>15702.8693360187</v>
+        <f aca="false">V83*założenia!$C$6</f>
+        <v>15800</v>
       </c>
       <c r="W177" s="49" t="n">
-        <f aca="false">W83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">W83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="X177" s="49" t="n">
-        <f aca="false">X83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">X83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Y177" s="49" t="n">
-        <f aca="false">Y83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Y83*założenia!$C$6</f>
         <v>0</v>
       </c>
       <c r="Z177" s="49" t="n">
-        <f aca="false">Z83*(założenia!$C$6-założenia!$C$19)</f>
+        <f aca="false">Z83*założenia!$C$6</f>
         <v>0</v>
       </c>
     </row>
@@ -39611,99 +39625,99 @@
       </c>
       <c r="C178" s="49" t="n">
         <f aca="false">SUM(D178:Z178)</f>
-        <v>132960</v>
+        <v>130678.784927454</v>
       </c>
       <c r="D178" s="49" t="n">
-        <f aca="false">D84*założenia!$C$7</f>
+        <f aca="false">D84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="E178" s="49" t="n">
-        <f aca="false">E84*założenia!$C$7</f>
+        <f aca="false">E84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="F178" s="49" t="n">
-        <f aca="false">F84*założenia!$C$7</f>
+        <f aca="false">F84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="G178" s="49" t="n">
-        <f aca="false">G84*założenia!$C$7</f>
+        <f aca="false">G84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="H178" s="49" t="n">
-        <f aca="false">H84*założenia!$C$7</f>
+        <f aca="false">H84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="I178" s="49" t="n">
-        <f aca="false">I84*założenia!$C$7</f>
+        <f aca="false">I84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="J178" s="49" t="n">
-        <f aca="false">J84*założenia!$C$7</f>
+        <f aca="false">J84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="K178" s="49" t="n">
-        <f aca="false">K84*założenia!$C$7</f>
+        <f aca="false">K84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="L178" s="49" t="n">
-        <f aca="false">L84*założenia!$C$7</f>
+        <f aca="false">L84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="M178" s="49" t="n">
-        <f aca="false">M84*założenia!$C$7</f>
+        <f aca="false">M84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="N178" s="49" t="n">
-        <f aca="false">N84*założenia!$C$7</f>
+        <f aca="false">N84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="O178" s="49" t="n">
-        <f aca="false">O84*założenia!$C$7</f>
+        <f aca="false">O84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="P178" s="49" t="n">
-        <f aca="false">P84*założenia!$C$7</f>
+        <f aca="false">P84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="Q178" s="49" t="n">
-        <f aca="false">Q84*założenia!$C$7</f>
+        <f aca="false">Q84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="R178" s="49" t="n">
-        <f aca="false">R84*założenia!$C$7</f>
+        <f aca="false">R84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="S178" s="49" t="n">
-        <f aca="false">S84*założenia!$C$7</f>
+        <f aca="false">S84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="T178" s="49" t="n">
-        <f aca="false">T84*założenia!$C$7</f>
+        <f aca="false">T84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="U178" s="49" t="n">
-        <f aca="false">U84*założenia!$C$7</f>
+        <f aca="false">U84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="V178" s="49" t="n">
-        <f aca="false">V84*założenia!$C$7</f>
+        <f aca="false">V84*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="W178" s="49" t="n">
-        <f aca="false">W84*założenia!$C$7</f>
-        <v>33240</v>
+        <f aca="false">W84*(założenia!$C$7-założenia!$C$19)</f>
+        <v>32669.6962318634</v>
       </c>
       <c r="X178" s="49" t="n">
-        <f aca="false">X84*założenia!$C$7</f>
-        <v>33240</v>
+        <f aca="false">X84*(założenia!$C$7-założenia!$C$19)</f>
+        <v>32669.6962318634</v>
       </c>
       <c r="Y178" s="49" t="n">
-        <f aca="false">Y84*założenia!$C$7</f>
-        <v>33240</v>
+        <f aca="false">Y84*(założenia!$C$7-założenia!$C$19)</f>
+        <v>32669.6962318634</v>
       </c>
       <c r="Z178" s="49" t="n">
-        <f aca="false">Z84*założenia!$C$7</f>
-        <v>33240</v>
+        <f aca="false">Z84*(założenia!$C$7-założenia!$C$19)</f>
+        <v>32669.6962318634</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39715,99 +39729,99 @@
       </c>
       <c r="C179" s="49" t="n">
         <f aca="false">SUM(D179:Z179)</f>
-        <v>22632</v>
+        <v>22243.6993116586</v>
       </c>
       <c r="D179" s="49" t="n">
-        <f aca="false">D85*założenia!$C$7</f>
+        <f aca="false">D85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="E179" s="49" t="n">
-        <f aca="false">E85*założenia!$C$7</f>
+        <f aca="false">E85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="F179" s="49" t="n">
-        <f aca="false">F85*założenia!$C$7</f>
+        <f aca="false">F85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="G179" s="49" t="n">
-        <f aca="false">G85*założenia!$C$7</f>
+        <f aca="false">G85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="H179" s="49" t="n">
-        <f aca="false">H85*założenia!$C$7</f>
+        <f aca="false">H85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="I179" s="49" t="n">
-        <f aca="false">I85*założenia!$C$7</f>
+        <f aca="false">I85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="J179" s="49" t="n">
-        <f aca="false">J85*założenia!$C$7</f>
+        <f aca="false">J85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="K179" s="49" t="n">
-        <f aca="false">K85*założenia!$C$7</f>
+        <f aca="false">K85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="L179" s="49" t="n">
-        <f aca="false">L85*założenia!$C$7</f>
+        <f aca="false">L85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="M179" s="49" t="n">
-        <f aca="false">M85*założenia!$C$7</f>
+        <f aca="false">M85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="N179" s="49" t="n">
-        <f aca="false">N85*założenia!$C$7</f>
+        <f aca="false">N85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="O179" s="49" t="n">
-        <f aca="false">O85*założenia!$C$7</f>
+        <f aca="false">O85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="P179" s="49" t="n">
-        <f aca="false">P85*założenia!$C$7</f>
+        <f aca="false">P85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="Q179" s="49" t="n">
-        <f aca="false">Q85*założenia!$C$7</f>
+        <f aca="false">Q85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="R179" s="49" t="n">
-        <f aca="false">R85*założenia!$C$7</f>
+        <f aca="false">R85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="S179" s="49" t="n">
-        <f aca="false">S85*założenia!$C$7</f>
+        <f aca="false">S85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="T179" s="49" t="n">
-        <f aca="false">T85*założenia!$C$7</f>
+        <f aca="false">T85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="U179" s="49" t="n">
-        <f aca="false">U85*założenia!$C$7</f>
+        <f aca="false">U85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="V179" s="49" t="n">
-        <f aca="false">V85*założenia!$C$7</f>
+        <f aca="false">V85*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="W179" s="49" t="n">
-        <f aca="false">W85*założenia!$C$7</f>
-        <v>5658</v>
+        <f aca="false">W85*(założenia!$C$7-założenia!$C$19)</f>
+        <v>5560.92482791466</v>
       </c>
       <c r="X179" s="49" t="n">
-        <f aca="false">X85*założenia!$C$7</f>
-        <v>5658</v>
+        <f aca="false">X85*(założenia!$C$7-założenia!$C$19)</f>
+        <v>5560.92482791466</v>
       </c>
       <c r="Y179" s="49" t="n">
-        <f aca="false">Y85*założenia!$C$7</f>
-        <v>5658</v>
+        <f aca="false">Y85*(założenia!$C$7-założenia!$C$19)</f>
+        <v>5560.92482791466</v>
       </c>
       <c r="Z179" s="49" t="n">
-        <f aca="false">Z85*założenia!$C$7</f>
-        <v>5658</v>
+        <f aca="false">Z85*(założenia!$C$7-założenia!$C$19)</f>
+        <v>5560.92482791466</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39819,99 +39833,99 @@
       </c>
       <c r="C180" s="49" t="n">
         <f aca="false">SUM(D180:Z180)</f>
-        <v>65064</v>
+        <v>63947.6869924778</v>
       </c>
       <c r="D180" s="49" t="n">
-        <f aca="false">D86*założenia!$C$7</f>
+        <f aca="false">D86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="E180" s="49" t="n">
-        <f aca="false">E86*założenia!$C$7</f>
+        <f aca="false">E86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="F180" s="49" t="n">
-        <f aca="false">F86*założenia!$C$7</f>
+        <f aca="false">F86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="G180" s="49" t="n">
-        <f aca="false">G86*założenia!$C$7</f>
+        <f aca="false">G86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="H180" s="49" t="n">
-        <f aca="false">H86*założenia!$C$7</f>
+        <f aca="false">H86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="I180" s="49" t="n">
-        <f aca="false">I86*założenia!$C$7</f>
+        <f aca="false">I86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="J180" s="49" t="n">
-        <f aca="false">J86*założenia!$C$7</f>
+        <f aca="false">J86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="K180" s="49" t="n">
-        <f aca="false">K86*założenia!$C$7</f>
+        <f aca="false">K86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="L180" s="49" t="n">
-        <f aca="false">L86*założenia!$C$7</f>
+        <f aca="false">L86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="M180" s="49" t="n">
-        <f aca="false">M86*założenia!$C$7</f>
+        <f aca="false">M86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="N180" s="49" t="n">
-        <f aca="false">N86*założenia!$C$7</f>
+        <f aca="false">N86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="O180" s="49" t="n">
-        <f aca="false">O86*założenia!$C$7</f>
+        <f aca="false">O86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="P180" s="49" t="n">
-        <f aca="false">P86*założenia!$C$7</f>
+        <f aca="false">P86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="Q180" s="49" t="n">
-        <f aca="false">Q86*założenia!$C$7</f>
+        <f aca="false">Q86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="R180" s="49" t="n">
-        <f aca="false">R86*założenia!$C$7</f>
+        <f aca="false">R86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="S180" s="49" t="n">
-        <f aca="false">S86*założenia!$C$7</f>
+        <f aca="false">S86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="T180" s="49" t="n">
-        <f aca="false">T86*założenia!$C$7</f>
+        <f aca="false">T86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="U180" s="49" t="n">
-        <f aca="false">U86*założenia!$C$7</f>
+        <f aca="false">U86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="V180" s="49" t="n">
-        <f aca="false">V86*założenia!$C$7</f>
+        <f aca="false">V86*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="W180" s="49" t="n">
-        <f aca="false">W86*założenia!$C$7</f>
-        <v>16266</v>
+        <f aca="false">W86*(założenia!$C$7-założenia!$C$19)</f>
+        <v>15986.9217481194</v>
       </c>
       <c r="X180" s="49" t="n">
-        <f aca="false">X86*założenia!$C$7</f>
-        <v>16266</v>
+        <f aca="false">X86*(założenia!$C$7-założenia!$C$19)</f>
+        <v>15986.9217481194</v>
       </c>
       <c r="Y180" s="49" t="n">
-        <f aca="false">Y86*założenia!$C$7</f>
-        <v>16266</v>
+        <f aca="false">Y86*(założenia!$C$7-założenia!$C$19)</f>
+        <v>15986.9217481194</v>
       </c>
       <c r="Z180" s="49" t="n">
-        <f aca="false">Z86*założenia!$C$7</f>
-        <v>16266</v>
+        <f aca="false">Z86*(założenia!$C$7-założenia!$C$19)</f>
+        <v>15986.9217481194</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39923,99 +39937,99 @@
       </c>
       <c r="C181" s="49" t="n">
         <f aca="false">SUM(D181:Z181)</f>
-        <v>49500</v>
+        <v>48650.7209229013</v>
       </c>
       <c r="D181" s="49" t="n">
-        <f aca="false">D87*założenia!$C$7</f>
+        <f aca="false">D87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="E181" s="49" t="n">
-        <f aca="false">E87*założenia!$C$7</f>
+        <f aca="false">E87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="F181" s="49" t="n">
-        <f aca="false">F87*założenia!$C$7</f>
+        <f aca="false">F87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="G181" s="49" t="n">
-        <f aca="false">G87*założenia!$C$7</f>
+        <f aca="false">G87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="H181" s="49" t="n">
-        <f aca="false">H87*założenia!$C$7</f>
+        <f aca="false">H87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="I181" s="49" t="n">
-        <f aca="false">I87*założenia!$C$7</f>
+        <f aca="false">I87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="J181" s="49" t="n">
-        <f aca="false">J87*założenia!$C$7</f>
+        <f aca="false">J87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="K181" s="49" t="n">
-        <f aca="false">K87*założenia!$C$7</f>
+        <f aca="false">K87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="L181" s="49" t="n">
-        <f aca="false">L87*założenia!$C$7</f>
+        <f aca="false">L87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="M181" s="49" t="n">
-        <f aca="false">M87*założenia!$C$7</f>
+        <f aca="false">M87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="N181" s="49" t="n">
-        <f aca="false">N87*założenia!$C$7</f>
+        <f aca="false">N87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="O181" s="49" t="n">
-        <f aca="false">O87*założenia!$C$7</f>
+        <f aca="false">O87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="P181" s="49" t="n">
-        <f aca="false">P87*założenia!$C$7</f>
+        <f aca="false">P87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="Q181" s="49" t="n">
-        <f aca="false">Q87*założenia!$C$7</f>
+        <f aca="false">Q87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="R181" s="49" t="n">
-        <f aca="false">R87*założenia!$C$7</f>
+        <f aca="false">R87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="S181" s="49" t="n">
-        <f aca="false">S87*założenia!$C$7</f>
+        <f aca="false">S87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="T181" s="49" t="n">
-        <f aca="false">T87*założenia!$C$7</f>
+        <f aca="false">T87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="U181" s="49" t="n">
-        <f aca="false">U87*założenia!$C$7</f>
+        <f aca="false">U87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="V181" s="49" t="n">
-        <f aca="false">V87*założenia!$C$7</f>
+        <f aca="false">V87*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="W181" s="49" t="n">
-        <f aca="false">W87*założenia!$C$7</f>
-        <v>12375</v>
+        <f aca="false">W87*(założenia!$C$7-założenia!$C$19)</f>
+        <v>12162.6802307253</v>
       </c>
       <c r="X181" s="49" t="n">
-        <f aca="false">X87*założenia!$C$7</f>
-        <v>12375</v>
+        <f aca="false">X87*(założenia!$C$7-założenia!$C$19)</f>
+        <v>12162.6802307253</v>
       </c>
       <c r="Y181" s="49" t="n">
-        <f aca="false">Y87*założenia!$C$7</f>
-        <v>12375</v>
+        <f aca="false">Y87*(założenia!$C$7-założenia!$C$19)</f>
+        <v>12162.6802307253</v>
       </c>
       <c r="Z181" s="49" t="n">
-        <f aca="false">Z87*założenia!$C$7</f>
-        <v>12375</v>
+        <f aca="false">Z87*(założenia!$C$7-założenia!$C$19)</f>
+        <v>12162.6802307253</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40027,99 +40041,99 @@
       </c>
       <c r="C182" s="49" t="n">
         <f aca="false">SUM(D182:Z182)</f>
-        <v>17856</v>
+        <v>17549.6418747338</v>
       </c>
       <c r="D182" s="49" t="n">
-        <f aca="false">D88*założenia!$C$7</f>
+        <f aca="false">D88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="E182" s="49" t="n">
-        <f aca="false">E88*założenia!$C$7</f>
+        <f aca="false">E88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="F182" s="49" t="n">
-        <f aca="false">F88*założenia!$C$7</f>
+        <f aca="false">F88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="G182" s="49" t="n">
-        <f aca="false">G88*założenia!$C$7</f>
+        <f aca="false">G88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="H182" s="49" t="n">
-        <f aca="false">H88*założenia!$C$7</f>
+        <f aca="false">H88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="I182" s="49" t="n">
-        <f aca="false">I88*założenia!$C$7</f>
+        <f aca="false">I88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="J182" s="49" t="n">
-        <f aca="false">J88*założenia!$C$7</f>
+        <f aca="false">J88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="K182" s="49" t="n">
-        <f aca="false">K88*założenia!$C$7</f>
+        <f aca="false">K88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="L182" s="49" t="n">
-        <f aca="false">L88*założenia!$C$7</f>
+        <f aca="false">L88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="M182" s="49" t="n">
-        <f aca="false">M88*założenia!$C$7</f>
+        <f aca="false">M88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="N182" s="49" t="n">
-        <f aca="false">N88*założenia!$C$7</f>
+        <f aca="false">N88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="O182" s="49" t="n">
-        <f aca="false">O88*założenia!$C$7</f>
+        <f aca="false">O88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="P182" s="49" t="n">
-        <f aca="false">P88*założenia!$C$7</f>
+        <f aca="false">P88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="Q182" s="49" t="n">
-        <f aca="false">Q88*założenia!$C$7</f>
+        <f aca="false">Q88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="R182" s="49" t="n">
-        <f aca="false">R88*założenia!$C$7</f>
+        <f aca="false">R88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="S182" s="49" t="n">
-        <f aca="false">S88*założenia!$C$7</f>
+        <f aca="false">S88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="T182" s="49" t="n">
-        <f aca="false">T88*założenia!$C$7</f>
+        <f aca="false">T88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="U182" s="49" t="n">
-        <f aca="false">U88*założenia!$C$7</f>
+        <f aca="false">U88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="V182" s="49" t="n">
-        <f aca="false">V88*założenia!$C$7</f>
+        <f aca="false">V88*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="W182" s="49" t="n">
-        <f aca="false">W88*założenia!$C$7</f>
-        <v>4464</v>
+        <f aca="false">W88*(założenia!$C$7-założenia!$C$19)</f>
+        <v>4387.41046868346</v>
       </c>
       <c r="X182" s="49" t="n">
-        <f aca="false">X88*założenia!$C$7</f>
-        <v>4464</v>
+        <f aca="false">X88*(założenia!$C$7-założenia!$C$19)</f>
+        <v>4387.41046868346</v>
       </c>
       <c r="Y182" s="49" t="n">
-        <f aca="false">Y88*założenia!$C$7</f>
-        <v>4464</v>
+        <f aca="false">Y88*(założenia!$C$7-założenia!$C$19)</f>
+        <v>4387.41046868346</v>
       </c>
       <c r="Z182" s="49" t="n">
-        <f aca="false">Z88*założenia!$C$7</f>
-        <v>4464</v>
+        <f aca="false">Z88*(założenia!$C$7-założenia!$C$19)</f>
+        <v>4387.41046868346</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40131,99 +40145,99 @@
       </c>
       <c r="C183" s="49" t="n">
         <f aca="false">SUM(D183:Z183)</f>
-        <v>49500</v>
+        <v>48650.7209229013</v>
       </c>
       <c r="D183" s="49" t="n">
-        <f aca="false">D89*założenia!$C$7</f>
+        <f aca="false">D89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="E183" s="49" t="n">
-        <f aca="false">E89*założenia!$C$7</f>
+        <f aca="false">E89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="F183" s="49" t="n">
-        <f aca="false">F89*założenia!$C$7</f>
+        <f aca="false">F89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="G183" s="49" t="n">
-        <f aca="false">G89*założenia!$C$7</f>
+        <f aca="false">G89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="H183" s="49" t="n">
-        <f aca="false">H89*założenia!$C$7</f>
+        <f aca="false">H89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="I183" s="49" t="n">
-        <f aca="false">I89*założenia!$C$7</f>
+        <f aca="false">I89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="J183" s="49" t="n">
-        <f aca="false">J89*założenia!$C$7</f>
+        <f aca="false">J89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="K183" s="49" t="n">
-        <f aca="false">K89*założenia!$C$7</f>
+        <f aca="false">K89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="L183" s="49" t="n">
-        <f aca="false">L89*założenia!$C$7</f>
+        <f aca="false">L89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="M183" s="49" t="n">
-        <f aca="false">M89*założenia!$C$7</f>
+        <f aca="false">M89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="N183" s="49" t="n">
-        <f aca="false">N89*założenia!$C$7</f>
+        <f aca="false">N89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="O183" s="49" t="n">
-        <f aca="false">O89*założenia!$C$7</f>
+        <f aca="false">O89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="P183" s="49" t="n">
-        <f aca="false">P89*założenia!$C$7</f>
+        <f aca="false">P89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="Q183" s="49" t="n">
-        <f aca="false">Q89*założenia!$C$7</f>
+        <f aca="false">Q89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="R183" s="49" t="n">
-        <f aca="false">R89*założenia!$C$7</f>
+        <f aca="false">R89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="S183" s="49" t="n">
-        <f aca="false">S89*założenia!$C$7</f>
+        <f aca="false">S89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="T183" s="49" t="n">
-        <f aca="false">T89*założenia!$C$7</f>
+        <f aca="false">T89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="U183" s="49" t="n">
-        <f aca="false">U89*założenia!$C$7</f>
+        <f aca="false">U89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="V183" s="49" t="n">
-        <f aca="false">V89*założenia!$C$7</f>
+        <f aca="false">V89*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="W183" s="49" t="n">
-        <f aca="false">W89*założenia!$C$7</f>
-        <v>12375</v>
+        <f aca="false">W89*(założenia!$C$7-założenia!$C$19)</f>
+        <v>12162.6802307253</v>
       </c>
       <c r="X183" s="49" t="n">
-        <f aca="false">X89*założenia!$C$7</f>
-        <v>12375</v>
+        <f aca="false">X89*(założenia!$C$7-założenia!$C$19)</f>
+        <v>12162.6802307253</v>
       </c>
       <c r="Y183" s="49" t="n">
-        <f aca="false">Y89*założenia!$C$7</f>
-        <v>12375</v>
+        <f aca="false">Y89*(założenia!$C$7-założenia!$C$19)</f>
+        <v>12162.6802307253</v>
       </c>
       <c r="Z183" s="49" t="n">
-        <f aca="false">Z89*założenia!$C$7</f>
-        <v>12375</v>
+        <f aca="false">Z89*(założenia!$C$7-założenia!$C$19)</f>
+        <v>12162.6802307253</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40235,99 +40249,99 @@
       </c>
       <c r="C184" s="49" t="n">
         <f aca="false">SUM(D184:Z184)</f>
-        <v>1714.284</v>
+        <v>1684.87176700192</v>
       </c>
       <c r="D184" s="49" t="n">
-        <f aca="false">D90*założenia!$C$7</f>
+        <f aca="false">D90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="E184" s="49" t="n">
-        <f aca="false">E90*założenia!$C$7</f>
+        <f aca="false">E90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="F184" s="49" t="n">
-        <f aca="false">F90*założenia!$C$7</f>
+        <f aca="false">F90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="G184" s="49" t="n">
-        <f aca="false">G90*założenia!$C$7</f>
+        <f aca="false">G90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="H184" s="49" t="n">
-        <f aca="false">H90*założenia!$C$7</f>
+        <f aca="false">H90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="I184" s="49" t="n">
-        <f aca="false">I90*założenia!$C$7</f>
+        <f aca="false">I90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="J184" s="49" t="n">
-        <f aca="false">J90*założenia!$C$7</f>
+        <f aca="false">J90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="K184" s="49" t="n">
-        <f aca="false">K90*założenia!$C$7</f>
+        <f aca="false">K90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="L184" s="49" t="n">
-        <f aca="false">L90*założenia!$C$7</f>
+        <f aca="false">L90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="M184" s="49" t="n">
-        <f aca="false">M90*założenia!$C$7</f>
+        <f aca="false">M90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="N184" s="49" t="n">
-        <f aca="false">N90*założenia!$C$7</f>
+        <f aca="false">N90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="O184" s="49" t="n">
-        <f aca="false">O90*założenia!$C$7</f>
+        <f aca="false">O90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="P184" s="49" t="n">
-        <f aca="false">P90*założenia!$C$7</f>
+        <f aca="false">P90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="Q184" s="49" t="n">
-        <f aca="false">Q90*założenia!$C$7</f>
+        <f aca="false">Q90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="R184" s="49" t="n">
-        <f aca="false">R90*założenia!$C$7</f>
+        <f aca="false">R90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="S184" s="49" t="n">
-        <f aca="false">S90*założenia!$C$7</f>
+        <f aca="false">S90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="T184" s="49" t="n">
-        <f aca="false">T90*założenia!$C$7</f>
+        <f aca="false">T90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="U184" s="49" t="n">
-        <f aca="false">U90*założenia!$C$7</f>
+        <f aca="false">U90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="V184" s="49" t="n">
-        <f aca="false">V90*założenia!$C$7</f>
+        <f aca="false">V90*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="W184" s="49" t="n">
-        <f aca="false">W90*założenia!$C$7</f>
-        <v>428.571</v>
+        <f aca="false">W90*(założenia!$C$7-założenia!$C$19)</f>
+        <v>421.217941750479</v>
       </c>
       <c r="X184" s="49" t="n">
-        <f aca="false">X90*założenia!$C$7</f>
-        <v>428.571</v>
+        <f aca="false">X90*(założenia!$C$7-założenia!$C$19)</f>
+        <v>421.217941750479</v>
       </c>
       <c r="Y184" s="49" t="n">
-        <f aca="false">Y90*założenia!$C$7</f>
-        <v>428.571</v>
+        <f aca="false">Y90*(założenia!$C$7-założenia!$C$19)</f>
+        <v>421.217941750479</v>
       </c>
       <c r="Z184" s="49" t="n">
-        <f aca="false">Z90*założenia!$C$7</f>
-        <v>428.571</v>
+        <f aca="false">Z90*(założenia!$C$7-założenia!$C$19)</f>
+        <v>421.217941750479</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40339,99 +40353,99 @@
       </c>
       <c r="C185" s="49" t="n">
         <f aca="false">SUM(D185:Z185)</f>
-        <v>47400</v>
+        <v>46586.750944354</v>
       </c>
       <c r="D185" s="49" t="n">
-        <f aca="false">D91*założenia!$C$7</f>
+        <f aca="false">D91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="E185" s="49" t="n">
-        <f aca="false">E91*założenia!$C$7</f>
+        <f aca="false">E91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="F185" s="49" t="n">
-        <f aca="false">F91*założenia!$C$7</f>
+        <f aca="false">F91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="G185" s="49" t="n">
-        <f aca="false">G91*założenia!$C$7</f>
+        <f aca="false">G91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="H185" s="49" t="n">
-        <f aca="false">H91*założenia!$C$7</f>
+        <f aca="false">H91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="I185" s="49" t="n">
-        <f aca="false">I91*założenia!$C$7</f>
+        <f aca="false">I91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="J185" s="49" t="n">
-        <f aca="false">J91*założenia!$C$7</f>
+        <f aca="false">J91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="K185" s="49" t="n">
-        <f aca="false">K91*założenia!$C$7</f>
+        <f aca="false">K91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="L185" s="49" t="n">
-        <f aca="false">L91*założenia!$C$7</f>
+        <f aca="false">L91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="M185" s="49" t="n">
-        <f aca="false">M91*założenia!$C$7</f>
+        <f aca="false">M91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="N185" s="49" t="n">
-        <f aca="false">N91*założenia!$C$7</f>
+        <f aca="false">N91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="O185" s="49" t="n">
-        <f aca="false">O91*założenia!$C$7</f>
+        <f aca="false">O91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="P185" s="49" t="n">
-        <f aca="false">P91*założenia!$C$7</f>
+        <f aca="false">P91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="Q185" s="49" t="n">
-        <f aca="false">Q91*założenia!$C$7</f>
+        <f aca="false">Q91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="R185" s="49" t="n">
-        <f aca="false">R91*założenia!$C$7</f>
+        <f aca="false">R91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="S185" s="49" t="n">
-        <f aca="false">S91*założenia!$C$7</f>
+        <f aca="false">S91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="T185" s="49" t="n">
-        <f aca="false">T91*założenia!$C$7</f>
+        <f aca="false">T91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="U185" s="49" t="n">
-        <f aca="false">U91*założenia!$C$7</f>
+        <f aca="false">U91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="V185" s="49" t="n">
-        <f aca="false">V91*założenia!$C$7</f>
+        <f aca="false">V91*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="W185" s="49" t="n">
-        <f aca="false">W91*założenia!$C$7</f>
-        <v>11850</v>
+        <f aca="false">W91*(założenia!$C$7-założenia!$C$19)</f>
+        <v>11646.6877360885</v>
       </c>
       <c r="X185" s="49" t="n">
-        <f aca="false">X91*założenia!$C$7</f>
-        <v>11850</v>
+        <f aca="false">X91*(założenia!$C$7-założenia!$C$19)</f>
+        <v>11646.6877360885</v>
       </c>
       <c r="Y185" s="49" t="n">
-        <f aca="false">Y91*założenia!$C$7</f>
-        <v>11850</v>
+        <f aca="false">Y91*(założenia!$C$7-założenia!$C$19)</f>
+        <v>11646.6877360885</v>
       </c>
       <c r="Z185" s="49" t="n">
-        <f aca="false">Z91*założenia!$C$7</f>
-        <v>11850</v>
+        <f aca="false">Z91*(założenia!$C$7-założenia!$C$19)</f>
+        <v>11646.6877360885</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40443,104 +40457,104 @@
       </c>
       <c r="C186" s="49" t="n">
         <f aca="false">SUM(D186:Z186)</f>
-        <v>11808</v>
+        <v>11605.4083365175</v>
       </c>
       <c r="D186" s="49" t="n">
-        <f aca="false">D92*założenia!$C$7</f>
+        <f aca="false">D92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="E186" s="49" t="n">
-        <f aca="false">E92*założenia!$C$7</f>
+        <f aca="false">E92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="F186" s="49" t="n">
-        <f aca="false">F92*założenia!$C$7</f>
+        <f aca="false">F92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="G186" s="49" t="n">
-        <f aca="false">G92*założenia!$C$7</f>
+        <f aca="false">G92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="H186" s="49" t="n">
-        <f aca="false">H92*założenia!$C$7</f>
+        <f aca="false">H92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="I186" s="49" t="n">
-        <f aca="false">I92*założenia!$C$7</f>
+        <f aca="false">I92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="J186" s="49" t="n">
-        <f aca="false">J92*założenia!$C$7</f>
+        <f aca="false">J92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="K186" s="49" t="n">
-        <f aca="false">K92*założenia!$C$7</f>
+        <f aca="false">K92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="L186" s="49" t="n">
-        <f aca="false">L92*założenia!$C$7</f>
+        <f aca="false">L92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="M186" s="49" t="n">
-        <f aca="false">M92*założenia!$C$7</f>
+        <f aca="false">M92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="N186" s="49" t="n">
-        <f aca="false">N92*założenia!$C$7</f>
+        <f aca="false">N92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="O186" s="49" t="n">
-        <f aca="false">O92*założenia!$C$7</f>
+        <f aca="false">O92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="P186" s="49" t="n">
-        <f aca="false">P92*założenia!$C$7</f>
+        <f aca="false">P92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="Q186" s="49" t="n">
-        <f aca="false">Q92*założenia!$C$7</f>
+        <f aca="false">Q92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="R186" s="49" t="n">
-        <f aca="false">R92*założenia!$C$7</f>
+        <f aca="false">R92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="S186" s="49" t="n">
-        <f aca="false">S92*założenia!$C$7</f>
+        <f aca="false">S92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="T186" s="49" t="n">
-        <f aca="false">T92*założenia!$C$7</f>
+        <f aca="false">T92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="U186" s="49" t="n">
-        <f aca="false">U92*założenia!$C$7</f>
+        <f aca="false">U92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="V186" s="49" t="n">
-        <f aca="false">V92*założenia!$C$7</f>
+        <f aca="false">V92*(założenia!$C$7-założenia!$C$19)</f>
         <v>0</v>
       </c>
       <c r="W186" s="49" t="n">
-        <f aca="false">W92*założenia!$C$7</f>
-        <v>2952</v>
+        <f aca="false">W92*(założenia!$C$7-założenia!$C$19)</f>
+        <v>2901.35208412939</v>
       </c>
       <c r="X186" s="49" t="n">
-        <f aca="false">X92*założenia!$C$7</f>
-        <v>2952</v>
+        <f aca="false">X92*(założenia!$C$7-założenia!$C$19)</f>
+        <v>2901.35208412939</v>
       </c>
       <c r="Y186" s="49" t="n">
-        <f aca="false">Y92*założenia!$C$7</f>
-        <v>2952</v>
+        <f aca="false">Y92*(założenia!$C$7-założenia!$C$19)</f>
+        <v>2901.35208412939</v>
       </c>
       <c r="Z186" s="49" t="n">
-        <f aca="false">Z92*założenia!$C$7</f>
-        <v>2952</v>
+        <f aca="false">Z92*(założenia!$C$7-założenia!$C$19)</f>
+        <v>2901.35208412939</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="40" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B187" s="40" t="n">
         <v>1</v>
@@ -40644,14 +40658,14 @@
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="40" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B188" s="40" t="n">
         <v>2</v>
       </c>
       <c r="C188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,C$150:C$186)</f>
-        <v>810408.96</v>
+        <v>810408.93</v>
       </c>
       <c r="D188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,D$150:D$186)</f>
@@ -40675,27 +40689,27 @@
       </c>
       <c r="I188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,I$150:I$186)</f>
-        <v>134502.571666667</v>
+        <v>134770.518333333</v>
       </c>
       <c r="J188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,J$150:J$186)</f>
-        <v>134502.571666667</v>
+        <v>134770.518333333</v>
       </c>
       <c r="K188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,K$150:K$186)</f>
-        <v>134502.571666667</v>
+        <v>134770.518333333</v>
       </c>
       <c r="L188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,L$150:L$186)</f>
-        <v>134502.571666667</v>
+        <v>134770.518333333</v>
       </c>
       <c r="M188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,M$150:M$186)</f>
-        <v>134502.571666667</v>
+        <v>134770.518333333</v>
       </c>
       <c r="N188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,N$150:N$186)</f>
-        <v>137896.101666667</v>
+        <v>136556.338333333</v>
       </c>
       <c r="O188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,O$150:O$186)</f>
@@ -40748,14 +40762,14 @@
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="40" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B189" s="40" t="n">
         <v>3</v>
       </c>
       <c r="C189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,C$150:C$186)</f>
-        <v>1105163.396</v>
+        <v>1111999.424</v>
       </c>
       <c r="D189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,D$150:D$186)</f>
@@ -40803,35 +40817,35 @@
       </c>
       <c r="O189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,O$150:O$186)</f>
-        <v>134103.923350954</v>
+        <v>134933.428</v>
       </c>
       <c r="P189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,P$150:P$186)</f>
-        <v>134103.923350954</v>
+        <v>134933.428</v>
       </c>
       <c r="Q189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,Q$150:Q$186)</f>
-        <v>139492.591549682</v>
+        <v>140355.428</v>
       </c>
       <c r="R189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,R$150:R$186)</f>
-        <v>139492.591549682</v>
+        <v>140355.428</v>
       </c>
       <c r="S189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,S$150:S$186)</f>
-        <v>139492.591549682</v>
+        <v>140355.428</v>
       </c>
       <c r="T189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,T$150:T$186)</f>
-        <v>139492.591549682</v>
+        <v>140355.428</v>
       </c>
       <c r="U189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,U$150:U$186)</f>
-        <v>139492.591549682</v>
+        <v>140355.428</v>
       </c>
       <c r="V189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,V$150:V$186)</f>
-        <v>139492.591549682</v>
+        <v>140355.428</v>
       </c>
       <c r="W189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,W$150:W$186)</f>
@@ -40852,14 +40866,14 @@
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="40" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B190" s="40" t="n">
         <v>4</v>
       </c>
       <c r="C190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,C$150:C$186)</f>
-        <v>398434.284</v>
+        <v>391598.286</v>
       </c>
       <c r="D190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,D$150:D$186)</f>
@@ -40939,19 +40953,19 @@
       </c>
       <c r="W190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,W$150:W$186)</f>
-        <v>99608.571</v>
+        <v>97899.5715</v>
       </c>
       <c r="X190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,X$150:X$186)</f>
-        <v>99608.571</v>
+        <v>97899.5715</v>
       </c>
       <c r="Y190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,Y$150:Y$186)</f>
-        <v>99608.571</v>
+        <v>97899.5715</v>
       </c>
       <c r="Z190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,Z$150:Z$186)</f>
-        <v>99608.571</v>
+        <v>97899.5715</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40985,80 +40999,80 @@
       </c>
       <c r="I191" s="63" t="n">
         <f aca="false">SUM(I187:I190)</f>
-        <v>134502.571666667</v>
+        <v>134770.518333333</v>
       </c>
       <c r="J191" s="63" t="n">
         <f aca="false">SUM(J187:J190)</f>
-        <v>134502.571666667</v>
+        <v>134770.518333333</v>
       </c>
       <c r="K191" s="63" t="n">
         <f aca="false">SUM(K187:K190)</f>
-        <v>134502.571666667</v>
+        <v>134770.518333333</v>
       </c>
       <c r="L191" s="63" t="n">
         <f aca="false">SUM(L187:L190)</f>
-        <v>134502.571666667</v>
+        <v>134770.518333333</v>
       </c>
       <c r="M191" s="63" t="n">
         <f aca="false">SUM(M187:M190)</f>
-        <v>134502.571666667</v>
+        <v>134770.518333333</v>
       </c>
       <c r="N191" s="63" t="n">
         <f aca="false">SUM(N187:N190)</f>
-        <v>137896.101666667</v>
+        <v>136556.338333333</v>
       </c>
       <c r="O191" s="63" t="n">
         <f aca="false">SUM(O187:O190)</f>
-        <v>134103.923350954</v>
+        <v>134933.428</v>
       </c>
       <c r="P191" s="63" t="n">
         <f aca="false">SUM(P187:P190)</f>
-        <v>134103.923350954</v>
+        <v>134933.428</v>
       </c>
       <c r="Q191" s="63" t="n">
         <f aca="false">SUM(Q187:Q190)</f>
-        <v>139492.591549682</v>
+        <v>140355.428</v>
       </c>
       <c r="R191" s="63" t="n">
         <f aca="false">SUM(R187:R190)</f>
-        <v>139492.591549682</v>
+        <v>140355.428</v>
       </c>
       <c r="S191" s="63" t="n">
         <f aca="false">SUM(S187:S190)</f>
-        <v>139492.591549682</v>
+        <v>140355.428</v>
       </c>
       <c r="T191" s="63" t="n">
         <f aca="false">SUM(T187:T190)</f>
-        <v>139492.591549682</v>
+        <v>140355.428</v>
       </c>
       <c r="U191" s="63" t="n">
         <f aca="false">SUM(U187:U190)</f>
-        <v>139492.591549682</v>
+        <v>140355.428</v>
       </c>
       <c r="V191" s="63" t="n">
         <f aca="false">SUM(V187:V190)</f>
-        <v>139492.591549682</v>
+        <v>140355.428</v>
       </c>
       <c r="W191" s="63" t="n">
         <f aca="false">SUM(W187:W190)</f>
-        <v>99608.571</v>
+        <v>97899.5715</v>
       </c>
       <c r="X191" s="63" t="n">
         <f aca="false">SUM(X187:X190)</f>
-        <v>99608.571</v>
+        <v>97899.5715</v>
       </c>
       <c r="Y191" s="63" t="n">
         <f aca="false">SUM(Y187:Y190)</f>
-        <v>99608.571</v>
+        <v>97899.5715</v>
       </c>
       <c r="Z191" s="63" t="n">
         <f aca="false">SUM(Z187:Z190)</f>
-        <v>99608.571</v>
+        <v>97899.5715</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="40" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B192" s="40"/>
       <c r="C192" s="63" t="n">
@@ -41087,27 +41101,27 @@
       </c>
       <c r="I192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,I98*$C$191/$C$97)</f>
-        <v>32110.6912421468</v>
+        <v>32174.6608822624</v>
       </c>
       <c r="J192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,J98*$C$191/$C$97)</f>
-        <v>32110.6912421468</v>
+        <v>32174.6608822624</v>
       </c>
       <c r="K192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,K98*$C$191/$C$97)</f>
-        <v>32110.6912421468</v>
+        <v>32174.6608822624</v>
       </c>
       <c r="L192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,L98*$C$191/$C$97)</f>
-        <v>32110.6912421468</v>
+        <v>32174.6608822624</v>
       </c>
       <c r="M192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,M98*$C$191/$C$97)</f>
-        <v>32110.6912421468</v>
+        <v>32174.6608822624</v>
       </c>
       <c r="N192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,N98*$C$191/$C$97)</f>
-        <v>32920.8506927005</v>
+        <v>32601.0024921226</v>
       </c>
       <c r="O192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,O98*$C$191/$C$97)</f>
@@ -41160,7 +41174,7 @@
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="40" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B193" s="40"/>
       <c r="C193" s="63" t="n">
@@ -41189,80 +41203,80 @@
       </c>
       <c r="I193" s="63" t="n">
         <f aca="false">I191+I192</f>
-        <v>166613.262908813</v>
+        <v>166945.179215596</v>
       </c>
       <c r="J193" s="63" t="n">
         <f aca="false">J191+J192</f>
-        <v>166613.262908813</v>
+        <v>166945.179215596</v>
       </c>
       <c r="K193" s="63" t="n">
         <f aca="false">K191+K192</f>
-        <v>166613.262908813</v>
+        <v>166945.179215596</v>
       </c>
       <c r="L193" s="63" t="n">
         <f aca="false">L191+L192</f>
-        <v>166613.262908813</v>
+        <v>166945.179215596</v>
       </c>
       <c r="M193" s="63" t="n">
         <f aca="false">M191+M192</f>
-        <v>166613.262908813</v>
+        <v>166945.179215596</v>
       </c>
       <c r="N193" s="63" t="n">
         <f aca="false">N191+N192</f>
-        <v>170816.952359367</v>
+        <v>169157.340825456</v>
       </c>
       <c r="O193" s="63" t="n">
         <f aca="false">O191+O192</f>
-        <v>166317.475704083</v>
+        <v>167146.980353129</v>
       </c>
       <c r="P193" s="63" t="n">
         <f aca="false">P191+P192</f>
-        <v>166317.475704083</v>
+        <v>167146.980353129</v>
       </c>
       <c r="Q193" s="63" t="n">
         <f aca="false">Q191+Q192</f>
-        <v>173000.57392988</v>
+        <v>173863.410380198</v>
       </c>
       <c r="R193" s="63" t="n">
         <f aca="false">R191+R192</f>
-        <v>173000.57392988</v>
+        <v>173863.410380198</v>
       </c>
       <c r="S193" s="63" t="n">
         <f aca="false">S191+S192</f>
-        <v>173000.57392988</v>
+        <v>173863.410380198</v>
       </c>
       <c r="T193" s="63" t="n">
         <f aca="false">T191+T192</f>
-        <v>173000.57392988</v>
+        <v>173863.410380198</v>
       </c>
       <c r="U193" s="63" t="n">
         <f aca="false">U191+U192</f>
-        <v>173000.57392988</v>
+        <v>173863.410380198</v>
       </c>
       <c r="V193" s="63" t="n">
         <f aca="false">V191+V192</f>
-        <v>173000.57392988</v>
+        <v>173863.410380198</v>
       </c>
       <c r="W193" s="63" t="n">
         <f aca="false">W191+W192</f>
-        <v>131315.52421675</v>
+        <v>129606.52471675</v>
       </c>
       <c r="X193" s="63" t="n">
         <f aca="false">X191+X192</f>
-        <v>131315.52421675</v>
+        <v>129606.52471675</v>
       </c>
       <c r="Y193" s="63" t="n">
         <f aca="false">Y191+Y192</f>
-        <v>131315.52421675</v>
+        <v>129606.52471675</v>
       </c>
       <c r="Z193" s="63" t="n">
         <f aca="false">Z191+Z192</f>
-        <v>131315.52421675</v>
+        <v>129606.52471675</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="40" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B194" s="40"/>
       <c r="C194" s="63"/>
@@ -41288,71 +41302,71 @@
       </c>
       <c r="I194" s="63" t="n">
         <f aca="false">H194+I193</f>
-        <v>966762.67915093</v>
+        <v>967094.595457712</v>
       </c>
       <c r="J194" s="63" t="n">
         <f aca="false">I194+J193</f>
-        <v>1133375.94205974</v>
+        <v>1134039.77467331</v>
       </c>
       <c r="K194" s="63" t="n">
         <f aca="false">J194+K193</f>
-        <v>1299989.20496856</v>
+        <v>1300984.9538889</v>
       </c>
       <c r="L194" s="63" t="n">
         <f aca="false">K194+L193</f>
-        <v>1466602.46787737</v>
+        <v>1467930.1331045</v>
       </c>
       <c r="M194" s="63" t="n">
         <f aca="false">L194+M193</f>
-        <v>1633215.73078618</v>
+        <v>1634875.31232009</v>
       </c>
       <c r="N194" s="63" t="n">
         <f aca="false">M194+N193</f>
-        <v>1804032.68314555</v>
+        <v>1804032.65314555</v>
       </c>
       <c r="O194" s="63" t="n">
         <f aca="false">N194+O193</f>
-        <v>1970350.15884963</v>
+        <v>1971179.63349868</v>
       </c>
       <c r="P194" s="63" t="n">
         <f aca="false">O194+P193</f>
-        <v>2136667.63455372</v>
+        <v>2138326.61385181</v>
       </c>
       <c r="Q194" s="63" t="n">
         <f aca="false">P194+Q193</f>
-        <v>2309668.2084836</v>
+        <v>2312190.02423201</v>
       </c>
       <c r="R194" s="63" t="n">
         <f aca="false">Q194+R193</f>
-        <v>2482668.78241348</v>
+        <v>2486053.4346122</v>
       </c>
       <c r="S194" s="63" t="n">
         <f aca="false">R194+S193</f>
-        <v>2655669.35634336</v>
+        <v>2659916.8449924</v>
       </c>
       <c r="T194" s="63" t="n">
         <f aca="false">S194+T193</f>
-        <v>2828669.93027324</v>
+        <v>2833780.2553726</v>
       </c>
       <c r="U194" s="63" t="n">
         <f aca="false">T194+U193</f>
-        <v>3001670.50420312</v>
+        <v>3007643.6657528</v>
       </c>
       <c r="V194" s="63" t="n">
         <f aca="false">U194+V193</f>
-        <v>3174671.078133</v>
+        <v>3181507.076133</v>
       </c>
       <c r="W194" s="63" t="n">
         <f aca="false">V194+W193</f>
-        <v>3305986.60234975</v>
+        <v>3311113.60084975</v>
       </c>
       <c r="X194" s="63" t="n">
         <f aca="false">W194+X193</f>
-        <v>3437302.1265665</v>
+        <v>3440720.1255665</v>
       </c>
       <c r="Y194" s="63" t="n">
         <f aca="false">X194+Y193</f>
-        <v>3568617.65078325</v>
+        <v>3570326.65028325</v>
       </c>
       <c r="Z194" s="63" t="n">
         <f aca="false">Y194+Z193</f>
@@ -41389,23 +41403,23 @@
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="67"/>
       <c r="B1" s="68" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C1" s="68"/>
       <c r="D1" s="68"/>
       <c r="E1" s="68" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F1" s="68"/>
       <c r="G1" s="68"/>
       <c r="H1" s="69"/>
       <c r="I1" s="68" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J1" s="68"/>
       <c r="K1" s="68"/>
       <c r="L1" s="68" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="M1" s="68"/>
       <c r="N1" s="68"/>
@@ -41445,17 +41459,17 @@
         <v>117</v>
       </c>
       <c r="L2" s="67" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="M2" s="67" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="N2" s="67" t="s">
         <v>117</v>
       </c>
       <c r="O2" s="69"/>
       <c r="P2" s="67" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -42066,7 +42080,7 @@
       </c>
       <c r="E13" s="71" t="n">
         <f aca="false">SUM(E14:E23)</f>
-        <v>1013986.84</v>
+        <v>1013524.62</v>
       </c>
       <c r="F13" s="71" t="n">
         <f aca="false">SUM(F14:F23)</f>
@@ -42074,7 +42088,7 @@
       </c>
       <c r="G13" s="71" t="n">
         <f aca="false">SUM(G14:G23)</f>
-        <v>810408.96</v>
+        <v>810408.93</v>
       </c>
       <c r="H13" s="63"/>
       <c r="I13" s="71" t="n">
@@ -42091,7 +42105,7 @@
       </c>
       <c r="L13" s="71" t="n">
         <f aca="false">E13-I13</f>
-        <v>-212948.87</v>
+        <v>-213411.09</v>
       </c>
       <c r="M13" s="71" t="n">
         <f aca="false">F13-J13</f>
@@ -42099,7 +42113,7 @@
       </c>
       <c r="N13" s="71" t="n">
         <f aca="false">G13-K13</f>
-        <v>-152739.6</v>
+        <v>-152739.63</v>
       </c>
       <c r="O13" s="40"/>
       <c r="P13" s="70" t="str">
@@ -42538,15 +42552,15 @@
       </c>
       <c r="E21" s="74" t="n">
         <f aca="false">ROUND(F21*założenia!$C$8,2)</f>
-        <v>5217.55</v>
+        <v>2745.7</v>
       </c>
       <c r="F21" s="74" t="n">
         <f aca="false">założenia!$C$14</f>
-        <v>4241.91</v>
+        <v>2232.28</v>
       </c>
       <c r="G21" s="74" t="n">
         <f aca="false">założenia!$C$9</f>
-        <v>3393.53</v>
+        <v>1785.82</v>
       </c>
       <c r="H21" s="49"/>
       <c r="I21" s="73" t="n">
@@ -42563,15 +42577,15 @@
       </c>
       <c r="L21" s="73" t="n">
         <f aca="false">E21-I21</f>
-        <v>-117782.45</v>
+        <v>-120254.3</v>
       </c>
       <c r="M21" s="73" t="n">
         <f aca="false">F21-J21</f>
-        <v>-95758.09</v>
+        <v>-97767.72</v>
       </c>
       <c r="N21" s="73" t="n">
         <f aca="false">G21-K21</f>
-        <v>-76606.47</v>
+        <v>-78214.18</v>
       </c>
       <c r="O21" s="41"/>
       <c r="P21" s="72" t="str">
@@ -42596,16 +42610,16 @@
         <v>1820.88</v>
       </c>
       <c r="E22" s="74" t="n">
-        <f aca="false">B22</f>
-        <v>2276.08</v>
+        <f aca="false">I22</f>
+        <v>4285.71</v>
       </c>
       <c r="F22" s="74" t="n">
-        <f aca="false">C22</f>
-        <v>2276.08</v>
+        <f aca="false">J22</f>
+        <v>4285.71</v>
       </c>
       <c r="G22" s="74" t="n">
-        <f aca="false">D22</f>
-        <v>1820.88</v>
+        <f aca="false">K22</f>
+        <v>3428.56</v>
       </c>
       <c r="H22" s="49"/>
       <c r="I22" s="73" t="n">
@@ -42622,15 +42636,15 @@
       </c>
       <c r="L22" s="73" t="n">
         <f aca="false">E22-I22</f>
-        <v>-2009.63</v>
+        <v>0</v>
       </c>
       <c r="M22" s="73" t="n">
         <f aca="false">F22-J22</f>
-        <v>-2009.63</v>
+        <v>0</v>
       </c>
       <c r="N22" s="73" t="n">
         <f aca="false">G22-K22</f>
-        <v>-1607.68</v>
+        <v>0</v>
       </c>
       <c r="O22" s="41"/>
       <c r="P22" s="72" t="str">
@@ -42723,7 +42737,7 @@
       </c>
       <c r="G24" s="71" t="n">
         <f aca="false">SUM(G25:G33)</f>
-        <v>1105163.4</v>
+        <v>1111999.42</v>
       </c>
       <c r="H24" s="63"/>
       <c r="I24" s="71" t="n">
@@ -42748,7 +42762,7 @@
       </c>
       <c r="N24" s="71" t="n">
         <f aca="false">G24-K24</f>
-        <v>222014.84</v>
+        <v>228850.86</v>
       </c>
       <c r="O24" s="40"/>
       <c r="P24" s="70" t="str">
@@ -42781,8 +42795,8 @@
         <v>443200</v>
       </c>
       <c r="G25" s="74" t="n">
-        <f aca="false">ROUND(założenia!$C$13-(G4+G5+G6+G7+G8+G9+G10+G11+G12+G14+G15+G16+G17+G18+G19+G20+G21+G22+G23+G26+G27+G28+G29+G30+G31+G32+G33+G35+G36+G37+G38+G39+G40+G41+G42+G43),2)</f>
-        <v>352380.34</v>
+        <f aca="false">ROUND('budżet po miesiącach'!$C$169,2)</f>
+        <v>354560</v>
       </c>
       <c r="H25" s="49"/>
       <c r="I25" s="73" t="n">
@@ -42807,16 +42821,13 @@
       </c>
       <c r="N25" s="73" t="n">
         <f aca="false">G25-K25</f>
-        <v>86460.34</v>
+        <v>88640</v>
       </c>
       <c r="O25" s="41"/>
       <c r="P25" s="72" t="str">
         <f aca="false">IF(AND(E25&gt;=B25-0.005,F25&gt;=C25-0.005,G25&gt;=D25-0.005),"OK","&lt; narastająco")</f>
         <v>OK</v>
       </c>
-      <c r="Q25" s="55" t="s">
-        <v>246</v>
-      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="72" t="s">
@@ -42844,7 +42855,7 @@
       </c>
       <c r="G26" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$170,2)</f>
-        <v>119961.97</v>
+        <v>120704</v>
       </c>
       <c r="H26" s="49"/>
       <c r="I26" s="73" t="n">
@@ -42869,7 +42880,7 @@
       </c>
       <c r="N26" s="73" t="n">
         <f aca="false">G26-K26</f>
-        <v>29433.97</v>
+        <v>30176</v>
       </c>
       <c r="O26" s="41"/>
       <c r="P26" s="72" t="str">
@@ -42903,7 +42914,7 @@
       </c>
       <c r="G27" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$171,2)</f>
-        <v>161660.05</v>
+        <v>162660</v>
       </c>
       <c r="H27" s="49"/>
       <c r="I27" s="73" t="n">
@@ -42928,7 +42939,7 @@
       </c>
       <c r="N27" s="73" t="n">
         <f aca="false">G27-K27</f>
-        <v>31532.05</v>
+        <v>32532</v>
       </c>
       <c r="O27" s="41"/>
       <c r="P27" s="72" t="str">
@@ -42962,7 +42973,7 @@
       </c>
       <c r="G28" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$172,2)</f>
-        <v>131188.53</v>
+        <v>132000</v>
       </c>
       <c r="H28" s="49"/>
       <c r="I28" s="73" t="n">
@@ -42987,7 +42998,7 @@
       </c>
       <c r="N28" s="73" t="n">
         <f aca="false">G28-K28</f>
-        <v>32188.53</v>
+        <v>33000</v>
       </c>
       <c r="O28" s="41"/>
       <c r="P28" s="72" t="str">
@@ -43021,7 +43032,7 @@
       </c>
       <c r="G29" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$173,2)</f>
-        <v>47323.28</v>
+        <v>47616</v>
       </c>
       <c r="H29" s="49"/>
       <c r="I29" s="73" t="n">
@@ -43046,7 +43057,7 @@
       </c>
       <c r="N29" s="73" t="n">
         <f aca="false">G29-K29</f>
-        <v>11611.28</v>
+        <v>11904</v>
       </c>
       <c r="O29" s="41"/>
       <c r="P29" s="72" t="str">
@@ -43080,7 +43091,7 @@
       </c>
       <c r="G30" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$174,2)</f>
-        <v>131188.53</v>
+        <v>132000</v>
       </c>
       <c r="H30" s="49"/>
       <c r="I30" s="73" t="n">
@@ -43105,7 +43116,7 @@
       </c>
       <c r="N30" s="73" t="n">
         <f aca="false">G30-K30</f>
-        <v>32188.53</v>
+        <v>33000</v>
       </c>
       <c r="O30" s="41"/>
       <c r="P30" s="72" t="str">
@@ -43139,7 +43150,7 @@
       </c>
       <c r="G31" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$175,2)</f>
-        <v>31294.43</v>
+        <v>31488</v>
       </c>
       <c r="H31" s="49"/>
       <c r="I31" s="73" t="n">
@@ -43164,7 +43175,7 @@
       </c>
       <c r="N31" s="73" t="n">
         <f aca="false">G31-K31</f>
-        <v>-33337.57</v>
+        <v>-33144</v>
       </c>
       <c r="O31" s="41"/>
       <c r="P31" s="72" t="str">
@@ -43198,7 +43209,7 @@
       </c>
       <c r="G32" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$176,2)</f>
-        <v>4543.32</v>
+        <v>4571.42</v>
       </c>
       <c r="H32" s="49"/>
       <c r="I32" s="73" t="n">
@@ -43223,7 +43234,7 @@
       </c>
       <c r="N32" s="73" t="n">
         <f aca="false">G32-K32</f>
-        <v>1114.76</v>
+        <v>1142.86</v>
       </c>
       <c r="O32" s="41"/>
       <c r="P32" s="72" t="str">
@@ -43257,7 +43268,7 @@
       </c>
       <c r="G33" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$177,2)</f>
-        <v>125622.95</v>
+        <v>126400</v>
       </c>
       <c r="H33" s="49"/>
       <c r="I33" s="73" t="n">
@@ -43282,7 +43293,7 @@
       </c>
       <c r="N33" s="73" t="n">
         <f aca="false">G33-K33</f>
-        <v>30822.95</v>
+        <v>31600</v>
       </c>
       <c r="O33" s="41"/>
       <c r="P33" s="72" t="str">
@@ -43316,7 +43327,7 @@
       </c>
       <c r="G34" s="71" t="n">
         <f aca="false">SUM(G35:G43)</f>
-        <v>398434.28</v>
+        <v>391598.29</v>
       </c>
       <c r="H34" s="63"/>
       <c r="I34" s="71" t="n">
@@ -43341,7 +43352,7 @@
       </c>
       <c r="N34" s="71" t="n">
         <f aca="false">G34-K34</f>
-        <v>-20508</v>
+        <v>-27343.9900000001</v>
       </c>
       <c r="O34" s="40"/>
       <c r="P34" s="70" t="str">
@@ -43374,8 +43385,8 @@
         <v>221600</v>
       </c>
       <c r="G35" s="74" t="n">
-        <f aca="false">ROUND('budżet po miesiącach'!$C$178,2)</f>
-        <v>132960</v>
+        <f aca="false">ROUND(założenia!$C$13-(G4+G5+G6+G7+G8+G9+G10+G11+G12+G14+G15+G16+G17+G18+G19+G20+G21+G22+G23+G25+G26+G27+G28+G29+G30+G31+G32+G33+G36+G37+G38+G39+G40+G41+G42+G43),2)</f>
+        <v>130678.79</v>
       </c>
       <c r="H35" s="49"/>
       <c r="I35" s="73" t="n">
@@ -43400,13 +43411,16 @@
       </c>
       <c r="N35" s="73" t="n">
         <f aca="false">G35-K35</f>
-        <v>0</v>
+        <v>-2281.21000000001</v>
       </c>
       <c r="O35" s="41"/>
       <c r="P35" s="72" t="str">
         <f aca="false">IF(AND(E35&gt;=B35-0.005,F35&gt;=C35-0.005,G35&gt;=D35-0.005),"OK","&lt; narastająco")</f>
         <v>OK</v>
       </c>
+      <c r="Q35" s="55" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="72" t="s">
@@ -43434,7 +43448,7 @@
       </c>
       <c r="G36" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$179,2)</f>
-        <v>22632</v>
+        <v>22243.7</v>
       </c>
       <c r="H36" s="49"/>
       <c r="I36" s="73" t="n">
@@ -43459,7 +43473,7 @@
       </c>
       <c r="N36" s="73" t="n">
         <f aca="false">G36-K36</f>
-        <v>0</v>
+        <v>-388.299999999999</v>
       </c>
       <c r="O36" s="41"/>
       <c r="P36" s="72" t="str">
@@ -43493,7 +43507,7 @@
       </c>
       <c r="G37" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$180,2)</f>
-        <v>65064</v>
+        <v>63947.69</v>
       </c>
       <c r="H37" s="49"/>
       <c r="I37" s="73" t="n">
@@ -43518,7 +43532,7 @@
       </c>
       <c r="N37" s="73" t="n">
         <f aca="false">G37-K37</f>
-        <v>0</v>
+        <v>-1116.31</v>
       </c>
       <c r="O37" s="41"/>
       <c r="P37" s="72" t="str">
@@ -43552,7 +43566,7 @@
       </c>
       <c r="G38" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$181,2)</f>
-        <v>49500</v>
+        <v>48650.72</v>
       </c>
       <c r="H38" s="49"/>
       <c r="I38" s="73" t="n">
@@ -43577,7 +43591,7 @@
       </c>
       <c r="N38" s="73" t="n">
         <f aca="false">G38-K38</f>
-        <v>0</v>
+        <v>-849.279999999999</v>
       </c>
       <c r="O38" s="41"/>
       <c r="P38" s="72" t="str">
@@ -43611,7 +43625,7 @@
       </c>
       <c r="G39" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$182,2)</f>
-        <v>17856</v>
+        <v>17549.64</v>
       </c>
       <c r="H39" s="49"/>
       <c r="I39" s="73" t="n">
@@ -43636,7 +43650,7 @@
       </c>
       <c r="N39" s="73" t="n">
         <f aca="false">G39-K39</f>
-        <v>0</v>
+        <v>-306.360000000001</v>
       </c>
       <c r="O39" s="41"/>
       <c r="P39" s="72" t="str">
@@ -43670,7 +43684,7 @@
       </c>
       <c r="G40" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$183,2)</f>
-        <v>49500</v>
+        <v>48650.72</v>
       </c>
       <c r="H40" s="49"/>
       <c r="I40" s="73" t="n">
@@ -43695,7 +43709,7 @@
       </c>
       <c r="N40" s="73" t="n">
         <f aca="false">G40-K40</f>
-        <v>0</v>
+        <v>-849.279999999999</v>
       </c>
       <c r="O40" s="41"/>
       <c r="P40" s="72" t="str">
@@ -43729,7 +43743,7 @@
       </c>
       <c r="G41" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$184,2)</f>
-        <v>1714.28</v>
+        <v>1684.87</v>
       </c>
       <c r="H41" s="49"/>
       <c r="I41" s="73" t="n">
@@ -43754,7 +43768,7 @@
       </c>
       <c r="N41" s="73" t="n">
         <f aca="false">G41-K41</f>
-        <v>0</v>
+        <v>-29.4100000000001</v>
       </c>
       <c r="O41" s="41"/>
       <c r="P41" s="72" t="str">
@@ -43788,7 +43802,7 @@
       </c>
       <c r="G42" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$185,2)</f>
-        <v>47400</v>
+        <v>46586.75</v>
       </c>
       <c r="H42" s="49"/>
       <c r="I42" s="73" t="n">
@@ -43813,7 +43827,7 @@
       </c>
       <c r="N42" s="73" t="n">
         <f aca="false">G42-K42</f>
-        <v>0</v>
+        <v>-813.25</v>
       </c>
       <c r="O42" s="41"/>
       <c r="P42" s="72" t="str">
@@ -43847,7 +43861,7 @@
       </c>
       <c r="G43" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$186,2)</f>
-        <v>11808</v>
+        <v>11605.41</v>
       </c>
       <c r="H43" s="49"/>
       <c r="I43" s="73" t="n">
@@ -43872,7 +43886,7 @@
       </c>
       <c r="N43" s="73" t="n">
         <f aca="false">G43-K43</f>
-        <v>-20508</v>
+        <v>-20710.59</v>
       </c>
       <c r="O43" s="41"/>
       <c r="P43" s="72" t="str">
@@ -43882,54 +43896,54 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="75" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="53" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B47" s="53" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C47" s="53" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D47" s="53" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E47" s="53" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F47" s="53" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G47" s="53" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="H47" s="76"/>
       <c r="I47" s="53" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="J47" s="53" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="K47" s="53" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="L47" s="53" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="M47" s="53" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="N47" s="53" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="41" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B48" s="73" t="n">
         <f aca="false">B3+B13+B24+B34</f>
@@ -43945,7 +43959,7 @@
       </c>
       <c r="E48" s="73" t="n">
         <f aca="false">E3+E13+E24+E34</f>
-        <v>3875468.13</v>
+        <v>3875005.91</v>
       </c>
       <c r="F48" s="73" t="n">
         <f aca="false">F3+F13+F24+F34</f>
@@ -43970,7 +43984,7 @@
       </c>
       <c r="L48" s="73" t="n">
         <f aca="false">E48-I48</f>
-        <v>-22024.3599999999</v>
+        <v>-22486.5800000001</v>
       </c>
       <c r="M48" s="73" t="n">
         <f aca="false">F48-J48</f>
@@ -43983,7 +43997,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B49" s="73" t="n">
         <f aca="false">Podsumowanie!D130</f>
@@ -44037,7 +44051,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="40" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B50" s="46" t="n">
         <f aca="false">B48+B49</f>
@@ -44053,7 +44067,7 @@
       </c>
       <c r="E50" s="46" t="n">
         <f aca="false">E48+E49</f>
-        <v>4844091.25</v>
+        <v>4843629.03</v>
       </c>
       <c r="F50" s="46" t="n">
         <f aca="false">F48+F49</f>
@@ -44078,7 +44092,7 @@
       </c>
       <c r="L50" s="46" t="n">
         <f aca="false">E50-I50</f>
-        <v>-22024.3600000003</v>
+        <v>-22486.5800000001</v>
       </c>
       <c r="M50" s="46" t="n">
         <f aca="false">F50-J50</f>
@@ -44091,7 +44105,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="41" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B51" s="73"/>
       <c r="C51" s="73"/>
@@ -44115,7 +44129,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="41" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B52" s="73"/>
       <c r="C52" s="73"/>
@@ -44139,7 +44153,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="40" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B53" s="46"/>
       <c r="C53" s="46"/>

</xml_diff>

<commit_message>
Fixed intensities (80/60), Z4 qualified costs reduced to fit dofinansowanie limit
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3QuwGR9tgiXrdWSSrWcuu
</commit_message>
<xml_diff>
--- a/Wniosek_o_platnosc_str26-34.xlsx
+++ b/Wniosek_o_platnosc_str26-34.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1119" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="268">
   <si>
     <t xml:space="preserve">Wniosek o płatność – PODSUMOWANIE (PDF str. 27–34)</t>
   </si>
@@ -504,31 +504,34 @@
     <t xml:space="preserve">Cel dofinansowanie – koszty bezpośrednie (PDF)</t>
   </si>
   <si>
-    <t xml:space="preserve">Pozostaje na licencjach – kwalifikowalne (cel − wszystkie pozostałe pozycje)</t>
+    <t xml:space="preserve">Licencje – kwalifikowalne po zmianie (przyjęto 0: dofinansowanie nie może wzrosnąć)</t>
   </si>
   <si>
-    <t xml:space="preserve">Z4 – kwalifikowalne razem (prognoza)</t>
+    <t xml:space="preserve">Z4 – kwalifikowalne planowane (stawka × etat), przed obniżeniem</t>
   </si>
   <si>
-    <t xml:space="preserve">Z3 – dofinansowanie przy pełnej intensywności (Z3 × 80%)</t>
+    <t xml:space="preserve">Z3 – dofinansowanie (80% kosztów kwalifikowalnych)</t>
   </si>
   <si>
-    <t xml:space="preserve">Dofinansowanie pozostałe: Z1+Z2 (wykonanie, poz. 2.9 wg planu, z licencją) + Z4 przy pełnej intensywności</t>
+    <t xml:space="preserve">Dofinansowanie Z1+Z2 (wykonanie, poz. 2.9 wg planu, licencje) + Z3</t>
   </si>
   <si>
-    <t xml:space="preserve">Nadwyżka dofinansowania ponad cel (do obniżenia w Z4), zł</t>
+    <t xml:space="preserve">Dofinansowanie dostępne dla Z4 = cel D bezpośrednie − C17</t>
   </si>
   <si>
-    <t xml:space="preserve">Obniżenie intensywności Z4 (60% minus ta wartość)</t>
+    <t xml:space="preserve">Współczynnik obniżenia kosztów kwalifikowalnych Z4 (Z4 = C15 × C19, tak by D = 60% mieściło się w C18)</t>
   </si>
   <si>
     <t xml:space="preserve">TEST: koszt wakatu grafika w Z4 (stawka × miesiące Z4), gdyby został</t>
   </si>
   <si>
-    <t xml:space="preserve">TEST: reszta na licencjach, gdyby wakat w Z4 został</t>
+    <t xml:space="preserve">TEST: dofinansowanie (60%), które dodałby wakat w Z4</t>
   </si>
   <si>
     <t xml:space="preserve">TEST: wniosek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z4 – kwalifikowalne po obniżeniu</t>
   </si>
   <si>
     <t xml:space="preserve">KONTROLE</t>
@@ -546,10 +549,10 @@
     <t xml:space="preserve">różnica</t>
   </si>
   <si>
-    <t xml:space="preserve">Kwalifikowalne razem = cel</t>
+    <t xml:space="preserve">Kwalifikowalne razem nie przekraczają celu</t>
   </si>
   <si>
-    <t xml:space="preserve">Dofinansowanie razem = cel</t>
+    <t xml:space="preserve">Dofinansowanie razem nie przekracza celu (nie może wzrosnąć)</t>
   </si>
   <si>
     <t xml:space="preserve">Z1 i Z2 w nowym budżecie = wydatki narastająco, bez poz. 2.9 i licencji (suma różnic)</t>
@@ -573,13 +576,13 @@
     <t xml:space="preserve">1. Oś czasu: było Z1 m 1–5, Z2 m 6–11, Z3 m 12–17, Z4 m 18–21 (21 m-cy). Będzie Z1 m 1–5, Z2 m 6–11, Z3 m 12–19 (8 m-cy), Z4 m 20–23 (23 m-ce).</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Cel: wydatki kwalifikowalne razem 4 843 115,61 zł i dofinansowanie razem 3 699 933,17 zł bez zmian vs budżet pierwotny. Wartość ogółem może się zmienić (VAT licencji).</t>
+    <t xml:space="preserve">2. Cel: dofinansowanie razem (3 699 933,17 zł) nie może wzrosnąć; wydatki kwalifikowalne razem (4 843 115,61 zł) mogą się zmniejszyć, ale nie wzrosnąć. Stałe zasady: intensywność Z1–Z3 = 80%, Z4 = 60%, koszty pośrednie = 25% kwalifikowalnych oraz 25% dofinansowania kosztów bezpośrednich (pochodne – nie są sterowane ręcznie).</t>
   </si>
   <si>
     <t xml:space="preserve">3. Z1 i Z2 w nowym budżecie = wydatki narastająco (ogółem, kwalifikowalne, dofinansowanie) per pozycja, z wyjątkiem poz. 2.9 (amortyzacja laptopów w Z2) – bez zmian wg planu: 4 285,71 zł. Poz. 2.1 (Ekspert AI, Z2): przyjęto 332 400 zł kwalifikowalnych / 265 920 zł dofinansowania (PARP wstrzymał wypłatę, budżet nie jest tracony).</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Licencje (Z2): wykonanie 0, więc całość uwalnia środki. Na licencjach zostaje tylko reszta, która domyka sumę kwalifikowalnych do celu (C14); dofinansowanie tej reszty = reszta × 80% (C9); nadwyżkę dofinansowania koryguje się w Z3 (punkt 11).</t>
+    <t xml:space="preserve">4. Licencje (Z2): wykonanie 0, więc całość uwalnia środki. Po zmianie 0 zł (C14) – przy stałych intensywnościach budżet nie mieści ani reszty na licencjach, ani wakatu grafika w Z4.</t>
   </si>
   <si>
     <t xml:space="preserve">5. Z3 i Z4 = prognoza: stawka × etat × miesiące (arkusz „plan etatów”). Z3 nie jest przycinane.</t>
@@ -594,16 +597,16 @@
     <t xml:space="preserve">8. Big Data Engineer: 1 etat w Z1–Z3, 0,5 etatu w Z4 (37 720 zł, zgodnie z PDF).</t>
   </si>
   <si>
-    <t xml:space="preserve">9. Grafik-Ilustrator: wakat (8 545 zł/mies.) wyzerowany w całym projekcie, w tym w Z4; zostaje Suska (4 920 zł/mies.). Test w C20:C22 pokazuje, czy przy pozostawieniu wakatu w Z4 budżet by wystarczył.</t>
+    <t xml:space="preserve">9. Grafik-Ilustrator: wakat (8 545 zł/mies.) wyzerowany w całym projekcie, w tym w Z4; zostaje Suska (4 920 zł/mies.). Test w C20:C22 pokazuje, że wakat w Z4 nie mieści się w limicie dofinansowania.</t>
   </si>
   <si>
     <t xml:space="preserve">10. Amortyzacja laptopów: 714,29 zł/mies.; wydłużenie Z3 do 8 m-cy zwiększa amortyzację Z3 (5 714,29 zł). Z4 bez zmian.</t>
   </si>
   <si>
-    <t xml:space="preserve">11. Dofinansowanie: Z3 dokładnie 80% kosztów kwalifikowalnych (poz. 3.1–3.9), Z1 i Z2 jak wykonanie. Suma dofinansowania nie może przekroczyć 3 699 933,17 zł, a środki z wakatu w Z4 (60%) trafiają do Z3 (80%), więc nadwyżkę z C18 odjęto od dofinansowania Z4 (równomiernie, intensywność Z4 spada o C19). Własny wkład w Z4 rośnie o tę kwotę. Alternatywa: obniżyć dofinansowanie w innym miejscu (np. koszty pośrednie).</t>
+    <t xml:space="preserve">11. Dofinansowanie: Z1–Z3 po 80%, Z4 po 60% (bez żadnych korekt intensywności). Przy pełnej prognozie Z3 i Z4 dofinansowanie przekroczyłoby cel, dlatego kwalifikowalne Z4 obniżono jednolitym współczynnikiem C19 do kwoty mieszczącej się w limicie dofinansowania (C18). Kwalifikowalne razem spadają poniżej celu – różnica to niewykorzystany budżet.</t>
   </si>
   <si>
-    <t xml:space="preserve">12. Koszty pośrednie: 25% kwalifikowalnych kosztów bezpośrednich – bez zmian, bo suma bezpośrednich bez zmian.</t>
+    <t xml:space="preserve">12. Koszty pośrednie: 25% kwalifikowalnych kosztów bezpośrednich; dofinansowanie do nich = ta sama proporcja co w kosztach bezpośrednich (25% dofinansowania bezpośredniego, zaokrąglone w dół). Zmieniają się wraz z kosztami bezpośrednimi.</t>
   </si>
   <si>
     <t xml:space="preserve">14. Daty zadań (PDF): Z1 2025-10-01 – 2026-02-28, Z2 2026-03-01 – 2026-08-31, Z3 2026-09-01 – 2027-04-30, Z4 2027-05-01 – 2027-08-31 (poprawione).</t>
@@ -831,7 +834,7 @@
     <t xml:space="preserve">Różnica nowy − cel</t>
   </si>
   <si>
-    <t xml:space="preserve">Status (tolerancja 0,05 zł – zaokrąglenia)</t>
+    <t xml:space="preserve">Status (kwota nie może przekroczyć celu)</t>
   </si>
 </sst>
 </file>
@@ -1096,7 +1099,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="78">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1281,7 +1284,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1403,6 +1406,10 @@
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -12090,7 +12097,7 @@
       </c>
       <c r="C9" s="44" t="n">
         <f aca="false">ROUND(C14*C5,2)</f>
-        <v>1785.82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12132,8 +12139,7 @@
         <v>157</v>
       </c>
       <c r="C14" s="46" t="n">
-        <f aca="false">ROUND(C12-('nowy format 2'!F4+'nowy format 2'!F5+'nowy format 2'!F6+'nowy format 2'!F7+'nowy format 2'!F8+'nowy format 2'!F9+'nowy format 2'!F10+'nowy format 2'!F11+'nowy format 2'!F12+'nowy format 2'!F14+'nowy format 2'!F15+'nowy format 2'!F16+'nowy format 2'!F17+'nowy format 2'!F18+'nowy format 2'!F19+'nowy format 2'!F20+'nowy format 2'!F22+'nowy format 2'!F23+'nowy format 2'!F25+'nowy format 2'!F26+'nowy format 2'!F27+'nowy format 2'!F28+'nowy format 2'!F29+'nowy format 2'!F30+'nowy format 2'!F31+'nowy format 2'!F32+'nowy format 2'!F33+'nowy format 2'!F35+'nowy format 2'!F36+'nowy format 2'!F37+'nowy format 2'!F38+'nowy format 2'!F39+'nowy format 2'!F40+'nowy format 2'!F41+'nowy format 2'!F42+'nowy format 2'!F43),2)</f>
-        <v>2232.28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12141,7 +12147,7 @@
         <v>158</v>
       </c>
       <c r="C15" s="44" t="n">
-        <f aca="false">'nowy format 2'!F34</f>
+        <f aca="false">SUMIF('plan etatów'!$C$78:$C$114,4,'plan etatów'!$AA$78:$AA$114)</f>
         <v>664057.14</v>
       </c>
     </row>
@@ -12150,8 +12156,8 @@
         <v>159</v>
       </c>
       <c r="C16" s="44" t="n">
-        <f aca="false">'nowy format 2'!F24*C6</f>
-        <v>1111999.424</v>
+        <f aca="false">'nowy format 2'!G24</f>
+        <v>1111999.42</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12159,8 +12165,8 @@
         <v>160</v>
       </c>
       <c r="C17" s="44" t="n">
-        <f aca="false">'nowy format 2'!G4+'nowy format 2'!G5+'nowy format 2'!G6+'nowy format 2'!G7+'nowy format 2'!G8+'nowy format 2'!G9+'nowy format 2'!G10+'nowy format 2'!G11+'nowy format 2'!G12+'nowy format 2'!G14+'nowy format 2'!G15+'nowy format 2'!G16+'nowy format 2'!G17+'nowy format 2'!G18+'nowy format 2'!G19+'nowy format 2'!G20+'nowy format 2'!G21+'nowy format 2'!G22+'nowy format 2'!G23+C15*C7</f>
-        <v>1854783.114</v>
+        <f aca="false">'nowy format 2'!G4+'nowy format 2'!G5+'nowy format 2'!G6+'nowy format 2'!G7+'nowy format 2'!G8+'nowy format 2'!G9+'nowy format 2'!G10+'nowy format 2'!G11+'nowy format 2'!G12+'nowy format 2'!G14+'nowy format 2'!G15+'nowy format 2'!G16+'nowy format 2'!G17+'nowy format 2'!G18+'nowy format 2'!G19+'nowy format 2'!G20+'nowy format 2'!G21+'nowy format 2'!G22+'nowy format 2'!G23+C16</f>
+        <v>2566562.43</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12168,8 +12174,8 @@
         <v>161</v>
       </c>
       <c r="C18" s="44" t="n">
-        <f aca="false">C16+C17-C13</f>
-        <v>6835.99800000014</v>
+        <f aca="false">C13-C17</f>
+        <v>393384.11</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12177,8 +12183,8 @@
         <v>162</v>
       </c>
       <c r="C19" s="47" t="n">
-        <f aca="false">C18/C15</f>
-        <v>0.0102942918436208</v>
+        <f aca="false">MIN(1,ROUNDDOWN(C18/C7,2)/C15)</f>
+        <v>0.987324946163518</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12195,8 +12201,8 @@
         <v>164</v>
       </c>
       <c r="C21" s="44" t="n">
-        <f aca="false">C14-C20</f>
-        <v>-31947.72</v>
+        <f aca="false">C20*C7</f>
+        <v>20508</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12204,51 +12210,60 @@
         <v>165</v>
       </c>
       <c r="C22" s="48" t="str">
-        <f aca="false">IF(C21&lt;0,"NIE WYSTARCZA – wakat grafika w Z4 zdjęty","wystarcza – wakat można zostawić")</f>
-        <v>NIE WYSTARCZA – wakat grafika w Z4 zdjęty</v>
+        <f aca="false">IF(C21&gt;MAX(0,C18-C15*C7),"wakat w Z4 nie mieści się w limicie dofinansowania – zdjęty","mieści się")</f>
+        <v>wakat w Z4 nie mieści się w limicie dofinansowania – zdjęty</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="41" t="s">
+        <v>166</v>
+      </c>
+      <c r="C23" s="44" t="n">
+        <f aca="false">ROUND(C15*C19,2)</f>
+        <v>655640.18</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="40" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C24" s="40" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D24" s="40" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E24" s="40" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F24" s="40" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="41" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C25" s="49" t="n">
         <f aca="false">'nowy format 2'!F50</f>
-        <v>4843115.61</v>
+        <v>4829804.08</v>
       </c>
       <c r="D25" s="49" t="n">
         <f aca="false">C10</f>
         <v>4843115.61</v>
       </c>
       <c r="E25" s="40" t="str">
-        <f aca="false">IF(ABS(C25-D25)&lt;=0.05,"OK","BŁĄD")</f>
+        <f aca="false">IF(C25&lt;=D25+0.005,"OK","BŁĄD")</f>
         <v>OK</v>
       </c>
       <c r="F25" s="49" t="n">
         <f aca="false">ROUND(C25-D25,2)</f>
-        <v>0</v>
+        <v>-13311.53</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="41" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C26" s="49" t="n">
         <f aca="false">'nowy format 2'!G50</f>
@@ -12259,7 +12274,7 @@
         <v>3699933.17</v>
       </c>
       <c r="E26" s="40" t="str">
-        <f aca="false">IF(ABS(C26-D26)&lt;=0.05,"OK","BŁĄD")</f>
+        <f aca="false">IF(C26&lt;=D26+0.005,"OK","BŁĄD")</f>
         <v>OK</v>
       </c>
       <c r="F26" s="49" t="n">
@@ -12269,7 +12284,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="41" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C27" s="49" t="n">
         <f aca="false">ABS('nowy format 2'!E4-'nowy format 2'!B4)+ABS('nowy format 2'!F4-'nowy format 2'!C4)+ABS('nowy format 2'!G4-'nowy format 2'!D4)+ABS('nowy format 2'!E5-'nowy format 2'!B5)+ABS('nowy format 2'!F5-'nowy format 2'!C5)+ABS('nowy format 2'!G5-'nowy format 2'!D5)+ABS('nowy format 2'!E6-'nowy format 2'!B6)+ABS('nowy format 2'!F6-'nowy format 2'!C6)+ABS('nowy format 2'!G6-'nowy format 2'!D6)+ABS('nowy format 2'!E7-'nowy format 2'!B7)+ABS('nowy format 2'!F7-'nowy format 2'!C7)+ABS('nowy format 2'!G7-'nowy format 2'!D7)+ABS('nowy format 2'!E8-'nowy format 2'!B8)+ABS('nowy format 2'!F8-'nowy format 2'!C8)+ABS('nowy format 2'!G8-'nowy format 2'!D8)+ABS('nowy format 2'!E9-'nowy format 2'!B9)+ABS('nowy format 2'!F9-'nowy format 2'!C9)+ABS('nowy format 2'!G9-'nowy format 2'!D9)+ABS('nowy format 2'!E10-'nowy format 2'!B10)+ABS('nowy format 2'!F10-'nowy format 2'!C10)+ABS('nowy format 2'!G10-'nowy format 2'!D10)+ABS('nowy format 2'!E11-'nowy format 2'!B11)+ABS('nowy format 2'!F11-'nowy format 2'!C11)+ABS('nowy format 2'!G11-'nowy format 2'!D11)+ABS('nowy format 2'!E12-'nowy format 2'!B12)+ABS('nowy format 2'!F12-'nowy format 2'!C12)+ABS('nowy format 2'!G12-'nowy format 2'!D12)+ABS('nowy format 2'!E14-'nowy format 2'!B14)+ABS('nowy format 2'!F14-'nowy format 2'!C14)+ABS('nowy format 2'!G14-'nowy format 2'!D14)+ABS('nowy format 2'!E15-'nowy format 2'!B15)+ABS('nowy format 2'!F15-'nowy format 2'!C15)+ABS('nowy format 2'!G15-'nowy format 2'!D15)+ABS('nowy format 2'!E16-'nowy format 2'!B16)+ABS('nowy format 2'!F16-'nowy format 2'!C16)+ABS('nowy format 2'!G16-'nowy format 2'!D16)+ABS('nowy format 2'!E17-'nowy format 2'!B17)+ABS('nowy format 2'!F17-'nowy format 2'!C17)+ABS('nowy format 2'!G17-'nowy format 2'!D17)+ABS('nowy format 2'!E18-'nowy format 2'!B18)+ABS('nowy format 2'!F18-'nowy format 2'!C18)+ABS('nowy format 2'!G18-'nowy format 2'!D18)+ABS('nowy format 2'!E19-'nowy format 2'!B19)+ABS('nowy format 2'!F19-'nowy format 2'!C19)+ABS('nowy format 2'!G19-'nowy format 2'!D19)+ABS('nowy format 2'!E20-'nowy format 2'!B20)+ABS('nowy format 2'!F20-'nowy format 2'!C20)+ABS('nowy format 2'!G20-'nowy format 2'!D20)+ABS('nowy format 2'!E23-'nowy format 2'!B23)+ABS('nowy format 2'!F23-'nowy format 2'!C23)+ABS('nowy format 2'!G23-'nowy format 2'!D23)</f>
@@ -12284,15 +12299,15 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="41" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C28" s="49" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!C97,2)</f>
-        <v>3874492.49</v>
+        <v>3863843.25</v>
       </c>
       <c r="D28" s="49" t="n">
         <f aca="false">'nowy format 2'!F48</f>
-        <v>3874492.49</v>
+        <v>3863843.26</v>
       </c>
       <c r="E28" s="40" t="str">
         <f aca="false">IF(ABS(C28-D28)&lt;=0.05,"OK","BŁĄD")</f>
@@ -12302,7 +12317,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="41" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C29" s="49" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!C50,2)</f>
@@ -12320,7 +12335,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="41" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C30" s="49" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!C144,2)</f>
@@ -12338,7 +12353,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="41" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C31" s="49" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!C191,2)</f>
@@ -12356,12 +12371,12 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="40" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="50" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B34" s="50"/>
       <c r="C34" s="50"/>
@@ -12371,7 +12386,7 @@
     </row>
     <row r="35" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="50" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B35" s="50"/>
       <c r="C35" s="50"/>
@@ -12381,7 +12396,7 @@
     </row>
     <row r="36" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="50" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B36" s="50"/>
       <c r="C36" s="50"/>
@@ -12391,7 +12406,7 @@
     </row>
     <row r="37" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="50" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B37" s="50"/>
       <c r="C37" s="50"/>
@@ -12401,7 +12416,7 @@
     </row>
     <row r="38" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="50" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B38" s="50"/>
       <c r="C38" s="50"/>
@@ -12411,7 +12426,7 @@
     </row>
     <row r="39" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="50" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B39" s="50"/>
       <c r="C39" s="50"/>
@@ -12421,7 +12436,7 @@
     </row>
     <row r="40" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="50" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B40" s="50"/>
       <c r="C40" s="50"/>
@@ -12431,7 +12446,7 @@
     </row>
     <row r="41" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="50" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B41" s="50"/>
       <c r="C41" s="50"/>
@@ -12441,7 +12456,7 @@
     </row>
     <row r="42" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="50" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B42" s="50"/>
       <c r="C42" s="50"/>
@@ -12451,7 +12466,7 @@
     </row>
     <row r="43" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="50" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B43" s="50"/>
       <c r="C43" s="50"/>
@@ -12461,7 +12476,7 @@
     </row>
     <row r="44" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="50" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B44" s="50"/>
       <c r="C44" s="50"/>
@@ -12471,7 +12486,7 @@
     </row>
     <row r="45" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="50" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B45" s="50"/>
       <c r="C45" s="50"/>
@@ -12481,7 +12496,7 @@
     </row>
     <row r="46" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="50" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B46" s="50"/>
       <c r="C46" s="50"/>
@@ -12491,7 +12506,7 @@
     </row>
     <row r="47" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="50" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B47" s="50"/>
       <c r="C47" s="50"/>
@@ -12543,37 +12558,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="39" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="51" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="40" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B3" s="40" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C3" s="40" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D3" s="40" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E3" s="40" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F3" s="40" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="41" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B4" s="52" t="n">
         <v>1</v>
@@ -12588,12 +12603,12 @@
         <v>5</v>
       </c>
       <c r="F4" s="41" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="41" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B5" s="52" t="n">
         <v>6</v>
@@ -12608,12 +12623,12 @@
         <v>11</v>
       </c>
       <c r="F5" s="41" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="41" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B6" s="52" t="n">
         <v>12</v>
@@ -12628,12 +12643,12 @@
         <v>19</v>
       </c>
       <c r="F6" s="41" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="41" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B7" s="52" t="n">
         <v>18</v>
@@ -12648,23 +12663,23 @@
         <v>23</v>
       </c>
       <c r="F7" s="41" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="40" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="53" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B10" s="53" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C10" s="53" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D10" s="53" t="n">
         <v>1</v>
@@ -12736,12 +12751,12 @@
         <v>23</v>
       </c>
       <c r="AA10" s="53" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="41" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B11" s="54" t="n">
         <v>27700</v>
@@ -13203,7 +13218,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="41" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B17" s="54" t="n">
         <v>19750</v>
@@ -13357,7 +13372,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="41" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B19" s="54" t="n">
         <f aca="false">ROUND(4285.71/6,4)</f>
@@ -13435,18 +13450,18 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="40" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="53" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B23" s="53" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C23" s="53" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D23" s="53" t="n">
         <v>1</v>
@@ -13518,12 +13533,12 @@
         <v>23</v>
       </c>
       <c r="AA23" s="53" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="41" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B24" s="54" t="n">
         <v>27700</v>
@@ -13675,7 +13690,7 @@
         <v>0.5</v>
       </c>
       <c r="AB25" s="55" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13755,7 +13770,7 @@
         <v>2</v>
       </c>
       <c r="AB26" s="55" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13835,7 +13850,7 @@
         <v>1</v>
       </c>
       <c r="AB27" s="55" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13994,7 +14009,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="41" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B30" s="54" t="n">
         <v>19750</v>
@@ -14148,7 +14163,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="41" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B32" s="54" t="n">
         <f aca="false">ROUND(4285.71/6,4)</f>
@@ -14224,23 +14239,23 @@
         <v>1</v>
       </c>
       <c r="AB32" s="55" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="40" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="53" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B36" s="53" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C36" s="53" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D36" s="53" t="n">
         <v>1</v>
@@ -14312,7 +14327,7 @@
         <v>23</v>
       </c>
       <c r="AA36" s="53" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18142,18 +18157,18 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="40" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="53" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B77" s="53" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C77" s="53" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D77" s="53" t="n">
         <v>1</v>
@@ -18225,7 +18240,7 @@
         <v>23</v>
       </c>
       <c r="AA77" s="53" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22080,17 +22095,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="39" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="51" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="58" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B3" s="59"/>
       <c r="C3" s="59"/>
@@ -22189,13 +22204,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="58" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B4" s="59" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C4" s="59" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D4" s="59" t="n">
         <v>1</v>
@@ -22269,7 +22284,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="58" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B5" s="59"/>
       <c r="C5" s="59"/>
@@ -22368,7 +22383,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="58" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B6" s="59"/>
       <c r="C6" s="59"/>
@@ -22495,7 +22510,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="60" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B8" s="61"/>
       <c r="C8" s="62"/>
@@ -26373,7 +26388,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="40" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B46" s="40" t="n">
         <v>1</v>
@@ -26477,7 +26492,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="40" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B47" s="40" t="n">
         <v>2</v>
@@ -26581,7 +26596,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="40" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B48" s="40" t="n">
         <v>3</v>
@@ -26685,7 +26700,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="40" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B49" s="40" t="n">
         <v>4</v>
@@ -26891,7 +26906,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="40" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B51" s="40"/>
       <c r="C51" s="63" t="n">
@@ -26993,7 +27008,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="40" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B52" s="40"/>
       <c r="C52" s="63" t="n">
@@ -27095,7 +27110,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="40" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B53" s="40"/>
       <c r="C53" s="63"/>
@@ -27222,7 +27237,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="64" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B55" s="65"/>
       <c r="C55" s="66"/>
@@ -28923,7 +28938,7 @@
       </c>
       <c r="C72" s="49" t="n">
         <f aca="false">SUM(D72:Z72)</f>
-        <v>2232.28</v>
+        <v>0</v>
       </c>
       <c r="D72" s="49" t="n">
         <f aca="false">IF(D$4='plan etatów'!$E$5,założenia!$C$14,0)</f>
@@ -28967,7 +28982,7 @@
       </c>
       <c r="N72" s="49" t="n">
         <f aca="false">IF(N$4='plan etatów'!$E$5,założenia!$C$14,0)</f>
-        <v>2232.28</v>
+        <v>0</v>
       </c>
       <c r="O72" s="49" t="n">
         <f aca="false">IF(O$4='plan etatów'!$E$5,założenia!$C$14,0)</f>
@@ -30171,99 +30186,99 @@
       </c>
       <c r="C84" s="49" t="n">
         <f aca="false">SUM(D84:Z84)</f>
-        <v>221600</v>
+        <v>218791.208069836</v>
       </c>
       <c r="D84" s="49" t="n">
-        <f aca="false">'plan etatów'!D106</f>
+        <f aca="false">'plan etatów'!D106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="E84" s="49" t="n">
-        <f aca="false">'plan etatów'!E106</f>
+        <f aca="false">'plan etatów'!E106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="F84" s="49" t="n">
-        <f aca="false">'plan etatów'!F106</f>
+        <f aca="false">'plan etatów'!F106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="G84" s="49" t="n">
-        <f aca="false">'plan etatów'!G106</f>
+        <f aca="false">'plan etatów'!G106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="H84" s="49" t="n">
-        <f aca="false">'plan etatów'!H106</f>
+        <f aca="false">'plan etatów'!H106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="I84" s="49" t="n">
-        <f aca="false">'plan etatów'!I106</f>
+        <f aca="false">'plan etatów'!I106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="J84" s="49" t="n">
-        <f aca="false">'plan etatów'!J106</f>
+        <f aca="false">'plan etatów'!J106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="K84" s="49" t="n">
-        <f aca="false">'plan etatów'!K106</f>
+        <f aca="false">'plan etatów'!K106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="L84" s="49" t="n">
-        <f aca="false">'plan etatów'!L106</f>
+        <f aca="false">'plan etatów'!L106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="M84" s="49" t="n">
-        <f aca="false">'plan etatów'!M106</f>
+        <f aca="false">'plan etatów'!M106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="N84" s="49" t="n">
-        <f aca="false">'plan etatów'!N106</f>
+        <f aca="false">'plan etatów'!N106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="O84" s="49" t="n">
-        <f aca="false">'plan etatów'!O106</f>
+        <f aca="false">'plan etatów'!O106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="P84" s="49" t="n">
-        <f aca="false">'plan etatów'!P106</f>
+        <f aca="false">'plan etatów'!P106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="Q84" s="49" t="n">
-        <f aca="false">'plan etatów'!Q106</f>
+        <f aca="false">'plan etatów'!Q106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="R84" s="49" t="n">
-        <f aca="false">'plan etatów'!R106</f>
+        <f aca="false">'plan etatów'!R106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="S84" s="49" t="n">
-        <f aca="false">'plan etatów'!S106</f>
+        <f aca="false">'plan etatów'!S106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="T84" s="49" t="n">
-        <f aca="false">'plan etatów'!T106</f>
+        <f aca="false">'plan etatów'!T106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="U84" s="49" t="n">
-        <f aca="false">'plan etatów'!U106</f>
+        <f aca="false">'plan etatów'!U106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="V84" s="49" t="n">
-        <f aca="false">'plan etatów'!V106</f>
+        <f aca="false">'plan etatów'!V106*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="W84" s="49" t="n">
-        <f aca="false">'plan etatów'!W106</f>
-        <v>55400</v>
+        <f aca="false">'plan etatów'!W106*założenia!$C$19</f>
+        <v>54697.8020174589</v>
       </c>
       <c r="X84" s="49" t="n">
-        <f aca="false">'plan etatów'!X106</f>
-        <v>55400</v>
+        <f aca="false">'plan etatów'!X106*założenia!$C$19</f>
+        <v>54697.8020174589</v>
       </c>
       <c r="Y84" s="49" t="n">
-        <f aca="false">'plan etatów'!Y106</f>
-        <v>55400</v>
+        <f aca="false">'plan etatów'!Y106*założenia!$C$19</f>
+        <v>54697.8020174589</v>
       </c>
       <c r="Z84" s="49" t="n">
-        <f aca="false">'plan etatów'!Z106</f>
-        <v>55400</v>
+        <f aca="false">'plan etatów'!Z106*założenia!$C$19</f>
+        <v>54697.8020174589</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30275,99 +30290,99 @@
       </c>
       <c r="C85" s="49" t="n">
         <f aca="false">SUM(D85:Z85)</f>
-        <v>37720</v>
+        <v>37241.8969692879</v>
       </c>
       <c r="D85" s="49" t="n">
-        <f aca="false">'plan etatów'!D107</f>
+        <f aca="false">'plan etatów'!D107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="E85" s="49" t="n">
-        <f aca="false">'plan etatów'!E107</f>
+        <f aca="false">'plan etatów'!E107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="F85" s="49" t="n">
-        <f aca="false">'plan etatów'!F107</f>
+        <f aca="false">'plan etatów'!F107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="G85" s="49" t="n">
-        <f aca="false">'plan etatów'!G107</f>
+        <f aca="false">'plan etatów'!G107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="H85" s="49" t="n">
-        <f aca="false">'plan etatów'!H107</f>
+        <f aca="false">'plan etatów'!H107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="I85" s="49" t="n">
-        <f aca="false">'plan etatów'!I107</f>
+        <f aca="false">'plan etatów'!I107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="J85" s="49" t="n">
-        <f aca="false">'plan etatów'!J107</f>
+        <f aca="false">'plan etatów'!J107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="K85" s="49" t="n">
-        <f aca="false">'plan etatów'!K107</f>
+        <f aca="false">'plan etatów'!K107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="L85" s="49" t="n">
-        <f aca="false">'plan etatów'!L107</f>
+        <f aca="false">'plan etatów'!L107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="M85" s="49" t="n">
-        <f aca="false">'plan etatów'!M107</f>
+        <f aca="false">'plan etatów'!M107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="N85" s="49" t="n">
-        <f aca="false">'plan etatów'!N107</f>
+        <f aca="false">'plan etatów'!N107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="O85" s="49" t="n">
-        <f aca="false">'plan etatów'!O107</f>
+        <f aca="false">'plan etatów'!O107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="P85" s="49" t="n">
-        <f aca="false">'plan etatów'!P107</f>
+        <f aca="false">'plan etatów'!P107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="Q85" s="49" t="n">
-        <f aca="false">'plan etatów'!Q107</f>
+        <f aca="false">'plan etatów'!Q107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="R85" s="49" t="n">
-        <f aca="false">'plan etatów'!R107</f>
+        <f aca="false">'plan etatów'!R107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="S85" s="49" t="n">
-        <f aca="false">'plan etatów'!S107</f>
+        <f aca="false">'plan etatów'!S107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="T85" s="49" t="n">
-        <f aca="false">'plan etatów'!T107</f>
+        <f aca="false">'plan etatów'!T107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="U85" s="49" t="n">
-        <f aca="false">'plan etatów'!U107</f>
+        <f aca="false">'plan etatów'!U107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="V85" s="49" t="n">
-        <f aca="false">'plan etatów'!V107</f>
+        <f aca="false">'plan etatów'!V107*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="W85" s="49" t="n">
-        <f aca="false">'plan etatów'!W107</f>
-        <v>9430</v>
+        <f aca="false">'plan etatów'!W107*założenia!$C$19</f>
+        <v>9310.47424232198</v>
       </c>
       <c r="X85" s="49" t="n">
-        <f aca="false">'plan etatów'!X107</f>
-        <v>9430</v>
+        <f aca="false">'plan etatów'!X107*założenia!$C$19</f>
+        <v>9310.47424232198</v>
       </c>
       <c r="Y85" s="49" t="n">
-        <f aca="false">'plan etatów'!Y107</f>
-        <v>9430</v>
+        <f aca="false">'plan etatów'!Y107*założenia!$C$19</f>
+        <v>9310.47424232198</v>
       </c>
       <c r="Z85" s="49" t="n">
-        <f aca="false">'plan etatów'!Z107</f>
-        <v>9430</v>
+        <f aca="false">'plan etatów'!Z107*założenia!$C$19</f>
+        <v>9310.47424232198</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30379,99 +30394,99 @@
       </c>
       <c r="C86" s="49" t="n">
         <f aca="false">SUM(D86:Z86)</f>
-        <v>108440</v>
+        <v>107065.517161972</v>
       </c>
       <c r="D86" s="49" t="n">
-        <f aca="false">'plan etatów'!D108</f>
+        <f aca="false">'plan etatów'!D108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="E86" s="49" t="n">
-        <f aca="false">'plan etatów'!E108</f>
+        <f aca="false">'plan etatów'!E108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="F86" s="49" t="n">
-        <f aca="false">'plan etatów'!F108</f>
+        <f aca="false">'plan etatów'!F108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="G86" s="49" t="n">
-        <f aca="false">'plan etatów'!G108</f>
+        <f aca="false">'plan etatów'!G108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="H86" s="49" t="n">
-        <f aca="false">'plan etatów'!H108</f>
+        <f aca="false">'plan etatów'!H108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="I86" s="49" t="n">
-        <f aca="false">'plan etatów'!I108</f>
+        <f aca="false">'plan etatów'!I108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="J86" s="49" t="n">
-        <f aca="false">'plan etatów'!J108</f>
+        <f aca="false">'plan etatów'!J108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="K86" s="49" t="n">
-        <f aca="false">'plan etatów'!K108</f>
+        <f aca="false">'plan etatów'!K108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="L86" s="49" t="n">
-        <f aca="false">'plan etatów'!L108</f>
+        <f aca="false">'plan etatów'!L108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="M86" s="49" t="n">
-        <f aca="false">'plan etatów'!M108</f>
+        <f aca="false">'plan etatów'!M108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="N86" s="49" t="n">
-        <f aca="false">'plan etatów'!N108</f>
+        <f aca="false">'plan etatów'!N108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="O86" s="49" t="n">
-        <f aca="false">'plan etatów'!O108</f>
+        <f aca="false">'plan etatów'!O108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="P86" s="49" t="n">
-        <f aca="false">'plan etatów'!P108</f>
+        <f aca="false">'plan etatów'!P108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="Q86" s="49" t="n">
-        <f aca="false">'plan etatów'!Q108</f>
+        <f aca="false">'plan etatów'!Q108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="R86" s="49" t="n">
-        <f aca="false">'plan etatów'!R108</f>
+        <f aca="false">'plan etatów'!R108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="S86" s="49" t="n">
-        <f aca="false">'plan etatów'!S108</f>
+        <f aca="false">'plan etatów'!S108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="T86" s="49" t="n">
-        <f aca="false">'plan etatów'!T108</f>
+        <f aca="false">'plan etatów'!T108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="U86" s="49" t="n">
-        <f aca="false">'plan etatów'!U108</f>
+        <f aca="false">'plan etatów'!U108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="V86" s="49" t="n">
-        <f aca="false">'plan etatów'!V108</f>
+        <f aca="false">'plan etatów'!V108*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="W86" s="49" t="n">
-        <f aca="false">'plan etatów'!W108</f>
-        <v>27110</v>
+        <f aca="false">'plan etatów'!W108*założenia!$C$19</f>
+        <v>26766.379290493</v>
       </c>
       <c r="X86" s="49" t="n">
-        <f aca="false">'plan etatów'!X108</f>
-        <v>27110</v>
+        <f aca="false">'plan etatów'!X108*założenia!$C$19</f>
+        <v>26766.379290493</v>
       </c>
       <c r="Y86" s="49" t="n">
-        <f aca="false">'plan etatów'!Y108</f>
-        <v>27110</v>
+        <f aca="false">'plan etatów'!Y108*założenia!$C$19</f>
+        <v>26766.379290493</v>
       </c>
       <c r="Z86" s="49" t="n">
-        <f aca="false">'plan etatów'!Z108</f>
-        <v>27110</v>
+        <f aca="false">'plan etatów'!Z108*założenia!$C$19</f>
+        <v>26766.379290493</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30483,99 +30498,99 @@
       </c>
       <c r="C87" s="49" t="n">
         <f aca="false">SUM(D87:Z87)</f>
-        <v>82500</v>
+        <v>81454.3080584903</v>
       </c>
       <c r="D87" s="49" t="n">
-        <f aca="false">'plan etatów'!D109</f>
+        <f aca="false">'plan etatów'!D109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="E87" s="49" t="n">
-        <f aca="false">'plan etatów'!E109</f>
+        <f aca="false">'plan etatów'!E109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="F87" s="49" t="n">
-        <f aca="false">'plan etatów'!F109</f>
+        <f aca="false">'plan etatów'!F109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="G87" s="49" t="n">
-        <f aca="false">'plan etatów'!G109</f>
+        <f aca="false">'plan etatów'!G109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="H87" s="49" t="n">
-        <f aca="false">'plan etatów'!H109</f>
+        <f aca="false">'plan etatów'!H109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="I87" s="49" t="n">
-        <f aca="false">'plan etatów'!I109</f>
+        <f aca="false">'plan etatów'!I109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="J87" s="49" t="n">
-        <f aca="false">'plan etatów'!J109</f>
+        <f aca="false">'plan etatów'!J109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="K87" s="49" t="n">
-        <f aca="false">'plan etatów'!K109</f>
+        <f aca="false">'plan etatów'!K109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="L87" s="49" t="n">
-        <f aca="false">'plan etatów'!L109</f>
+        <f aca="false">'plan etatów'!L109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="M87" s="49" t="n">
-        <f aca="false">'plan etatów'!M109</f>
+        <f aca="false">'plan etatów'!M109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="N87" s="49" t="n">
-        <f aca="false">'plan etatów'!N109</f>
+        <f aca="false">'plan etatów'!N109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="O87" s="49" t="n">
-        <f aca="false">'plan etatów'!O109</f>
+        <f aca="false">'plan etatów'!O109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="P87" s="49" t="n">
-        <f aca="false">'plan etatów'!P109</f>
+        <f aca="false">'plan etatów'!P109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="Q87" s="49" t="n">
-        <f aca="false">'plan etatów'!Q109</f>
+        <f aca="false">'plan etatów'!Q109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="R87" s="49" t="n">
-        <f aca="false">'plan etatów'!R109</f>
+        <f aca="false">'plan etatów'!R109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="S87" s="49" t="n">
-        <f aca="false">'plan etatów'!S109</f>
+        <f aca="false">'plan etatów'!S109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="T87" s="49" t="n">
-        <f aca="false">'plan etatów'!T109</f>
+        <f aca="false">'plan etatów'!T109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="U87" s="49" t="n">
-        <f aca="false">'plan etatów'!U109</f>
+        <f aca="false">'plan etatów'!U109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="V87" s="49" t="n">
-        <f aca="false">'plan etatów'!V109</f>
+        <f aca="false">'plan etatów'!V109*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="W87" s="49" t="n">
-        <f aca="false">'plan etatów'!W109</f>
-        <v>20625</v>
+        <f aca="false">'plan etatów'!W109*założenia!$C$19</f>
+        <v>20363.5770146226</v>
       </c>
       <c r="X87" s="49" t="n">
-        <f aca="false">'plan etatów'!X109</f>
-        <v>20625</v>
+        <f aca="false">'plan etatów'!X109*założenia!$C$19</f>
+        <v>20363.5770146226</v>
       </c>
       <c r="Y87" s="49" t="n">
-        <f aca="false">'plan etatów'!Y109</f>
-        <v>20625</v>
+        <f aca="false">'plan etatów'!Y109*założenia!$C$19</f>
+        <v>20363.5770146226</v>
       </c>
       <c r="Z87" s="49" t="n">
-        <f aca="false">'plan etatów'!Z109</f>
-        <v>20625</v>
+        <f aca="false">'plan etatów'!Z109*założenia!$C$19</f>
+        <v>20363.5770146226</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30587,99 +30602,99 @@
       </c>
       <c r="C88" s="49" t="n">
         <f aca="false">SUM(D88:Z88)</f>
-        <v>29760</v>
+        <v>29382.7903978263</v>
       </c>
       <c r="D88" s="49" t="n">
-        <f aca="false">'plan etatów'!D110</f>
+        <f aca="false">'plan etatów'!D110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="E88" s="49" t="n">
-        <f aca="false">'plan etatów'!E110</f>
+        <f aca="false">'plan etatów'!E110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="F88" s="49" t="n">
-        <f aca="false">'plan etatów'!F110</f>
+        <f aca="false">'plan etatów'!F110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="G88" s="49" t="n">
-        <f aca="false">'plan etatów'!G110</f>
+        <f aca="false">'plan etatów'!G110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="H88" s="49" t="n">
-        <f aca="false">'plan etatów'!H110</f>
+        <f aca="false">'plan etatów'!H110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="I88" s="49" t="n">
-        <f aca="false">'plan etatów'!I110</f>
+        <f aca="false">'plan etatów'!I110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="J88" s="49" t="n">
-        <f aca="false">'plan etatów'!J110</f>
+        <f aca="false">'plan etatów'!J110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="K88" s="49" t="n">
-        <f aca="false">'plan etatów'!K110</f>
+        <f aca="false">'plan etatów'!K110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="L88" s="49" t="n">
-        <f aca="false">'plan etatów'!L110</f>
+        <f aca="false">'plan etatów'!L110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="M88" s="49" t="n">
-        <f aca="false">'plan etatów'!M110</f>
+        <f aca="false">'plan etatów'!M110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="N88" s="49" t="n">
-        <f aca="false">'plan etatów'!N110</f>
+        <f aca="false">'plan etatów'!N110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="O88" s="49" t="n">
-        <f aca="false">'plan etatów'!O110</f>
+        <f aca="false">'plan etatów'!O110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="P88" s="49" t="n">
-        <f aca="false">'plan etatów'!P110</f>
+        <f aca="false">'plan etatów'!P110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="Q88" s="49" t="n">
-        <f aca="false">'plan etatów'!Q110</f>
+        <f aca="false">'plan etatów'!Q110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="R88" s="49" t="n">
-        <f aca="false">'plan etatów'!R110</f>
+        <f aca="false">'plan etatów'!R110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="S88" s="49" t="n">
-        <f aca="false">'plan etatów'!S110</f>
+        <f aca="false">'plan etatów'!S110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="T88" s="49" t="n">
-        <f aca="false">'plan etatów'!T110</f>
+        <f aca="false">'plan etatów'!T110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="U88" s="49" t="n">
-        <f aca="false">'plan etatów'!U110</f>
+        <f aca="false">'plan etatów'!U110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="V88" s="49" t="n">
-        <f aca="false">'plan etatów'!V110</f>
+        <f aca="false">'plan etatów'!V110*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="W88" s="49" t="n">
-        <f aca="false">'plan etatów'!W110</f>
-        <v>7440</v>
+        <f aca="false">'plan etatów'!W110*założenia!$C$19</f>
+        <v>7345.69759945658</v>
       </c>
       <c r="X88" s="49" t="n">
-        <f aca="false">'plan etatów'!X110</f>
-        <v>7440</v>
+        <f aca="false">'plan etatów'!X110*założenia!$C$19</f>
+        <v>7345.69759945658</v>
       </c>
       <c r="Y88" s="49" t="n">
-        <f aca="false">'plan etatów'!Y110</f>
-        <v>7440</v>
+        <f aca="false">'plan etatów'!Y110*założenia!$C$19</f>
+        <v>7345.69759945658</v>
       </c>
       <c r="Z88" s="49" t="n">
-        <f aca="false">'plan etatów'!Z110</f>
-        <v>7440</v>
+        <f aca="false">'plan etatów'!Z110*założenia!$C$19</f>
+        <v>7345.69759945658</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30691,99 +30706,99 @@
       </c>
       <c r="C89" s="49" t="n">
         <f aca="false">SUM(D89:Z89)</f>
-        <v>82500</v>
+        <v>81454.3080584903</v>
       </c>
       <c r="D89" s="49" t="n">
-        <f aca="false">'plan etatów'!D111</f>
+        <f aca="false">'plan etatów'!D111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="E89" s="49" t="n">
-        <f aca="false">'plan etatów'!E111</f>
+        <f aca="false">'plan etatów'!E111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="F89" s="49" t="n">
-        <f aca="false">'plan etatów'!F111</f>
+        <f aca="false">'plan etatów'!F111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="G89" s="49" t="n">
-        <f aca="false">'plan etatów'!G111</f>
+        <f aca="false">'plan etatów'!G111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="H89" s="49" t="n">
-        <f aca="false">'plan etatów'!H111</f>
+        <f aca="false">'plan etatów'!H111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="I89" s="49" t="n">
-        <f aca="false">'plan etatów'!I111</f>
+        <f aca="false">'plan etatów'!I111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="J89" s="49" t="n">
-        <f aca="false">'plan etatów'!J111</f>
+        <f aca="false">'plan etatów'!J111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="K89" s="49" t="n">
-        <f aca="false">'plan etatów'!K111</f>
+        <f aca="false">'plan etatów'!K111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="L89" s="49" t="n">
-        <f aca="false">'plan etatów'!L111</f>
+        <f aca="false">'plan etatów'!L111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="M89" s="49" t="n">
-        <f aca="false">'plan etatów'!M111</f>
+        <f aca="false">'plan etatów'!M111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="N89" s="49" t="n">
-        <f aca="false">'plan etatów'!N111</f>
+        <f aca="false">'plan etatów'!N111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="O89" s="49" t="n">
-        <f aca="false">'plan etatów'!O111</f>
+        <f aca="false">'plan etatów'!O111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="P89" s="49" t="n">
-        <f aca="false">'plan etatów'!P111</f>
+        <f aca="false">'plan etatów'!P111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="Q89" s="49" t="n">
-        <f aca="false">'plan etatów'!Q111</f>
+        <f aca="false">'plan etatów'!Q111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="R89" s="49" t="n">
-        <f aca="false">'plan etatów'!R111</f>
+        <f aca="false">'plan etatów'!R111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="S89" s="49" t="n">
-        <f aca="false">'plan etatów'!S111</f>
+        <f aca="false">'plan etatów'!S111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="T89" s="49" t="n">
-        <f aca="false">'plan etatów'!T111</f>
+        <f aca="false">'plan etatów'!T111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="U89" s="49" t="n">
-        <f aca="false">'plan etatów'!U111</f>
+        <f aca="false">'plan etatów'!U111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="V89" s="49" t="n">
-        <f aca="false">'plan etatów'!V111</f>
+        <f aca="false">'plan etatów'!V111*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="W89" s="49" t="n">
-        <f aca="false">'plan etatów'!W111</f>
-        <v>20625</v>
+        <f aca="false">'plan etatów'!W111*założenia!$C$19</f>
+        <v>20363.5770146226</v>
       </c>
       <c r="X89" s="49" t="n">
-        <f aca="false">'plan etatów'!X111</f>
-        <v>20625</v>
+        <f aca="false">'plan etatów'!X111*założenia!$C$19</f>
+        <v>20363.5770146226</v>
       </c>
       <c r="Y89" s="49" t="n">
-        <f aca="false">'plan etatów'!Y111</f>
-        <v>20625</v>
+        <f aca="false">'plan etatów'!Y111*założenia!$C$19</f>
+        <v>20363.5770146226</v>
       </c>
       <c r="Z89" s="49" t="n">
-        <f aca="false">'plan etatów'!Z111</f>
-        <v>20625</v>
+        <f aca="false">'plan etatów'!Z111*założenia!$C$19</f>
+        <v>20363.5770146226</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30795,99 +30810,99 @@
       </c>
       <c r="C90" s="49" t="n">
         <f aca="false">SUM(D90:Z90)</f>
-        <v>2857.14</v>
+        <v>2820.92559668164</v>
       </c>
       <c r="D90" s="49" t="n">
-        <f aca="false">'plan etatów'!D112</f>
+        <f aca="false">'plan etatów'!D112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="E90" s="49" t="n">
-        <f aca="false">'plan etatów'!E112</f>
+        <f aca="false">'plan etatów'!E112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="F90" s="49" t="n">
-        <f aca="false">'plan etatów'!F112</f>
+        <f aca="false">'plan etatów'!F112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="G90" s="49" t="n">
-        <f aca="false">'plan etatów'!G112</f>
+        <f aca="false">'plan etatów'!G112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="H90" s="49" t="n">
-        <f aca="false">'plan etatów'!H112</f>
+        <f aca="false">'plan etatów'!H112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="I90" s="49" t="n">
-        <f aca="false">'plan etatów'!I112</f>
+        <f aca="false">'plan etatów'!I112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="J90" s="49" t="n">
-        <f aca="false">'plan etatów'!J112</f>
+        <f aca="false">'plan etatów'!J112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="K90" s="49" t="n">
-        <f aca="false">'plan etatów'!K112</f>
+        <f aca="false">'plan etatów'!K112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="L90" s="49" t="n">
-        <f aca="false">'plan etatów'!L112</f>
+        <f aca="false">'plan etatów'!L112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="M90" s="49" t="n">
-        <f aca="false">'plan etatów'!M112</f>
+        <f aca="false">'plan etatów'!M112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="N90" s="49" t="n">
-        <f aca="false">'plan etatów'!N112</f>
+        <f aca="false">'plan etatów'!N112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="O90" s="49" t="n">
-        <f aca="false">'plan etatów'!O112</f>
+        <f aca="false">'plan etatów'!O112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="P90" s="49" t="n">
-        <f aca="false">'plan etatów'!P112</f>
+        <f aca="false">'plan etatów'!P112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="Q90" s="49" t="n">
-        <f aca="false">'plan etatów'!Q112</f>
+        <f aca="false">'plan etatów'!Q112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="R90" s="49" t="n">
-        <f aca="false">'plan etatów'!R112</f>
+        <f aca="false">'plan etatów'!R112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="S90" s="49" t="n">
-        <f aca="false">'plan etatów'!S112</f>
+        <f aca="false">'plan etatów'!S112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="T90" s="49" t="n">
-        <f aca="false">'plan etatów'!T112</f>
+        <f aca="false">'plan etatów'!T112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="U90" s="49" t="n">
-        <f aca="false">'plan etatów'!U112</f>
+        <f aca="false">'plan etatów'!U112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="V90" s="49" t="n">
-        <f aca="false">'plan etatów'!V112</f>
+        <f aca="false">'plan etatów'!V112*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="W90" s="49" t="n">
-        <f aca="false">'plan etatów'!W112</f>
-        <v>714.285</v>
+        <f aca="false">'plan etatów'!W112*założenia!$C$19</f>
+        <v>705.231399170409</v>
       </c>
       <c r="X90" s="49" t="n">
-        <f aca="false">'plan etatów'!X112</f>
-        <v>714.285</v>
+        <f aca="false">'plan etatów'!X112*założenia!$C$19</f>
+        <v>705.231399170409</v>
       </c>
       <c r="Y90" s="49" t="n">
-        <f aca="false">'plan etatów'!Y112</f>
-        <v>714.285</v>
+        <f aca="false">'plan etatów'!Y112*założenia!$C$19</f>
+        <v>705.231399170409</v>
       </c>
       <c r="Z90" s="49" t="n">
-        <f aca="false">'plan etatów'!Z112</f>
-        <v>714.285</v>
+        <f aca="false">'plan etatów'!Z112*założenia!$C$19</f>
+        <v>705.231399170409</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30899,99 +30914,99 @@
       </c>
       <c r="C91" s="49" t="n">
         <f aca="false">SUM(D91:Z91)</f>
-        <v>79000</v>
+        <v>77998.670746918</v>
       </c>
       <c r="D91" s="49" t="n">
-        <f aca="false">'plan etatów'!D113</f>
+        <f aca="false">'plan etatów'!D113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="E91" s="49" t="n">
-        <f aca="false">'plan etatów'!E113</f>
+        <f aca="false">'plan etatów'!E113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="F91" s="49" t="n">
-        <f aca="false">'plan etatów'!F113</f>
+        <f aca="false">'plan etatów'!F113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="G91" s="49" t="n">
-        <f aca="false">'plan etatów'!G113</f>
+        <f aca="false">'plan etatów'!G113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="H91" s="49" t="n">
-        <f aca="false">'plan etatów'!H113</f>
+        <f aca="false">'plan etatów'!H113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="I91" s="49" t="n">
-        <f aca="false">'plan etatów'!I113</f>
+        <f aca="false">'plan etatów'!I113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="J91" s="49" t="n">
-        <f aca="false">'plan etatów'!J113</f>
+        <f aca="false">'plan etatów'!J113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="K91" s="49" t="n">
-        <f aca="false">'plan etatów'!K113</f>
+        <f aca="false">'plan etatów'!K113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="L91" s="49" t="n">
-        <f aca="false">'plan etatów'!L113</f>
+        <f aca="false">'plan etatów'!L113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="M91" s="49" t="n">
-        <f aca="false">'plan etatów'!M113</f>
+        <f aca="false">'plan etatów'!M113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="N91" s="49" t="n">
-        <f aca="false">'plan etatów'!N113</f>
+        <f aca="false">'plan etatów'!N113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="O91" s="49" t="n">
-        <f aca="false">'plan etatów'!O113</f>
+        <f aca="false">'plan etatów'!O113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="P91" s="49" t="n">
-        <f aca="false">'plan etatów'!P113</f>
+        <f aca="false">'plan etatów'!P113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="Q91" s="49" t="n">
-        <f aca="false">'plan etatów'!Q113</f>
+        <f aca="false">'plan etatów'!Q113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="R91" s="49" t="n">
-        <f aca="false">'plan etatów'!R113</f>
+        <f aca="false">'plan etatów'!R113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="S91" s="49" t="n">
-        <f aca="false">'plan etatów'!S113</f>
+        <f aca="false">'plan etatów'!S113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="T91" s="49" t="n">
-        <f aca="false">'plan etatów'!T113</f>
+        <f aca="false">'plan etatów'!T113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="U91" s="49" t="n">
-        <f aca="false">'plan etatów'!U113</f>
+        <f aca="false">'plan etatów'!U113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="V91" s="49" t="n">
-        <f aca="false">'plan etatów'!V113</f>
+        <f aca="false">'plan etatów'!V113*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="W91" s="49" t="n">
-        <f aca="false">'plan etatów'!W113</f>
-        <v>19750</v>
+        <f aca="false">'plan etatów'!W113*założenia!$C$19</f>
+        <v>19499.6676867295</v>
       </c>
       <c r="X91" s="49" t="n">
-        <f aca="false">'plan etatów'!X113</f>
-        <v>19750</v>
+        <f aca="false">'plan etatów'!X113*założenia!$C$19</f>
+        <v>19499.6676867295</v>
       </c>
       <c r="Y91" s="49" t="n">
-        <f aca="false">'plan etatów'!Y113</f>
-        <v>19750</v>
+        <f aca="false">'plan etatów'!Y113*założenia!$C$19</f>
+        <v>19499.6676867295</v>
       </c>
       <c r="Z91" s="49" t="n">
-        <f aca="false">'plan etatów'!Z113</f>
-        <v>19750</v>
+        <f aca="false">'plan etatów'!Z113*założenia!$C$19</f>
+        <v>19499.6676867295</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31003,104 +31018,104 @@
       </c>
       <c r="C92" s="49" t="n">
         <f aca="false">SUM(D92:Z92)</f>
-        <v>19680</v>
+        <v>19430.554940498</v>
       </c>
       <c r="D92" s="49" t="n">
-        <f aca="false">'plan etatów'!D114</f>
+        <f aca="false">'plan etatów'!D114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="E92" s="49" t="n">
-        <f aca="false">'plan etatów'!E114</f>
+        <f aca="false">'plan etatów'!E114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="F92" s="49" t="n">
-        <f aca="false">'plan etatów'!F114</f>
+        <f aca="false">'plan etatów'!F114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="G92" s="49" t="n">
-        <f aca="false">'plan etatów'!G114</f>
+        <f aca="false">'plan etatów'!G114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="H92" s="49" t="n">
-        <f aca="false">'plan etatów'!H114</f>
+        <f aca="false">'plan etatów'!H114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="I92" s="49" t="n">
-        <f aca="false">'plan etatów'!I114</f>
+        <f aca="false">'plan etatów'!I114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="J92" s="49" t="n">
-        <f aca="false">'plan etatów'!J114</f>
+        <f aca="false">'plan etatów'!J114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="K92" s="49" t="n">
-        <f aca="false">'plan etatów'!K114</f>
+        <f aca="false">'plan etatów'!K114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="L92" s="49" t="n">
-        <f aca="false">'plan etatów'!L114</f>
+        <f aca="false">'plan etatów'!L114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="M92" s="49" t="n">
-        <f aca="false">'plan etatów'!M114</f>
+        <f aca="false">'plan etatów'!M114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="N92" s="49" t="n">
-        <f aca="false">'plan etatów'!N114</f>
+        <f aca="false">'plan etatów'!N114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="O92" s="49" t="n">
-        <f aca="false">'plan etatów'!O114</f>
+        <f aca="false">'plan etatów'!O114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="P92" s="49" t="n">
-        <f aca="false">'plan etatów'!P114</f>
+        <f aca="false">'plan etatów'!P114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="Q92" s="49" t="n">
-        <f aca="false">'plan etatów'!Q114</f>
+        <f aca="false">'plan etatów'!Q114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="R92" s="49" t="n">
-        <f aca="false">'plan etatów'!R114</f>
+        <f aca="false">'plan etatów'!R114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="S92" s="49" t="n">
-        <f aca="false">'plan etatów'!S114</f>
+        <f aca="false">'plan etatów'!S114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="T92" s="49" t="n">
-        <f aca="false">'plan etatów'!T114</f>
+        <f aca="false">'plan etatów'!T114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="U92" s="49" t="n">
-        <f aca="false">'plan etatów'!U114</f>
+        <f aca="false">'plan etatów'!U114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="V92" s="49" t="n">
-        <f aca="false">'plan etatów'!V114</f>
+        <f aca="false">'plan etatów'!V114*założenia!$C$19</f>
         <v>0</v>
       </c>
       <c r="W92" s="49" t="n">
-        <f aca="false">'plan etatów'!W114</f>
-        <v>4920</v>
+        <f aca="false">'plan etatów'!W114*założenia!$C$19</f>
+        <v>4857.63873512451</v>
       </c>
       <c r="X92" s="49" t="n">
-        <f aca="false">'plan etatów'!X114</f>
-        <v>4920</v>
+        <f aca="false">'plan etatów'!X114*założenia!$C$19</f>
+        <v>4857.63873512451</v>
       </c>
       <c r="Y92" s="49" t="n">
-        <f aca="false">'plan etatów'!Y114</f>
-        <v>4920</v>
+        <f aca="false">'plan etatów'!Y114*założenia!$C$19</f>
+        <v>4857.63873512451</v>
       </c>
       <c r="Z92" s="49" t="n">
-        <f aca="false">'plan etatów'!Z114</f>
-        <v>4920</v>
+        <f aca="false">'plan etatów'!Z114*założenia!$C$19</f>
+        <v>4857.63873512451</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="40" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B93" s="40" t="n">
         <v>1</v>
@@ -31204,14 +31219,14 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="40" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B94" s="40" t="n">
         <v>2</v>
       </c>
       <c r="C94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,C$56:C$92)</f>
-        <v>1013011.2</v>
+        <v>1010778.92</v>
       </c>
       <c r="D94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,D$56:D$92)</f>
@@ -31255,7 +31270,7 @@
       </c>
       <c r="N94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,N$56:N$92)</f>
-        <v>170695.433333333</v>
+        <v>168463.153333333</v>
       </c>
       <c r="O94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,O$56:O$92)</f>
@@ -31308,7 +31323,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="40" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B95" s="40" t="n">
         <v>3</v>
@@ -31412,14 +31427,14 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="40" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B96" s="40" t="n">
         <v>4</v>
       </c>
       <c r="C96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,C$56:C$92)</f>
-        <v>664057.14</v>
+        <v>655640.18</v>
       </c>
       <c r="D96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,D$56:D$92)</f>
@@ -31499,19 +31514,19 @@
       </c>
       <c r="W96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,W$56:W$92)</f>
-        <v>166014.285</v>
+        <v>163910.045</v>
       </c>
       <c r="X96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,X$56:X$92)</f>
-        <v>166014.285</v>
+        <v>163910.045</v>
       </c>
       <c r="Y96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,Y$56:Y$92)</f>
-        <v>166014.285</v>
+        <v>163910.045</v>
       </c>
       <c r="Z96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,Z$56:Z$92)</f>
-        <v>166014.285</v>
+        <v>163910.045</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31521,7 +31536,7 @@
       <c r="B97" s="40"/>
       <c r="C97" s="63" t="n">
         <f aca="false">SUM(C93:C96)</f>
-        <v>3874492.49</v>
+        <v>3863843.25</v>
       </c>
       <c r="D97" s="63" t="n">
         <f aca="false">SUM(D93:D96)</f>
@@ -31565,7 +31580,7 @@
       </c>
       <c r="N97" s="63" t="n">
         <f aca="false">SUM(N93:N96)</f>
-        <v>170695.433333333</v>
+        <v>168463.153333333</v>
       </c>
       <c r="O97" s="63" t="n">
         <f aca="false">SUM(O93:O96)</f>
@@ -31601,29 +31616,29 @@
       </c>
       <c r="W97" s="63" t="n">
         <f aca="false">SUM(W93:W96)</f>
-        <v>166014.285</v>
+        <v>163910.045</v>
       </c>
       <c r="X97" s="63" t="n">
         <f aca="false">SUM(X93:X96)</f>
-        <v>166014.285</v>
+        <v>163910.045</v>
       </c>
       <c r="Y97" s="63" t="n">
         <f aca="false">SUM(Y93:Y96)</f>
-        <v>166014.285</v>
+        <v>163910.045</v>
       </c>
       <c r="Z97" s="63" t="n">
         <f aca="false">SUM(Z93:Z96)</f>
-        <v>166014.285</v>
+        <v>163910.045</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="40" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B98" s="40"/>
       <c r="C98" s="63" t="n">
         <f aca="false">0.25*C97</f>
-        <v>968623.1225</v>
+        <v>965960.8125</v>
       </c>
       <c r="D98" s="63" t="n">
         <f aca="false">0.25*D97</f>
@@ -31667,7 +31682,7 @@
       </c>
       <c r="N98" s="63" t="n">
         <f aca="false">0.25*N97</f>
-        <v>42673.8583333333</v>
+        <v>42115.7883333333</v>
       </c>
       <c r="O98" s="63" t="n">
         <f aca="false">0.25*O97</f>
@@ -31703,29 +31718,29 @@
       </c>
       <c r="W98" s="63" t="n">
         <f aca="false">0.25*W97</f>
-        <v>41503.57125</v>
+        <v>40977.51125</v>
       </c>
       <c r="X98" s="63" t="n">
         <f aca="false">0.25*X97</f>
-        <v>41503.57125</v>
+        <v>40977.51125</v>
       </c>
       <c r="Y98" s="63" t="n">
         <f aca="false">0.25*Y97</f>
-        <v>41503.57125</v>
+        <v>40977.51125</v>
       </c>
       <c r="Z98" s="63" t="n">
         <f aca="false">0.25*Z97</f>
-        <v>41503.57125</v>
+        <v>40977.51125</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="40" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B99" s="40"/>
       <c r="C99" s="63" t="n">
         <f aca="false">C97+C98</f>
-        <v>4843115.6125</v>
+        <v>4829804.0625</v>
       </c>
       <c r="D99" s="63" t="n">
         <f aca="false">D97+D98</f>
@@ -31769,7 +31784,7 @@
       </c>
       <c r="N99" s="63" t="n">
         <f aca="false">N97+N98</f>
-        <v>213369.291666667</v>
+        <v>210578.941666667</v>
       </c>
       <c r="O99" s="63" t="n">
         <f aca="false">O97+O98</f>
@@ -31805,24 +31820,24 @@
       </c>
       <c r="W99" s="63" t="n">
         <f aca="false">W97+W98</f>
-        <v>207517.85625</v>
+        <v>204887.55625</v>
       </c>
       <c r="X99" s="63" t="n">
         <f aca="false">X97+X98</f>
-        <v>207517.85625</v>
+        <v>204887.55625</v>
       </c>
       <c r="Y99" s="63" t="n">
         <f aca="false">Y97+Y98</f>
-        <v>207517.85625</v>
+        <v>204887.55625</v>
       </c>
       <c r="Z99" s="63" t="n">
         <f aca="false">Z97+Z98</f>
-        <v>207517.85625</v>
+        <v>204887.55625</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="40" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B100" s="40"/>
       <c r="C100" s="63"/>
@@ -31868,55 +31883,55 @@
       </c>
       <c r="N100" s="63" t="n">
         <f aca="false">M100+N99</f>
-        <v>2275545.0875</v>
+        <v>2272754.7375</v>
       </c>
       <c r="O100" s="63" t="n">
         <f aca="false">N100+O99</f>
-        <v>2486378.56875</v>
+        <v>2483588.21875</v>
       </c>
       <c r="P100" s="63" t="n">
         <f aca="false">O100+P99</f>
-        <v>2697212.05</v>
+        <v>2694421.7</v>
       </c>
       <c r="Q100" s="63" t="n">
         <f aca="false">P100+Q99</f>
-        <v>2916517.40625</v>
+        <v>2913727.05625</v>
       </c>
       <c r="R100" s="63" t="n">
         <f aca="false">Q100+R99</f>
-        <v>3135822.7625</v>
+        <v>3133032.4125</v>
       </c>
       <c r="S100" s="63" t="n">
         <f aca="false">R100+S99</f>
-        <v>3355128.11875</v>
+        <v>3352337.76875</v>
       </c>
       <c r="T100" s="63" t="n">
         <f aca="false">S100+T99</f>
-        <v>3574433.475</v>
+        <v>3571643.125</v>
       </c>
       <c r="U100" s="63" t="n">
         <f aca="false">T100+U99</f>
-        <v>3793738.83125</v>
+        <v>3790948.48125</v>
       </c>
       <c r="V100" s="63" t="n">
         <f aca="false">U100+V99</f>
-        <v>4013044.1875</v>
+        <v>4010253.8375</v>
       </c>
       <c r="W100" s="63" t="n">
         <f aca="false">V100+W99</f>
-        <v>4220562.04375</v>
+        <v>4215141.39375</v>
       </c>
       <c r="X100" s="63" t="n">
         <f aca="false">W100+X99</f>
-        <v>4428079.9</v>
+        <v>4420028.95</v>
       </c>
       <c r="Y100" s="63" t="n">
         <f aca="false">X100+Y99</f>
-        <v>4635597.75625</v>
+        <v>4624916.50625</v>
       </c>
       <c r="Z100" s="63" t="n">
         <f aca="false">Y100+Z99</f>
-        <v>4843115.6125</v>
+        <v>4829804.0625</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31949,7 +31964,7 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="60" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B102" s="61"/>
       <c r="C102" s="62"/>
@@ -35827,7 +35842,7 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="40" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B140" s="40" t="n">
         <v>1</v>
@@ -35931,7 +35946,7 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="40" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B141" s="40" t="n">
         <v>2</v>
@@ -36035,7 +36050,7 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="40" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B142" s="40" t="n">
         <v>3</v>
@@ -36139,7 +36154,7 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="40" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B143" s="40" t="n">
         <v>4</v>
@@ -36345,7 +36360,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="40" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B145" s="40"/>
       <c r="C145" s="63" t="n">
@@ -36447,7 +36462,7 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="40" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B146" s="40"/>
       <c r="C146" s="63" t="n">
@@ -36549,7 +36564,7 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="40" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B147" s="40"/>
       <c r="C147" s="63"/>
@@ -36676,7 +36691,7 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="64" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B149" s="65"/>
       <c r="C149" s="66"/>
@@ -38377,7 +38392,7 @@
       </c>
       <c r="C166" s="49" t="n">
         <f aca="false">SUM(D166:Z166)</f>
-        <v>1785.82</v>
+        <v>0</v>
       </c>
       <c r="D166" s="49" t="n">
         <f aca="false">IF(D$4='plan etatów'!$E$5,założenia!$C$9,0)</f>
@@ -38421,7 +38436,7 @@
       </c>
       <c r="N166" s="49" t="n">
         <f aca="false">IF(N$4='plan etatów'!$E$5,założenia!$C$9,0)</f>
-        <v>1785.82</v>
+        <v>0</v>
       </c>
       <c r="O166" s="49" t="n">
         <f aca="false">IF(O$4='plan etatów'!$E$5,założenia!$C$9,0)</f>
@@ -39625,99 +39640,99 @@
       </c>
       <c r="C178" s="49" t="n">
         <f aca="false">SUM(D178:Z178)</f>
-        <v>130678.784927454</v>
+        <v>131274.724841901</v>
       </c>
       <c r="D178" s="49" t="n">
-        <f aca="false">D84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">D84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="E178" s="49" t="n">
-        <f aca="false">E84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">E84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="F178" s="49" t="n">
-        <f aca="false">F84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">F84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="G178" s="49" t="n">
-        <f aca="false">G84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">G84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="H178" s="49" t="n">
-        <f aca="false">H84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">H84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="I178" s="49" t="n">
-        <f aca="false">I84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">I84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="J178" s="49" t="n">
-        <f aca="false">J84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">J84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="K178" s="49" t="n">
-        <f aca="false">K84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">K84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="L178" s="49" t="n">
-        <f aca="false">L84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">L84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="M178" s="49" t="n">
-        <f aca="false">M84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">M84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="N178" s="49" t="n">
-        <f aca="false">N84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">N84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="O178" s="49" t="n">
-        <f aca="false">O84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">O84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="P178" s="49" t="n">
-        <f aca="false">P84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">P84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="Q178" s="49" t="n">
-        <f aca="false">Q84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">Q84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="R178" s="49" t="n">
-        <f aca="false">R84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">R84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="S178" s="49" t="n">
-        <f aca="false">S84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">S84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="T178" s="49" t="n">
-        <f aca="false">T84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">T84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="U178" s="49" t="n">
-        <f aca="false">U84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">U84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="V178" s="49" t="n">
-        <f aca="false">V84*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">V84*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="W178" s="49" t="n">
-        <f aca="false">W84*(założenia!$C$7-założenia!$C$19)</f>
-        <v>32669.6962318634</v>
+        <f aca="false">W84*założenia!$C$7</f>
+        <v>32818.6812104754</v>
       </c>
       <c r="X178" s="49" t="n">
-        <f aca="false">X84*(założenia!$C$7-założenia!$C$19)</f>
-        <v>32669.6962318634</v>
+        <f aca="false">X84*założenia!$C$7</f>
+        <v>32818.6812104754</v>
       </c>
       <c r="Y178" s="49" t="n">
-        <f aca="false">Y84*(założenia!$C$7-założenia!$C$19)</f>
-        <v>32669.6962318634</v>
+        <f aca="false">Y84*założenia!$C$7</f>
+        <v>32818.6812104754</v>
       </c>
       <c r="Z178" s="49" t="n">
-        <f aca="false">Z84*(założenia!$C$7-założenia!$C$19)</f>
-        <v>32669.6962318634</v>
+        <f aca="false">Z84*założenia!$C$7</f>
+        <v>32818.6812104754</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39729,99 +39744,99 @@
       </c>
       <c r="C179" s="49" t="n">
         <f aca="false">SUM(D179:Z179)</f>
-        <v>22243.6993116586</v>
+        <v>22345.1381815727</v>
       </c>
       <c r="D179" s="49" t="n">
-        <f aca="false">D85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">D85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="E179" s="49" t="n">
-        <f aca="false">E85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">E85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="F179" s="49" t="n">
-        <f aca="false">F85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">F85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="G179" s="49" t="n">
-        <f aca="false">G85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">G85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="H179" s="49" t="n">
-        <f aca="false">H85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">H85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="I179" s="49" t="n">
-        <f aca="false">I85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">I85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="J179" s="49" t="n">
-        <f aca="false">J85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">J85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="K179" s="49" t="n">
-        <f aca="false">K85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">K85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="L179" s="49" t="n">
-        <f aca="false">L85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">L85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="M179" s="49" t="n">
-        <f aca="false">M85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">M85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="N179" s="49" t="n">
-        <f aca="false">N85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">N85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="O179" s="49" t="n">
-        <f aca="false">O85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">O85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="P179" s="49" t="n">
-        <f aca="false">P85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">P85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="Q179" s="49" t="n">
-        <f aca="false">Q85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">Q85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="R179" s="49" t="n">
-        <f aca="false">R85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">R85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="S179" s="49" t="n">
-        <f aca="false">S85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">S85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="T179" s="49" t="n">
-        <f aca="false">T85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">T85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="U179" s="49" t="n">
-        <f aca="false">U85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">U85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="V179" s="49" t="n">
-        <f aca="false">V85*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">V85*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="W179" s="49" t="n">
-        <f aca="false">W85*(założenia!$C$7-założenia!$C$19)</f>
-        <v>5560.92482791466</v>
+        <f aca="false">W85*założenia!$C$7</f>
+        <v>5586.28454539319</v>
       </c>
       <c r="X179" s="49" t="n">
-        <f aca="false">X85*(założenia!$C$7-założenia!$C$19)</f>
-        <v>5560.92482791466</v>
+        <f aca="false">X85*założenia!$C$7</f>
+        <v>5586.28454539319</v>
       </c>
       <c r="Y179" s="49" t="n">
-        <f aca="false">Y85*(założenia!$C$7-założenia!$C$19)</f>
-        <v>5560.92482791466</v>
+        <f aca="false">Y85*założenia!$C$7</f>
+        <v>5586.28454539319</v>
       </c>
       <c r="Z179" s="49" t="n">
-        <f aca="false">Z85*(założenia!$C$7-założenia!$C$19)</f>
-        <v>5560.92482791466</v>
+        <f aca="false">Z85*założenia!$C$7</f>
+        <v>5586.28454539319</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39833,99 +39848,99 @@
       </c>
       <c r="C180" s="49" t="n">
         <f aca="false">SUM(D180:Z180)</f>
-        <v>63947.6869924778</v>
+        <v>64239.3102971832</v>
       </c>
       <c r="D180" s="49" t="n">
-        <f aca="false">D86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">D86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="E180" s="49" t="n">
-        <f aca="false">E86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">E86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="F180" s="49" t="n">
-        <f aca="false">F86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">F86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="G180" s="49" t="n">
-        <f aca="false">G86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">G86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="H180" s="49" t="n">
-        <f aca="false">H86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">H86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="I180" s="49" t="n">
-        <f aca="false">I86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">I86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="J180" s="49" t="n">
-        <f aca="false">J86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">J86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="K180" s="49" t="n">
-        <f aca="false">K86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">K86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="L180" s="49" t="n">
-        <f aca="false">L86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">L86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="M180" s="49" t="n">
-        <f aca="false">M86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">M86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="N180" s="49" t="n">
-        <f aca="false">N86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">N86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="O180" s="49" t="n">
-        <f aca="false">O86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">O86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="P180" s="49" t="n">
-        <f aca="false">P86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">P86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="Q180" s="49" t="n">
-        <f aca="false">Q86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">Q86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="R180" s="49" t="n">
-        <f aca="false">R86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">R86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="S180" s="49" t="n">
-        <f aca="false">S86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">S86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="T180" s="49" t="n">
-        <f aca="false">T86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">T86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="U180" s="49" t="n">
-        <f aca="false">U86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">U86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="V180" s="49" t="n">
-        <f aca="false">V86*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">V86*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="W180" s="49" t="n">
-        <f aca="false">W86*(założenia!$C$7-założenia!$C$19)</f>
-        <v>15986.9217481194</v>
+        <f aca="false">W86*założenia!$C$7</f>
+        <v>16059.8275742958</v>
       </c>
       <c r="X180" s="49" t="n">
-        <f aca="false">X86*(założenia!$C$7-założenia!$C$19)</f>
-        <v>15986.9217481194</v>
+        <f aca="false">X86*założenia!$C$7</f>
+        <v>16059.8275742958</v>
       </c>
       <c r="Y180" s="49" t="n">
-        <f aca="false">Y86*(założenia!$C$7-założenia!$C$19)</f>
-        <v>15986.9217481194</v>
+        <f aca="false">Y86*założenia!$C$7</f>
+        <v>16059.8275742958</v>
       </c>
       <c r="Z180" s="49" t="n">
-        <f aca="false">Z86*(założenia!$C$7-założenia!$C$19)</f>
-        <v>15986.9217481194</v>
+        <f aca="false">Z86*założenia!$C$7</f>
+        <v>16059.8275742958</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39937,99 +39952,99 @@
       </c>
       <c r="C181" s="49" t="n">
         <f aca="false">SUM(D181:Z181)</f>
-        <v>48650.7209229013</v>
+        <v>48872.5848350942</v>
       </c>
       <c r="D181" s="49" t="n">
-        <f aca="false">D87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">D87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="E181" s="49" t="n">
-        <f aca="false">E87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">E87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="F181" s="49" t="n">
-        <f aca="false">F87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">F87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="G181" s="49" t="n">
-        <f aca="false">G87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">G87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="H181" s="49" t="n">
-        <f aca="false">H87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">H87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="I181" s="49" t="n">
-        <f aca="false">I87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">I87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="J181" s="49" t="n">
-        <f aca="false">J87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">J87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="K181" s="49" t="n">
-        <f aca="false">K87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">K87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="L181" s="49" t="n">
-        <f aca="false">L87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">L87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="M181" s="49" t="n">
-        <f aca="false">M87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">M87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="N181" s="49" t="n">
-        <f aca="false">N87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">N87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="O181" s="49" t="n">
-        <f aca="false">O87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">O87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="P181" s="49" t="n">
-        <f aca="false">P87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">P87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="Q181" s="49" t="n">
-        <f aca="false">Q87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">Q87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="R181" s="49" t="n">
-        <f aca="false">R87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">R87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="S181" s="49" t="n">
-        <f aca="false">S87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">S87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="T181" s="49" t="n">
-        <f aca="false">T87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">T87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="U181" s="49" t="n">
-        <f aca="false">U87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">U87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="V181" s="49" t="n">
-        <f aca="false">V87*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">V87*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="W181" s="49" t="n">
-        <f aca="false">W87*(założenia!$C$7-założenia!$C$19)</f>
-        <v>12162.6802307253</v>
+        <f aca="false">W87*założenia!$C$7</f>
+        <v>12218.1462087735</v>
       </c>
       <c r="X181" s="49" t="n">
-        <f aca="false">X87*(założenia!$C$7-założenia!$C$19)</f>
-        <v>12162.6802307253</v>
+        <f aca="false">X87*założenia!$C$7</f>
+        <v>12218.1462087735</v>
       </c>
       <c r="Y181" s="49" t="n">
-        <f aca="false">Y87*(założenia!$C$7-założenia!$C$19)</f>
-        <v>12162.6802307253</v>
+        <f aca="false">Y87*założenia!$C$7</f>
+        <v>12218.1462087735</v>
       </c>
       <c r="Z181" s="49" t="n">
-        <f aca="false">Z87*(założenia!$C$7-założenia!$C$19)</f>
-        <v>12162.6802307253</v>
+        <f aca="false">Z87*założenia!$C$7</f>
+        <v>12218.1462087735</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40041,99 +40056,99 @@
       </c>
       <c r="C182" s="49" t="n">
         <f aca="false">SUM(D182:Z182)</f>
-        <v>17549.6418747338</v>
+        <v>17629.6742386958</v>
       </c>
       <c r="D182" s="49" t="n">
-        <f aca="false">D88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">D88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="E182" s="49" t="n">
-        <f aca="false">E88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">E88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="F182" s="49" t="n">
-        <f aca="false">F88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">F88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="G182" s="49" t="n">
-        <f aca="false">G88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">G88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="H182" s="49" t="n">
-        <f aca="false">H88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">H88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="I182" s="49" t="n">
-        <f aca="false">I88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">I88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="J182" s="49" t="n">
-        <f aca="false">J88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">J88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="K182" s="49" t="n">
-        <f aca="false">K88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">K88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="L182" s="49" t="n">
-        <f aca="false">L88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">L88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="M182" s="49" t="n">
-        <f aca="false">M88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">M88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="N182" s="49" t="n">
-        <f aca="false">N88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">N88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="O182" s="49" t="n">
-        <f aca="false">O88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">O88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="P182" s="49" t="n">
-        <f aca="false">P88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">P88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="Q182" s="49" t="n">
-        <f aca="false">Q88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">Q88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="R182" s="49" t="n">
-        <f aca="false">R88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">R88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="S182" s="49" t="n">
-        <f aca="false">S88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">S88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="T182" s="49" t="n">
-        <f aca="false">T88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">T88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="U182" s="49" t="n">
-        <f aca="false">U88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">U88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="V182" s="49" t="n">
-        <f aca="false">V88*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">V88*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="W182" s="49" t="n">
-        <f aca="false">W88*(założenia!$C$7-założenia!$C$19)</f>
-        <v>4387.41046868346</v>
+        <f aca="false">W88*założenia!$C$7</f>
+        <v>4407.41855967395</v>
       </c>
       <c r="X182" s="49" t="n">
-        <f aca="false">X88*(założenia!$C$7-założenia!$C$19)</f>
-        <v>4387.41046868346</v>
+        <f aca="false">X88*założenia!$C$7</f>
+        <v>4407.41855967395</v>
       </c>
       <c r="Y182" s="49" t="n">
-        <f aca="false">Y88*(założenia!$C$7-założenia!$C$19)</f>
-        <v>4387.41046868346</v>
+        <f aca="false">Y88*założenia!$C$7</f>
+        <v>4407.41855967395</v>
       </c>
       <c r="Z182" s="49" t="n">
-        <f aca="false">Z88*(założenia!$C$7-założenia!$C$19)</f>
-        <v>4387.41046868346</v>
+        <f aca="false">Z88*założenia!$C$7</f>
+        <v>4407.41855967395</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40145,99 +40160,99 @@
       </c>
       <c r="C183" s="49" t="n">
         <f aca="false">SUM(D183:Z183)</f>
-        <v>48650.7209229013</v>
+        <v>48872.5848350942</v>
       </c>
       <c r="D183" s="49" t="n">
-        <f aca="false">D89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">D89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="E183" s="49" t="n">
-        <f aca="false">E89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">E89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="F183" s="49" t="n">
-        <f aca="false">F89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">F89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="G183" s="49" t="n">
-        <f aca="false">G89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">G89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="H183" s="49" t="n">
-        <f aca="false">H89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">H89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="I183" s="49" t="n">
-        <f aca="false">I89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">I89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="J183" s="49" t="n">
-        <f aca="false">J89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">J89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="K183" s="49" t="n">
-        <f aca="false">K89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">K89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="L183" s="49" t="n">
-        <f aca="false">L89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">L89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="M183" s="49" t="n">
-        <f aca="false">M89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">M89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="N183" s="49" t="n">
-        <f aca="false">N89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">N89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="O183" s="49" t="n">
-        <f aca="false">O89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">O89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="P183" s="49" t="n">
-        <f aca="false">P89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">P89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="Q183" s="49" t="n">
-        <f aca="false">Q89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">Q89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="R183" s="49" t="n">
-        <f aca="false">R89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">R89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="S183" s="49" t="n">
-        <f aca="false">S89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">S89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="T183" s="49" t="n">
-        <f aca="false">T89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">T89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="U183" s="49" t="n">
-        <f aca="false">U89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">U89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="V183" s="49" t="n">
-        <f aca="false">V89*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">V89*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="W183" s="49" t="n">
-        <f aca="false">W89*(założenia!$C$7-założenia!$C$19)</f>
-        <v>12162.6802307253</v>
+        <f aca="false">W89*założenia!$C$7</f>
+        <v>12218.1462087735</v>
       </c>
       <c r="X183" s="49" t="n">
-        <f aca="false">X89*(założenia!$C$7-założenia!$C$19)</f>
-        <v>12162.6802307253</v>
+        <f aca="false">X89*założenia!$C$7</f>
+        <v>12218.1462087735</v>
       </c>
       <c r="Y183" s="49" t="n">
-        <f aca="false">Y89*(założenia!$C$7-założenia!$C$19)</f>
-        <v>12162.6802307253</v>
+        <f aca="false">Y89*założenia!$C$7</f>
+        <v>12218.1462087735</v>
       </c>
       <c r="Z183" s="49" t="n">
-        <f aca="false">Z89*(założenia!$C$7-założenia!$C$19)</f>
-        <v>12162.6802307253</v>
+        <f aca="false">Z89*założenia!$C$7</f>
+        <v>12218.1462087735</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40249,99 +40264,99 @@
       </c>
       <c r="C184" s="49" t="n">
         <f aca="false">SUM(D184:Z184)</f>
-        <v>1684.87176700192</v>
+        <v>1692.55535800898</v>
       </c>
       <c r="D184" s="49" t="n">
-        <f aca="false">D90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">D90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="E184" s="49" t="n">
-        <f aca="false">E90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">E90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="F184" s="49" t="n">
-        <f aca="false">F90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">F90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="G184" s="49" t="n">
-        <f aca="false">G90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">G90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="H184" s="49" t="n">
-        <f aca="false">H90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">H90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="I184" s="49" t="n">
-        <f aca="false">I90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">I90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="J184" s="49" t="n">
-        <f aca="false">J90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">J90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="K184" s="49" t="n">
-        <f aca="false">K90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">K90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="L184" s="49" t="n">
-        <f aca="false">L90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">L90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="M184" s="49" t="n">
-        <f aca="false">M90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">M90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="N184" s="49" t="n">
-        <f aca="false">N90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">N90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="O184" s="49" t="n">
-        <f aca="false">O90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">O90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="P184" s="49" t="n">
-        <f aca="false">P90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">P90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="Q184" s="49" t="n">
-        <f aca="false">Q90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">Q90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="R184" s="49" t="n">
-        <f aca="false">R90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">R90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="S184" s="49" t="n">
-        <f aca="false">S90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">S90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="T184" s="49" t="n">
-        <f aca="false">T90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">T90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="U184" s="49" t="n">
-        <f aca="false">U90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">U90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="V184" s="49" t="n">
-        <f aca="false">V90*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">V90*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="W184" s="49" t="n">
-        <f aca="false">W90*(założenia!$C$7-założenia!$C$19)</f>
-        <v>421.217941750479</v>
+        <f aca="false">W90*założenia!$C$7</f>
+        <v>423.138839502245</v>
       </c>
       <c r="X184" s="49" t="n">
-        <f aca="false">X90*(założenia!$C$7-założenia!$C$19)</f>
-        <v>421.217941750479</v>
+        <f aca="false">X90*założenia!$C$7</f>
+        <v>423.138839502245</v>
       </c>
       <c r="Y184" s="49" t="n">
-        <f aca="false">Y90*(założenia!$C$7-założenia!$C$19)</f>
-        <v>421.217941750479</v>
+        <f aca="false">Y90*założenia!$C$7</f>
+        <v>423.138839502245</v>
       </c>
       <c r="Z184" s="49" t="n">
-        <f aca="false">Z90*(założenia!$C$7-założenia!$C$19)</f>
-        <v>421.217941750479</v>
+        <f aca="false">Z90*założenia!$C$7</f>
+        <v>423.138839502245</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40353,99 +40368,99 @@
       </c>
       <c r="C185" s="49" t="n">
         <f aca="false">SUM(D185:Z185)</f>
-        <v>46586.750944354</v>
+        <v>46799.2024481508</v>
       </c>
       <c r="D185" s="49" t="n">
-        <f aca="false">D91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">D91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="E185" s="49" t="n">
-        <f aca="false">E91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">E91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="F185" s="49" t="n">
-        <f aca="false">F91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">F91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="G185" s="49" t="n">
-        <f aca="false">G91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">G91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="H185" s="49" t="n">
-        <f aca="false">H91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">H91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="I185" s="49" t="n">
-        <f aca="false">I91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">I91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="J185" s="49" t="n">
-        <f aca="false">J91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">J91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="K185" s="49" t="n">
-        <f aca="false">K91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">K91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="L185" s="49" t="n">
-        <f aca="false">L91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">L91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="M185" s="49" t="n">
-        <f aca="false">M91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">M91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="N185" s="49" t="n">
-        <f aca="false">N91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">N91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="O185" s="49" t="n">
-        <f aca="false">O91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">O91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="P185" s="49" t="n">
-        <f aca="false">P91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">P91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="Q185" s="49" t="n">
-        <f aca="false">Q91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">Q91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="R185" s="49" t="n">
-        <f aca="false">R91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">R91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="S185" s="49" t="n">
-        <f aca="false">S91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">S91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="T185" s="49" t="n">
-        <f aca="false">T91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">T91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="U185" s="49" t="n">
-        <f aca="false">U91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">U91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="V185" s="49" t="n">
-        <f aca="false">V91*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">V91*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="W185" s="49" t="n">
-        <f aca="false">W91*(założenia!$C$7-założenia!$C$19)</f>
-        <v>11646.6877360885</v>
+        <f aca="false">W91*założenia!$C$7</f>
+        <v>11699.8006120377</v>
       </c>
       <c r="X185" s="49" t="n">
-        <f aca="false">X91*(założenia!$C$7-założenia!$C$19)</f>
-        <v>11646.6877360885</v>
+        <f aca="false">X91*założenia!$C$7</f>
+        <v>11699.8006120377</v>
       </c>
       <c r="Y185" s="49" t="n">
-        <f aca="false">Y91*(założenia!$C$7-założenia!$C$19)</f>
-        <v>11646.6877360885</v>
+        <f aca="false">Y91*założenia!$C$7</f>
+        <v>11699.8006120377</v>
       </c>
       <c r="Z185" s="49" t="n">
-        <f aca="false">Z91*(założenia!$C$7-założenia!$C$19)</f>
-        <v>11646.6877360885</v>
+        <f aca="false">Z91*założenia!$C$7</f>
+        <v>11699.8006120377</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40457,104 +40472,104 @@
       </c>
       <c r="C186" s="49" t="n">
         <f aca="false">SUM(D186:Z186)</f>
-        <v>11605.4083365175</v>
+        <v>11658.3329642988</v>
       </c>
       <c r="D186" s="49" t="n">
-        <f aca="false">D92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">D92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="E186" s="49" t="n">
-        <f aca="false">E92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">E92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="F186" s="49" t="n">
-        <f aca="false">F92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">F92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="G186" s="49" t="n">
-        <f aca="false">G92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">G92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="H186" s="49" t="n">
-        <f aca="false">H92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">H92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="I186" s="49" t="n">
-        <f aca="false">I92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">I92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="J186" s="49" t="n">
-        <f aca="false">J92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">J92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="K186" s="49" t="n">
-        <f aca="false">K92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">K92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="L186" s="49" t="n">
-        <f aca="false">L92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">L92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="M186" s="49" t="n">
-        <f aca="false">M92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">M92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="N186" s="49" t="n">
-        <f aca="false">N92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">N92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="O186" s="49" t="n">
-        <f aca="false">O92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">O92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="P186" s="49" t="n">
-        <f aca="false">P92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">P92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="Q186" s="49" t="n">
-        <f aca="false">Q92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">Q92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="R186" s="49" t="n">
-        <f aca="false">R92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">R92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="S186" s="49" t="n">
-        <f aca="false">S92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">S92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="T186" s="49" t="n">
-        <f aca="false">T92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">T92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="U186" s="49" t="n">
-        <f aca="false">U92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">U92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="V186" s="49" t="n">
-        <f aca="false">V92*(założenia!$C$7-założenia!$C$19)</f>
+        <f aca="false">V92*założenia!$C$7</f>
         <v>0</v>
       </c>
       <c r="W186" s="49" t="n">
-        <f aca="false">W92*(założenia!$C$7-założenia!$C$19)</f>
-        <v>2901.35208412939</v>
+        <f aca="false">W92*założenia!$C$7</f>
+        <v>2914.58324107471</v>
       </c>
       <c r="X186" s="49" t="n">
-        <f aca="false">X92*(założenia!$C$7-założenia!$C$19)</f>
-        <v>2901.35208412939</v>
+        <f aca="false">X92*założenia!$C$7</f>
+        <v>2914.58324107471</v>
       </c>
       <c r="Y186" s="49" t="n">
-        <f aca="false">Y92*(założenia!$C$7-założenia!$C$19)</f>
-        <v>2901.35208412939</v>
+        <f aca="false">Y92*założenia!$C$7</f>
+        <v>2914.58324107471</v>
       </c>
       <c r="Z186" s="49" t="n">
-        <f aca="false">Z92*(założenia!$C$7-założenia!$C$19)</f>
-        <v>2901.35208412939</v>
+        <f aca="false">Z92*założenia!$C$7</f>
+        <v>2914.58324107471</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="40" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B187" s="40" t="n">
         <v>1</v>
@@ -40658,14 +40673,14 @@
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="40" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B188" s="40" t="n">
         <v>2</v>
       </c>
       <c r="C188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,C$150:C$186)</f>
-        <v>810408.93</v>
+        <v>808623.11</v>
       </c>
       <c r="D188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,D$150:D$186)</f>
@@ -40709,7 +40724,7 @@
       </c>
       <c r="N188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,N$150:N$186)</f>
-        <v>136556.338333333</v>
+        <v>134770.518333333</v>
       </c>
       <c r="O188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,O$150:O$186)</f>
@@ -40762,7 +40777,7 @@
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="40" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B189" s="40" t="n">
         <v>3</v>
@@ -40866,14 +40881,14 @@
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="40" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B190" s="40" t="n">
         <v>4</v>
       </c>
       <c r="C190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,C$150:C$186)</f>
-        <v>391598.286</v>
+        <v>393384.108</v>
       </c>
       <c r="D190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,D$150:D$186)</f>
@@ -40953,19 +40968,19 @@
       </c>
       <c r="W190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,W$150:W$186)</f>
-        <v>97899.5715</v>
+        <v>98346.027</v>
       </c>
       <c r="X190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,X$150:X$186)</f>
-        <v>97899.5715</v>
+        <v>98346.027</v>
       </c>
       <c r="Y190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,Y$150:Y$186)</f>
-        <v>97899.5715</v>
+        <v>98346.027</v>
       </c>
       <c r="Z190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,Z$150:Z$186)</f>
-        <v>97899.5715</v>
+        <v>98346.027</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40975,7 +40990,7 @@
       <c r="B191" s="40"/>
       <c r="C191" s="63" t="n">
         <f aca="false">SUM(C187:C190)</f>
-        <v>2959946.54</v>
+        <v>2959946.542</v>
       </c>
       <c r="D191" s="63" t="n">
         <f aca="false">SUM(D187:D190)</f>
@@ -41019,7 +41034,7 @@
       </c>
       <c r="N191" s="63" t="n">
         <f aca="false">SUM(N187:N190)</f>
-        <v>136556.338333333</v>
+        <v>134770.518333333</v>
       </c>
       <c r="O191" s="63" t="n">
         <f aca="false">SUM(O187:O190)</f>
@@ -41055,322 +41070,322 @@
       </c>
       <c r="W191" s="63" t="n">
         <f aca="false">SUM(W187:W190)</f>
-        <v>97899.5715</v>
+        <v>98346.027</v>
       </c>
       <c r="X191" s="63" t="n">
         <f aca="false">SUM(X187:X190)</f>
-        <v>97899.5715</v>
+        <v>98346.027</v>
       </c>
       <c r="Y191" s="63" t="n">
         <f aca="false">SUM(Y187:Y190)</f>
-        <v>97899.5715</v>
+        <v>98346.027</v>
       </c>
       <c r="Z191" s="63" t="n">
         <f aca="false">SUM(Z187:Z190)</f>
-        <v>97899.5715</v>
+        <v>98346.027</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="40" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B192" s="40"/>
       <c r="C192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,C98*$C$191/$C$97)</f>
-        <v>739986.635</v>
+        <v>739986.6355</v>
       </c>
       <c r="D192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,D98*$C$191/$C$97)</f>
-        <v>31359.675174367</v>
+        <v>31446.1064211191</v>
       </c>
       <c r="E192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,E98*$C$191/$C$97)</f>
-        <v>31359.675174367</v>
+        <v>31446.1064211191</v>
       </c>
       <c r="F192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,F98*$C$191/$C$97)</f>
-        <v>31359.675174367</v>
+        <v>31446.1064211191</v>
       </c>
       <c r="G192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,G98*$C$191/$C$97)</f>
-        <v>30065.2453595076</v>
+        <v>30148.1089933264</v>
       </c>
       <c r="H192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,H98*$C$191/$C$97)</f>
-        <v>30065.2453595076</v>
+        <v>30148.1089933264</v>
       </c>
       <c r="I192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,I98*$C$191/$C$97)</f>
-        <v>32174.6608822624</v>
+        <v>32263.3383331102</v>
       </c>
       <c r="J192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,J98*$C$191/$C$97)</f>
-        <v>32174.6608822624</v>
+        <v>32263.3383331102</v>
       </c>
       <c r="K192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,K98*$C$191/$C$97)</f>
-        <v>32174.6608822624</v>
+        <v>32263.3383331102</v>
       </c>
       <c r="L192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,L98*$C$191/$C$97)</f>
-        <v>32174.6608822624</v>
+        <v>32263.3383331102</v>
       </c>
       <c r="M192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,M98*$C$191/$C$97)</f>
-        <v>32174.6608822624</v>
+        <v>32263.3383331102</v>
       </c>
       <c r="N192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,N98*$C$191/$C$97)</f>
-        <v>32601.0024921226</v>
+        <v>32263.3383331102</v>
       </c>
       <c r="O192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,O98*$C$191/$C$97)</f>
-        <v>32213.5523531286</v>
+        <v>32302.3369938084</v>
       </c>
       <c r="P192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,P98*$C$191/$C$97)</f>
-        <v>32213.5523531286</v>
+        <v>32302.3369938084</v>
       </c>
       <c r="Q192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,Q98*$C$191/$C$97)</f>
-        <v>33507.9823801984</v>
+        <v>33600.3346343962</v>
       </c>
       <c r="R192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,R98*$C$191/$C$97)</f>
-        <v>33507.9823801984</v>
+        <v>33600.3346343962</v>
       </c>
       <c r="S192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,S98*$C$191/$C$97)</f>
-        <v>33507.9823801984</v>
+        <v>33600.3346343962</v>
       </c>
       <c r="T192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,T98*$C$191/$C$97)</f>
-        <v>33507.9823801984</v>
+        <v>33600.3346343962</v>
       </c>
       <c r="U192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,U98*$C$191/$C$97)</f>
-        <v>33507.9823801984</v>
+        <v>33600.3346343962</v>
       </c>
       <c r="V192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,V98*$C$191/$C$97)</f>
-        <v>33507.9823801984</v>
+        <v>33600.3346343962</v>
       </c>
       <c r="W192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,W98*$C$191/$C$97)</f>
-        <v>31706.9532167505</v>
+        <v>31391.3466143337</v>
       </c>
       <c r="X192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,X98*$C$191/$C$97)</f>
-        <v>31706.9532167505</v>
+        <v>31391.3466143337</v>
       </c>
       <c r="Y192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,Y98*$C$191/$C$97)</f>
-        <v>31706.9532167505</v>
+        <v>31391.3466143337</v>
       </c>
       <c r="Z192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,Z98*$C$191/$C$97)</f>
-        <v>31706.9532167505</v>
+        <v>31391.3466143337</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="40" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B193" s="40"/>
       <c r="C193" s="63" t="n">
         <f aca="false">C191+C192</f>
-        <v>3699933.175</v>
+        <v>3699933.1775</v>
       </c>
       <c r="D193" s="63" t="n">
         <f aca="false">D191+D192</f>
-        <v>162716.454729923</v>
+        <v>162802.885976675</v>
       </c>
       <c r="E193" s="63" t="n">
         <f aca="false">E191+E192</f>
-        <v>162716.454729923</v>
+        <v>162802.885976675</v>
       </c>
       <c r="F193" s="63" t="n">
         <f aca="false">F191+F192</f>
-        <v>162716.454729923</v>
+        <v>162802.885976675</v>
       </c>
       <c r="G193" s="63" t="n">
         <f aca="false">G191+G192</f>
-        <v>156000.026026174</v>
+        <v>156082.889659993</v>
       </c>
       <c r="H193" s="63" t="n">
         <f aca="false">H191+H192</f>
-        <v>156000.026026174</v>
+        <v>156082.889659993</v>
       </c>
       <c r="I193" s="63" t="n">
         <f aca="false">I191+I192</f>
-        <v>166945.179215596</v>
+        <v>167033.856666444</v>
       </c>
       <c r="J193" s="63" t="n">
         <f aca="false">J191+J192</f>
-        <v>166945.179215596</v>
+        <v>167033.856666444</v>
       </c>
       <c r="K193" s="63" t="n">
         <f aca="false">K191+K192</f>
-        <v>166945.179215596</v>
+        <v>167033.856666444</v>
       </c>
       <c r="L193" s="63" t="n">
         <f aca="false">L191+L192</f>
-        <v>166945.179215596</v>
+        <v>167033.856666444</v>
       </c>
       <c r="M193" s="63" t="n">
         <f aca="false">M191+M192</f>
-        <v>166945.179215596</v>
+        <v>167033.856666444</v>
       </c>
       <c r="N193" s="63" t="n">
         <f aca="false">N191+N192</f>
-        <v>169157.340825456</v>
+        <v>167033.856666444</v>
       </c>
       <c r="O193" s="63" t="n">
         <f aca="false">O191+O192</f>
-        <v>167146.980353129</v>
+        <v>167235.764993808</v>
       </c>
       <c r="P193" s="63" t="n">
         <f aca="false">P191+P192</f>
-        <v>167146.980353129</v>
+        <v>167235.764993808</v>
       </c>
       <c r="Q193" s="63" t="n">
         <f aca="false">Q191+Q192</f>
-        <v>173863.410380198</v>
+        <v>173955.762634396</v>
       </c>
       <c r="R193" s="63" t="n">
         <f aca="false">R191+R192</f>
-        <v>173863.410380198</v>
+        <v>173955.762634396</v>
       </c>
       <c r="S193" s="63" t="n">
         <f aca="false">S191+S192</f>
-        <v>173863.410380198</v>
+        <v>173955.762634396</v>
       </c>
       <c r="T193" s="63" t="n">
         <f aca="false">T191+T192</f>
-        <v>173863.410380198</v>
+        <v>173955.762634396</v>
       </c>
       <c r="U193" s="63" t="n">
         <f aca="false">U191+U192</f>
-        <v>173863.410380198</v>
+        <v>173955.762634396</v>
       </c>
       <c r="V193" s="63" t="n">
         <f aca="false">V191+V192</f>
-        <v>173863.410380198</v>
+        <v>173955.762634396</v>
       </c>
       <c r="W193" s="63" t="n">
         <f aca="false">W191+W192</f>
-        <v>129606.52471675</v>
+        <v>129737.373614334</v>
       </c>
       <c r="X193" s="63" t="n">
         <f aca="false">X191+X192</f>
-        <v>129606.52471675</v>
+        <v>129737.373614334</v>
       </c>
       <c r="Y193" s="63" t="n">
         <f aca="false">Y191+Y192</f>
-        <v>129606.52471675</v>
+        <v>129737.373614334</v>
       </c>
       <c r="Z193" s="63" t="n">
         <f aca="false">Z191+Z192</f>
-        <v>129606.52471675</v>
+        <v>129737.373614334</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="40" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B194" s="40"/>
       <c r="C194" s="63"/>
       <c r="D194" s="63" t="n">
         <f aca="false">D193</f>
-        <v>162716.454729923</v>
+        <v>162802.885976675</v>
       </c>
       <c r="E194" s="63" t="n">
         <f aca="false">D194+E193</f>
-        <v>325432.909459845</v>
+        <v>325605.771953349</v>
       </c>
       <c r="F194" s="63" t="n">
         <f aca="false">E194+F193</f>
-        <v>488149.364189768</v>
+        <v>488408.657930024</v>
       </c>
       <c r="G194" s="63" t="n">
         <f aca="false">F194+G193</f>
-        <v>644149.390215942</v>
+        <v>644491.547590017</v>
       </c>
       <c r="H194" s="63" t="n">
         <f aca="false">G194+H193</f>
-        <v>800149.416242116</v>
+        <v>800574.43725001</v>
       </c>
       <c r="I194" s="63" t="n">
         <f aca="false">H194+I193</f>
-        <v>967094.595457712</v>
+        <v>967608.293916454</v>
       </c>
       <c r="J194" s="63" t="n">
         <f aca="false">I194+J193</f>
-        <v>1134039.77467331</v>
+        <v>1134642.1505829</v>
       </c>
       <c r="K194" s="63" t="n">
         <f aca="false">J194+K193</f>
-        <v>1300984.9538889</v>
+        <v>1301676.00724934</v>
       </c>
       <c r="L194" s="63" t="n">
         <f aca="false">K194+L193</f>
-        <v>1467930.1331045</v>
+        <v>1468709.86391578</v>
       </c>
       <c r="M194" s="63" t="n">
         <f aca="false">L194+M193</f>
-        <v>1634875.31232009</v>
+        <v>1635743.72058223</v>
       </c>
       <c r="N194" s="63" t="n">
         <f aca="false">M194+N193</f>
-        <v>1804032.65314555</v>
+        <v>1802777.57724867</v>
       </c>
       <c r="O194" s="63" t="n">
         <f aca="false">N194+O193</f>
-        <v>1971179.63349868</v>
+        <v>1970013.34224248</v>
       </c>
       <c r="P194" s="63" t="n">
         <f aca="false">O194+P193</f>
-        <v>2138326.61385181</v>
+        <v>2137249.10723629</v>
       </c>
       <c r="Q194" s="63" t="n">
         <f aca="false">P194+Q193</f>
-        <v>2312190.02423201</v>
+        <v>2311204.86987068</v>
       </c>
       <c r="R194" s="63" t="n">
         <f aca="false">Q194+R193</f>
-        <v>2486053.4346122</v>
+        <v>2485160.63250508</v>
       </c>
       <c r="S194" s="63" t="n">
         <f aca="false">R194+S193</f>
-        <v>2659916.8449924</v>
+        <v>2659116.39513948</v>
       </c>
       <c r="T194" s="63" t="n">
         <f aca="false">S194+T193</f>
-        <v>2833780.2553726</v>
+        <v>2833072.15777387</v>
       </c>
       <c r="U194" s="63" t="n">
         <f aca="false">T194+U193</f>
-        <v>3007643.6657528</v>
+        <v>3007027.92040827</v>
       </c>
       <c r="V194" s="63" t="n">
         <f aca="false">U194+V193</f>
-        <v>3181507.076133</v>
+        <v>3180983.68304266</v>
       </c>
       <c r="W194" s="63" t="n">
         <f aca="false">V194+W193</f>
-        <v>3311113.60084975</v>
+        <v>3310721.056657</v>
       </c>
       <c r="X194" s="63" t="n">
         <f aca="false">W194+X193</f>
-        <v>3440720.1255665</v>
+        <v>3440458.43027133</v>
       </c>
       <c r="Y194" s="63" t="n">
         <f aca="false">X194+Y193</f>
-        <v>3570326.65028325</v>
+        <v>3570195.80388567</v>
       </c>
       <c r="Z194" s="63" t="n">
         <f aca="false">Y194+Z193</f>
-        <v>3699933.175</v>
+        <v>3699933.1775</v>
       </c>
     </row>
   </sheetData>
@@ -41403,23 +41418,23 @@
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="67"/>
       <c r="B1" s="68" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C1" s="68"/>
       <c r="D1" s="68"/>
       <c r="E1" s="68" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F1" s="68"/>
       <c r="G1" s="68"/>
       <c r="H1" s="69"/>
       <c r="I1" s="68" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="J1" s="68"/>
       <c r="K1" s="68"/>
       <c r="L1" s="68" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="M1" s="68"/>
       <c r="N1" s="68"/>
@@ -41459,17 +41474,17 @@
         <v>117</v>
       </c>
       <c r="L2" s="67" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="M2" s="67" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="N2" s="67" t="s">
         <v>117</v>
       </c>
       <c r="O2" s="69"/>
       <c r="P2" s="67" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -42080,15 +42095,15 @@
       </c>
       <c r="E13" s="71" t="n">
         <f aca="false">SUM(E14:E23)</f>
-        <v>1013524.62</v>
+        <v>1010778.92</v>
       </c>
       <c r="F13" s="71" t="n">
         <f aca="false">SUM(F14:F23)</f>
-        <v>1013011.2</v>
+        <v>1010778.92</v>
       </c>
       <c r="G13" s="71" t="n">
         <f aca="false">SUM(G14:G23)</f>
-        <v>810408.93</v>
+        <v>808623.11</v>
       </c>
       <c r="H13" s="63"/>
       <c r="I13" s="71" t="n">
@@ -42105,15 +42120,15 @@
       </c>
       <c r="L13" s="71" t="n">
         <f aca="false">E13-I13</f>
-        <v>-213411.09</v>
+        <v>-216156.79</v>
       </c>
       <c r="M13" s="71" t="n">
         <f aca="false">F13-J13</f>
-        <v>-190924.51</v>
+        <v>-193156.79</v>
       </c>
       <c r="N13" s="71" t="n">
         <f aca="false">G13-K13</f>
-        <v>-152739.63</v>
+        <v>-154525.45</v>
       </c>
       <c r="O13" s="40"/>
       <c r="P13" s="70" t="str">
@@ -42552,15 +42567,15 @@
       </c>
       <c r="E21" s="74" t="n">
         <f aca="false">ROUND(F21*założenia!$C$8,2)</f>
-        <v>2745.7</v>
+        <v>0</v>
       </c>
       <c r="F21" s="74" t="n">
         <f aca="false">założenia!$C$14</f>
-        <v>2232.28</v>
+        <v>0</v>
       </c>
       <c r="G21" s="74" t="n">
         <f aca="false">założenia!$C$9</f>
-        <v>1785.82</v>
+        <v>0</v>
       </c>
       <c r="H21" s="49"/>
       <c r="I21" s="73" t="n">
@@ -42577,15 +42592,15 @@
       </c>
       <c r="L21" s="73" t="n">
         <f aca="false">E21-I21</f>
-        <v>-120254.3</v>
+        <v>-123000</v>
       </c>
       <c r="M21" s="73" t="n">
         <f aca="false">F21-J21</f>
-        <v>-97767.72</v>
+        <v>-100000</v>
       </c>
       <c r="N21" s="73" t="n">
         <f aca="false">G21-K21</f>
-        <v>-78214.18</v>
+        <v>-80000</v>
       </c>
       <c r="O21" s="41"/>
       <c r="P21" s="72" t="str">
@@ -43319,15 +43334,15 @@
       </c>
       <c r="E34" s="71" t="n">
         <f aca="false">SUM(E35:E43)</f>
-        <v>664057.14</v>
+        <v>655640.19</v>
       </c>
       <c r="F34" s="71" t="n">
         <f aca="false">SUM(F35:F43)</f>
-        <v>664057.14</v>
+        <v>655640.19</v>
       </c>
       <c r="G34" s="71" t="n">
         <f aca="false">SUM(G35:G43)</f>
-        <v>391598.29</v>
+        <v>393384.11</v>
       </c>
       <c r="H34" s="63"/>
       <c r="I34" s="71" t="n">
@@ -43344,15 +43359,15 @@
       </c>
       <c r="L34" s="71" t="n">
         <f aca="false">E34-I34</f>
-        <v>-34180</v>
+        <v>-42596.95</v>
       </c>
       <c r="M34" s="71" t="n">
         <f aca="false">F34-J34</f>
-        <v>-34180</v>
+        <v>-42596.95</v>
       </c>
       <c r="N34" s="71" t="n">
         <f aca="false">G34-K34</f>
-        <v>-27343.9900000001</v>
+        <v>-25558.17</v>
       </c>
       <c r="O34" s="40"/>
       <c r="P34" s="70" t="str">
@@ -43378,15 +43393,15 @@
       </c>
       <c r="E35" s="74" t="n">
         <f aca="false">F35</f>
-        <v>221600</v>
+        <v>218791.21</v>
       </c>
       <c r="F35" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$84,2)</f>
-        <v>221600</v>
+        <v>218791.21</v>
       </c>
       <c r="G35" s="74" t="n">
         <f aca="false">ROUND(założenia!$C$13-(G4+G5+G6+G7+G8+G9+G10+G11+G12+G14+G15+G16+G17+G18+G19+G20+G21+G22+G23+G25+G26+G27+G28+G29+G30+G31+G32+G33+G36+G37+G38+G39+G40+G41+G42+G43),2)</f>
-        <v>130678.79</v>
+        <v>131274.74</v>
       </c>
       <c r="H35" s="49"/>
       <c r="I35" s="73" t="n">
@@ -43403,15 +43418,15 @@
       </c>
       <c r="L35" s="73" t="n">
         <f aca="false">E35-I35</f>
-        <v>0</v>
+        <v>-2808.79000000001</v>
       </c>
       <c r="M35" s="73" t="n">
         <f aca="false">F35-J35</f>
-        <v>0</v>
+        <v>-2808.79000000001</v>
       </c>
       <c r="N35" s="73" t="n">
         <f aca="false">G35-K35</f>
-        <v>-2281.21000000001</v>
+        <v>-1685.26000000001</v>
       </c>
       <c r="O35" s="41"/>
       <c r="P35" s="72" t="str">
@@ -43419,7 +43434,7 @@
         <v>OK</v>
       </c>
       <c r="Q35" s="55" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43440,15 +43455,15 @@
       </c>
       <c r="E36" s="74" t="n">
         <f aca="false">F36</f>
-        <v>37720</v>
+        <v>37241.9</v>
       </c>
       <c r="F36" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$85,2)</f>
-        <v>37720</v>
+        <v>37241.9</v>
       </c>
       <c r="G36" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$179,2)</f>
-        <v>22243.7</v>
+        <v>22345.14</v>
       </c>
       <c r="H36" s="49"/>
       <c r="I36" s="73" t="n">
@@ -43465,15 +43480,15 @@
       </c>
       <c r="L36" s="73" t="n">
         <f aca="false">E36-I36</f>
-        <v>0</v>
+        <v>-478.099999999999</v>
       </c>
       <c r="M36" s="73" t="n">
         <f aca="false">F36-J36</f>
-        <v>0</v>
+        <v>-478.099999999999</v>
       </c>
       <c r="N36" s="73" t="n">
         <f aca="false">G36-K36</f>
-        <v>-388.299999999999</v>
+        <v>-286.860000000001</v>
       </c>
       <c r="O36" s="41"/>
       <c r="P36" s="72" t="str">
@@ -43499,15 +43514,15 @@
       </c>
       <c r="E37" s="74" t="n">
         <f aca="false">F37</f>
-        <v>108440</v>
+        <v>107065.52</v>
       </c>
       <c r="F37" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$86,2)</f>
-        <v>108440</v>
+        <v>107065.52</v>
       </c>
       <c r="G37" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$180,2)</f>
-        <v>63947.69</v>
+        <v>64239.31</v>
       </c>
       <c r="H37" s="49"/>
       <c r="I37" s="73" t="n">
@@ -43524,15 +43539,15 @@
       </c>
       <c r="L37" s="73" t="n">
         <f aca="false">E37-I37</f>
-        <v>0</v>
+        <v>-1374.48</v>
       </c>
       <c r="M37" s="73" t="n">
         <f aca="false">F37-J37</f>
-        <v>0</v>
+        <v>-1374.48</v>
       </c>
       <c r="N37" s="73" t="n">
         <f aca="false">G37-K37</f>
-        <v>-1116.31</v>
+        <v>-824.690000000002</v>
       </c>
       <c r="O37" s="41"/>
       <c r="P37" s="72" t="str">
@@ -43558,15 +43573,15 @@
       </c>
       <c r="E38" s="74" t="n">
         <f aca="false">F38</f>
-        <v>82500</v>
+        <v>81454.31</v>
       </c>
       <c r="F38" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$87,2)</f>
-        <v>82500</v>
+        <v>81454.31</v>
       </c>
       <c r="G38" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$181,2)</f>
-        <v>48650.72</v>
+        <v>48872.58</v>
       </c>
       <c r="H38" s="49"/>
       <c r="I38" s="73" t="n">
@@ -43583,15 +43598,15 @@
       </c>
       <c r="L38" s="73" t="n">
         <f aca="false">E38-I38</f>
-        <v>0</v>
+        <v>-1045.69</v>
       </c>
       <c r="M38" s="73" t="n">
         <f aca="false">F38-J38</f>
-        <v>0</v>
+        <v>-1045.69</v>
       </c>
       <c r="N38" s="73" t="n">
         <f aca="false">G38-K38</f>
-        <v>-849.279999999999</v>
+        <v>-627.419999999998</v>
       </c>
       <c r="O38" s="41"/>
       <c r="P38" s="72" t="str">
@@ -43617,15 +43632,15 @@
       </c>
       <c r="E39" s="74" t="n">
         <f aca="false">F39</f>
-        <v>29760</v>
+        <v>29382.79</v>
       </c>
       <c r="F39" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$88,2)</f>
-        <v>29760</v>
+        <v>29382.79</v>
       </c>
       <c r="G39" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$182,2)</f>
-        <v>17549.64</v>
+        <v>17629.67</v>
       </c>
       <c r="H39" s="49"/>
       <c r="I39" s="73" t="n">
@@ -43642,15 +43657,15 @@
       </c>
       <c r="L39" s="73" t="n">
         <f aca="false">E39-I39</f>
-        <v>0</v>
+        <v>-377.209999999999</v>
       </c>
       <c r="M39" s="73" t="n">
         <f aca="false">F39-J39</f>
-        <v>0</v>
+        <v>-377.209999999999</v>
       </c>
       <c r="N39" s="73" t="n">
         <f aca="false">G39-K39</f>
-        <v>-306.360000000001</v>
+        <v>-226.330000000002</v>
       </c>
       <c r="O39" s="41"/>
       <c r="P39" s="72" t="str">
@@ -43676,15 +43691,15 @@
       </c>
       <c r="E40" s="74" t="n">
         <f aca="false">F40</f>
-        <v>82500</v>
+        <v>81454.31</v>
       </c>
       <c r="F40" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$89,2)</f>
-        <v>82500</v>
+        <v>81454.31</v>
       </c>
       <c r="G40" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$183,2)</f>
-        <v>48650.72</v>
+        <v>48872.58</v>
       </c>
       <c r="H40" s="49"/>
       <c r="I40" s="73" t="n">
@@ -43701,15 +43716,15 @@
       </c>
       <c r="L40" s="73" t="n">
         <f aca="false">E40-I40</f>
-        <v>0</v>
+        <v>-1045.69</v>
       </c>
       <c r="M40" s="73" t="n">
         <f aca="false">F40-J40</f>
-        <v>0</v>
+        <v>-1045.69</v>
       </c>
       <c r="N40" s="73" t="n">
         <f aca="false">G40-K40</f>
-        <v>-849.279999999999</v>
+        <v>-627.419999999998</v>
       </c>
       <c r="O40" s="41"/>
       <c r="P40" s="72" t="str">
@@ -43735,15 +43750,15 @@
       </c>
       <c r="E41" s="74" t="n">
         <f aca="false">F41</f>
-        <v>2857.14</v>
+        <v>2820.93</v>
       </c>
       <c r="F41" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$90,2)</f>
-        <v>2857.14</v>
+        <v>2820.93</v>
       </c>
       <c r="G41" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$184,2)</f>
-        <v>1684.87</v>
+        <v>1692.56</v>
       </c>
       <c r="H41" s="49"/>
       <c r="I41" s="73" t="n">
@@ -43760,15 +43775,15 @@
       </c>
       <c r="L41" s="73" t="n">
         <f aca="false">E41-I41</f>
-        <v>0</v>
+        <v>-36.21</v>
       </c>
       <c r="M41" s="73" t="n">
         <f aca="false">F41-J41</f>
-        <v>0</v>
+        <v>-36.21</v>
       </c>
       <c r="N41" s="73" t="n">
         <f aca="false">G41-K41</f>
-        <v>-29.4100000000001</v>
+        <v>-21.72</v>
       </c>
       <c r="O41" s="41"/>
       <c r="P41" s="72" t="str">
@@ -43794,15 +43809,15 @@
       </c>
       <c r="E42" s="74" t="n">
         <f aca="false">F42</f>
-        <v>79000</v>
+        <v>77998.67</v>
       </c>
       <c r="F42" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$91,2)</f>
-        <v>79000</v>
+        <v>77998.67</v>
       </c>
       <c r="G42" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$185,2)</f>
-        <v>46586.75</v>
+        <v>46799.2</v>
       </c>
       <c r="H42" s="49"/>
       <c r="I42" s="73" t="n">
@@ -43819,15 +43834,15 @@
       </c>
       <c r="L42" s="73" t="n">
         <f aca="false">E42-I42</f>
-        <v>0</v>
+        <v>-1001.33</v>
       </c>
       <c r="M42" s="73" t="n">
         <f aca="false">F42-J42</f>
-        <v>0</v>
+        <v>-1001.33</v>
       </c>
       <c r="N42" s="73" t="n">
         <f aca="false">G42-K42</f>
-        <v>-813.25</v>
+        <v>-600.800000000003</v>
       </c>
       <c r="O42" s="41"/>
       <c r="P42" s="72" t="str">
@@ -43853,15 +43868,15 @@
       </c>
       <c r="E43" s="74" t="n">
         <f aca="false">F43</f>
-        <v>19680</v>
+        <v>19430.55</v>
       </c>
       <c r="F43" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$92,2)</f>
-        <v>19680</v>
+        <v>19430.55</v>
       </c>
       <c r="G43" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$186,2)</f>
-        <v>11605.41</v>
+        <v>11658.33</v>
       </c>
       <c r="H43" s="49"/>
       <c r="I43" s="73" t="n">
@@ -43878,15 +43893,15 @@
       </c>
       <c r="L43" s="73" t="n">
         <f aca="false">E43-I43</f>
-        <v>-34180</v>
+        <v>-34429.45</v>
       </c>
       <c r="M43" s="73" t="n">
         <f aca="false">F43-J43</f>
-        <v>-34180</v>
+        <v>-34429.45</v>
       </c>
       <c r="N43" s="73" t="n">
         <f aca="false">G43-K43</f>
-        <v>-20710.59</v>
+        <v>-20657.67</v>
       </c>
       <c r="O43" s="41"/>
       <c r="P43" s="72" t="str">
@@ -43896,54 +43911,54 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="75" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="53" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B47" s="53" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C47" s="53" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D47" s="53" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E47" s="53" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F47" s="53" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G47" s="53" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H47" s="76"/>
       <c r="I47" s="53" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="J47" s="53" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K47" s="53" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="L47" s="53" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="M47" s="53" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="N47" s="53" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B48" s="73" t="n">
         <f aca="false">B3+B13+B24+B34</f>
@@ -43959,11 +43974,11 @@
       </c>
       <c r="E48" s="73" t="n">
         <f aca="false">E3+E13+E24+E34</f>
-        <v>3875005.91</v>
+        <v>3863843.26</v>
       </c>
       <c r="F48" s="73" t="n">
         <f aca="false">F3+F13+F24+F34</f>
-        <v>3874492.49</v>
+        <v>3863843.26</v>
       </c>
       <c r="G48" s="73" t="n">
         <f aca="false">G3+G13+G24+G34</f>
@@ -43984,11 +43999,11 @@
       </c>
       <c r="L48" s="73" t="n">
         <f aca="false">E48-I48</f>
-        <v>-22486.5800000001</v>
+        <v>-33649.23</v>
       </c>
       <c r="M48" s="73" t="n">
         <f aca="false">F48-J48</f>
-        <v>0</v>
+        <v>-10649.23</v>
       </c>
       <c r="N48" s="73" t="n">
         <f aca="false">G48-K48</f>
@@ -43997,7 +44012,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="41" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B49" s="73" t="n">
         <f aca="false">Podsumowanie!D130</f>
@@ -44013,14 +44028,14 @@
       </c>
       <c r="E49" s="73" t="n">
         <f aca="false">F49</f>
-        <v>968623.12</v>
+        <v>965960.82</v>
       </c>
       <c r="F49" s="73" t="n">
         <f aca="false">ROUND(0.25*F48,2)</f>
-        <v>968623.12</v>
+        <v>965960.82</v>
       </c>
       <c r="G49" s="73" t="n">
-        <f aca="false">ROUND(F49*G48/F48,2)</f>
+        <f aca="false">ROUNDDOWN(F49*G48/F48,2)</f>
         <v>739986.63</v>
       </c>
       <c r="H49" s="41"/>
@@ -44038,11 +44053,11 @@
       </c>
       <c r="L49" s="73" t="n">
         <f aca="false">E49-I49</f>
-        <v>0</v>
+        <v>-2662.30000000005</v>
       </c>
       <c r="M49" s="73" t="n">
         <f aca="false">F49-J49</f>
-        <v>0</v>
+        <v>-2662.30000000005</v>
       </c>
       <c r="N49" s="73" t="n">
         <f aca="false">G49-K49</f>
@@ -44051,61 +44066,61 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="40" t="s">
-        <v>235</v>
-      </c>
-      <c r="B50" s="46" t="n">
+        <v>236</v>
+      </c>
+      <c r="B50" s="77" t="n">
         <f aca="false">B48+B49</f>
         <v>2186266.46</v>
       </c>
-      <c r="C50" s="46" t="n">
+      <c r="C50" s="77" t="n">
         <f aca="false">C48+C49</f>
         <v>2144716.46</v>
       </c>
-      <c r="D50" s="46" t="n">
+      <c r="D50" s="77" t="n">
         <f aca="false">D48+D49</f>
         <v>1715773.16</v>
       </c>
-      <c r="E50" s="46" t="n">
+      <c r="E50" s="77" t="n">
         <f aca="false">E48+E49</f>
-        <v>4843629.03</v>
-      </c>
-      <c r="F50" s="46" t="n">
+        <v>4829804.08</v>
+      </c>
+      <c r="F50" s="77" t="n">
         <f aca="false">F48+F49</f>
-        <v>4843115.61</v>
-      </c>
-      <c r="G50" s="46" t="n">
+        <v>4829804.08</v>
+      </c>
+      <c r="G50" s="77" t="n">
         <f aca="false">G48+G49</f>
         <v>3699933.17</v>
       </c>
       <c r="H50" s="40"/>
-      <c r="I50" s="46" t="n">
+      <c r="I50" s="77" t="n">
         <f aca="false">I48+I49</f>
         <v>4866115.61</v>
       </c>
-      <c r="J50" s="46" t="n">
+      <c r="J50" s="77" t="n">
         <f aca="false">J48+J49</f>
         <v>4843115.61</v>
       </c>
-      <c r="K50" s="46" t="n">
+      <c r="K50" s="77" t="n">
         <f aca="false">K48+K49</f>
         <v>3699933.17</v>
       </c>
-      <c r="L50" s="46" t="n">
+      <c r="L50" s="77" t="n">
         <f aca="false">E50-I50</f>
-        <v>-22486.5800000001</v>
-      </c>
-      <c r="M50" s="46" t="n">
+        <v>-36311.5300000003</v>
+      </c>
+      <c r="M50" s="77" t="n">
         <f aca="false">F50-J50</f>
-        <v>0</v>
-      </c>
-      <c r="N50" s="46" t="n">
+        <v>-13311.5300000003</v>
+      </c>
+      <c r="N50" s="77" t="n">
         <f aca="false">G50-K50</f>
         <v>0</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="41" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B51" s="73"/>
       <c r="C51" s="73"/>
@@ -44129,7 +44144,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="41" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B52" s="73"/>
       <c r="C52" s="73"/>
@@ -44137,7 +44152,7 @@
       <c r="E52" s="73"/>
       <c r="F52" s="73" t="n">
         <f aca="false">ROUND(F50-F51,2)</f>
-        <v>0</v>
+        <v>-13311.53</v>
       </c>
       <c r="G52" s="73" t="n">
         <f aca="false">ROUND(G50-G51,2)</f>
@@ -44153,27 +44168,27 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="40" t="s">
-        <v>266</v>
-      </c>
-      <c r="B53" s="46"/>
-      <c r="C53" s="46"/>
-      <c r="D53" s="46"/>
-      <c r="E53" s="46"/>
-      <c r="F53" s="46" t="str">
-        <f aca="false">IF(ABS(F52)&lt;=0.05,"OK","BŁĄD")</f>
+        <v>267</v>
+      </c>
+      <c r="B53" s="77"/>
+      <c r="C53" s="77"/>
+      <c r="D53" s="77"/>
+      <c r="E53" s="77"/>
+      <c r="F53" s="77" t="str">
+        <f aca="false">IF(F52&lt;=0.005,"OK","BŁĄD")</f>
         <v>OK</v>
       </c>
-      <c r="G53" s="46" t="str">
-        <f aca="false">IF(ABS(G52)&lt;=0.05,"OK","BŁĄD")</f>
+      <c r="G53" s="77" t="str">
+        <f aca="false">IF(G52&lt;=0.005,"OK","BŁĄD")</f>
         <v>OK</v>
       </c>
       <c r="H53" s="40"/>
-      <c r="I53" s="46"/>
-      <c r="J53" s="46"/>
-      <c r="K53" s="46"/>
-      <c r="L53" s="46"/>
-      <c r="M53" s="46"/>
-      <c r="N53" s="46"/>
+      <c r="I53" s="77"/>
+      <c r="J53" s="77"/>
+      <c r="K53" s="77"/>
+      <c r="L53" s="77"/>
+      <c r="M53" s="77"/>
+      <c r="N53" s="77"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Amortization 569.02/month; freed difference goes to Z4, not licences
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3QuwGR9tgiXrdWSSrWcuu
</commit_message>
<xml_diff>
--- a/Wniosek_o_platnosc_str26-34.xlsx
+++ b/Wniosek_o_platnosc_str26-34.xlsx
@@ -507,19 +507,19 @@
     <t xml:space="preserve">Licencje – kwalifikowalne po zmianie (przyjęto 0: dofinansowanie nie może wzrosnąć)</t>
   </si>
   <si>
-    <t xml:space="preserve">Z4 – kwalifikowalne planowane (stawka × etat), przed obniżeniem</t>
+    <t xml:space="preserve">Z4 – kwalifikowalne osobowe (stawka × etat, bez amortyzacji), przed obniżeniem</t>
   </si>
   <si>
     <t xml:space="preserve">Z3 – dofinansowanie (80% kosztów kwalifikowalnych)</t>
   </si>
   <si>
-    <t xml:space="preserve">Dofinansowanie Z1+Z2 (wykonanie, poz. 2.9 wg planu, licencje) + Z3</t>
+    <t xml:space="preserve">Dofinansowanie Z1+Z2 (wykonanie, poz. 2.9 wg stawki, licencje) + Z3</t>
   </si>
   <si>
-    <t xml:space="preserve">Dofinansowanie dostępne dla Z4 = cel D bezpośrednie − C17</t>
+    <t xml:space="preserve">Dofinansowanie dostępne dla osobowych Z4 = cel D bezpośrednie − C17 − dofinansowanie amortyzacji Z4</t>
   </si>
   <si>
-    <t xml:space="preserve">Współczynnik obniżenia kosztów kwalifikowalnych Z4 (Z4 = C15 × C19, tak by D = 60% mieściło się w C18)</t>
+    <t xml:space="preserve">Współczynnik obniżenia osobowych kosztów kwalifikowalnych Z4 (= C15 × C19, tak by D = 60% mieściło się w C18; amortyzacja bez obniżenia)</t>
   </si>
   <si>
     <t xml:space="preserve">TEST: koszt wakatu grafika w Z4 (stawka × miesiące Z4), gdyby został</t>
@@ -531,7 +531,7 @@
     <t xml:space="preserve">TEST: wniosek</t>
   </si>
   <si>
-    <t xml:space="preserve">Z4 – kwalifikowalne po obniżeniu</t>
+    <t xml:space="preserve">Z4 – kwalifikowalne osobowe po obniżeniu</t>
   </si>
   <si>
     <t xml:space="preserve">KONTROLE</t>
@@ -579,7 +579,7 @@
     <t xml:space="preserve">2. Cel: dofinansowanie razem (3 699 933,17 zł) nie może wzrosnąć; wydatki kwalifikowalne razem (4 843 115,61 zł) mogą się zmniejszyć, ale nie wzrosnąć. Stałe zasady: intensywność Z1–Z3 = 80%, Z4 = 60%, koszty pośrednie = 25% kwalifikowalnych oraz 25% dofinansowania kosztów bezpośrednich (pochodne – nie są sterowane ręcznie).</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Z1 i Z2 w nowym budżecie = wydatki narastająco (ogółem, kwalifikowalne, dofinansowanie) per pozycja, z wyjątkiem poz. 2.9 (amortyzacja laptopów w Z2) – bez zmian wg planu: 4 285,71 zł. Poz. 2.1 (Ekspert AI, Z2): przyjęto 332 400 zł kwalifikowalnych / 265 920 zł dofinansowania (PARP wstrzymał wypłatę, budżet nie jest tracony).</t>
+    <t xml:space="preserve">3. Z1 i Z2 w nowym budżecie = wydatki narastająco (ogółem, kwalifikowalne, dofinansowanie) per pozycja, z wyjątkiem poz. 2.9 (amortyzacja laptopów w Z2) – liczona wg stawki 569,02 zł/mies. × 6 m-cy. Poz. 2.1 (Ekspert AI, Z2): przyjęto 332 400 zł kwalifikowalnych / 265 920 zł dofinansowania (PARP wstrzymał wypłatę, budżet nie jest tracony).</t>
   </si>
   <si>
     <t xml:space="preserve">4. Licencje (Z2): wykonanie 0, więc całość uwalnia środki. Po zmianie 0 zł (C14) – przy stałych intensywnościach budżet nie mieści ani reszty na licencjach, ani wakatu grafika w Z4.</t>
@@ -600,7 +600,7 @@
     <t xml:space="preserve">9. Grafik-Ilustrator: wakat (8 545 zł/mies.) wyzerowany w całym projekcie, w tym w Z4; zostaje Suska (4 920 zł/mies.). Test w C20:C22 pokazuje, że wakat w Z4 nie mieści się w limicie dofinansowania.</t>
   </si>
   <si>
-    <t xml:space="preserve">10. Amortyzacja laptopów: 714,29 zł/mies.; wydłużenie Z3 do 8 m-cy zwiększa amortyzację Z3 (5 714,29 zł). Z4 bez zmian.</t>
+    <t xml:space="preserve">10. Amortyzacja laptopów: 569,02 zł/mies. (Z1 wykonanie 2 276,08 = 4 × 569,02). Poz. 2.9 (Z2, 6 m-cy) = 3 414,12 zł, poz. 3.8 (Z3, 8 m-cy) = 4 552,16 zł, poz. 4.7 (Z4, 4 m-ce) = 2 276,08 zł. Uwolniona różnica nie trafia na licencje – zwiększa kwalifikowalne Z4 (mniejsze obniżenie, współczynnik C19), w granicach limitu dofinansowania.</t>
   </si>
   <si>
     <t xml:space="preserve">11. Dofinansowanie: Z1–Z3 po 80%, Z4 po 60% (bez żadnych korekt intensywności). Przy pełnej prognozie Z3 i Z4 dofinansowanie przekroczyłoby cel, dlatego kwalifikowalne Z4 obniżono jednolitym współczynnikiem C19 do kwoty mieszczącej się w limicie dofinansowania (C18). Kwalifikowalne razem spadają poniżej celu – różnica to niewykorzystany budżet.</t>
@@ -678,7 +678,7 @@
     <t xml:space="preserve">Architekt rozwiązań chmurowych</t>
   </si>
   <si>
-    <t xml:space="preserve">Amortyzacja laptopów (1 = 714,29/mies.)</t>
+    <t xml:space="preserve">Amortyzacja laptopów (stawka = amortyzacja miesięczna)</t>
   </si>
   <si>
     <t xml:space="preserve">FTE – BĘDZIE (nowy budżet)</t>
@@ -12147,8 +12147,8 @@
         <v>158</v>
       </c>
       <c r="C15" s="44" t="n">
-        <f aca="false">SUMIF('plan etatów'!$C$78:$C$114,4,'plan etatów'!$AA$78:$AA$114)</f>
-        <v>664057.14</v>
+        <f aca="false">'plan etatów'!AA106+'plan etatów'!AA107+'plan etatów'!AA108+'plan etatów'!AA109+'plan etatów'!AA110+'plan etatów'!AA111+'plan etatów'!AA113+'plan etatów'!AA114</f>
+        <v>661200</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12157,7 +12157,7 @@
       </c>
       <c r="C16" s="44" t="n">
         <f aca="false">'nowy format 2'!G24</f>
-        <v>1111999.42</v>
+        <v>1111069.73</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="C17" s="44" t="n">
         <f aca="false">'nowy format 2'!G4+'nowy format 2'!G5+'nowy format 2'!G6+'nowy format 2'!G7+'nowy format 2'!G8+'nowy format 2'!G9+'nowy format 2'!G10+'nowy format 2'!G11+'nowy format 2'!G12+'nowy format 2'!G14+'nowy format 2'!G15+'nowy format 2'!G16+'nowy format 2'!G17+'nowy format 2'!G18+'nowy format 2'!G19+'nowy format 2'!G20+'nowy format 2'!G21+'nowy format 2'!G22+'nowy format 2'!G23+C16</f>
-        <v>2566562.43</v>
+        <v>2564935.48</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12174,8 +12174,8 @@
         <v>161</v>
       </c>
       <c r="C18" s="44" t="n">
-        <f aca="false">C13-C17</f>
-        <v>393384.11</v>
+        <f aca="false">C13-C17-C7*('plan etatów'!AA112)</f>
+        <v>393645.412</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12184,7 +12184,7 @@
       </c>
       <c r="C19" s="47" t="n">
         <f aca="false">MIN(1,ROUNDDOWN(C18/C7,2)/C15)</f>
-        <v>0.987324946163518</v>
+        <v>0.992249969751966</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12220,7 +12220,7 @@
       </c>
       <c r="C23" s="44" t="n">
         <f aca="false">ROUND(C15*C19,2)</f>
-        <v>655640.18</v>
+        <v>656075.68</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12246,7 +12246,7 @@
       </c>
       <c r="C25" s="49" t="n">
         <f aca="false">'nowy format 2'!F50</f>
-        <v>4829804.08</v>
+        <v>4830651.4</v>
       </c>
       <c r="D25" s="49" t="n">
         <f aca="false">C10</f>
@@ -12258,7 +12258,7 @@
       </c>
       <c r="F25" s="49" t="n">
         <f aca="false">ROUND(C25-D25,2)</f>
-        <v>-13311.53</v>
+        <v>-12464.21</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12303,11 +12303,11 @@
       </c>
       <c r="C28" s="49" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!C97,2)</f>
-        <v>3863843.25</v>
+        <v>3864521.12</v>
       </c>
       <c r="D28" s="49" t="n">
         <f aca="false">'nowy format 2'!F48</f>
-        <v>3863843.26</v>
+        <v>3864521.12</v>
       </c>
       <c r="E28" s="40" t="str">
         <f aca="false">IF(ABS(C28-D28)&lt;=0.05,"OK","BŁĄD")</f>
@@ -12357,7 +12357,7 @@
       </c>
       <c r="C31" s="49" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!C191,2)</f>
-        <v>2959946.54</v>
+        <v>2959946.53</v>
       </c>
       <c r="D31" s="49" t="n">
         <f aca="false">'nowy format 2'!G48</f>
@@ -14166,8 +14166,7 @@
         <v>215</v>
       </c>
       <c r="B32" s="54" t="n">
-        <f aca="false">ROUND(4285.71/6,4)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="D32" s="52" t="n">
         <v>1</v>
@@ -18980,23 +18979,23 @@
       </c>
       <c r="D85" s="56" t="n">
         <f aca="false">IF(AND(D$77&gt;=$D$4,D$77&lt;=$E$4),$B$32*D32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="E85" s="56" t="n">
         <f aca="false">IF(AND(E$77&gt;=$D$4,E$77&lt;=$E$4),$B$32*E32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="F85" s="56" t="n">
         <f aca="false">IF(AND(F$77&gt;=$D$4,F$77&lt;=$E$4),$B$32*F32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="G85" s="56" t="n">
         <f aca="false">IF(AND(G$77&gt;=$D$4,G$77&lt;=$E$4),$B$32*G32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="H85" s="56" t="n">
         <f aca="false">IF(AND(H$77&gt;=$D$4,H$77&lt;=$E$4),$B$32*H32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="I85" s="56" t="n">
         <f aca="false">IF(AND(I$77&gt;=$D$4,I$77&lt;=$E$4),$B$32*I32,0)</f>
@@ -19072,7 +19071,7 @@
       </c>
       <c r="AA85" s="57" t="n">
         <f aca="false">SUM(D85:Z85)</f>
-        <v>3571.425</v>
+        <v>2845.1</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20017,27 +20016,27 @@
       </c>
       <c r="I95" s="56" t="n">
         <f aca="false">IF(AND(I$77&gt;=$D$5,I$77&lt;=$E$5),$B$32*I32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="J95" s="56" t="n">
         <f aca="false">IF(AND(J$77&gt;=$D$5,J$77&lt;=$E$5),$B$32*J32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="K95" s="56" t="n">
         <f aca="false">IF(AND(K$77&gt;=$D$5,K$77&lt;=$E$5),$B$32*K32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="L95" s="56" t="n">
         <f aca="false">IF(AND(L$77&gt;=$D$5,L$77&lt;=$E$5),$B$32*L32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="M95" s="56" t="n">
         <f aca="false">IF(AND(M$77&gt;=$D$5,M$77&lt;=$E$5),$B$32*M32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="N95" s="56" t="n">
         <f aca="false">IF(AND(N$77&gt;=$D$5,N$77&lt;=$E$5),$B$32*N32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="O95" s="56" t="n">
         <f aca="false">IF(AND(O$77&gt;=$D$5,O$77&lt;=$E$5),$B$32*O32,0)</f>
@@ -20089,7 +20088,7 @@
       </c>
       <c r="AA95" s="57" t="n">
         <f aca="false">SUM(D95:Z95)</f>
-        <v>4285.71</v>
+        <v>3414.12</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20977,35 +20976,35 @@
       </c>
       <c r="O104" s="56" t="n">
         <f aca="false">IF(AND(O$77&gt;=$D$6,O$77&lt;=$E$6),$B$32*O32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="P104" s="56" t="n">
         <f aca="false">IF(AND(P$77&gt;=$D$6,P$77&lt;=$E$6),$B$32*P32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="Q104" s="56" t="n">
         <f aca="false">IF(AND(Q$77&gt;=$D$6,Q$77&lt;=$E$6),$B$32*Q32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="R104" s="56" t="n">
         <f aca="false">IF(AND(R$77&gt;=$D$6,R$77&lt;=$E$6),$B$32*R32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="S104" s="56" t="n">
         <f aca="false">IF(AND(S$77&gt;=$D$6,S$77&lt;=$E$6),$B$32*S32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="T104" s="56" t="n">
         <f aca="false">IF(AND(T$77&gt;=$D$6,T$77&lt;=$E$6),$B$32*T32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="U104" s="56" t="n">
         <f aca="false">IF(AND(U$77&gt;=$D$6,U$77&lt;=$E$6),$B$32*U32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="V104" s="56" t="n">
         <f aca="false">IF(AND(V$77&gt;=$D$6,V$77&lt;=$E$6),$B$32*V32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="W104" s="56" t="n">
         <f aca="false">IF(AND(W$77&gt;=$D$6,W$77&lt;=$E$6),$B$32*W32,0)</f>
@@ -21025,7 +21024,7 @@
       </c>
       <c r="AA104" s="57" t="n">
         <f aca="false">SUM(D104:Z104)</f>
-        <v>5714.28</v>
+        <v>4552.16</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21841,23 +21840,23 @@
       </c>
       <c r="W112" s="56" t="n">
         <f aca="false">IF(AND(W$77&gt;=$D$7,W$77&lt;=$E$7),$B$32*W32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="X112" s="56" t="n">
         <f aca="false">IF(AND(X$77&gt;=$D$7,X$77&lt;=$E$7),$B$32*X32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="Y112" s="56" t="n">
         <f aca="false">IF(AND(Y$77&gt;=$D$7,Y$77&lt;=$E$7),$B$32*Y32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="Z112" s="56" t="n">
         <f aca="false">IF(AND(Z$77&gt;=$D$7,Z$77&lt;=$E$7),$B$32*Z32,0)</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="AA112" s="57" t="n">
         <f aca="false">SUM(D112:Z112)</f>
-        <v>2857.14</v>
+        <v>2276.08</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29042,98 +29041,98 @@
       </c>
       <c r="C73" s="49" t="n">
         <f aca="false">SUM(D73:Z73)</f>
-        <v>4285.71</v>
+        <v>3414.12</v>
       </c>
       <c r="D73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!D95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!D95</f>
         <v>0</v>
       </c>
       <c r="E73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!E95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!E95</f>
         <v>0</v>
       </c>
       <c r="F73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!F95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!F95</f>
         <v>0</v>
       </c>
       <c r="G73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!G95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!G95</f>
         <v>0</v>
       </c>
       <c r="H73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!H95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!H95</f>
         <v>0</v>
       </c>
       <c r="I73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!I95/'plan etatów'!$AA$95)</f>
-        <v>714.285</v>
+        <f aca="false">'plan etatów'!I95</f>
+        <v>569.02</v>
       </c>
       <c r="J73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!J95/'plan etatów'!$AA$95)</f>
-        <v>714.285</v>
+        <f aca="false">'plan etatów'!J95</f>
+        <v>569.02</v>
       </c>
       <c r="K73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!K95/'plan etatów'!$AA$95)</f>
-        <v>714.285</v>
+        <f aca="false">'plan etatów'!K95</f>
+        <v>569.02</v>
       </c>
       <c r="L73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!L95/'plan etatów'!$AA$95)</f>
-        <v>714.285</v>
+        <f aca="false">'plan etatów'!L95</f>
+        <v>569.02</v>
       </c>
       <c r="M73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!M95/'plan etatów'!$AA$95)</f>
-        <v>714.285</v>
+        <f aca="false">'plan etatów'!M95</f>
+        <v>569.02</v>
       </c>
       <c r="N73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!N95/'plan etatów'!$AA$95)</f>
-        <v>714.285</v>
+        <f aca="false">'plan etatów'!N95</f>
+        <v>569.02</v>
       </c>
       <c r="O73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!O95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!O95</f>
         <v>0</v>
       </c>
       <c r="P73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!P95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!P95</f>
         <v>0</v>
       </c>
       <c r="Q73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!Q95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!Q95</f>
         <v>0</v>
       </c>
       <c r="R73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!R95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!R95</f>
         <v>0</v>
       </c>
       <c r="S73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!S95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!S95</f>
         <v>0</v>
       </c>
       <c r="T73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!T95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!T95</f>
         <v>0</v>
       </c>
       <c r="U73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!U95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!U95</f>
         <v>0</v>
       </c>
       <c r="V73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!V95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!V95</f>
         <v>0</v>
       </c>
       <c r="W73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!W95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!W95</f>
         <v>0</v>
       </c>
       <c r="X73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!X95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!X95</f>
         <v>0</v>
       </c>
       <c r="Y73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!Y95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!Y95</f>
         <v>0</v>
       </c>
       <c r="Z73" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$J$22*'plan etatów'!Z95/'plan etatów'!$AA$95)</f>
+        <f aca="false">'plan etatów'!Z95</f>
         <v>0</v>
       </c>
     </row>
@@ -29978,7 +29977,7 @@
       </c>
       <c r="C82" s="49" t="n">
         <f aca="false">SUM(D82:Z82)</f>
-        <v>5714.28</v>
+        <v>4552.16</v>
       </c>
       <c r="D82" s="49" t="n">
         <f aca="false">'plan etatów'!D104</f>
@@ -30026,35 +30025,35 @@
       </c>
       <c r="O82" s="49" t="n">
         <f aca="false">'plan etatów'!O104</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="P82" s="49" t="n">
         <f aca="false">'plan etatów'!P104</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="Q82" s="49" t="n">
         <f aca="false">'plan etatów'!Q104</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="R82" s="49" t="n">
         <f aca="false">'plan etatów'!R104</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="S82" s="49" t="n">
         <f aca="false">'plan etatów'!S104</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="T82" s="49" t="n">
         <f aca="false">'plan etatów'!T104</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="U82" s="49" t="n">
         <f aca="false">'plan etatów'!U104</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="V82" s="49" t="n">
         <f aca="false">'plan etatów'!V104</f>
-        <v>714.285</v>
+        <v>569.02</v>
       </c>
       <c r="W82" s="49" t="n">
         <f aca="false">'plan etatów'!W104</f>
@@ -30186,7 +30185,7 @@
       </c>
       <c r="C84" s="49" t="n">
         <f aca="false">SUM(D84:Z84)</f>
-        <v>218791.208069836</v>
+        <v>219882.593297036</v>
       </c>
       <c r="D84" s="49" t="n">
         <f aca="false">'plan etatów'!D106*założenia!$C$19</f>
@@ -30266,19 +30265,19 @@
       </c>
       <c r="W84" s="49" t="n">
         <f aca="false">'plan etatów'!W106*założenia!$C$19</f>
-        <v>54697.8020174589</v>
+        <v>54970.6483242589</v>
       </c>
       <c r="X84" s="49" t="n">
         <f aca="false">'plan etatów'!X106*założenia!$C$19</f>
-        <v>54697.8020174589</v>
+        <v>54970.6483242589</v>
       </c>
       <c r="Y84" s="49" t="n">
         <f aca="false">'plan etatów'!Y106*założenia!$C$19</f>
-        <v>54697.8020174589</v>
+        <v>54970.6483242589</v>
       </c>
       <c r="Z84" s="49" t="n">
         <f aca="false">'plan etatów'!Z106*założenia!$C$19</f>
-        <v>54697.8020174589</v>
+        <v>54970.6483242589</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30290,7 +30289,7 @@
       </c>
       <c r="C85" s="49" t="n">
         <f aca="false">SUM(D85:Z85)</f>
-        <v>37241.8969692879</v>
+        <v>37427.6688590442</v>
       </c>
       <c r="D85" s="49" t="n">
         <f aca="false">'plan etatów'!D107*założenia!$C$19</f>
@@ -30370,19 +30369,19 @@
       </c>
       <c r="W85" s="49" t="n">
         <f aca="false">'plan etatów'!W107*założenia!$C$19</f>
-        <v>9310.47424232198</v>
+        <v>9356.91721476104</v>
       </c>
       <c r="X85" s="49" t="n">
         <f aca="false">'plan etatów'!X107*założenia!$C$19</f>
-        <v>9310.47424232198</v>
+        <v>9356.91721476104</v>
       </c>
       <c r="Y85" s="49" t="n">
         <f aca="false">'plan etatów'!Y107*założenia!$C$19</f>
-        <v>9310.47424232198</v>
+        <v>9356.91721476104</v>
       </c>
       <c r="Z85" s="49" t="n">
         <f aca="false">'plan etatów'!Z107*założenia!$C$19</f>
-        <v>9310.47424232198</v>
+        <v>9356.91721476104</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30394,7 +30393,7 @@
       </c>
       <c r="C86" s="49" t="n">
         <f aca="false">SUM(D86:Z86)</f>
-        <v>107065.517161972</v>
+        <v>107599.586719903</v>
       </c>
       <c r="D86" s="49" t="n">
         <f aca="false">'plan etatów'!D108*założenia!$C$19</f>
@@ -30474,19 +30473,19 @@
       </c>
       <c r="W86" s="49" t="n">
         <f aca="false">'plan etatów'!W108*założenia!$C$19</f>
-        <v>26766.379290493</v>
+        <v>26899.8966799758</v>
       </c>
       <c r="X86" s="49" t="n">
         <f aca="false">'plan etatów'!X108*założenia!$C$19</f>
-        <v>26766.379290493</v>
+        <v>26899.8966799758</v>
       </c>
       <c r="Y86" s="49" t="n">
         <f aca="false">'plan etatów'!Y108*założenia!$C$19</f>
-        <v>26766.379290493</v>
+        <v>26899.8966799758</v>
       </c>
       <c r="Z86" s="49" t="n">
         <f aca="false">'plan etatów'!Z108*założenia!$C$19</f>
-        <v>26766.379290493</v>
+        <v>26899.8966799758</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30498,7 +30497,7 @@
       </c>
       <c r="C87" s="49" t="n">
         <f aca="false">SUM(D87:Z87)</f>
-        <v>81454.3080584903</v>
+        <v>81860.6225045372</v>
       </c>
       <c r="D87" s="49" t="n">
         <f aca="false">'plan etatów'!D109*założenia!$C$19</f>
@@ -30578,19 +30577,19 @@
       </c>
       <c r="W87" s="49" t="n">
         <f aca="false">'plan etatów'!W109*założenia!$C$19</f>
-        <v>20363.5770146226</v>
+        <v>20465.1556261343</v>
       </c>
       <c r="X87" s="49" t="n">
         <f aca="false">'plan etatów'!X109*założenia!$C$19</f>
-        <v>20363.5770146226</v>
+        <v>20465.1556261343</v>
       </c>
       <c r="Y87" s="49" t="n">
         <f aca="false">'plan etatów'!Y109*założenia!$C$19</f>
-        <v>20363.5770146226</v>
+        <v>20465.1556261343</v>
       </c>
       <c r="Z87" s="49" t="n">
         <f aca="false">'plan etatów'!Z109*założenia!$C$19</f>
-        <v>20363.5770146226</v>
+        <v>20465.1556261343</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30602,7 +30601,7 @@
       </c>
       <c r="C88" s="49" t="n">
         <f aca="false">SUM(D88:Z88)</f>
-        <v>29382.7903978263</v>
+        <v>29529.3590998185</v>
       </c>
       <c r="D88" s="49" t="n">
         <f aca="false">'plan etatów'!D110*założenia!$C$19</f>
@@ -30682,19 +30681,19 @@
       </c>
       <c r="W88" s="49" t="n">
         <f aca="false">'plan etatów'!W110*założenia!$C$19</f>
-        <v>7345.69759945658</v>
+        <v>7382.33977495463</v>
       </c>
       <c r="X88" s="49" t="n">
         <f aca="false">'plan etatów'!X110*założenia!$C$19</f>
-        <v>7345.69759945658</v>
+        <v>7382.33977495463</v>
       </c>
       <c r="Y88" s="49" t="n">
         <f aca="false">'plan etatów'!Y110*założenia!$C$19</f>
-        <v>7345.69759945658</v>
+        <v>7382.33977495463</v>
       </c>
       <c r="Z88" s="49" t="n">
         <f aca="false">'plan etatów'!Z110*założenia!$C$19</f>
-        <v>7345.69759945658</v>
+        <v>7382.33977495463</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30706,7 +30705,7 @@
       </c>
       <c r="C89" s="49" t="n">
         <f aca="false">SUM(D89:Z89)</f>
-        <v>81454.3080584903</v>
+        <v>81860.6225045372</v>
       </c>
       <c r="D89" s="49" t="n">
         <f aca="false">'plan etatów'!D111*założenia!$C$19</f>
@@ -30786,19 +30785,19 @@
       </c>
       <c r="W89" s="49" t="n">
         <f aca="false">'plan etatów'!W111*założenia!$C$19</f>
-        <v>20363.5770146226</v>
+        <v>20465.1556261343</v>
       </c>
       <c r="X89" s="49" t="n">
         <f aca="false">'plan etatów'!X111*założenia!$C$19</f>
-        <v>20363.5770146226</v>
+        <v>20465.1556261343</v>
       </c>
       <c r="Y89" s="49" t="n">
         <f aca="false">'plan etatów'!Y111*założenia!$C$19</f>
-        <v>20363.5770146226</v>
+        <v>20465.1556261343</v>
       </c>
       <c r="Z89" s="49" t="n">
         <f aca="false">'plan etatów'!Z111*założenia!$C$19</f>
-        <v>20363.5770146226</v>
+        <v>20465.1556261343</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30810,99 +30809,99 @@
       </c>
       <c r="C90" s="49" t="n">
         <f aca="false">SUM(D90:Z90)</f>
-        <v>2820.92559668164</v>
+        <v>2276.08</v>
       </c>
       <c r="D90" s="49" t="n">
-        <f aca="false">'plan etatów'!D112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!D112</f>
         <v>0</v>
       </c>
       <c r="E90" s="49" t="n">
-        <f aca="false">'plan etatów'!E112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!E112</f>
         <v>0</v>
       </c>
       <c r="F90" s="49" t="n">
-        <f aca="false">'plan etatów'!F112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!F112</f>
         <v>0</v>
       </c>
       <c r="G90" s="49" t="n">
-        <f aca="false">'plan etatów'!G112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!G112</f>
         <v>0</v>
       </c>
       <c r="H90" s="49" t="n">
-        <f aca="false">'plan etatów'!H112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!H112</f>
         <v>0</v>
       </c>
       <c r="I90" s="49" t="n">
-        <f aca="false">'plan etatów'!I112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!I112</f>
         <v>0</v>
       </c>
       <c r="J90" s="49" t="n">
-        <f aca="false">'plan etatów'!J112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!J112</f>
         <v>0</v>
       </c>
       <c r="K90" s="49" t="n">
-        <f aca="false">'plan etatów'!K112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!K112</f>
         <v>0</v>
       </c>
       <c r="L90" s="49" t="n">
-        <f aca="false">'plan etatów'!L112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!L112</f>
         <v>0</v>
       </c>
       <c r="M90" s="49" t="n">
-        <f aca="false">'plan etatów'!M112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!M112</f>
         <v>0</v>
       </c>
       <c r="N90" s="49" t="n">
-        <f aca="false">'plan etatów'!N112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!N112</f>
         <v>0</v>
       </c>
       <c r="O90" s="49" t="n">
-        <f aca="false">'plan etatów'!O112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!O112</f>
         <v>0</v>
       </c>
       <c r="P90" s="49" t="n">
-        <f aca="false">'plan etatów'!P112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!P112</f>
         <v>0</v>
       </c>
       <c r="Q90" s="49" t="n">
-        <f aca="false">'plan etatów'!Q112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!Q112</f>
         <v>0</v>
       </c>
       <c r="R90" s="49" t="n">
-        <f aca="false">'plan etatów'!R112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!R112</f>
         <v>0</v>
       </c>
       <c r="S90" s="49" t="n">
-        <f aca="false">'plan etatów'!S112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!S112</f>
         <v>0</v>
       </c>
       <c r="T90" s="49" t="n">
-        <f aca="false">'plan etatów'!T112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!T112</f>
         <v>0</v>
       </c>
       <c r="U90" s="49" t="n">
-        <f aca="false">'plan etatów'!U112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!U112</f>
         <v>0</v>
       </c>
       <c r="V90" s="49" t="n">
-        <f aca="false">'plan etatów'!V112*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!V112</f>
         <v>0</v>
       </c>
       <c r="W90" s="49" t="n">
-        <f aca="false">'plan etatów'!W112*założenia!$C$19</f>
-        <v>705.231399170409</v>
+        <f aca="false">'plan etatów'!W112</f>
+        <v>569.02</v>
       </c>
       <c r="X90" s="49" t="n">
-        <f aca="false">'plan etatów'!X112*założenia!$C$19</f>
-        <v>705.231399170409</v>
+        <f aca="false">'plan etatów'!X112</f>
+        <v>569.02</v>
       </c>
       <c r="Y90" s="49" t="n">
-        <f aca="false">'plan etatów'!Y112*założenia!$C$19</f>
-        <v>705.231399170409</v>
+        <f aca="false">'plan etatów'!Y112</f>
+        <v>569.02</v>
       </c>
       <c r="Z90" s="49" t="n">
-        <f aca="false">'plan etatów'!Z112*założenia!$C$19</f>
-        <v>705.231399170409</v>
+        <f aca="false">'plan etatów'!Z112</f>
+        <v>569.02</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30914,7 +30913,7 @@
       </c>
       <c r="C91" s="49" t="n">
         <f aca="false">SUM(D91:Z91)</f>
-        <v>77998.670746918</v>
+        <v>78387.7476104053</v>
       </c>
       <c r="D91" s="49" t="n">
         <f aca="false">'plan etatów'!D113*założenia!$C$19</f>
@@ -30994,19 +30993,19 @@
       </c>
       <c r="W91" s="49" t="n">
         <f aca="false">'plan etatów'!W113*założenia!$C$19</f>
-        <v>19499.6676867295</v>
+        <v>19596.9369026013</v>
       </c>
       <c r="X91" s="49" t="n">
         <f aca="false">'plan etatów'!X113*założenia!$C$19</f>
-        <v>19499.6676867295</v>
+        <v>19596.9369026013</v>
       </c>
       <c r="Y91" s="49" t="n">
         <f aca="false">'plan etatów'!Y113*założenia!$C$19</f>
-        <v>19499.6676867295</v>
+        <v>19596.9369026013</v>
       </c>
       <c r="Z91" s="49" t="n">
         <f aca="false">'plan etatów'!Z113*założenia!$C$19</f>
-        <v>19499.6676867295</v>
+        <v>19596.9369026013</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31018,7 +31017,7 @@
       </c>
       <c r="C92" s="49" t="n">
         <f aca="false">SUM(D92:Z92)</f>
-        <v>19430.554940498</v>
+        <v>19527.4794047187</v>
       </c>
       <c r="D92" s="49" t="n">
         <f aca="false">'plan etatów'!D114*założenia!$C$19</f>
@@ -31098,19 +31097,19 @@
       </c>
       <c r="W92" s="49" t="n">
         <f aca="false">'plan etatów'!W114*założenia!$C$19</f>
-        <v>4857.63873512451</v>
+        <v>4881.86985117967</v>
       </c>
       <c r="X92" s="49" t="n">
         <f aca="false">'plan etatów'!X114*założenia!$C$19</f>
-        <v>4857.63873512451</v>
+        <v>4881.86985117967</v>
       </c>
       <c r="Y92" s="49" t="n">
         <f aca="false">'plan etatów'!Y114*założenia!$C$19</f>
-        <v>4857.63873512451</v>
+        <v>4881.86985117967</v>
       </c>
       <c r="Z92" s="49" t="n">
         <f aca="false">'plan etatów'!Z114*założenia!$C$19</f>
-        <v>4857.63873512451</v>
+        <v>4881.86985117967</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31226,7 +31225,7 @@
       </c>
       <c r="C94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,C$56:C$92)</f>
-        <v>1010778.92</v>
+        <v>1009907.33</v>
       </c>
       <c r="D94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,D$56:D$92)</f>
@@ -31250,27 +31249,27 @@
       </c>
       <c r="I94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,I$56:I$92)</f>
-        <v>168463.153333333</v>
+        <v>168317.888333333</v>
       </c>
       <c r="J94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,J$56:J$92)</f>
-        <v>168463.153333333</v>
+        <v>168317.888333333</v>
       </c>
       <c r="K94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,K$56:K$92)</f>
-        <v>168463.153333333</v>
+        <v>168317.888333333</v>
       </c>
       <c r="L94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,L$56:L$92)</f>
-        <v>168463.153333333</v>
+        <v>168317.888333333</v>
       </c>
       <c r="M94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,M$56:M$92)</f>
-        <v>168463.153333333</v>
+        <v>168317.888333333</v>
       </c>
       <c r="N94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,N$56:N$92)</f>
-        <v>168463.153333333</v>
+        <v>168317.888333333</v>
       </c>
       <c r="O94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,O$56:O$92)</f>
@@ -31330,7 +31329,7 @@
       </c>
       <c r="C95" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,3,C$56:C$92)</f>
-        <v>1389999.28</v>
+        <v>1388837.16</v>
       </c>
       <c r="D95" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,3,D$56:D$92)</f>
@@ -31378,35 +31377,35 @@
       </c>
       <c r="O95" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,3,O$56:O$92)</f>
-        <v>168666.785</v>
+        <v>168521.52</v>
       </c>
       <c r="P95" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,3,P$56:P$92)</f>
-        <v>168666.785</v>
+        <v>168521.52</v>
       </c>
       <c r="Q95" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,3,Q$56:Q$92)</f>
-        <v>175444.285</v>
+        <v>175299.02</v>
       </c>
       <c r="R95" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,3,R$56:R$92)</f>
-        <v>175444.285</v>
+        <v>175299.02</v>
       </c>
       <c r="S95" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,3,S$56:S$92)</f>
-        <v>175444.285</v>
+        <v>175299.02</v>
       </c>
       <c r="T95" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,3,T$56:T$92)</f>
-        <v>175444.285</v>
+        <v>175299.02</v>
       </c>
       <c r="U95" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,3,U$56:U$92)</f>
-        <v>175444.285</v>
+        <v>175299.02</v>
       </c>
       <c r="V95" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,3,V$56:V$92)</f>
-        <v>175444.285</v>
+        <v>175299.02</v>
       </c>
       <c r="W95" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,3,W$56:W$92)</f>
@@ -31434,7 +31433,7 @@
       </c>
       <c r="C96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,C$56:C$92)</f>
-        <v>655640.18</v>
+        <v>658351.76</v>
       </c>
       <c r="D96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,D$56:D$92)</f>
@@ -31514,19 +31513,19 @@
       </c>
       <c r="W96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,W$56:W$92)</f>
-        <v>163910.045</v>
+        <v>164587.94</v>
       </c>
       <c r="X96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,X$56:X$92)</f>
-        <v>163910.045</v>
+        <v>164587.94</v>
       </c>
       <c r="Y96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,Y$56:Y$92)</f>
-        <v>163910.045</v>
+        <v>164587.94</v>
       </c>
       <c r="Z96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,Z$56:Z$92)</f>
-        <v>163910.045</v>
+        <v>164587.94</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31536,7 +31535,7 @@
       <c r="B97" s="40"/>
       <c r="C97" s="63" t="n">
         <f aca="false">SUM(C93:C96)</f>
-        <v>3863843.25</v>
+        <v>3864521.12</v>
       </c>
       <c r="D97" s="63" t="n">
         <f aca="false">SUM(D93:D96)</f>
@@ -31560,75 +31559,75 @@
       </c>
       <c r="I97" s="63" t="n">
         <f aca="false">SUM(I93:I96)</f>
-        <v>168463.153333333</v>
+        <v>168317.888333333</v>
       </c>
       <c r="J97" s="63" t="n">
         <f aca="false">SUM(J93:J96)</f>
-        <v>168463.153333333</v>
+        <v>168317.888333333</v>
       </c>
       <c r="K97" s="63" t="n">
         <f aca="false">SUM(K93:K96)</f>
-        <v>168463.153333333</v>
+        <v>168317.888333333</v>
       </c>
       <c r="L97" s="63" t="n">
         <f aca="false">SUM(L93:L96)</f>
-        <v>168463.153333333</v>
+        <v>168317.888333333</v>
       </c>
       <c r="M97" s="63" t="n">
         <f aca="false">SUM(M93:M96)</f>
-        <v>168463.153333333</v>
+        <v>168317.888333333</v>
       </c>
       <c r="N97" s="63" t="n">
         <f aca="false">SUM(N93:N96)</f>
-        <v>168463.153333333</v>
+        <v>168317.888333333</v>
       </c>
       <c r="O97" s="63" t="n">
         <f aca="false">SUM(O93:O96)</f>
-        <v>168666.785</v>
+        <v>168521.52</v>
       </c>
       <c r="P97" s="63" t="n">
         <f aca="false">SUM(P93:P96)</f>
-        <v>168666.785</v>
+        <v>168521.52</v>
       </c>
       <c r="Q97" s="63" t="n">
         <f aca="false">SUM(Q93:Q96)</f>
-        <v>175444.285</v>
+        <v>175299.02</v>
       </c>
       <c r="R97" s="63" t="n">
         <f aca="false">SUM(R93:R96)</f>
-        <v>175444.285</v>
+        <v>175299.02</v>
       </c>
       <c r="S97" s="63" t="n">
         <f aca="false">SUM(S93:S96)</f>
-        <v>175444.285</v>
+        <v>175299.02</v>
       </c>
       <c r="T97" s="63" t="n">
         <f aca="false">SUM(T93:T96)</f>
-        <v>175444.285</v>
+        <v>175299.02</v>
       </c>
       <c r="U97" s="63" t="n">
         <f aca="false">SUM(U93:U96)</f>
-        <v>175444.285</v>
+        <v>175299.02</v>
       </c>
       <c r="V97" s="63" t="n">
         <f aca="false">SUM(V93:V96)</f>
-        <v>175444.285</v>
+        <v>175299.02</v>
       </c>
       <c r="W97" s="63" t="n">
         <f aca="false">SUM(W93:W96)</f>
-        <v>163910.045</v>
+        <v>164587.94</v>
       </c>
       <c r="X97" s="63" t="n">
         <f aca="false">SUM(X93:X96)</f>
-        <v>163910.045</v>
+        <v>164587.94</v>
       </c>
       <c r="Y97" s="63" t="n">
         <f aca="false">SUM(Y93:Y96)</f>
-        <v>163910.045</v>
+        <v>164587.94</v>
       </c>
       <c r="Z97" s="63" t="n">
         <f aca="false">SUM(Z93:Z96)</f>
-        <v>163910.045</v>
+        <v>164587.94</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31638,7 +31637,7 @@
       <c r="B98" s="40"/>
       <c r="C98" s="63" t="n">
         <f aca="false">0.25*C97</f>
-        <v>965960.8125</v>
+        <v>966130.28</v>
       </c>
       <c r="D98" s="63" t="n">
         <f aca="false">0.25*D97</f>
@@ -31662,75 +31661,75 @@
       </c>
       <c r="I98" s="63" t="n">
         <f aca="false">0.25*I97</f>
-        <v>42115.7883333333</v>
+        <v>42079.4720833333</v>
       </c>
       <c r="J98" s="63" t="n">
         <f aca="false">0.25*J97</f>
-        <v>42115.7883333333</v>
+        <v>42079.4720833333</v>
       </c>
       <c r="K98" s="63" t="n">
         <f aca="false">0.25*K97</f>
-        <v>42115.7883333333</v>
+        <v>42079.4720833333</v>
       </c>
       <c r="L98" s="63" t="n">
         <f aca="false">0.25*L97</f>
-        <v>42115.7883333333</v>
+        <v>42079.4720833333</v>
       </c>
       <c r="M98" s="63" t="n">
         <f aca="false">0.25*M97</f>
-        <v>42115.7883333333</v>
+        <v>42079.4720833333</v>
       </c>
       <c r="N98" s="63" t="n">
         <f aca="false">0.25*N97</f>
-        <v>42115.7883333333</v>
+        <v>42079.4720833333</v>
       </c>
       <c r="O98" s="63" t="n">
         <f aca="false">0.25*O97</f>
-        <v>42166.69625</v>
+        <v>42130.38</v>
       </c>
       <c r="P98" s="63" t="n">
         <f aca="false">0.25*P97</f>
-        <v>42166.69625</v>
+        <v>42130.38</v>
       </c>
       <c r="Q98" s="63" t="n">
         <f aca="false">0.25*Q97</f>
-        <v>43861.07125</v>
+        <v>43824.755</v>
       </c>
       <c r="R98" s="63" t="n">
         <f aca="false">0.25*R97</f>
-        <v>43861.07125</v>
+        <v>43824.755</v>
       </c>
       <c r="S98" s="63" t="n">
         <f aca="false">0.25*S97</f>
-        <v>43861.07125</v>
+        <v>43824.755</v>
       </c>
       <c r="T98" s="63" t="n">
         <f aca="false">0.25*T97</f>
-        <v>43861.07125</v>
+        <v>43824.755</v>
       </c>
       <c r="U98" s="63" t="n">
         <f aca="false">0.25*U97</f>
-        <v>43861.07125</v>
+        <v>43824.755</v>
       </c>
       <c r="V98" s="63" t="n">
         <f aca="false">0.25*V97</f>
-        <v>43861.07125</v>
+        <v>43824.755</v>
       </c>
       <c r="W98" s="63" t="n">
         <f aca="false">0.25*W97</f>
-        <v>40977.51125</v>
+        <v>41146.985</v>
       </c>
       <c r="X98" s="63" t="n">
         <f aca="false">0.25*X97</f>
-        <v>40977.51125</v>
+        <v>41146.985</v>
       </c>
       <c r="Y98" s="63" t="n">
         <f aca="false">0.25*Y97</f>
-        <v>40977.51125</v>
+        <v>41146.985</v>
       </c>
       <c r="Z98" s="63" t="n">
         <f aca="false">0.25*Z97</f>
-        <v>40977.51125</v>
+        <v>41146.985</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31740,7 +31739,7 @@
       <c r="B99" s="40"/>
       <c r="C99" s="63" t="n">
         <f aca="false">C97+C98</f>
-        <v>4829804.0625</v>
+        <v>4830651.4</v>
       </c>
       <c r="D99" s="63" t="n">
         <f aca="false">D97+D98</f>
@@ -31764,75 +31763,75 @@
       </c>
       <c r="I99" s="63" t="n">
         <f aca="false">I97+I98</f>
-        <v>210578.941666667</v>
+        <v>210397.360416667</v>
       </c>
       <c r="J99" s="63" t="n">
         <f aca="false">J97+J98</f>
-        <v>210578.941666667</v>
+        <v>210397.360416667</v>
       </c>
       <c r="K99" s="63" t="n">
         <f aca="false">K97+K98</f>
-        <v>210578.941666667</v>
+        <v>210397.360416667</v>
       </c>
       <c r="L99" s="63" t="n">
         <f aca="false">L97+L98</f>
-        <v>210578.941666667</v>
+        <v>210397.360416667</v>
       </c>
       <c r="M99" s="63" t="n">
         <f aca="false">M97+M98</f>
-        <v>210578.941666667</v>
+        <v>210397.360416667</v>
       </c>
       <c r="N99" s="63" t="n">
         <f aca="false">N97+N98</f>
-        <v>210578.941666667</v>
+        <v>210397.360416667</v>
       </c>
       <c r="O99" s="63" t="n">
         <f aca="false">O97+O98</f>
-        <v>210833.48125</v>
+        <v>210651.9</v>
       </c>
       <c r="P99" s="63" t="n">
         <f aca="false">P97+P98</f>
-        <v>210833.48125</v>
+        <v>210651.9</v>
       </c>
       <c r="Q99" s="63" t="n">
         <f aca="false">Q97+Q98</f>
-        <v>219305.35625</v>
+        <v>219123.775</v>
       </c>
       <c r="R99" s="63" t="n">
         <f aca="false">R97+R98</f>
-        <v>219305.35625</v>
+        <v>219123.775</v>
       </c>
       <c r="S99" s="63" t="n">
         <f aca="false">S97+S98</f>
-        <v>219305.35625</v>
+        <v>219123.775</v>
       </c>
       <c r="T99" s="63" t="n">
         <f aca="false">T97+T98</f>
-        <v>219305.35625</v>
+        <v>219123.775</v>
       </c>
       <c r="U99" s="63" t="n">
         <f aca="false">U97+U98</f>
-        <v>219305.35625</v>
+        <v>219123.775</v>
       </c>
       <c r="V99" s="63" t="n">
         <f aca="false">V97+V98</f>
-        <v>219305.35625</v>
+        <v>219123.775</v>
       </c>
       <c r="W99" s="63" t="n">
         <f aca="false">W97+W98</f>
-        <v>204887.55625</v>
+        <v>205734.925</v>
       </c>
       <c r="X99" s="63" t="n">
         <f aca="false">X97+X98</f>
-        <v>204887.55625</v>
+        <v>205734.925</v>
       </c>
       <c r="Y99" s="63" t="n">
         <f aca="false">Y97+Y98</f>
-        <v>204887.55625</v>
+        <v>205734.925</v>
       </c>
       <c r="Z99" s="63" t="n">
         <f aca="false">Z97+Z98</f>
-        <v>204887.55625</v>
+        <v>205734.925</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31863,75 +31862,75 @@
       </c>
       <c r="I100" s="63" t="n">
         <f aca="false">H100+I99</f>
-        <v>1219860.02916667</v>
+        <v>1219678.44791667</v>
       </c>
       <c r="J100" s="63" t="n">
         <f aca="false">I100+J99</f>
-        <v>1430438.97083333</v>
+        <v>1430075.80833333</v>
       </c>
       <c r="K100" s="63" t="n">
         <f aca="false">J100+K99</f>
-        <v>1641017.9125</v>
+        <v>1640473.16875</v>
       </c>
       <c r="L100" s="63" t="n">
         <f aca="false">K100+L99</f>
-        <v>1851596.85416667</v>
+        <v>1850870.52916667</v>
       </c>
       <c r="M100" s="63" t="n">
         <f aca="false">L100+M99</f>
-        <v>2062175.79583333</v>
+        <v>2061267.88958333</v>
       </c>
       <c r="N100" s="63" t="n">
         <f aca="false">M100+N99</f>
-        <v>2272754.7375</v>
+        <v>2271665.25</v>
       </c>
       <c r="O100" s="63" t="n">
         <f aca="false">N100+O99</f>
-        <v>2483588.21875</v>
+        <v>2482317.15</v>
       </c>
       <c r="P100" s="63" t="n">
         <f aca="false">O100+P99</f>
-        <v>2694421.7</v>
+        <v>2692969.05</v>
       </c>
       <c r="Q100" s="63" t="n">
         <f aca="false">P100+Q99</f>
-        <v>2913727.05625</v>
+        <v>2912092.825</v>
       </c>
       <c r="R100" s="63" t="n">
         <f aca="false">Q100+R99</f>
-        <v>3133032.4125</v>
+        <v>3131216.6</v>
       </c>
       <c r="S100" s="63" t="n">
         <f aca="false">R100+S99</f>
-        <v>3352337.76875</v>
+        <v>3350340.375</v>
       </c>
       <c r="T100" s="63" t="n">
         <f aca="false">S100+T99</f>
-        <v>3571643.125</v>
+        <v>3569464.15</v>
       </c>
       <c r="U100" s="63" t="n">
         <f aca="false">T100+U99</f>
-        <v>3790948.48125</v>
+        <v>3788587.925</v>
       </c>
       <c r="V100" s="63" t="n">
         <f aca="false">U100+V99</f>
-        <v>4010253.8375</v>
+        <v>4007711.7</v>
       </c>
       <c r="W100" s="63" t="n">
         <f aca="false">V100+W99</f>
-        <v>4215141.39375</v>
+        <v>4213446.625</v>
       </c>
       <c r="X100" s="63" t="n">
         <f aca="false">W100+X99</f>
-        <v>4420028.95</v>
+        <v>4419181.55</v>
       </c>
       <c r="Y100" s="63" t="n">
         <f aca="false">X100+Y99</f>
-        <v>4624916.50625</v>
+        <v>4624916.475</v>
       </c>
       <c r="Z100" s="63" t="n">
         <f aca="false">Y100+Z99</f>
-        <v>4829804.0625</v>
+        <v>4830651.4</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -38496,98 +38495,98 @@
       </c>
       <c r="C167" s="49" t="n">
         <f aca="false">SUM(D167:Z167)</f>
-        <v>3428.56</v>
+        <v>2731.296</v>
       </c>
       <c r="D167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!D95/'plan etatów'!$AA$95)</f>
+        <f aca="false">D73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="E167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!E95/'plan etatów'!$AA$95)</f>
+        <f aca="false">E73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="F167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!F95/'plan etatów'!$AA$95)</f>
+        <f aca="false">F73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="G167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!G95/'plan etatów'!$AA$95)</f>
+        <f aca="false">G73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="H167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!H95/'plan etatów'!$AA$95)</f>
+        <f aca="false">H73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="I167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!I95/'plan etatów'!$AA$95)</f>
-        <v>571.426666666667</v>
+        <f aca="false">I73*założenia!$C$5</f>
+        <v>455.216</v>
       </c>
       <c r="J167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!J95/'plan etatów'!$AA$95)</f>
-        <v>571.426666666667</v>
+        <f aca="false">J73*założenia!$C$5</f>
+        <v>455.216</v>
       </c>
       <c r="K167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!K95/'plan etatów'!$AA$95)</f>
-        <v>571.426666666667</v>
+        <f aca="false">K73*założenia!$C$5</f>
+        <v>455.216</v>
       </c>
       <c r="L167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!L95/'plan etatów'!$AA$95)</f>
-        <v>571.426666666667</v>
+        <f aca="false">L73*założenia!$C$5</f>
+        <v>455.216</v>
       </c>
       <c r="M167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!M95/'plan etatów'!$AA$95)</f>
-        <v>571.426666666667</v>
+        <f aca="false">M73*założenia!$C$5</f>
+        <v>455.216</v>
       </c>
       <c r="N167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!N95/'plan etatów'!$AA$95)</f>
-        <v>571.426666666667</v>
+        <f aca="false">N73*założenia!$C$5</f>
+        <v>455.216</v>
       </c>
       <c r="O167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!O95/'plan etatów'!$AA$95)</f>
+        <f aca="false">O73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="P167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!P95/'plan etatów'!$AA$95)</f>
+        <f aca="false">P73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="Q167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!Q95/'plan etatów'!$AA$95)</f>
+        <f aca="false">Q73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="R167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!R95/'plan etatów'!$AA$95)</f>
+        <f aca="false">R73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="S167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!S95/'plan etatów'!$AA$95)</f>
+        <f aca="false">S73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="T167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!T95/'plan etatów'!$AA$95)</f>
+        <f aca="false">T73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="U167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!U95/'plan etatów'!$AA$95)</f>
+        <f aca="false">U73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="V167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!V95/'plan etatów'!$AA$95)</f>
+        <f aca="false">V73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="W167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!W95/'plan etatów'!$AA$95)</f>
+        <f aca="false">W73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="X167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!X95/'plan etatów'!$AA$95)</f>
+        <f aca="false">X73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="Y167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!Y95/'plan etatów'!$AA$95)</f>
+        <f aca="false">Y73*założenia!$C$5</f>
         <v>0</v>
       </c>
       <c r="Z167" s="49" t="n">
-        <f aca="false">IF('plan etatów'!$AA$95=0,0,'nowy format 2'!$K$22*'plan etatów'!Z95/'plan etatów'!$AA$95)</f>
+        <f aca="false">Z73*założenia!$C$5</f>
         <v>0</v>
       </c>
     </row>
@@ -39432,7 +39431,7 @@
       </c>
       <c r="C176" s="49" t="n">
         <f aca="false">SUM(D176:Z176)</f>
-        <v>4571.424</v>
+        <v>3641.728</v>
       </c>
       <c r="D176" s="49" t="n">
         <f aca="false">D82*założenia!$C$6</f>
@@ -39480,35 +39479,35 @@
       </c>
       <c r="O176" s="49" t="n">
         <f aca="false">O82*założenia!$C$6</f>
-        <v>571.428</v>
+        <v>455.216</v>
       </c>
       <c r="P176" s="49" t="n">
         <f aca="false">P82*założenia!$C$6</f>
-        <v>571.428</v>
+        <v>455.216</v>
       </c>
       <c r="Q176" s="49" t="n">
         <f aca="false">Q82*założenia!$C$6</f>
-        <v>571.428</v>
+        <v>455.216</v>
       </c>
       <c r="R176" s="49" t="n">
         <f aca="false">R82*założenia!$C$6</f>
-        <v>571.428</v>
+        <v>455.216</v>
       </c>
       <c r="S176" s="49" t="n">
         <f aca="false">S82*założenia!$C$6</f>
-        <v>571.428</v>
+        <v>455.216</v>
       </c>
       <c r="T176" s="49" t="n">
         <f aca="false">T82*założenia!$C$6</f>
-        <v>571.428</v>
+        <v>455.216</v>
       </c>
       <c r="U176" s="49" t="n">
         <f aca="false">U82*założenia!$C$6</f>
-        <v>571.428</v>
+        <v>455.216</v>
       </c>
       <c r="V176" s="49" t="n">
         <f aca="false">V82*założenia!$C$6</f>
-        <v>571.428</v>
+        <v>455.216</v>
       </c>
       <c r="W176" s="49" t="n">
         <f aca="false">W82*założenia!$C$6</f>
@@ -39640,7 +39639,7 @@
       </c>
       <c r="C178" s="49" t="n">
         <f aca="false">SUM(D178:Z178)</f>
-        <v>131274.724841901</v>
+        <v>131929.555978221</v>
       </c>
       <c r="D178" s="49" t="n">
         <f aca="false">D84*założenia!$C$7</f>
@@ -39720,19 +39719,19 @@
       </c>
       <c r="W178" s="49" t="n">
         <f aca="false">W84*założenia!$C$7</f>
-        <v>32818.6812104754</v>
+        <v>32982.3889945554</v>
       </c>
       <c r="X178" s="49" t="n">
         <f aca="false">X84*założenia!$C$7</f>
-        <v>32818.6812104754</v>
+        <v>32982.3889945554</v>
       </c>
       <c r="Y178" s="49" t="n">
         <f aca="false">Y84*założenia!$C$7</f>
-        <v>32818.6812104754</v>
+        <v>32982.3889945554</v>
       </c>
       <c r="Z178" s="49" t="n">
         <f aca="false">Z84*założenia!$C$7</f>
-        <v>32818.6812104754</v>
+        <v>32982.3889945554</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39744,7 +39743,7 @@
       </c>
       <c r="C179" s="49" t="n">
         <f aca="false">SUM(D179:Z179)</f>
-        <v>22345.1381815727</v>
+        <v>22456.6013154265</v>
       </c>
       <c r="D179" s="49" t="n">
         <f aca="false">D85*założenia!$C$7</f>
@@ -39824,19 +39823,19 @@
       </c>
       <c r="W179" s="49" t="n">
         <f aca="false">W85*założenia!$C$7</f>
-        <v>5586.28454539319</v>
+        <v>5614.15032885663</v>
       </c>
       <c r="X179" s="49" t="n">
         <f aca="false">X85*założenia!$C$7</f>
-        <v>5586.28454539319</v>
+        <v>5614.15032885663</v>
       </c>
       <c r="Y179" s="49" t="n">
         <f aca="false">Y85*założenia!$C$7</f>
-        <v>5586.28454539319</v>
+        <v>5614.15032885663</v>
       </c>
       <c r="Z179" s="49" t="n">
         <f aca="false">Z85*założenia!$C$7</f>
-        <v>5586.28454539319</v>
+        <v>5614.15032885663</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39848,7 +39847,7 @@
       </c>
       <c r="C180" s="49" t="n">
         <f aca="false">SUM(D180:Z180)</f>
-        <v>64239.3102971832</v>
+        <v>64559.7520319419</v>
       </c>
       <c r="D180" s="49" t="n">
         <f aca="false">D86*założenia!$C$7</f>
@@ -39928,19 +39927,19 @@
       </c>
       <c r="W180" s="49" t="n">
         <f aca="false">W86*założenia!$C$7</f>
-        <v>16059.8275742958</v>
+        <v>16139.9380079855</v>
       </c>
       <c r="X180" s="49" t="n">
         <f aca="false">X86*założenia!$C$7</f>
-        <v>16059.8275742958</v>
+        <v>16139.9380079855</v>
       </c>
       <c r="Y180" s="49" t="n">
         <f aca="false">Y86*założenia!$C$7</f>
-        <v>16059.8275742958</v>
+        <v>16139.9380079855</v>
       </c>
       <c r="Z180" s="49" t="n">
         <f aca="false">Z86*założenia!$C$7</f>
-        <v>16059.8275742958</v>
+        <v>16139.9380079855</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39952,7 +39951,7 @@
       </c>
       <c r="C181" s="49" t="n">
         <f aca="false">SUM(D181:Z181)</f>
-        <v>48872.5848350942</v>
+        <v>49116.3735027223</v>
       </c>
       <c r="D181" s="49" t="n">
         <f aca="false">D87*założenia!$C$7</f>
@@ -40032,19 +40031,19 @@
       </c>
       <c r="W181" s="49" t="n">
         <f aca="false">W87*założenia!$C$7</f>
-        <v>12218.1462087735</v>
+        <v>12279.0933756806</v>
       </c>
       <c r="X181" s="49" t="n">
         <f aca="false">X87*założenia!$C$7</f>
-        <v>12218.1462087735</v>
+        <v>12279.0933756806</v>
       </c>
       <c r="Y181" s="49" t="n">
         <f aca="false">Y87*założenia!$C$7</f>
-        <v>12218.1462087735</v>
+        <v>12279.0933756806</v>
       </c>
       <c r="Z181" s="49" t="n">
         <f aca="false">Z87*założenia!$C$7</f>
-        <v>12218.1462087735</v>
+        <v>12279.0933756806</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40056,7 +40055,7 @@
       </c>
       <c r="C182" s="49" t="n">
         <f aca="false">SUM(D182:Z182)</f>
-        <v>17629.6742386958</v>
+        <v>17717.6154598911</v>
       </c>
       <c r="D182" s="49" t="n">
         <f aca="false">D88*założenia!$C$7</f>
@@ -40136,19 +40135,19 @@
       </c>
       <c r="W182" s="49" t="n">
         <f aca="false">W88*założenia!$C$7</f>
-        <v>4407.41855967395</v>
+        <v>4429.40386497278</v>
       </c>
       <c r="X182" s="49" t="n">
         <f aca="false">X88*założenia!$C$7</f>
-        <v>4407.41855967395</v>
+        <v>4429.40386497278</v>
       </c>
       <c r="Y182" s="49" t="n">
         <f aca="false">Y88*założenia!$C$7</f>
-        <v>4407.41855967395</v>
+        <v>4429.40386497278</v>
       </c>
       <c r="Z182" s="49" t="n">
         <f aca="false">Z88*założenia!$C$7</f>
-        <v>4407.41855967395</v>
+        <v>4429.40386497278</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40160,7 +40159,7 @@
       </c>
       <c r="C183" s="49" t="n">
         <f aca="false">SUM(D183:Z183)</f>
-        <v>48872.5848350942</v>
+        <v>49116.3735027223</v>
       </c>
       <c r="D183" s="49" t="n">
         <f aca="false">D89*założenia!$C$7</f>
@@ -40240,19 +40239,19 @@
       </c>
       <c r="W183" s="49" t="n">
         <f aca="false">W89*założenia!$C$7</f>
-        <v>12218.1462087735</v>
+        <v>12279.0933756806</v>
       </c>
       <c r="X183" s="49" t="n">
         <f aca="false">X89*założenia!$C$7</f>
-        <v>12218.1462087735</v>
+        <v>12279.0933756806</v>
       </c>
       <c r="Y183" s="49" t="n">
         <f aca="false">Y89*założenia!$C$7</f>
-        <v>12218.1462087735</v>
+        <v>12279.0933756806</v>
       </c>
       <c r="Z183" s="49" t="n">
         <f aca="false">Z89*założenia!$C$7</f>
-        <v>12218.1462087735</v>
+        <v>12279.0933756806</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40264,7 +40263,7 @@
       </c>
       <c r="C184" s="49" t="n">
         <f aca="false">SUM(D184:Z184)</f>
-        <v>1692.55535800898</v>
+        <v>1365.648</v>
       </c>
       <c r="D184" s="49" t="n">
         <f aca="false">D90*założenia!$C$7</f>
@@ -40344,19 +40343,19 @@
       </c>
       <c r="W184" s="49" t="n">
         <f aca="false">W90*założenia!$C$7</f>
-        <v>423.138839502245</v>
+        <v>341.412</v>
       </c>
       <c r="X184" s="49" t="n">
         <f aca="false">X90*założenia!$C$7</f>
-        <v>423.138839502245</v>
+        <v>341.412</v>
       </c>
       <c r="Y184" s="49" t="n">
         <f aca="false">Y90*założenia!$C$7</f>
-        <v>423.138839502245</v>
+        <v>341.412</v>
       </c>
       <c r="Z184" s="49" t="n">
         <f aca="false">Z90*założenia!$C$7</f>
-        <v>423.138839502245</v>
+        <v>341.412</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40368,7 +40367,7 @@
       </c>
       <c r="C185" s="49" t="n">
         <f aca="false">SUM(D185:Z185)</f>
-        <v>46799.2024481508</v>
+        <v>47032.6485662432</v>
       </c>
       <c r="D185" s="49" t="n">
         <f aca="false">D91*założenia!$C$7</f>
@@ -40448,19 +40447,19 @@
       </c>
       <c r="W185" s="49" t="n">
         <f aca="false">W91*założenia!$C$7</f>
-        <v>11699.8006120377</v>
+        <v>11758.1621415608</v>
       </c>
       <c r="X185" s="49" t="n">
         <f aca="false">X91*założenia!$C$7</f>
-        <v>11699.8006120377</v>
+        <v>11758.1621415608</v>
       </c>
       <c r="Y185" s="49" t="n">
         <f aca="false">Y91*założenia!$C$7</f>
-        <v>11699.8006120377</v>
+        <v>11758.1621415608</v>
       </c>
       <c r="Z185" s="49" t="n">
         <f aca="false">Z91*założenia!$C$7</f>
-        <v>11699.8006120377</v>
+        <v>11758.1621415608</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40472,7 +40471,7 @@
       </c>
       <c r="C186" s="49" t="n">
         <f aca="false">SUM(D186:Z186)</f>
-        <v>11658.3329642988</v>
+        <v>11716.4876428312</v>
       </c>
       <c r="D186" s="49" t="n">
         <f aca="false">D92*założenia!$C$7</f>
@@ -40552,19 +40551,19 @@
       </c>
       <c r="W186" s="49" t="n">
         <f aca="false">W92*założenia!$C$7</f>
-        <v>2914.58324107471</v>
+        <v>2929.1219107078</v>
       </c>
       <c r="X186" s="49" t="n">
         <f aca="false">X92*założenia!$C$7</f>
-        <v>2914.58324107471</v>
+        <v>2929.1219107078</v>
       </c>
       <c r="Y186" s="49" t="n">
         <f aca="false">Y92*założenia!$C$7</f>
-        <v>2914.58324107471</v>
+        <v>2929.1219107078</v>
       </c>
       <c r="Z186" s="49" t="n">
         <f aca="false">Z92*założenia!$C$7</f>
-        <v>2914.58324107471</v>
+        <v>2929.1219107078</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40680,7 +40679,7 @@
       </c>
       <c r="C188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,C$150:C$186)</f>
-        <v>808623.11</v>
+        <v>807925.846</v>
       </c>
       <c r="D188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,D$150:D$186)</f>
@@ -40704,27 +40703,27 @@
       </c>
       <c r="I188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,I$150:I$186)</f>
-        <v>134770.518333333</v>
+        <v>134654.307666667</v>
       </c>
       <c r="J188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,J$150:J$186)</f>
-        <v>134770.518333333</v>
+        <v>134654.307666667</v>
       </c>
       <c r="K188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,K$150:K$186)</f>
-        <v>134770.518333333</v>
+        <v>134654.307666667</v>
       </c>
       <c r="L188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,L$150:L$186)</f>
-        <v>134770.518333333</v>
+        <v>134654.307666667</v>
       </c>
       <c r="M188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,M$150:M$186)</f>
-        <v>134770.518333333</v>
+        <v>134654.307666667</v>
       </c>
       <c r="N188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,N$150:N$186)</f>
-        <v>134770.518333333</v>
+        <v>134654.307666667</v>
       </c>
       <c r="O188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,O$150:O$186)</f>
@@ -40784,7 +40783,7 @@
       </c>
       <c r="C189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,C$150:C$186)</f>
-        <v>1111999.424</v>
+        <v>1111069.728</v>
       </c>
       <c r="D189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,D$150:D$186)</f>
@@ -40832,35 +40831,35 @@
       </c>
       <c r="O189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,O$150:O$186)</f>
-        <v>134933.428</v>
+        <v>134817.216</v>
       </c>
       <c r="P189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,P$150:P$186)</f>
-        <v>134933.428</v>
+        <v>134817.216</v>
       </c>
       <c r="Q189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,Q$150:Q$186)</f>
-        <v>140355.428</v>
+        <v>140239.216</v>
       </c>
       <c r="R189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,R$150:R$186)</f>
-        <v>140355.428</v>
+        <v>140239.216</v>
       </c>
       <c r="S189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,S$150:S$186)</f>
-        <v>140355.428</v>
+        <v>140239.216</v>
       </c>
       <c r="T189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,T$150:T$186)</f>
-        <v>140355.428</v>
+        <v>140239.216</v>
       </c>
       <c r="U189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,U$150:U$186)</f>
-        <v>140355.428</v>
+        <v>140239.216</v>
       </c>
       <c r="V189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,V$150:V$186)</f>
-        <v>140355.428</v>
+        <v>140239.216</v>
       </c>
       <c r="W189" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,3,W$150:W$186)</f>
@@ -40888,7 +40887,7 @@
       </c>
       <c r="C190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,C$150:C$186)</f>
-        <v>393384.108</v>
+        <v>395011.056</v>
       </c>
       <c r="D190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,D$150:D$186)</f>
@@ -40968,19 +40967,19 @@
       </c>
       <c r="W190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,W$150:W$186)</f>
-        <v>98346.027</v>
+        <v>98752.764</v>
       </c>
       <c r="X190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,X$150:X$186)</f>
-        <v>98346.027</v>
+        <v>98752.764</v>
       </c>
       <c r="Y190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,Y$150:Y$186)</f>
-        <v>98346.027</v>
+        <v>98752.764</v>
       </c>
       <c r="Z190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,Z$150:Z$186)</f>
-        <v>98346.027</v>
+        <v>98752.764</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40990,7 +40989,7 @@
       <c r="B191" s="40"/>
       <c r="C191" s="63" t="n">
         <f aca="false">SUM(C187:C190)</f>
-        <v>2959946.542</v>
+        <v>2959946.53</v>
       </c>
       <c r="D191" s="63" t="n">
         <f aca="false">SUM(D187:D190)</f>
@@ -41014,75 +41013,75 @@
       </c>
       <c r="I191" s="63" t="n">
         <f aca="false">SUM(I187:I190)</f>
-        <v>134770.518333333</v>
+        <v>134654.307666667</v>
       </c>
       <c r="J191" s="63" t="n">
         <f aca="false">SUM(J187:J190)</f>
-        <v>134770.518333333</v>
+        <v>134654.307666667</v>
       </c>
       <c r="K191" s="63" t="n">
         <f aca="false">SUM(K187:K190)</f>
-        <v>134770.518333333</v>
+        <v>134654.307666667</v>
       </c>
       <c r="L191" s="63" t="n">
         <f aca="false">SUM(L187:L190)</f>
-        <v>134770.518333333</v>
+        <v>134654.307666667</v>
       </c>
       <c r="M191" s="63" t="n">
         <f aca="false">SUM(M187:M190)</f>
-        <v>134770.518333333</v>
+        <v>134654.307666667</v>
       </c>
       <c r="N191" s="63" t="n">
         <f aca="false">SUM(N187:N190)</f>
-        <v>134770.518333333</v>
+        <v>134654.307666667</v>
       </c>
       <c r="O191" s="63" t="n">
         <f aca="false">SUM(O187:O190)</f>
-        <v>134933.428</v>
+        <v>134817.216</v>
       </c>
       <c r="P191" s="63" t="n">
         <f aca="false">SUM(P187:P190)</f>
-        <v>134933.428</v>
+        <v>134817.216</v>
       </c>
       <c r="Q191" s="63" t="n">
         <f aca="false">SUM(Q187:Q190)</f>
-        <v>140355.428</v>
+        <v>140239.216</v>
       </c>
       <c r="R191" s="63" t="n">
         <f aca="false">SUM(R187:R190)</f>
-        <v>140355.428</v>
+        <v>140239.216</v>
       </c>
       <c r="S191" s="63" t="n">
         <f aca="false">SUM(S187:S190)</f>
-        <v>140355.428</v>
+        <v>140239.216</v>
       </c>
       <c r="T191" s="63" t="n">
         <f aca="false">SUM(T187:T190)</f>
-        <v>140355.428</v>
+        <v>140239.216</v>
       </c>
       <c r="U191" s="63" t="n">
         <f aca="false">SUM(U187:U190)</f>
-        <v>140355.428</v>
+        <v>140239.216</v>
       </c>
       <c r="V191" s="63" t="n">
         <f aca="false">SUM(V187:V190)</f>
-        <v>140355.428</v>
+        <v>140239.216</v>
       </c>
       <c r="W191" s="63" t="n">
         <f aca="false">SUM(W187:W190)</f>
-        <v>98346.027</v>
+        <v>98752.764</v>
       </c>
       <c r="X191" s="63" t="n">
         <f aca="false">SUM(X187:X190)</f>
-        <v>98346.027</v>
+        <v>98752.764</v>
       </c>
       <c r="Y191" s="63" t="n">
         <f aca="false">SUM(Y187:Y190)</f>
-        <v>98346.027</v>
+        <v>98752.764</v>
       </c>
       <c r="Z191" s="63" t="n">
         <f aca="false">SUM(Z187:Z190)</f>
-        <v>98346.027</v>
+        <v>98752.764</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -41092,99 +41091,99 @@
       <c r="B192" s="40"/>
       <c r="C192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,C98*$C$191/$C$97)</f>
-        <v>739986.6355</v>
+        <v>739986.6325</v>
       </c>
       <c r="D192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,D98*$C$191/$C$97)</f>
-        <v>31446.1064211191</v>
+        <v>31440.5903780996</v>
       </c>
       <c r="E192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,E98*$C$191/$C$97)</f>
-        <v>31446.1064211191</v>
+        <v>31440.5903780996</v>
       </c>
       <c r="F192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,F98*$C$191/$C$97)</f>
-        <v>31446.1064211191</v>
+        <v>31440.5903780996</v>
       </c>
       <c r="G192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,G98*$C$191/$C$97)</f>
-        <v>30148.1089933264</v>
+        <v>30142.8206353995</v>
       </c>
       <c r="H192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,H98*$C$191/$C$97)</f>
-        <v>30148.1089933264</v>
+        <v>30142.8206353995</v>
       </c>
       <c r="I192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,I98*$C$191/$C$97)</f>
-        <v>32263.3383331102</v>
+        <v>32229.8632895799</v>
       </c>
       <c r="J192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,J98*$C$191/$C$97)</f>
-        <v>32263.3383331102</v>
+        <v>32229.8632895799</v>
       </c>
       <c r="K192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,K98*$C$191/$C$97)</f>
-        <v>32263.3383331102</v>
+        <v>32229.8632895799</v>
       </c>
       <c r="L192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,L98*$C$191/$C$97)</f>
-        <v>32263.3383331102</v>
+        <v>32229.8632895799</v>
       </c>
       <c r="M192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,M98*$C$191/$C$97)</f>
-        <v>32263.3383331102</v>
+        <v>32229.8632895799</v>
       </c>
       <c r="N192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,N98*$C$191/$C$97)</f>
-        <v>32263.3383331102</v>
+        <v>32229.8632895799</v>
       </c>
       <c r="O192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,O98*$C$191/$C$97)</f>
-        <v>32302.3369938084</v>
+        <v>32268.855109422</v>
       </c>
       <c r="P192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,P98*$C$191/$C$97)</f>
-        <v>32302.3369938084</v>
+        <v>32268.855109422</v>
       </c>
       <c r="Q192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,Q98*$C$191/$C$97)</f>
-        <v>33600.3346343962</v>
+        <v>33566.62506488</v>
       </c>
       <c r="R192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,R98*$C$191/$C$97)</f>
-        <v>33600.3346343962</v>
+        <v>33566.62506488</v>
       </c>
       <c r="S192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,S98*$C$191/$C$97)</f>
-        <v>33600.3346343962</v>
+        <v>33566.62506488</v>
       </c>
       <c r="T192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,T98*$C$191/$C$97)</f>
-        <v>33600.3346343962</v>
+        <v>33566.62506488</v>
       </c>
       <c r="U192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,U98*$C$191/$C$97)</f>
-        <v>33600.3346343962</v>
+        <v>33566.62506488</v>
       </c>
       <c r="V192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,V98*$C$191/$C$97)</f>
-        <v>33600.3346343962</v>
+        <v>33566.62506488</v>
       </c>
       <c r="W192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,W98*$C$191/$C$97)</f>
-        <v>31391.3466143337</v>
+        <v>31515.6449373246</v>
       </c>
       <c r="X192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,X98*$C$191/$C$97)</f>
-        <v>31391.3466143337</v>
+        <v>31515.6449373246</v>
       </c>
       <c r="Y192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,Y98*$C$191/$C$97)</f>
-        <v>31391.3466143337</v>
+        <v>31515.6449373246</v>
       </c>
       <c r="Z192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,Z98*$C$191/$C$97)</f>
-        <v>31391.3466143337</v>
+        <v>31515.6449373246</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -41194,99 +41193,99 @@
       <c r="B193" s="40"/>
       <c r="C193" s="63" t="n">
         <f aca="false">C191+C192</f>
-        <v>3699933.1775</v>
+        <v>3699933.1625</v>
       </c>
       <c r="D193" s="63" t="n">
         <f aca="false">D191+D192</f>
-        <v>162802.885976675</v>
+        <v>162797.369933655</v>
       </c>
       <c r="E193" s="63" t="n">
         <f aca="false">E191+E192</f>
-        <v>162802.885976675</v>
+        <v>162797.369933655</v>
       </c>
       <c r="F193" s="63" t="n">
         <f aca="false">F191+F192</f>
-        <v>162802.885976675</v>
+        <v>162797.369933655</v>
       </c>
       <c r="G193" s="63" t="n">
         <f aca="false">G191+G192</f>
-        <v>156082.889659993</v>
+        <v>156077.601302066</v>
       </c>
       <c r="H193" s="63" t="n">
         <f aca="false">H191+H192</f>
-        <v>156082.889659993</v>
+        <v>156077.601302066</v>
       </c>
       <c r="I193" s="63" t="n">
         <f aca="false">I191+I192</f>
-        <v>167033.856666444</v>
+        <v>166884.170956247</v>
       </c>
       <c r="J193" s="63" t="n">
         <f aca="false">J191+J192</f>
-        <v>167033.856666444</v>
+        <v>166884.170956247</v>
       </c>
       <c r="K193" s="63" t="n">
         <f aca="false">K191+K192</f>
-        <v>167033.856666444</v>
+        <v>166884.170956247</v>
       </c>
       <c r="L193" s="63" t="n">
         <f aca="false">L191+L192</f>
-        <v>167033.856666444</v>
+        <v>166884.170956247</v>
       </c>
       <c r="M193" s="63" t="n">
         <f aca="false">M191+M192</f>
-        <v>167033.856666444</v>
+        <v>166884.170956247</v>
       </c>
       <c r="N193" s="63" t="n">
         <f aca="false">N191+N192</f>
-        <v>167033.856666444</v>
+        <v>166884.170956247</v>
       </c>
       <c r="O193" s="63" t="n">
         <f aca="false">O191+O192</f>
-        <v>167235.764993808</v>
+        <v>167086.071109422</v>
       </c>
       <c r="P193" s="63" t="n">
         <f aca="false">P191+P192</f>
-        <v>167235.764993808</v>
+        <v>167086.071109422</v>
       </c>
       <c r="Q193" s="63" t="n">
         <f aca="false">Q191+Q192</f>
-        <v>173955.762634396</v>
+        <v>173805.84106488</v>
       </c>
       <c r="R193" s="63" t="n">
         <f aca="false">R191+R192</f>
-        <v>173955.762634396</v>
+        <v>173805.84106488</v>
       </c>
       <c r="S193" s="63" t="n">
         <f aca="false">S191+S192</f>
-        <v>173955.762634396</v>
+        <v>173805.84106488</v>
       </c>
       <c r="T193" s="63" t="n">
         <f aca="false">T191+T192</f>
-        <v>173955.762634396</v>
+        <v>173805.84106488</v>
       </c>
       <c r="U193" s="63" t="n">
         <f aca="false">U191+U192</f>
-        <v>173955.762634396</v>
+        <v>173805.84106488</v>
       </c>
       <c r="V193" s="63" t="n">
         <f aca="false">V191+V192</f>
-        <v>173955.762634396</v>
+        <v>173805.84106488</v>
       </c>
       <c r="W193" s="63" t="n">
         <f aca="false">W191+W192</f>
-        <v>129737.373614334</v>
+        <v>130268.408937325</v>
       </c>
       <c r="X193" s="63" t="n">
         <f aca="false">X191+X192</f>
-        <v>129737.373614334</v>
+        <v>130268.408937325</v>
       </c>
       <c r="Y193" s="63" t="n">
         <f aca="false">Y191+Y192</f>
-        <v>129737.373614334</v>
+        <v>130268.408937325</v>
       </c>
       <c r="Z193" s="63" t="n">
         <f aca="false">Z191+Z192</f>
-        <v>129737.373614334</v>
+        <v>130268.408937325</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -41297,95 +41296,95 @@
       <c r="C194" s="63"/>
       <c r="D194" s="63" t="n">
         <f aca="false">D193</f>
-        <v>162802.885976675</v>
+        <v>162797.369933655</v>
       </c>
       <c r="E194" s="63" t="n">
         <f aca="false">D194+E193</f>
-        <v>325605.771953349</v>
+        <v>325594.73986731</v>
       </c>
       <c r="F194" s="63" t="n">
         <f aca="false">E194+F193</f>
-        <v>488408.657930024</v>
+        <v>488392.109800965</v>
       </c>
       <c r="G194" s="63" t="n">
         <f aca="false">F194+G193</f>
-        <v>644491.547590017</v>
+        <v>644469.711103032</v>
       </c>
       <c r="H194" s="63" t="n">
         <f aca="false">G194+H193</f>
-        <v>800574.43725001</v>
+        <v>800547.312405098</v>
       </c>
       <c r="I194" s="63" t="n">
         <f aca="false">H194+I193</f>
-        <v>967608.293916454</v>
+        <v>967431.483361344</v>
       </c>
       <c r="J194" s="63" t="n">
         <f aca="false">I194+J193</f>
-        <v>1134642.1505829</v>
+        <v>1134315.65431759</v>
       </c>
       <c r="K194" s="63" t="n">
         <f aca="false">J194+K193</f>
-        <v>1301676.00724934</v>
+        <v>1301199.82527384</v>
       </c>
       <c r="L194" s="63" t="n">
         <f aca="false">K194+L193</f>
-        <v>1468709.86391578</v>
+        <v>1468083.99623008</v>
       </c>
       <c r="M194" s="63" t="n">
         <f aca="false">L194+M193</f>
-        <v>1635743.72058223</v>
+        <v>1634968.16718633</v>
       </c>
       <c r="N194" s="63" t="n">
         <f aca="false">M194+N193</f>
-        <v>1802777.57724867</v>
+        <v>1801852.33814258</v>
       </c>
       <c r="O194" s="63" t="n">
         <f aca="false">N194+O193</f>
-        <v>1970013.34224248</v>
+        <v>1968938.409252</v>
       </c>
       <c r="P194" s="63" t="n">
         <f aca="false">O194+P193</f>
-        <v>2137249.10723629</v>
+        <v>2136024.48036142</v>
       </c>
       <c r="Q194" s="63" t="n">
         <f aca="false">P194+Q193</f>
-        <v>2311204.86987068</v>
+        <v>2309830.3214263</v>
       </c>
       <c r="R194" s="63" t="n">
         <f aca="false">Q194+R193</f>
-        <v>2485160.63250508</v>
+        <v>2483636.16249118</v>
       </c>
       <c r="S194" s="63" t="n">
         <f aca="false">R194+S193</f>
-        <v>2659116.39513948</v>
+        <v>2657442.00355606</v>
       </c>
       <c r="T194" s="63" t="n">
         <f aca="false">S194+T193</f>
-        <v>2833072.15777387</v>
+        <v>2831247.84462094</v>
       </c>
       <c r="U194" s="63" t="n">
         <f aca="false">T194+U193</f>
-        <v>3007027.92040827</v>
+        <v>3005053.68568582</v>
       </c>
       <c r="V194" s="63" t="n">
         <f aca="false">U194+V193</f>
-        <v>3180983.68304266</v>
+        <v>3178859.5267507</v>
       </c>
       <c r="W194" s="63" t="n">
         <f aca="false">V194+W193</f>
-        <v>3310721.056657</v>
+        <v>3309127.93568803</v>
       </c>
       <c r="X194" s="63" t="n">
         <f aca="false">W194+X193</f>
-        <v>3440458.43027133</v>
+        <v>3439396.34462535</v>
       </c>
       <c r="Y194" s="63" t="n">
         <f aca="false">X194+Y193</f>
-        <v>3570195.80388567</v>
+        <v>3569664.75356268</v>
       </c>
       <c r="Z194" s="63" t="n">
         <f aca="false">Y194+Z193</f>
-        <v>3699933.1775</v>
+        <v>3699933.1625</v>
       </c>
     </row>
   </sheetData>
@@ -42095,15 +42094,15 @@
       </c>
       <c r="E13" s="71" t="n">
         <f aca="false">SUM(E14:E23)</f>
-        <v>1010778.92</v>
+        <v>1009907.33</v>
       </c>
       <c r="F13" s="71" t="n">
         <f aca="false">SUM(F14:F23)</f>
-        <v>1010778.92</v>
+        <v>1009907.33</v>
       </c>
       <c r="G13" s="71" t="n">
         <f aca="false">SUM(G14:G23)</f>
-        <v>808623.11</v>
+        <v>807925.85</v>
       </c>
       <c r="H13" s="63"/>
       <c r="I13" s="71" t="n">
@@ -42120,15 +42119,15 @@
       </c>
       <c r="L13" s="71" t="n">
         <f aca="false">E13-I13</f>
-        <v>-216156.79</v>
+        <v>-217028.38</v>
       </c>
       <c r="M13" s="71" t="n">
         <f aca="false">F13-J13</f>
-        <v>-193156.79</v>
+        <v>-194028.38</v>
       </c>
       <c r="N13" s="71" t="n">
         <f aca="false">G13-K13</f>
-        <v>-154525.45</v>
+        <v>-155222.71</v>
       </c>
       <c r="O13" s="40"/>
       <c r="P13" s="70" t="str">
@@ -42625,16 +42624,16 @@
         <v>1820.88</v>
       </c>
       <c r="E22" s="74" t="n">
-        <f aca="false">I22</f>
-        <v>4285.71</v>
+        <f aca="false">F22</f>
+        <v>3414.12</v>
       </c>
       <c r="F22" s="74" t="n">
-        <f aca="false">J22</f>
-        <v>4285.71</v>
+        <f aca="false">ROUND('budżet po miesiącach'!$C$73,2)</f>
+        <v>3414.12</v>
       </c>
       <c r="G22" s="74" t="n">
-        <f aca="false">K22</f>
-        <v>3428.56</v>
+        <f aca="false">ROUND('budżet po miesiącach'!$C$167,2)</f>
+        <v>2731.3</v>
       </c>
       <c r="H22" s="49"/>
       <c r="I22" s="73" t="n">
@@ -42651,15 +42650,15 @@
       </c>
       <c r="L22" s="73" t="n">
         <f aca="false">E22-I22</f>
-        <v>0</v>
+        <v>-871.59</v>
       </c>
       <c r="M22" s="73" t="n">
         <f aca="false">F22-J22</f>
-        <v>0</v>
+        <v>-871.59</v>
       </c>
       <c r="N22" s="73" t="n">
         <f aca="false">G22-K22</f>
-        <v>0</v>
+        <v>-697.26</v>
       </c>
       <c r="O22" s="41"/>
       <c r="P22" s="72" t="str">
@@ -42744,15 +42743,15 @@
       </c>
       <c r="E24" s="71" t="n">
         <f aca="false">SUM(E25:E33)</f>
-        <v>1389999.28</v>
+        <v>1388837.16</v>
       </c>
       <c r="F24" s="71" t="n">
         <f aca="false">SUM(F25:F33)</f>
-        <v>1389999.28</v>
+        <v>1388837.16</v>
       </c>
       <c r="G24" s="71" t="n">
         <f aca="false">SUM(G25:G33)</f>
-        <v>1111999.42</v>
+        <v>1111069.73</v>
       </c>
       <c r="H24" s="63"/>
       <c r="I24" s="71" t="n">
@@ -42769,15 +42768,15 @@
       </c>
       <c r="L24" s="71" t="n">
         <f aca="false">E24-I24</f>
-        <v>286063.57</v>
+        <v>284901.45</v>
       </c>
       <c r="M24" s="71" t="n">
         <f aca="false">F24-J24</f>
-        <v>286063.57</v>
+        <v>284901.45</v>
       </c>
       <c r="N24" s="71" t="n">
         <f aca="false">G24-K24</f>
-        <v>228850.86</v>
+        <v>227921.17</v>
       </c>
       <c r="O24" s="40"/>
       <c r="P24" s="70" t="str">
@@ -43216,15 +43215,15 @@
       </c>
       <c r="E32" s="74" t="n">
         <f aca="false">F32</f>
-        <v>5714.28</v>
+        <v>4552.16</v>
       </c>
       <c r="F32" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$82,2)</f>
-        <v>5714.28</v>
+        <v>4552.16</v>
       </c>
       <c r="G32" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$176,2)</f>
-        <v>4571.42</v>
+        <v>3641.73</v>
       </c>
       <c r="H32" s="49"/>
       <c r="I32" s="73" t="n">
@@ -43241,15 +43240,15 @@
       </c>
       <c r="L32" s="73" t="n">
         <f aca="false">E32-I32</f>
-        <v>1428.57</v>
+        <v>266.45</v>
       </c>
       <c r="M32" s="73" t="n">
         <f aca="false">F32-J32</f>
-        <v>1428.57</v>
+        <v>266.45</v>
       </c>
       <c r="N32" s="73" t="n">
         <f aca="false">G32-K32</f>
-        <v>1142.86</v>
+        <v>213.17</v>
       </c>
       <c r="O32" s="41"/>
       <c r="P32" s="72" t="str">
@@ -43334,15 +43333,15 @@
       </c>
       <c r="E34" s="71" t="n">
         <f aca="false">SUM(E35:E43)</f>
-        <v>655640.19</v>
+        <v>658351.76</v>
       </c>
       <c r="F34" s="71" t="n">
         <f aca="false">SUM(F35:F43)</f>
-        <v>655640.19</v>
+        <v>658351.76</v>
       </c>
       <c r="G34" s="71" t="n">
         <f aca="false">SUM(G35:G43)</f>
-        <v>393384.11</v>
+        <v>395011.06</v>
       </c>
       <c r="H34" s="63"/>
       <c r="I34" s="71" t="n">
@@ -43359,15 +43358,15 @@
       </c>
       <c r="L34" s="71" t="n">
         <f aca="false">E34-I34</f>
-        <v>-42596.95</v>
+        <v>-39885.38</v>
       </c>
       <c r="M34" s="71" t="n">
         <f aca="false">F34-J34</f>
-        <v>-42596.95</v>
+        <v>-39885.38</v>
       </c>
       <c r="N34" s="71" t="n">
         <f aca="false">G34-K34</f>
-        <v>-25558.17</v>
+        <v>-23931.22</v>
       </c>
       <c r="O34" s="40"/>
       <c r="P34" s="70" t="str">
@@ -43393,15 +43392,15 @@
       </c>
       <c r="E35" s="74" t="n">
         <f aca="false">F35</f>
-        <v>218791.21</v>
+        <v>219882.59</v>
       </c>
       <c r="F35" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$84,2)</f>
-        <v>218791.21</v>
+        <v>219882.59</v>
       </c>
       <c r="G35" s="74" t="n">
         <f aca="false">ROUND(założenia!$C$13-(G4+G5+G6+G7+G8+G9+G10+G11+G12+G14+G15+G16+G17+G18+G19+G20+G21+G22+G23+G25+G26+G27+G28+G29+G30+G31+G32+G33+G36+G37+G38+G39+G40+G41+G42+G43),2)</f>
-        <v>131274.74</v>
+        <v>131929.56</v>
       </c>
       <c r="H35" s="49"/>
       <c r="I35" s="73" t="n">
@@ -43418,15 +43417,15 @@
       </c>
       <c r="L35" s="73" t="n">
         <f aca="false">E35-I35</f>
-        <v>-2808.79000000001</v>
+        <v>-1717.41</v>
       </c>
       <c r="M35" s="73" t="n">
         <f aca="false">F35-J35</f>
-        <v>-2808.79000000001</v>
+        <v>-1717.41</v>
       </c>
       <c r="N35" s="73" t="n">
         <f aca="false">G35-K35</f>
-        <v>-1685.26000000001</v>
+        <v>-1030.44</v>
       </c>
       <c r="O35" s="41"/>
       <c r="P35" s="72" t="str">
@@ -43455,15 +43454,15 @@
       </c>
       <c r="E36" s="74" t="n">
         <f aca="false">F36</f>
-        <v>37241.9</v>
+        <v>37427.67</v>
       </c>
       <c r="F36" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$85,2)</f>
-        <v>37241.9</v>
+        <v>37427.67</v>
       </c>
       <c r="G36" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$179,2)</f>
-        <v>22345.14</v>
+        <v>22456.6</v>
       </c>
       <c r="H36" s="49"/>
       <c r="I36" s="73" t="n">
@@ -43480,15 +43479,15 @@
       </c>
       <c r="L36" s="73" t="n">
         <f aca="false">E36-I36</f>
-        <v>-478.099999999999</v>
+        <v>-292.330000000002</v>
       </c>
       <c r="M36" s="73" t="n">
         <f aca="false">F36-J36</f>
-        <v>-478.099999999999</v>
+        <v>-292.330000000002</v>
       </c>
       <c r="N36" s="73" t="n">
         <f aca="false">G36-K36</f>
-        <v>-286.860000000001</v>
+        <v>-175.400000000001</v>
       </c>
       <c r="O36" s="41"/>
       <c r="P36" s="72" t="str">
@@ -43514,15 +43513,15 @@
       </c>
       <c r="E37" s="74" t="n">
         <f aca="false">F37</f>
-        <v>107065.52</v>
+        <v>107599.59</v>
       </c>
       <c r="F37" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$86,2)</f>
-        <v>107065.52</v>
+        <v>107599.59</v>
       </c>
       <c r="G37" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$180,2)</f>
-        <v>64239.31</v>
+        <v>64559.75</v>
       </c>
       <c r="H37" s="49"/>
       <c r="I37" s="73" t="n">
@@ -43539,15 +43538,15 @@
       </c>
       <c r="L37" s="73" t="n">
         <f aca="false">E37-I37</f>
-        <v>-1374.48</v>
+        <v>-840.410000000004</v>
       </c>
       <c r="M37" s="73" t="n">
         <f aca="false">F37-J37</f>
-        <v>-1374.48</v>
+        <v>-840.410000000004</v>
       </c>
       <c r="N37" s="73" t="n">
         <f aca="false">G37-K37</f>
-        <v>-824.690000000002</v>
+        <v>-504.25</v>
       </c>
       <c r="O37" s="41"/>
       <c r="P37" s="72" t="str">
@@ -43573,15 +43572,15 @@
       </c>
       <c r="E38" s="74" t="n">
         <f aca="false">F38</f>
-        <v>81454.31</v>
+        <v>81860.62</v>
       </c>
       <c r="F38" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$87,2)</f>
-        <v>81454.31</v>
+        <v>81860.62</v>
       </c>
       <c r="G38" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$181,2)</f>
-        <v>48872.58</v>
+        <v>49116.37</v>
       </c>
       <c r="H38" s="49"/>
       <c r="I38" s="73" t="n">
@@ -43598,15 +43597,15 @@
       </c>
       <c r="L38" s="73" t="n">
         <f aca="false">E38-I38</f>
-        <v>-1045.69</v>
+        <v>-639.380000000005</v>
       </c>
       <c r="M38" s="73" t="n">
         <f aca="false">F38-J38</f>
-        <v>-1045.69</v>
+        <v>-639.380000000005</v>
       </c>
       <c r="N38" s="73" t="n">
         <f aca="false">G38-K38</f>
-        <v>-627.419999999998</v>
+        <v>-383.629999999997</v>
       </c>
       <c r="O38" s="41"/>
       <c r="P38" s="72" t="str">
@@ -43632,15 +43631,15 @@
       </c>
       <c r="E39" s="74" t="n">
         <f aca="false">F39</f>
-        <v>29382.79</v>
+        <v>29529.36</v>
       </c>
       <c r="F39" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$88,2)</f>
-        <v>29382.79</v>
+        <v>29529.36</v>
       </c>
       <c r="G39" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$182,2)</f>
-        <v>17629.67</v>
+        <v>17717.62</v>
       </c>
       <c r="H39" s="49"/>
       <c r="I39" s="73" t="n">
@@ -43657,15 +43656,15 @@
       </c>
       <c r="L39" s="73" t="n">
         <f aca="false">E39-I39</f>
-        <v>-377.209999999999</v>
+        <v>-230.639999999999</v>
       </c>
       <c r="M39" s="73" t="n">
         <f aca="false">F39-J39</f>
-        <v>-377.209999999999</v>
+        <v>-230.639999999999</v>
       </c>
       <c r="N39" s="73" t="n">
         <f aca="false">G39-K39</f>
-        <v>-226.330000000002</v>
+        <v>-138.380000000001</v>
       </c>
       <c r="O39" s="41"/>
       <c r="P39" s="72" t="str">
@@ -43691,15 +43690,15 @@
       </c>
       <c r="E40" s="74" t="n">
         <f aca="false">F40</f>
-        <v>81454.31</v>
+        <v>81860.62</v>
       </c>
       <c r="F40" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$89,2)</f>
-        <v>81454.31</v>
+        <v>81860.62</v>
       </c>
       <c r="G40" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$183,2)</f>
-        <v>48872.58</v>
+        <v>49116.37</v>
       </c>
       <c r="H40" s="49"/>
       <c r="I40" s="73" t="n">
@@ -43716,15 +43715,15 @@
       </c>
       <c r="L40" s="73" t="n">
         <f aca="false">E40-I40</f>
-        <v>-1045.69</v>
+        <v>-639.380000000005</v>
       </c>
       <c r="M40" s="73" t="n">
         <f aca="false">F40-J40</f>
-        <v>-1045.69</v>
+        <v>-639.380000000005</v>
       </c>
       <c r="N40" s="73" t="n">
         <f aca="false">G40-K40</f>
-        <v>-627.419999999998</v>
+        <v>-383.629999999997</v>
       </c>
       <c r="O40" s="41"/>
       <c r="P40" s="72" t="str">
@@ -43750,15 +43749,15 @@
       </c>
       <c r="E41" s="74" t="n">
         <f aca="false">F41</f>
-        <v>2820.93</v>
+        <v>2276.08</v>
       </c>
       <c r="F41" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$90,2)</f>
-        <v>2820.93</v>
+        <v>2276.08</v>
       </c>
       <c r="G41" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$184,2)</f>
-        <v>1692.56</v>
+        <v>1365.65</v>
       </c>
       <c r="H41" s="49"/>
       <c r="I41" s="73" t="n">
@@ -43775,15 +43774,15 @@
       </c>
       <c r="L41" s="73" t="n">
         <f aca="false">E41-I41</f>
-        <v>-36.21</v>
+        <v>-581.06</v>
       </c>
       <c r="M41" s="73" t="n">
         <f aca="false">F41-J41</f>
-        <v>-36.21</v>
+        <v>-581.06</v>
       </c>
       <c r="N41" s="73" t="n">
         <f aca="false">G41-K41</f>
-        <v>-21.72</v>
+        <v>-348.63</v>
       </c>
       <c r="O41" s="41"/>
       <c r="P41" s="72" t="str">
@@ -43809,15 +43808,15 @@
       </c>
       <c r="E42" s="74" t="n">
         <f aca="false">F42</f>
-        <v>77998.67</v>
+        <v>78387.75</v>
       </c>
       <c r="F42" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$91,2)</f>
-        <v>77998.67</v>
+        <v>78387.75</v>
       </c>
       <c r="G42" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$185,2)</f>
-        <v>46799.2</v>
+        <v>47032.65</v>
       </c>
       <c r="H42" s="49"/>
       <c r="I42" s="73" t="n">
@@ -43834,15 +43833,15 @@
       </c>
       <c r="L42" s="73" t="n">
         <f aca="false">E42-I42</f>
-        <v>-1001.33</v>
+        <v>-612.25</v>
       </c>
       <c r="M42" s="73" t="n">
         <f aca="false">F42-J42</f>
-        <v>-1001.33</v>
+        <v>-612.25</v>
       </c>
       <c r="N42" s="73" t="n">
         <f aca="false">G42-K42</f>
-        <v>-600.800000000003</v>
+        <v>-367.349999999999</v>
       </c>
       <c r="O42" s="41"/>
       <c r="P42" s="72" t="str">
@@ -43868,15 +43867,15 @@
       </c>
       <c r="E43" s="74" t="n">
         <f aca="false">F43</f>
-        <v>19430.55</v>
+        <v>19527.48</v>
       </c>
       <c r="F43" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$92,2)</f>
-        <v>19430.55</v>
+        <v>19527.48</v>
       </c>
       <c r="G43" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$186,2)</f>
-        <v>11658.33</v>
+        <v>11716.49</v>
       </c>
       <c r="H43" s="49"/>
       <c r="I43" s="73" t="n">
@@ -43893,15 +43892,15 @@
       </c>
       <c r="L43" s="73" t="n">
         <f aca="false">E43-I43</f>
-        <v>-34429.45</v>
+        <v>-34332.52</v>
       </c>
       <c r="M43" s="73" t="n">
         <f aca="false">F43-J43</f>
-        <v>-34429.45</v>
+        <v>-34332.52</v>
       </c>
       <c r="N43" s="73" t="n">
         <f aca="false">G43-K43</f>
-        <v>-20657.67</v>
+        <v>-20599.51</v>
       </c>
       <c r="O43" s="41"/>
       <c r="P43" s="72" t="str">
@@ -43974,11 +43973,11 @@
       </c>
       <c r="E48" s="73" t="n">
         <f aca="false">E3+E13+E24+E34</f>
-        <v>3863843.26</v>
+        <v>3864521.12</v>
       </c>
       <c r="F48" s="73" t="n">
         <f aca="false">F3+F13+F24+F34</f>
-        <v>3863843.26</v>
+        <v>3864521.12</v>
       </c>
       <c r="G48" s="73" t="n">
         <f aca="false">G3+G13+G24+G34</f>
@@ -43999,11 +43998,11 @@
       </c>
       <c r="L48" s="73" t="n">
         <f aca="false">E48-I48</f>
-        <v>-33649.23</v>
+        <v>-32971.3700000001</v>
       </c>
       <c r="M48" s="73" t="n">
         <f aca="false">F48-J48</f>
-        <v>-10649.23</v>
+        <v>-9971.37000000011</v>
       </c>
       <c r="N48" s="73" t="n">
         <f aca="false">G48-K48</f>
@@ -44028,11 +44027,11 @@
       </c>
       <c r="E49" s="73" t="n">
         <f aca="false">F49</f>
-        <v>965960.82</v>
+        <v>966130.28</v>
       </c>
       <c r="F49" s="73" t="n">
         <f aca="false">ROUND(0.25*F48,2)</f>
-        <v>965960.82</v>
+        <v>966130.28</v>
       </c>
       <c r="G49" s="73" t="n">
         <f aca="false">ROUNDDOWN(F49*G48/F48,2)</f>
@@ -44053,11 +44052,11 @@
       </c>
       <c r="L49" s="73" t="n">
         <f aca="false">E49-I49</f>
-        <v>-2662.30000000005</v>
+        <v>-2492.83999999997</v>
       </c>
       <c r="M49" s="73" t="n">
         <f aca="false">F49-J49</f>
-        <v>-2662.30000000005</v>
+        <v>-2492.83999999997</v>
       </c>
       <c r="N49" s="73" t="n">
         <f aca="false">G49-K49</f>
@@ -44082,11 +44081,11 @@
       </c>
       <c r="E50" s="77" t="n">
         <f aca="false">E48+E49</f>
-        <v>4829804.08</v>
+        <v>4830651.4</v>
       </c>
       <c r="F50" s="77" t="n">
         <f aca="false">F48+F49</f>
-        <v>4829804.08</v>
+        <v>4830651.4</v>
       </c>
       <c r="G50" s="77" t="n">
         <f aca="false">G48+G49</f>
@@ -44107,11 +44106,11 @@
       </c>
       <c r="L50" s="77" t="n">
         <f aca="false">E50-I50</f>
-        <v>-36311.5300000003</v>
+        <v>-35464.21</v>
       </c>
       <c r="M50" s="77" t="n">
         <f aca="false">F50-J50</f>
-        <v>-13311.5300000003</v>
+        <v>-12464.21</v>
       </c>
       <c r="N50" s="77" t="n">
         <f aca="false">G50-K50</f>
@@ -44152,7 +44151,7 @@
       <c r="E52" s="73"/>
       <c r="F52" s="73" t="n">
         <f aca="false">ROUND(F50-F51,2)</f>
-        <v>-13311.53</v>
+        <v>-12464.21</v>
       </c>
       <c r="G52" s="73" t="n">
         <f aca="false">ROUND(G50-G51,2)</f>

</xml_diff>

<commit_message>
Licence 630.08 in Z2; Z4 differences only in laptop amortization and graphic designer
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3QuwGR9tgiXrdWSSrWcuu
</commit_message>
<xml_diff>
--- a/Wniosek_o_platnosc_str26-34.xlsx
+++ b/Wniosek_o_platnosc_str26-34.xlsx
@@ -504,10 +504,10 @@
     <t xml:space="preserve">Cel dofinansowanie – koszty bezpośrednie (PDF)</t>
   </si>
   <si>
-    <t xml:space="preserve">Licencje – kwalifikowalne po zmianie (przyjęto 0: dofinansowanie nie może wzrosnąć)</t>
+    <t xml:space="preserve">Licencje (Z2) – kwalifikowalne po zmianie (podane przez użytkownika)</t>
   </si>
   <si>
-    <t xml:space="preserve">Z4 – kwalifikowalne osobowe (stawka × etat, bez amortyzacji), przed obniżeniem</t>
+    <t xml:space="preserve">Z4 – Grafik-Ilustrator (poz. 4.9): kwalifikowalne planowane (Suska), przed obniżeniem</t>
   </si>
   <si>
     <t xml:space="preserve">Z3 – dofinansowanie (80% kosztów kwalifikowalnych)</t>
@@ -516,10 +516,10 @@
     <t xml:space="preserve">Dofinansowanie Z1+Z2 (wykonanie, poz. 2.9 wg stawki, licencje) + Z3</t>
   </si>
   <si>
-    <t xml:space="preserve">Dofinansowanie dostępne dla osobowych Z4 = cel D bezpośrednie − C17 − dofinansowanie amortyzacji Z4</t>
+    <t xml:space="preserve">Dofinansowanie dostępne dla poz. 4.9 = cel D bezpośrednie − C17 − dofinansowanie reszty Z4 (bez zmian vs pierwotny budżet, amortyzacja wg stawki)</t>
   </si>
   <si>
-    <t xml:space="preserve">Współczynnik obniżenia osobowych kosztów kwalifikowalnych Z4 (= C15 × C19, tak by D = 60% mieściło się w C18; amortyzacja bez obniżenia)</t>
+    <t xml:space="preserve">Współczynnik obniżenia kosztów poz. 4.9 (= C15 × C19, tak by D = 60% mieściło się w C18)</t>
   </si>
   <si>
     <t xml:space="preserve">TEST: koszt wakatu grafika w Z4 (stawka × miesiące Z4), gdyby został</t>
@@ -531,7 +531,7 @@
     <t xml:space="preserve">TEST: wniosek</t>
   </si>
   <si>
-    <t xml:space="preserve">Z4 – kwalifikowalne osobowe po obniżeniu</t>
+    <t xml:space="preserve">Z4 – poz. 4.9 Grafik: kwalifikowalne po obniżeniu</t>
   </si>
   <si>
     <t xml:space="preserve">KONTROLE</t>
@@ -582,7 +582,7 @@
     <t xml:space="preserve">3. Z1 i Z2 w nowym budżecie = wydatki narastająco (ogółem, kwalifikowalne, dofinansowanie) per pozycja, z wyjątkiem poz. 2.9 (amortyzacja laptopów w Z2) – liczona wg stawki 569,02 zł/mies. × 6 m-cy. Poz. 2.1 (Ekspert AI, Z2): przyjęto 332 400 zł kwalifikowalnych / 265 920 zł dofinansowania (PARP wstrzymał wypłatę, budżet nie jest tracony).</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Licencje (Z2): wykonanie 0, więc całość uwalnia środki. Po zmianie 0 zł (C14) – przy stałych intensywnościach budżet nie mieści ani reszty na licencjach, ani wakatu grafika w Z4.</t>
+    <t xml:space="preserve">4. Licencje (Z2): w nowym budżecie zostaje 630,08 zł kwalifikowalnych (podane przez użytkownika), dofinansowanie 80% = 504,06 zł, ogółem z VAT 775,00 zł. Brakująca wartość kwalifikowalnych jest zdejmowana z Z4 (poz. 4.9 Grafik).</t>
   </si>
   <si>
     <t xml:space="preserve">5. Z3 i Z4 = prognoza: stawka × etat × miesiące (arkusz „plan etatów”). Z3 nie jest przycinane.</t>
@@ -597,13 +597,13 @@
     <t xml:space="preserve">8. Big Data Engineer: 1 etat w Z1–Z3, 0,5 etatu w Z4 (37 720 zł, zgodnie z PDF).</t>
   </si>
   <si>
-    <t xml:space="preserve">9. Grafik-Ilustrator: wakat (8 545 zł/mies.) wyzerowany w całym projekcie, w tym w Z4; zostaje Suska (4 920 zł/mies.). Test w C20:C22 pokazuje, że wakat w Z4 nie mieści się w limicie dofinansowania.</t>
+    <t xml:space="preserve">9. Grafik-Ilustrator: wakat (8 545 zł/mies.) wyzerowany w całym projekcie, w tym w Z4; zostaje Suska (4 920 zł/mies.). Zadanie 3 jest składane w pełnej kwocie, a w Z4 różnice vs pierwotny budżet mogą dotyczyć tylko amortyzacji laptopów i grafika – dlatego obniżenie mieszczące się w limicie dofinansowania jest wyłącznie w poz. 4.9 (współczynnik C19).</t>
   </si>
   <si>
-    <t xml:space="preserve">10. Amortyzacja laptopów: 569,02 zł/mies. (Z1 wykonanie 2 276,08 = 4 × 569,02). Poz. 2.9 (Z2, 6 m-cy) = 3 414,12 zł, poz. 3.8 (Z3, 8 m-cy) = 4 552,16 zł, poz. 4.7 (Z4, 4 m-ce) = 2 276,08 zł. Uwolniona różnica nie trafia na licencje – zwiększa kwalifikowalne Z4 (mniejsze obniżenie, współczynnik C19), w granicach limitu dofinansowania.</t>
+    <t xml:space="preserve">10. Amortyzacja laptopów: 569,02 zł/mies. (Z1 wykonanie 2 276,08 = 4 × 569,02). Poz. 2.9 (Z2, 6 m-cy) = 3 414,12 zł, poz. 3.8 (Z3, 8 m-cy) = 4 552,16 zł, poz. 4.7 (Z4, 4 m-ce) = 2 276,08 zł.</t>
   </si>
   <si>
-    <t xml:space="preserve">11. Dofinansowanie: Z1–Z3 po 80%, Z4 po 60% (bez żadnych korekt intensywności). Przy pełnej prognozie Z3 i Z4 dofinansowanie przekroczyłoby cel, dlatego kwalifikowalne Z4 obniżono jednolitym współczynnikiem C19 do kwoty mieszczącej się w limicie dofinansowania (C18). Kwalifikowalne razem spadają poniżej celu – różnica to niewykorzystany budżet.</t>
+    <t xml:space="preserve">11. Dofinansowanie: Z1–Z3 po 80%, Z4 po 60% (bez żadnych korekt intensywności). Dofinansowanie razem nie może wzrosnąć, więc po odjęciu dofinansowania Z1, Z2 (z licencją 630,08 zł) i Z3 oraz pozostałych pozycji Z4 (bez zmian vs pierwotny budżet) na poz. 4.9 zostaje kwota z C18. Kwalifikowalne razem spadają poniżej celu – różnica to niewykorzystany budżet.</t>
   </si>
   <si>
     <t xml:space="preserve">12. Koszty pośrednie: 25% kwalifikowalnych kosztów bezpośrednich; dofinansowanie do nich = ta sama proporcja co w kosztach bezpośrednich (25% dofinansowania bezpośredniego, zaokrąglone w dół). Zmieniają się wraz z kosztami bezpośrednimi.</t>
@@ -12097,7 +12097,7 @@
       </c>
       <c r="C9" s="44" t="n">
         <f aca="false">ROUND(C14*C5,2)</f>
-        <v>0</v>
+        <v>504.06</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12139,7 +12139,7 @@
         <v>157</v>
       </c>
       <c r="C14" s="46" t="n">
-        <v>0</v>
+        <v>630.08</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12147,8 +12147,8 @@
         <v>158</v>
       </c>
       <c r="C15" s="44" t="n">
-        <f aca="false">'plan etatów'!AA106+'plan etatów'!AA107+'plan etatów'!AA108+'plan etatów'!AA109+'plan etatów'!AA110+'plan etatów'!AA111+'plan etatów'!AA113+'plan etatów'!AA114</f>
-        <v>661200</v>
+        <f aca="false">'plan etatów'!AA114</f>
+        <v>19680</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="C17" s="44" t="n">
         <f aca="false">'nowy format 2'!G4+'nowy format 2'!G5+'nowy format 2'!G6+'nowy format 2'!G7+'nowy format 2'!G8+'nowy format 2'!G9+'nowy format 2'!G10+'nowy format 2'!G11+'nowy format 2'!G12+'nowy format 2'!G14+'nowy format 2'!G15+'nowy format 2'!G16+'nowy format 2'!G17+'nowy format 2'!G18+'nowy format 2'!G19+'nowy format 2'!G20+'nowy format 2'!G21+'nowy format 2'!G22+'nowy format 2'!G23+C16</f>
-        <v>2564935.48</v>
+        <v>2565439.54</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12174,8 +12174,8 @@
         <v>161</v>
       </c>
       <c r="C18" s="44" t="n">
-        <f aca="false">C13-C17-C7*('plan etatów'!AA112)</f>
-        <v>393645.412</v>
+        <f aca="false">C13-C17-C7*('plan etatów'!AA106+'plan etatów'!AA107+'plan etatów'!AA108+'plan etatów'!AA109+'plan etatów'!AA110+'plan etatów'!AA111+'plan etatów'!AA112+'plan etatów'!AA113)</f>
+        <v>8229.35200000001</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12183,8 +12183,8 @@
         <v>162</v>
       </c>
       <c r="C19" s="47" t="n">
-        <f aca="false">MIN(1,ROUNDDOWN(C18/C7,2)/C15)</f>
-        <v>0.992249969751966</v>
+        <f aca="false">MIN(1,MAX(0,ROUNDDOWN(C18/C7,2)/C15))</f>
+        <v>0.696929878048781</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12220,7 +12220,7 @@
       </c>
       <c r="C23" s="44" t="n">
         <f aca="false">ROUND(C15*C19,2)</f>
-        <v>656075.68</v>
+        <v>13715.58</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12246,7 +12246,7 @@
       </c>
       <c r="C25" s="49" t="n">
         <f aca="false">'nowy format 2'!F50</f>
-        <v>4830651.4</v>
+        <v>4830388.88</v>
       </c>
       <c r="D25" s="49" t="n">
         <f aca="false">C10</f>
@@ -12258,7 +12258,7 @@
       </c>
       <c r="F25" s="49" t="n">
         <f aca="false">ROUND(C25-D25,2)</f>
-        <v>-12464.21</v>
+        <v>-12726.73</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12303,11 +12303,11 @@
       </c>
       <c r="C28" s="49" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!C97,2)</f>
-        <v>3864521.12</v>
+        <v>3864311.1</v>
       </c>
       <c r="D28" s="49" t="n">
         <f aca="false">'nowy format 2'!F48</f>
-        <v>3864521.12</v>
+        <v>3864311.1</v>
       </c>
       <c r="E28" s="40" t="str">
         <f aca="false">IF(ABS(C28-D28)&lt;=0.05,"OK","BŁĄD")</f>
@@ -28937,7 +28937,7 @@
       </c>
       <c r="C72" s="49" t="n">
         <f aca="false">SUM(D72:Z72)</f>
-        <v>0</v>
+        <v>630.08</v>
       </c>
       <c r="D72" s="49" t="n">
         <f aca="false">IF(D$4='plan etatów'!$E$5,założenia!$C$14,0)</f>
@@ -28981,7 +28981,7 @@
       </c>
       <c r="N72" s="49" t="n">
         <f aca="false">IF(N$4='plan etatów'!$E$5,założenia!$C$14,0)</f>
-        <v>0</v>
+        <v>630.08</v>
       </c>
       <c r="O72" s="49" t="n">
         <f aca="false">IF(O$4='plan etatów'!$E$5,założenia!$C$14,0)</f>
@@ -30185,99 +30185,99 @@
       </c>
       <c r="C84" s="49" t="n">
         <f aca="false">SUM(D84:Z84)</f>
-        <v>219882.593297036</v>
+        <v>221600</v>
       </c>
       <c r="D84" s="49" t="n">
-        <f aca="false">'plan etatów'!D106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!D106</f>
         <v>0</v>
       </c>
       <c r="E84" s="49" t="n">
-        <f aca="false">'plan etatów'!E106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!E106</f>
         <v>0</v>
       </c>
       <c r="F84" s="49" t="n">
-        <f aca="false">'plan etatów'!F106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!F106</f>
         <v>0</v>
       </c>
       <c r="G84" s="49" t="n">
-        <f aca="false">'plan etatów'!G106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!G106</f>
         <v>0</v>
       </c>
       <c r="H84" s="49" t="n">
-        <f aca="false">'plan etatów'!H106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!H106</f>
         <v>0</v>
       </c>
       <c r="I84" s="49" t="n">
-        <f aca="false">'plan etatów'!I106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!I106</f>
         <v>0</v>
       </c>
       <c r="J84" s="49" t="n">
-        <f aca="false">'plan etatów'!J106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!J106</f>
         <v>0</v>
       </c>
       <c r="K84" s="49" t="n">
-        <f aca="false">'plan etatów'!K106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!K106</f>
         <v>0</v>
       </c>
       <c r="L84" s="49" t="n">
-        <f aca="false">'plan etatów'!L106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!L106</f>
         <v>0</v>
       </c>
       <c r="M84" s="49" t="n">
-        <f aca="false">'plan etatów'!M106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!M106</f>
         <v>0</v>
       </c>
       <c r="N84" s="49" t="n">
-        <f aca="false">'plan etatów'!N106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!N106</f>
         <v>0</v>
       </c>
       <c r="O84" s="49" t="n">
-        <f aca="false">'plan etatów'!O106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!O106</f>
         <v>0</v>
       </c>
       <c r="P84" s="49" t="n">
-        <f aca="false">'plan etatów'!P106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!P106</f>
         <v>0</v>
       </c>
       <c r="Q84" s="49" t="n">
-        <f aca="false">'plan etatów'!Q106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!Q106</f>
         <v>0</v>
       </c>
       <c r="R84" s="49" t="n">
-        <f aca="false">'plan etatów'!R106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!R106</f>
         <v>0</v>
       </c>
       <c r="S84" s="49" t="n">
-        <f aca="false">'plan etatów'!S106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!S106</f>
         <v>0</v>
       </c>
       <c r="T84" s="49" t="n">
-        <f aca="false">'plan etatów'!T106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!T106</f>
         <v>0</v>
       </c>
       <c r="U84" s="49" t="n">
-        <f aca="false">'plan etatów'!U106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!U106</f>
         <v>0</v>
       </c>
       <c r="V84" s="49" t="n">
-        <f aca="false">'plan etatów'!V106*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!V106</f>
         <v>0</v>
       </c>
       <c r="W84" s="49" t="n">
-        <f aca="false">'plan etatów'!W106*założenia!$C$19</f>
-        <v>54970.6483242589</v>
+        <f aca="false">'plan etatów'!W106</f>
+        <v>55400</v>
       </c>
       <c r="X84" s="49" t="n">
-        <f aca="false">'plan etatów'!X106*założenia!$C$19</f>
-        <v>54970.6483242589</v>
+        <f aca="false">'plan etatów'!X106</f>
+        <v>55400</v>
       </c>
       <c r="Y84" s="49" t="n">
-        <f aca="false">'plan etatów'!Y106*założenia!$C$19</f>
-        <v>54970.6483242589</v>
+        <f aca="false">'plan etatów'!Y106</f>
+        <v>55400</v>
       </c>
       <c r="Z84" s="49" t="n">
-        <f aca="false">'plan etatów'!Z106*założenia!$C$19</f>
-        <v>54970.6483242589</v>
+        <f aca="false">'plan etatów'!Z106</f>
+        <v>55400</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30289,99 +30289,99 @@
       </c>
       <c r="C85" s="49" t="n">
         <f aca="false">SUM(D85:Z85)</f>
-        <v>37427.6688590442</v>
+        <v>37720</v>
       </c>
       <c r="D85" s="49" t="n">
-        <f aca="false">'plan etatów'!D107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!D107</f>
         <v>0</v>
       </c>
       <c r="E85" s="49" t="n">
-        <f aca="false">'plan etatów'!E107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!E107</f>
         <v>0</v>
       </c>
       <c r="F85" s="49" t="n">
-        <f aca="false">'plan etatów'!F107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!F107</f>
         <v>0</v>
       </c>
       <c r="G85" s="49" t="n">
-        <f aca="false">'plan etatów'!G107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!G107</f>
         <v>0</v>
       </c>
       <c r="H85" s="49" t="n">
-        <f aca="false">'plan etatów'!H107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!H107</f>
         <v>0</v>
       </c>
       <c r="I85" s="49" t="n">
-        <f aca="false">'plan etatów'!I107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!I107</f>
         <v>0</v>
       </c>
       <c r="J85" s="49" t="n">
-        <f aca="false">'plan etatów'!J107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!J107</f>
         <v>0</v>
       </c>
       <c r="K85" s="49" t="n">
-        <f aca="false">'plan etatów'!K107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!K107</f>
         <v>0</v>
       </c>
       <c r="L85" s="49" t="n">
-        <f aca="false">'plan etatów'!L107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!L107</f>
         <v>0</v>
       </c>
       <c r="M85" s="49" t="n">
-        <f aca="false">'plan etatów'!M107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!M107</f>
         <v>0</v>
       </c>
       <c r="N85" s="49" t="n">
-        <f aca="false">'plan etatów'!N107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!N107</f>
         <v>0</v>
       </c>
       <c r="O85" s="49" t="n">
-        <f aca="false">'plan etatów'!O107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!O107</f>
         <v>0</v>
       </c>
       <c r="P85" s="49" t="n">
-        <f aca="false">'plan etatów'!P107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!P107</f>
         <v>0</v>
       </c>
       <c r="Q85" s="49" t="n">
-        <f aca="false">'plan etatów'!Q107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!Q107</f>
         <v>0</v>
       </c>
       <c r="R85" s="49" t="n">
-        <f aca="false">'plan etatów'!R107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!R107</f>
         <v>0</v>
       </c>
       <c r="S85" s="49" t="n">
-        <f aca="false">'plan etatów'!S107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!S107</f>
         <v>0</v>
       </c>
       <c r="T85" s="49" t="n">
-        <f aca="false">'plan etatów'!T107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!T107</f>
         <v>0</v>
       </c>
       <c r="U85" s="49" t="n">
-        <f aca="false">'plan etatów'!U107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!U107</f>
         <v>0</v>
       </c>
       <c r="V85" s="49" t="n">
-        <f aca="false">'plan etatów'!V107*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!V107</f>
         <v>0</v>
       </c>
       <c r="W85" s="49" t="n">
-        <f aca="false">'plan etatów'!W107*założenia!$C$19</f>
-        <v>9356.91721476104</v>
+        <f aca="false">'plan etatów'!W107</f>
+        <v>9430</v>
       </c>
       <c r="X85" s="49" t="n">
-        <f aca="false">'plan etatów'!X107*założenia!$C$19</f>
-        <v>9356.91721476104</v>
+        <f aca="false">'plan etatów'!X107</f>
+        <v>9430</v>
       </c>
       <c r="Y85" s="49" t="n">
-        <f aca="false">'plan etatów'!Y107*założenia!$C$19</f>
-        <v>9356.91721476104</v>
+        <f aca="false">'plan etatów'!Y107</f>
+        <v>9430</v>
       </c>
       <c r="Z85" s="49" t="n">
-        <f aca="false">'plan etatów'!Z107*założenia!$C$19</f>
-        <v>9356.91721476104</v>
+        <f aca="false">'plan etatów'!Z107</f>
+        <v>9430</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30393,99 +30393,99 @@
       </c>
       <c r="C86" s="49" t="n">
         <f aca="false">SUM(D86:Z86)</f>
-        <v>107599.586719903</v>
+        <v>108440</v>
       </c>
       <c r="D86" s="49" t="n">
-        <f aca="false">'plan etatów'!D108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!D108</f>
         <v>0</v>
       </c>
       <c r="E86" s="49" t="n">
-        <f aca="false">'plan etatów'!E108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!E108</f>
         <v>0</v>
       </c>
       <c r="F86" s="49" t="n">
-        <f aca="false">'plan etatów'!F108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!F108</f>
         <v>0</v>
       </c>
       <c r="G86" s="49" t="n">
-        <f aca="false">'plan etatów'!G108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!G108</f>
         <v>0</v>
       </c>
       <c r="H86" s="49" t="n">
-        <f aca="false">'plan etatów'!H108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!H108</f>
         <v>0</v>
       </c>
       <c r="I86" s="49" t="n">
-        <f aca="false">'plan etatów'!I108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!I108</f>
         <v>0</v>
       </c>
       <c r="J86" s="49" t="n">
-        <f aca="false">'plan etatów'!J108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!J108</f>
         <v>0</v>
       </c>
       <c r="K86" s="49" t="n">
-        <f aca="false">'plan etatów'!K108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!K108</f>
         <v>0</v>
       </c>
       <c r="L86" s="49" t="n">
-        <f aca="false">'plan etatów'!L108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!L108</f>
         <v>0</v>
       </c>
       <c r="M86" s="49" t="n">
-        <f aca="false">'plan etatów'!M108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!M108</f>
         <v>0</v>
       </c>
       <c r="N86" s="49" t="n">
-        <f aca="false">'plan etatów'!N108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!N108</f>
         <v>0</v>
       </c>
       <c r="O86" s="49" t="n">
-        <f aca="false">'plan etatów'!O108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!O108</f>
         <v>0</v>
       </c>
       <c r="P86" s="49" t="n">
-        <f aca="false">'plan etatów'!P108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!P108</f>
         <v>0</v>
       </c>
       <c r="Q86" s="49" t="n">
-        <f aca="false">'plan etatów'!Q108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!Q108</f>
         <v>0</v>
       </c>
       <c r="R86" s="49" t="n">
-        <f aca="false">'plan etatów'!R108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!R108</f>
         <v>0</v>
       </c>
       <c r="S86" s="49" t="n">
-        <f aca="false">'plan etatów'!S108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!S108</f>
         <v>0</v>
       </c>
       <c r="T86" s="49" t="n">
-        <f aca="false">'plan etatów'!T108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!T108</f>
         <v>0</v>
       </c>
       <c r="U86" s="49" t="n">
-        <f aca="false">'plan etatów'!U108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!U108</f>
         <v>0</v>
       </c>
       <c r="V86" s="49" t="n">
-        <f aca="false">'plan etatów'!V108*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!V108</f>
         <v>0</v>
       </c>
       <c r="W86" s="49" t="n">
-        <f aca="false">'plan etatów'!W108*założenia!$C$19</f>
-        <v>26899.8966799758</v>
+        <f aca="false">'plan etatów'!W108</f>
+        <v>27110</v>
       </c>
       <c r="X86" s="49" t="n">
-        <f aca="false">'plan etatów'!X108*założenia!$C$19</f>
-        <v>26899.8966799758</v>
+        <f aca="false">'plan etatów'!X108</f>
+        <v>27110</v>
       </c>
       <c r="Y86" s="49" t="n">
-        <f aca="false">'plan etatów'!Y108*założenia!$C$19</f>
-        <v>26899.8966799758</v>
+        <f aca="false">'plan etatów'!Y108</f>
+        <v>27110</v>
       </c>
       <c r="Z86" s="49" t="n">
-        <f aca="false">'plan etatów'!Z108*założenia!$C$19</f>
-        <v>26899.8966799758</v>
+        <f aca="false">'plan etatów'!Z108</f>
+        <v>27110</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30497,99 +30497,99 @@
       </c>
       <c r="C87" s="49" t="n">
         <f aca="false">SUM(D87:Z87)</f>
-        <v>81860.6225045372</v>
+        <v>82500</v>
       </c>
       <c r="D87" s="49" t="n">
-        <f aca="false">'plan etatów'!D109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!D109</f>
         <v>0</v>
       </c>
       <c r="E87" s="49" t="n">
-        <f aca="false">'plan etatów'!E109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!E109</f>
         <v>0</v>
       </c>
       <c r="F87" s="49" t="n">
-        <f aca="false">'plan etatów'!F109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!F109</f>
         <v>0</v>
       </c>
       <c r="G87" s="49" t="n">
-        <f aca="false">'plan etatów'!G109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!G109</f>
         <v>0</v>
       </c>
       <c r="H87" s="49" t="n">
-        <f aca="false">'plan etatów'!H109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!H109</f>
         <v>0</v>
       </c>
       <c r="I87" s="49" t="n">
-        <f aca="false">'plan etatów'!I109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!I109</f>
         <v>0</v>
       </c>
       <c r="J87" s="49" t="n">
-        <f aca="false">'plan etatów'!J109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!J109</f>
         <v>0</v>
       </c>
       <c r="K87" s="49" t="n">
-        <f aca="false">'plan etatów'!K109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!K109</f>
         <v>0</v>
       </c>
       <c r="L87" s="49" t="n">
-        <f aca="false">'plan etatów'!L109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!L109</f>
         <v>0</v>
       </c>
       <c r="M87" s="49" t="n">
-        <f aca="false">'plan etatów'!M109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!M109</f>
         <v>0</v>
       </c>
       <c r="N87" s="49" t="n">
-        <f aca="false">'plan etatów'!N109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!N109</f>
         <v>0</v>
       </c>
       <c r="O87" s="49" t="n">
-        <f aca="false">'plan etatów'!O109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!O109</f>
         <v>0</v>
       </c>
       <c r="P87" s="49" t="n">
-        <f aca="false">'plan etatów'!P109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!P109</f>
         <v>0</v>
       </c>
       <c r="Q87" s="49" t="n">
-        <f aca="false">'plan etatów'!Q109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!Q109</f>
         <v>0</v>
       </c>
       <c r="R87" s="49" t="n">
-        <f aca="false">'plan etatów'!R109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!R109</f>
         <v>0</v>
       </c>
       <c r="S87" s="49" t="n">
-        <f aca="false">'plan etatów'!S109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!S109</f>
         <v>0</v>
       </c>
       <c r="T87" s="49" t="n">
-        <f aca="false">'plan etatów'!T109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!T109</f>
         <v>0</v>
       </c>
       <c r="U87" s="49" t="n">
-        <f aca="false">'plan etatów'!U109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!U109</f>
         <v>0</v>
       </c>
       <c r="V87" s="49" t="n">
-        <f aca="false">'plan etatów'!V109*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!V109</f>
         <v>0</v>
       </c>
       <c r="W87" s="49" t="n">
-        <f aca="false">'plan etatów'!W109*założenia!$C$19</f>
-        <v>20465.1556261343</v>
+        <f aca="false">'plan etatów'!W109</f>
+        <v>20625</v>
       </c>
       <c r="X87" s="49" t="n">
-        <f aca="false">'plan etatów'!X109*założenia!$C$19</f>
-        <v>20465.1556261343</v>
+        <f aca="false">'plan etatów'!X109</f>
+        <v>20625</v>
       </c>
       <c r="Y87" s="49" t="n">
-        <f aca="false">'plan etatów'!Y109*założenia!$C$19</f>
-        <v>20465.1556261343</v>
+        <f aca="false">'plan etatów'!Y109</f>
+        <v>20625</v>
       </c>
       <c r="Z87" s="49" t="n">
-        <f aca="false">'plan etatów'!Z109*założenia!$C$19</f>
-        <v>20465.1556261343</v>
+        <f aca="false">'plan etatów'!Z109</f>
+        <v>20625</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30601,99 +30601,99 @@
       </c>
       <c r="C88" s="49" t="n">
         <f aca="false">SUM(D88:Z88)</f>
-        <v>29529.3590998185</v>
+        <v>29760</v>
       </c>
       <c r="D88" s="49" t="n">
-        <f aca="false">'plan etatów'!D110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!D110</f>
         <v>0</v>
       </c>
       <c r="E88" s="49" t="n">
-        <f aca="false">'plan etatów'!E110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!E110</f>
         <v>0</v>
       </c>
       <c r="F88" s="49" t="n">
-        <f aca="false">'plan etatów'!F110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!F110</f>
         <v>0</v>
       </c>
       <c r="G88" s="49" t="n">
-        <f aca="false">'plan etatów'!G110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!G110</f>
         <v>0</v>
       </c>
       <c r="H88" s="49" t="n">
-        <f aca="false">'plan etatów'!H110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!H110</f>
         <v>0</v>
       </c>
       <c r="I88" s="49" t="n">
-        <f aca="false">'plan etatów'!I110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!I110</f>
         <v>0</v>
       </c>
       <c r="J88" s="49" t="n">
-        <f aca="false">'plan etatów'!J110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!J110</f>
         <v>0</v>
       </c>
       <c r="K88" s="49" t="n">
-        <f aca="false">'plan etatów'!K110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!K110</f>
         <v>0</v>
       </c>
       <c r="L88" s="49" t="n">
-        <f aca="false">'plan etatów'!L110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!L110</f>
         <v>0</v>
       </c>
       <c r="M88" s="49" t="n">
-        <f aca="false">'plan etatów'!M110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!M110</f>
         <v>0</v>
       </c>
       <c r="N88" s="49" t="n">
-        <f aca="false">'plan etatów'!N110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!N110</f>
         <v>0</v>
       </c>
       <c r="O88" s="49" t="n">
-        <f aca="false">'plan etatów'!O110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!O110</f>
         <v>0</v>
       </c>
       <c r="P88" s="49" t="n">
-        <f aca="false">'plan etatów'!P110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!P110</f>
         <v>0</v>
       </c>
       <c r="Q88" s="49" t="n">
-        <f aca="false">'plan etatów'!Q110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!Q110</f>
         <v>0</v>
       </c>
       <c r="R88" s="49" t="n">
-        <f aca="false">'plan etatów'!R110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!R110</f>
         <v>0</v>
       </c>
       <c r="S88" s="49" t="n">
-        <f aca="false">'plan etatów'!S110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!S110</f>
         <v>0</v>
       </c>
       <c r="T88" s="49" t="n">
-        <f aca="false">'plan etatów'!T110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!T110</f>
         <v>0</v>
       </c>
       <c r="U88" s="49" t="n">
-        <f aca="false">'plan etatów'!U110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!U110</f>
         <v>0</v>
       </c>
       <c r="V88" s="49" t="n">
-        <f aca="false">'plan etatów'!V110*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!V110</f>
         <v>0</v>
       </c>
       <c r="W88" s="49" t="n">
-        <f aca="false">'plan etatów'!W110*założenia!$C$19</f>
-        <v>7382.33977495463</v>
+        <f aca="false">'plan etatów'!W110</f>
+        <v>7440</v>
       </c>
       <c r="X88" s="49" t="n">
-        <f aca="false">'plan etatów'!X110*założenia!$C$19</f>
-        <v>7382.33977495463</v>
+        <f aca="false">'plan etatów'!X110</f>
+        <v>7440</v>
       </c>
       <c r="Y88" s="49" t="n">
-        <f aca="false">'plan etatów'!Y110*założenia!$C$19</f>
-        <v>7382.33977495463</v>
+        <f aca="false">'plan etatów'!Y110</f>
+        <v>7440</v>
       </c>
       <c r="Z88" s="49" t="n">
-        <f aca="false">'plan etatów'!Z110*założenia!$C$19</f>
-        <v>7382.33977495463</v>
+        <f aca="false">'plan etatów'!Z110</f>
+        <v>7440</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30705,99 +30705,99 @@
       </c>
       <c r="C89" s="49" t="n">
         <f aca="false">SUM(D89:Z89)</f>
-        <v>81860.6225045372</v>
+        <v>82500</v>
       </c>
       <c r="D89" s="49" t="n">
-        <f aca="false">'plan etatów'!D111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!D111</f>
         <v>0</v>
       </c>
       <c r="E89" s="49" t="n">
-        <f aca="false">'plan etatów'!E111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!E111</f>
         <v>0</v>
       </c>
       <c r="F89" s="49" t="n">
-        <f aca="false">'plan etatów'!F111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!F111</f>
         <v>0</v>
       </c>
       <c r="G89" s="49" t="n">
-        <f aca="false">'plan etatów'!G111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!G111</f>
         <v>0</v>
       </c>
       <c r="H89" s="49" t="n">
-        <f aca="false">'plan etatów'!H111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!H111</f>
         <v>0</v>
       </c>
       <c r="I89" s="49" t="n">
-        <f aca="false">'plan etatów'!I111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!I111</f>
         <v>0</v>
       </c>
       <c r="J89" s="49" t="n">
-        <f aca="false">'plan etatów'!J111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!J111</f>
         <v>0</v>
       </c>
       <c r="K89" s="49" t="n">
-        <f aca="false">'plan etatów'!K111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!K111</f>
         <v>0</v>
       </c>
       <c r="L89" s="49" t="n">
-        <f aca="false">'plan etatów'!L111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!L111</f>
         <v>0</v>
       </c>
       <c r="M89" s="49" t="n">
-        <f aca="false">'plan etatów'!M111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!M111</f>
         <v>0</v>
       </c>
       <c r="N89" s="49" t="n">
-        <f aca="false">'plan etatów'!N111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!N111</f>
         <v>0</v>
       </c>
       <c r="O89" s="49" t="n">
-        <f aca="false">'plan etatów'!O111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!O111</f>
         <v>0</v>
       </c>
       <c r="P89" s="49" t="n">
-        <f aca="false">'plan etatów'!P111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!P111</f>
         <v>0</v>
       </c>
       <c r="Q89" s="49" t="n">
-        <f aca="false">'plan etatów'!Q111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!Q111</f>
         <v>0</v>
       </c>
       <c r="R89" s="49" t="n">
-        <f aca="false">'plan etatów'!R111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!R111</f>
         <v>0</v>
       </c>
       <c r="S89" s="49" t="n">
-        <f aca="false">'plan etatów'!S111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!S111</f>
         <v>0</v>
       </c>
       <c r="T89" s="49" t="n">
-        <f aca="false">'plan etatów'!T111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!T111</f>
         <v>0</v>
       </c>
       <c r="U89" s="49" t="n">
-        <f aca="false">'plan etatów'!U111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!U111</f>
         <v>0</v>
       </c>
       <c r="V89" s="49" t="n">
-        <f aca="false">'plan etatów'!V111*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!V111</f>
         <v>0</v>
       </c>
       <c r="W89" s="49" t="n">
-        <f aca="false">'plan etatów'!W111*założenia!$C$19</f>
-        <v>20465.1556261343</v>
+        <f aca="false">'plan etatów'!W111</f>
+        <v>20625</v>
       </c>
       <c r="X89" s="49" t="n">
-        <f aca="false">'plan etatów'!X111*założenia!$C$19</f>
-        <v>20465.1556261343</v>
+        <f aca="false">'plan etatów'!X111</f>
+        <v>20625</v>
       </c>
       <c r="Y89" s="49" t="n">
-        <f aca="false">'plan etatów'!Y111*założenia!$C$19</f>
-        <v>20465.1556261343</v>
+        <f aca="false">'plan etatów'!Y111</f>
+        <v>20625</v>
       </c>
       <c r="Z89" s="49" t="n">
-        <f aca="false">'plan etatów'!Z111*założenia!$C$19</f>
-        <v>20465.1556261343</v>
+        <f aca="false">'plan etatów'!Z111</f>
+        <v>20625</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30913,99 +30913,99 @@
       </c>
       <c r="C91" s="49" t="n">
         <f aca="false">SUM(D91:Z91)</f>
-        <v>78387.7476104053</v>
+        <v>79000</v>
       </c>
       <c r="D91" s="49" t="n">
-        <f aca="false">'plan etatów'!D113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!D113</f>
         <v>0</v>
       </c>
       <c r="E91" s="49" t="n">
-        <f aca="false">'plan etatów'!E113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!E113</f>
         <v>0</v>
       </c>
       <c r="F91" s="49" t="n">
-        <f aca="false">'plan etatów'!F113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!F113</f>
         <v>0</v>
       </c>
       <c r="G91" s="49" t="n">
-        <f aca="false">'plan etatów'!G113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!G113</f>
         <v>0</v>
       </c>
       <c r="H91" s="49" t="n">
-        <f aca="false">'plan etatów'!H113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!H113</f>
         <v>0</v>
       </c>
       <c r="I91" s="49" t="n">
-        <f aca="false">'plan etatów'!I113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!I113</f>
         <v>0</v>
       </c>
       <c r="J91" s="49" t="n">
-        <f aca="false">'plan etatów'!J113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!J113</f>
         <v>0</v>
       </c>
       <c r="K91" s="49" t="n">
-        <f aca="false">'plan etatów'!K113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!K113</f>
         <v>0</v>
       </c>
       <c r="L91" s="49" t="n">
-        <f aca="false">'plan etatów'!L113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!L113</f>
         <v>0</v>
       </c>
       <c r="M91" s="49" t="n">
-        <f aca="false">'plan etatów'!M113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!M113</f>
         <v>0</v>
       </c>
       <c r="N91" s="49" t="n">
-        <f aca="false">'plan etatów'!N113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!N113</f>
         <v>0</v>
       </c>
       <c r="O91" s="49" t="n">
-        <f aca="false">'plan etatów'!O113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!O113</f>
         <v>0</v>
       </c>
       <c r="P91" s="49" t="n">
-        <f aca="false">'plan etatów'!P113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!P113</f>
         <v>0</v>
       </c>
       <c r="Q91" s="49" t="n">
-        <f aca="false">'plan etatów'!Q113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!Q113</f>
         <v>0</v>
       </c>
       <c r="R91" s="49" t="n">
-        <f aca="false">'plan etatów'!R113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!R113</f>
         <v>0</v>
       </c>
       <c r="S91" s="49" t="n">
-        <f aca="false">'plan etatów'!S113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!S113</f>
         <v>0</v>
       </c>
       <c r="T91" s="49" t="n">
-        <f aca="false">'plan etatów'!T113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!T113</f>
         <v>0</v>
       </c>
       <c r="U91" s="49" t="n">
-        <f aca="false">'plan etatów'!U113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!U113</f>
         <v>0</v>
       </c>
       <c r="V91" s="49" t="n">
-        <f aca="false">'plan etatów'!V113*założenia!$C$19</f>
+        <f aca="false">'plan etatów'!V113</f>
         <v>0</v>
       </c>
       <c r="W91" s="49" t="n">
-        <f aca="false">'plan etatów'!W113*założenia!$C$19</f>
-        <v>19596.9369026013</v>
+        <f aca="false">'plan etatów'!W113</f>
+        <v>19750</v>
       </c>
       <c r="X91" s="49" t="n">
-        <f aca="false">'plan etatów'!X113*założenia!$C$19</f>
-        <v>19596.9369026013</v>
+        <f aca="false">'plan etatów'!X113</f>
+        <v>19750</v>
       </c>
       <c r="Y91" s="49" t="n">
-        <f aca="false">'plan etatów'!Y113*założenia!$C$19</f>
-        <v>19596.9369026013</v>
+        <f aca="false">'plan etatów'!Y113</f>
+        <v>19750</v>
       </c>
       <c r="Z91" s="49" t="n">
-        <f aca="false">'plan etatów'!Z113*założenia!$C$19</f>
-        <v>19596.9369026013</v>
+        <f aca="false">'plan etatów'!Z113</f>
+        <v>19750</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31017,7 +31017,7 @@
       </c>
       <c r="C92" s="49" t="n">
         <f aca="false">SUM(D92:Z92)</f>
-        <v>19527.4794047187</v>
+        <v>13715.58</v>
       </c>
       <c r="D92" s="49" t="n">
         <f aca="false">'plan etatów'!D114*założenia!$C$19</f>
@@ -31097,19 +31097,19 @@
       </c>
       <c r="W92" s="49" t="n">
         <f aca="false">'plan etatów'!W114*założenia!$C$19</f>
-        <v>4881.86985117967</v>
+        <v>3428.895</v>
       </c>
       <c r="X92" s="49" t="n">
         <f aca="false">'plan etatów'!X114*założenia!$C$19</f>
-        <v>4881.86985117967</v>
+        <v>3428.895</v>
       </c>
       <c r="Y92" s="49" t="n">
         <f aca="false">'plan etatów'!Y114*założenia!$C$19</f>
-        <v>4881.86985117967</v>
+        <v>3428.895</v>
       </c>
       <c r="Z92" s="49" t="n">
         <f aca="false">'plan etatów'!Z114*założenia!$C$19</f>
-        <v>4881.86985117967</v>
+        <v>3428.895</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31225,7 +31225,7 @@
       </c>
       <c r="C94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,C$56:C$92)</f>
-        <v>1009907.33</v>
+        <v>1010537.41</v>
       </c>
       <c r="D94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,D$56:D$92)</f>
@@ -31269,7 +31269,7 @@
       </c>
       <c r="N94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,N$56:N$92)</f>
-        <v>168317.888333333</v>
+        <v>168947.968333333</v>
       </c>
       <c r="O94" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,2,O$56:O$92)</f>
@@ -31433,7 +31433,7 @@
       </c>
       <c r="C96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,C$56:C$92)</f>
-        <v>658351.76</v>
+        <v>657511.66</v>
       </c>
       <c r="D96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,D$56:D$92)</f>
@@ -31513,19 +31513,19 @@
       </c>
       <c r="W96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,W$56:W$92)</f>
-        <v>164587.94</v>
+        <v>164377.915</v>
       </c>
       <c r="X96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,X$56:X$92)</f>
-        <v>164587.94</v>
+        <v>164377.915</v>
       </c>
       <c r="Y96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,Y$56:Y$92)</f>
-        <v>164587.94</v>
+        <v>164377.915</v>
       </c>
       <c r="Z96" s="63" t="n">
         <f aca="false">SUMIF($B$56:$B$92,4,Z$56:Z$92)</f>
-        <v>164587.94</v>
+        <v>164377.915</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31535,7 +31535,7 @@
       <c r="B97" s="40"/>
       <c r="C97" s="63" t="n">
         <f aca="false">SUM(C93:C96)</f>
-        <v>3864521.12</v>
+        <v>3864311.1</v>
       </c>
       <c r="D97" s="63" t="n">
         <f aca="false">SUM(D93:D96)</f>
@@ -31579,7 +31579,7 @@
       </c>
       <c r="N97" s="63" t="n">
         <f aca="false">SUM(N93:N96)</f>
-        <v>168317.888333333</v>
+        <v>168947.968333333</v>
       </c>
       <c r="O97" s="63" t="n">
         <f aca="false">SUM(O93:O96)</f>
@@ -31615,19 +31615,19 @@
       </c>
       <c r="W97" s="63" t="n">
         <f aca="false">SUM(W93:W96)</f>
-        <v>164587.94</v>
+        <v>164377.915</v>
       </c>
       <c r="X97" s="63" t="n">
         <f aca="false">SUM(X93:X96)</f>
-        <v>164587.94</v>
+        <v>164377.915</v>
       </c>
       <c r="Y97" s="63" t="n">
         <f aca="false">SUM(Y93:Y96)</f>
-        <v>164587.94</v>
+        <v>164377.915</v>
       </c>
       <c r="Z97" s="63" t="n">
         <f aca="false">SUM(Z93:Z96)</f>
-        <v>164587.94</v>
+        <v>164377.915</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31637,7 +31637,7 @@
       <c r="B98" s="40"/>
       <c r="C98" s="63" t="n">
         <f aca="false">0.25*C97</f>
-        <v>966130.28</v>
+        <v>966077.775</v>
       </c>
       <c r="D98" s="63" t="n">
         <f aca="false">0.25*D97</f>
@@ -31681,7 +31681,7 @@
       </c>
       <c r="N98" s="63" t="n">
         <f aca="false">0.25*N97</f>
-        <v>42079.4720833333</v>
+        <v>42236.9920833333</v>
       </c>
       <c r="O98" s="63" t="n">
         <f aca="false">0.25*O97</f>
@@ -31717,19 +31717,19 @@
       </c>
       <c r="W98" s="63" t="n">
         <f aca="false">0.25*W97</f>
-        <v>41146.985</v>
+        <v>41094.47875</v>
       </c>
       <c r="X98" s="63" t="n">
         <f aca="false">0.25*X97</f>
-        <v>41146.985</v>
+        <v>41094.47875</v>
       </c>
       <c r="Y98" s="63" t="n">
         <f aca="false">0.25*Y97</f>
-        <v>41146.985</v>
+        <v>41094.47875</v>
       </c>
       <c r="Z98" s="63" t="n">
         <f aca="false">0.25*Z97</f>
-        <v>41146.985</v>
+        <v>41094.47875</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31739,7 +31739,7 @@
       <c r="B99" s="40"/>
       <c r="C99" s="63" t="n">
         <f aca="false">C97+C98</f>
-        <v>4830651.4</v>
+        <v>4830388.875</v>
       </c>
       <c r="D99" s="63" t="n">
         <f aca="false">D97+D98</f>
@@ -31783,7 +31783,7 @@
       </c>
       <c r="N99" s="63" t="n">
         <f aca="false">N97+N98</f>
-        <v>210397.360416667</v>
+        <v>211184.960416667</v>
       </c>
       <c r="O99" s="63" t="n">
         <f aca="false">O97+O98</f>
@@ -31819,19 +31819,19 @@
       </c>
       <c r="W99" s="63" t="n">
         <f aca="false">W97+W98</f>
-        <v>205734.925</v>
+        <v>205472.39375</v>
       </c>
       <c r="X99" s="63" t="n">
         <f aca="false">X97+X98</f>
-        <v>205734.925</v>
+        <v>205472.39375</v>
       </c>
       <c r="Y99" s="63" t="n">
         <f aca="false">Y97+Y98</f>
-        <v>205734.925</v>
+        <v>205472.39375</v>
       </c>
       <c r="Z99" s="63" t="n">
         <f aca="false">Z97+Z98</f>
-        <v>205734.925</v>
+        <v>205472.39375</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31882,55 +31882,55 @@
       </c>
       <c r="N100" s="63" t="n">
         <f aca="false">M100+N99</f>
-        <v>2271665.25</v>
+        <v>2272452.85</v>
       </c>
       <c r="O100" s="63" t="n">
         <f aca="false">N100+O99</f>
-        <v>2482317.15</v>
+        <v>2483104.75</v>
       </c>
       <c r="P100" s="63" t="n">
         <f aca="false">O100+P99</f>
-        <v>2692969.05</v>
+        <v>2693756.65</v>
       </c>
       <c r="Q100" s="63" t="n">
         <f aca="false">P100+Q99</f>
-        <v>2912092.825</v>
+        <v>2912880.425</v>
       </c>
       <c r="R100" s="63" t="n">
         <f aca="false">Q100+R99</f>
-        <v>3131216.6</v>
+        <v>3132004.2</v>
       </c>
       <c r="S100" s="63" t="n">
         <f aca="false">R100+S99</f>
-        <v>3350340.375</v>
+        <v>3351127.975</v>
       </c>
       <c r="T100" s="63" t="n">
         <f aca="false">S100+T99</f>
-        <v>3569464.15</v>
+        <v>3570251.75</v>
       </c>
       <c r="U100" s="63" t="n">
         <f aca="false">T100+U99</f>
-        <v>3788587.925</v>
+        <v>3789375.525</v>
       </c>
       <c r="V100" s="63" t="n">
         <f aca="false">U100+V99</f>
-        <v>4007711.7</v>
+        <v>4008499.3</v>
       </c>
       <c r="W100" s="63" t="n">
         <f aca="false">V100+W99</f>
-        <v>4213446.625</v>
+        <v>4213971.69375</v>
       </c>
       <c r="X100" s="63" t="n">
         <f aca="false">W100+X99</f>
-        <v>4419181.55</v>
+        <v>4419444.0875</v>
       </c>
       <c r="Y100" s="63" t="n">
         <f aca="false">X100+Y99</f>
-        <v>4624916.475</v>
+        <v>4624916.48125</v>
       </c>
       <c r="Z100" s="63" t="n">
         <f aca="false">Y100+Z99</f>
-        <v>4830651.4</v>
+        <v>4830388.875</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -38391,7 +38391,7 @@
       </c>
       <c r="C166" s="49" t="n">
         <f aca="false">SUM(D166:Z166)</f>
-        <v>0</v>
+        <v>504.06</v>
       </c>
       <c r="D166" s="49" t="n">
         <f aca="false">IF(D$4='plan etatów'!$E$5,założenia!$C$9,0)</f>
@@ -38435,7 +38435,7 @@
       </c>
       <c r="N166" s="49" t="n">
         <f aca="false">IF(N$4='plan etatów'!$E$5,założenia!$C$9,0)</f>
-        <v>0</v>
+        <v>504.06</v>
       </c>
       <c r="O166" s="49" t="n">
         <f aca="false">IF(O$4='plan etatów'!$E$5,założenia!$C$9,0)</f>
@@ -39639,7 +39639,7 @@
       </c>
       <c r="C178" s="49" t="n">
         <f aca="false">SUM(D178:Z178)</f>
-        <v>131929.555978221</v>
+        <v>132960</v>
       </c>
       <c r="D178" s="49" t="n">
         <f aca="false">D84*założenia!$C$7</f>
@@ -39719,19 +39719,19 @@
       </c>
       <c r="W178" s="49" t="n">
         <f aca="false">W84*założenia!$C$7</f>
-        <v>32982.3889945554</v>
+        <v>33240</v>
       </c>
       <c r="X178" s="49" t="n">
         <f aca="false">X84*założenia!$C$7</f>
-        <v>32982.3889945554</v>
+        <v>33240</v>
       </c>
       <c r="Y178" s="49" t="n">
         <f aca="false">Y84*założenia!$C$7</f>
-        <v>32982.3889945554</v>
+        <v>33240</v>
       </c>
       <c r="Z178" s="49" t="n">
         <f aca="false">Z84*założenia!$C$7</f>
-        <v>32982.3889945554</v>
+        <v>33240</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39743,7 +39743,7 @@
       </c>
       <c r="C179" s="49" t="n">
         <f aca="false">SUM(D179:Z179)</f>
-        <v>22456.6013154265</v>
+        <v>22632</v>
       </c>
       <c r="D179" s="49" t="n">
         <f aca="false">D85*założenia!$C$7</f>
@@ -39823,19 +39823,19 @@
       </c>
       <c r="W179" s="49" t="n">
         <f aca="false">W85*założenia!$C$7</f>
-        <v>5614.15032885663</v>
+        <v>5658</v>
       </c>
       <c r="X179" s="49" t="n">
         <f aca="false">X85*założenia!$C$7</f>
-        <v>5614.15032885663</v>
+        <v>5658</v>
       </c>
       <c r="Y179" s="49" t="n">
         <f aca="false">Y85*założenia!$C$7</f>
-        <v>5614.15032885663</v>
+        <v>5658</v>
       </c>
       <c r="Z179" s="49" t="n">
         <f aca="false">Z85*założenia!$C$7</f>
-        <v>5614.15032885663</v>
+        <v>5658</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39847,7 +39847,7 @@
       </c>
       <c r="C180" s="49" t="n">
         <f aca="false">SUM(D180:Z180)</f>
-        <v>64559.7520319419</v>
+        <v>65064</v>
       </c>
       <c r="D180" s="49" t="n">
         <f aca="false">D86*założenia!$C$7</f>
@@ -39927,19 +39927,19 @@
       </c>
       <c r="W180" s="49" t="n">
         <f aca="false">W86*założenia!$C$7</f>
-        <v>16139.9380079855</v>
+        <v>16266</v>
       </c>
       <c r="X180" s="49" t="n">
         <f aca="false">X86*założenia!$C$7</f>
-        <v>16139.9380079855</v>
+        <v>16266</v>
       </c>
       <c r="Y180" s="49" t="n">
         <f aca="false">Y86*założenia!$C$7</f>
-        <v>16139.9380079855</v>
+        <v>16266</v>
       </c>
       <c r="Z180" s="49" t="n">
         <f aca="false">Z86*założenia!$C$7</f>
-        <v>16139.9380079855</v>
+        <v>16266</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39951,7 +39951,7 @@
       </c>
       <c r="C181" s="49" t="n">
         <f aca="false">SUM(D181:Z181)</f>
-        <v>49116.3735027223</v>
+        <v>49500</v>
       </c>
       <c r="D181" s="49" t="n">
         <f aca="false">D87*założenia!$C$7</f>
@@ -40031,19 +40031,19 @@
       </c>
       <c r="W181" s="49" t="n">
         <f aca="false">W87*założenia!$C$7</f>
-        <v>12279.0933756806</v>
+        <v>12375</v>
       </c>
       <c r="X181" s="49" t="n">
         <f aca="false">X87*założenia!$C$7</f>
-        <v>12279.0933756806</v>
+        <v>12375</v>
       </c>
       <c r="Y181" s="49" t="n">
         <f aca="false">Y87*założenia!$C$7</f>
-        <v>12279.0933756806</v>
+        <v>12375</v>
       </c>
       <c r="Z181" s="49" t="n">
         <f aca="false">Z87*założenia!$C$7</f>
-        <v>12279.0933756806</v>
+        <v>12375</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40055,7 +40055,7 @@
       </c>
       <c r="C182" s="49" t="n">
         <f aca="false">SUM(D182:Z182)</f>
-        <v>17717.6154598911</v>
+        <v>17856</v>
       </c>
       <c r="D182" s="49" t="n">
         <f aca="false">D88*założenia!$C$7</f>
@@ -40135,19 +40135,19 @@
       </c>
       <c r="W182" s="49" t="n">
         <f aca="false">W88*założenia!$C$7</f>
-        <v>4429.40386497278</v>
+        <v>4464</v>
       </c>
       <c r="X182" s="49" t="n">
         <f aca="false">X88*założenia!$C$7</f>
-        <v>4429.40386497278</v>
+        <v>4464</v>
       </c>
       <c r="Y182" s="49" t="n">
         <f aca="false">Y88*założenia!$C$7</f>
-        <v>4429.40386497278</v>
+        <v>4464</v>
       </c>
       <c r="Z182" s="49" t="n">
         <f aca="false">Z88*założenia!$C$7</f>
-        <v>4429.40386497278</v>
+        <v>4464</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40159,7 +40159,7 @@
       </c>
       <c r="C183" s="49" t="n">
         <f aca="false">SUM(D183:Z183)</f>
-        <v>49116.3735027223</v>
+        <v>49500</v>
       </c>
       <c r="D183" s="49" t="n">
         <f aca="false">D89*założenia!$C$7</f>
@@ -40239,19 +40239,19 @@
       </c>
       <c r="W183" s="49" t="n">
         <f aca="false">W89*założenia!$C$7</f>
-        <v>12279.0933756806</v>
+        <v>12375</v>
       </c>
       <c r="X183" s="49" t="n">
         <f aca="false">X89*założenia!$C$7</f>
-        <v>12279.0933756806</v>
+        <v>12375</v>
       </c>
       <c r="Y183" s="49" t="n">
         <f aca="false">Y89*założenia!$C$7</f>
-        <v>12279.0933756806</v>
+        <v>12375</v>
       </c>
       <c r="Z183" s="49" t="n">
         <f aca="false">Z89*założenia!$C$7</f>
-        <v>12279.0933756806</v>
+        <v>12375</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40367,7 +40367,7 @@
       </c>
       <c r="C185" s="49" t="n">
         <f aca="false">SUM(D185:Z185)</f>
-        <v>47032.6485662432</v>
+        <v>47400</v>
       </c>
       <c r="D185" s="49" t="n">
         <f aca="false">D91*założenia!$C$7</f>
@@ -40447,19 +40447,19 @@
       </c>
       <c r="W185" s="49" t="n">
         <f aca="false">W91*założenia!$C$7</f>
-        <v>11758.1621415608</v>
+        <v>11850</v>
       </c>
       <c r="X185" s="49" t="n">
         <f aca="false">X91*założenia!$C$7</f>
-        <v>11758.1621415608</v>
+        <v>11850</v>
       </c>
       <c r="Y185" s="49" t="n">
         <f aca="false">Y91*założenia!$C$7</f>
-        <v>11758.1621415608</v>
+        <v>11850</v>
       </c>
       <c r="Z185" s="49" t="n">
         <f aca="false">Z91*założenia!$C$7</f>
-        <v>11758.1621415608</v>
+        <v>11850</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40471,7 +40471,7 @@
       </c>
       <c r="C186" s="49" t="n">
         <f aca="false">SUM(D186:Z186)</f>
-        <v>11716.4876428312</v>
+        <v>8229.348</v>
       </c>
       <c r="D186" s="49" t="n">
         <f aca="false">D92*założenia!$C$7</f>
@@ -40551,19 +40551,19 @@
       </c>
       <c r="W186" s="49" t="n">
         <f aca="false">W92*założenia!$C$7</f>
-        <v>2929.1219107078</v>
+        <v>2057.337</v>
       </c>
       <c r="X186" s="49" t="n">
         <f aca="false">X92*założenia!$C$7</f>
-        <v>2929.1219107078</v>
+        <v>2057.337</v>
       </c>
       <c r="Y186" s="49" t="n">
         <f aca="false">Y92*założenia!$C$7</f>
-        <v>2929.1219107078</v>
+        <v>2057.337</v>
       </c>
       <c r="Z186" s="49" t="n">
         <f aca="false">Z92*założenia!$C$7</f>
-        <v>2929.1219107078</v>
+        <v>2057.337</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40679,7 +40679,7 @@
       </c>
       <c r="C188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,C$150:C$186)</f>
-        <v>807925.846</v>
+        <v>808429.906</v>
       </c>
       <c r="D188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,D$150:D$186)</f>
@@ -40723,7 +40723,7 @@
       </c>
       <c r="N188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,N$150:N$186)</f>
-        <v>134654.307666667</v>
+        <v>135158.367666667</v>
       </c>
       <c r="O188" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,2,O$150:O$186)</f>
@@ -40887,7 +40887,7 @@
       </c>
       <c r="C190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,C$150:C$186)</f>
-        <v>395011.056</v>
+        <v>394506.996</v>
       </c>
       <c r="D190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,D$150:D$186)</f>
@@ -40967,19 +40967,19 @@
       </c>
       <c r="W190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,W$150:W$186)</f>
-        <v>98752.764</v>
+        <v>98626.749</v>
       </c>
       <c r="X190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,X$150:X$186)</f>
-        <v>98752.764</v>
+        <v>98626.749</v>
       </c>
       <c r="Y190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,Y$150:Y$186)</f>
-        <v>98752.764</v>
+        <v>98626.749</v>
       </c>
       <c r="Z190" s="63" t="n">
         <f aca="false">SUMIF($B$150:$B$186,4,Z$150:Z$186)</f>
-        <v>98752.764</v>
+        <v>98626.749</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -41033,7 +41033,7 @@
       </c>
       <c r="N191" s="63" t="n">
         <f aca="false">SUM(N187:N190)</f>
-        <v>134654.307666667</v>
+        <v>135158.367666667</v>
       </c>
       <c r="O191" s="63" t="n">
         <f aca="false">SUM(O187:O190)</f>
@@ -41069,19 +41069,19 @@
       </c>
       <c r="W191" s="63" t="n">
         <f aca="false">SUM(W187:W190)</f>
-        <v>98752.764</v>
+        <v>98626.749</v>
       </c>
       <c r="X191" s="63" t="n">
         <f aca="false">SUM(X187:X190)</f>
-        <v>98752.764</v>
+        <v>98626.749</v>
       </c>
       <c r="Y191" s="63" t="n">
         <f aca="false">SUM(Y187:Y190)</f>
-        <v>98752.764</v>
+        <v>98626.749</v>
       </c>
       <c r="Z191" s="63" t="n">
         <f aca="false">SUM(Z187:Z190)</f>
-        <v>98752.764</v>
+        <v>98626.749</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -41095,95 +41095,95 @@
       </c>
       <c r="D192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,D98*$C$191/$C$97)</f>
-        <v>31440.5903780996</v>
+        <v>31442.2991309977</v>
       </c>
       <c r="E192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,E98*$C$191/$C$97)</f>
-        <v>31440.5903780996</v>
+        <v>31442.2991309977</v>
       </c>
       <c r="F192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,F98*$C$191/$C$97)</f>
-        <v>31440.5903780996</v>
+        <v>31442.2991309977</v>
       </c>
       <c r="G192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,G98*$C$191/$C$97)</f>
-        <v>30142.8206353995</v>
+        <v>30144.4588562948</v>
       </c>
       <c r="H192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,H98*$C$191/$C$97)</f>
-        <v>30142.8206353995</v>
+        <v>30144.4588562948</v>
       </c>
       <c r="I192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,I98*$C$191/$C$97)</f>
-        <v>32229.8632895799</v>
+        <v>32231.6149383766</v>
       </c>
       <c r="J192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,J98*$C$191/$C$97)</f>
-        <v>32229.8632895799</v>
+        <v>32231.6149383766</v>
       </c>
       <c r="K192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,K98*$C$191/$C$97)</f>
-        <v>32229.8632895799</v>
+        <v>32231.6149383766</v>
       </c>
       <c r="L192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,L98*$C$191/$C$97)</f>
-        <v>32229.8632895799</v>
+        <v>32231.6149383766</v>
       </c>
       <c r="M192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,M98*$C$191/$C$97)</f>
-        <v>32229.8632895799</v>
+        <v>32231.6149383766</v>
       </c>
       <c r="N192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,N98*$C$191/$C$97)</f>
-        <v>32229.8632895799</v>
+        <v>32352.2705391654</v>
       </c>
       <c r="O192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,O98*$C$191/$C$97)</f>
-        <v>32268.855109422</v>
+        <v>32270.6088773705</v>
       </c>
       <c r="P192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,P98*$C$191/$C$97)</f>
-        <v>32268.855109422</v>
+        <v>32270.6088773705</v>
       </c>
       <c r="Q192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,Q98*$C$191/$C$97)</f>
-        <v>33566.62506488</v>
+        <v>33568.4493648428</v>
       </c>
       <c r="R192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,R98*$C$191/$C$97)</f>
-        <v>33566.62506488</v>
+        <v>33568.4493648428</v>
       </c>
       <c r="S192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,S98*$C$191/$C$97)</f>
-        <v>33566.62506488</v>
+        <v>33568.4493648428</v>
       </c>
       <c r="T192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,T98*$C$191/$C$97)</f>
-        <v>33566.62506488</v>
+        <v>33568.4493648428</v>
       </c>
       <c r="U192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,U98*$C$191/$C$97)</f>
-        <v>33566.62506488</v>
+        <v>33568.4493648428</v>
       </c>
       <c r="V192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,V98*$C$191/$C$97)</f>
-        <v>33566.62506488</v>
+        <v>33568.4493648428</v>
       </c>
       <c r="W192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,W98*$C$191/$C$97)</f>
-        <v>31515.6449373246</v>
+        <v>31477.1395548928</v>
       </c>
       <c r="X192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,X98*$C$191/$C$97)</f>
-        <v>31515.6449373246</v>
+        <v>31477.1395548928</v>
       </c>
       <c r="Y192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,Y98*$C$191/$C$97)</f>
-        <v>31515.6449373246</v>
+        <v>31477.1395548928</v>
       </c>
       <c r="Z192" s="63" t="n">
         <f aca="false">IF($C$97=0,0,Z98*$C$191/$C$97)</f>
-        <v>31515.6449373246</v>
+        <v>31477.1395548928</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -41197,95 +41197,95 @@
       </c>
       <c r="D193" s="63" t="n">
         <f aca="false">D191+D192</f>
-        <v>162797.369933655</v>
+        <v>162799.078686553</v>
       </c>
       <c r="E193" s="63" t="n">
         <f aca="false">E191+E192</f>
-        <v>162797.369933655</v>
+        <v>162799.078686553</v>
       </c>
       <c r="F193" s="63" t="n">
         <f aca="false">F191+F192</f>
-        <v>162797.369933655</v>
+        <v>162799.078686553</v>
       </c>
       <c r="G193" s="63" t="n">
         <f aca="false">G191+G192</f>
-        <v>156077.601302066</v>
+        <v>156079.239522961</v>
       </c>
       <c r="H193" s="63" t="n">
         <f aca="false">H191+H192</f>
-        <v>156077.601302066</v>
+        <v>156079.239522961</v>
       </c>
       <c r="I193" s="63" t="n">
         <f aca="false">I191+I192</f>
-        <v>166884.170956247</v>
+        <v>166885.922605043</v>
       </c>
       <c r="J193" s="63" t="n">
         <f aca="false">J191+J192</f>
-        <v>166884.170956247</v>
+        <v>166885.922605043</v>
       </c>
       <c r="K193" s="63" t="n">
         <f aca="false">K191+K192</f>
-        <v>166884.170956247</v>
+        <v>166885.922605043</v>
       </c>
       <c r="L193" s="63" t="n">
         <f aca="false">L191+L192</f>
-        <v>166884.170956247</v>
+        <v>166885.922605043</v>
       </c>
       <c r="M193" s="63" t="n">
         <f aca="false">M191+M192</f>
-        <v>166884.170956247</v>
+        <v>166885.922605043</v>
       </c>
       <c r="N193" s="63" t="n">
         <f aca="false">N191+N192</f>
-        <v>166884.170956247</v>
+        <v>167510.638205832</v>
       </c>
       <c r="O193" s="63" t="n">
         <f aca="false">O191+O192</f>
-        <v>167086.071109422</v>
+        <v>167087.824877371</v>
       </c>
       <c r="P193" s="63" t="n">
         <f aca="false">P191+P192</f>
-        <v>167086.071109422</v>
+        <v>167087.824877371</v>
       </c>
       <c r="Q193" s="63" t="n">
         <f aca="false">Q191+Q192</f>
-        <v>173805.84106488</v>
+        <v>173807.665364843</v>
       </c>
       <c r="R193" s="63" t="n">
         <f aca="false">R191+R192</f>
-        <v>173805.84106488</v>
+        <v>173807.665364843</v>
       </c>
       <c r="S193" s="63" t="n">
         <f aca="false">S191+S192</f>
-        <v>173805.84106488</v>
+        <v>173807.665364843</v>
       </c>
       <c r="T193" s="63" t="n">
         <f aca="false">T191+T192</f>
-        <v>173805.84106488</v>
+        <v>173807.665364843</v>
       </c>
       <c r="U193" s="63" t="n">
         <f aca="false">U191+U192</f>
-        <v>173805.84106488</v>
+        <v>173807.665364843</v>
       </c>
       <c r="V193" s="63" t="n">
         <f aca="false">V191+V192</f>
-        <v>173805.84106488</v>
+        <v>173807.665364843</v>
       </c>
       <c r="W193" s="63" t="n">
         <f aca="false">W191+W192</f>
-        <v>130268.408937325</v>
+        <v>130103.888554893</v>
       </c>
       <c r="X193" s="63" t="n">
         <f aca="false">X191+X192</f>
-        <v>130268.408937325</v>
+        <v>130103.888554893</v>
       </c>
       <c r="Y193" s="63" t="n">
         <f aca="false">Y191+Y192</f>
-        <v>130268.408937325</v>
+        <v>130103.888554893</v>
       </c>
       <c r="Z193" s="63" t="n">
         <f aca="false">Z191+Z192</f>
-        <v>130268.408937325</v>
+        <v>130103.888554893</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -41296,91 +41296,91 @@
       <c r="C194" s="63"/>
       <c r="D194" s="63" t="n">
         <f aca="false">D193</f>
-        <v>162797.369933655</v>
+        <v>162799.078686553</v>
       </c>
       <c r="E194" s="63" t="n">
         <f aca="false">D194+E193</f>
-        <v>325594.73986731</v>
+        <v>325598.157373106</v>
       </c>
       <c r="F194" s="63" t="n">
         <f aca="false">E194+F193</f>
-        <v>488392.109800965</v>
+        <v>488397.23605966</v>
       </c>
       <c r="G194" s="63" t="n">
         <f aca="false">F194+G193</f>
-        <v>644469.711103032</v>
+        <v>644476.475582621</v>
       </c>
       <c r="H194" s="63" t="n">
         <f aca="false">G194+H193</f>
-        <v>800547.312405098</v>
+        <v>800555.715105583</v>
       </c>
       <c r="I194" s="63" t="n">
         <f aca="false">H194+I193</f>
-        <v>967431.483361344</v>
+        <v>967441.637710626</v>
       </c>
       <c r="J194" s="63" t="n">
         <f aca="false">I194+J193</f>
-        <v>1134315.65431759</v>
+        <v>1134327.56031567</v>
       </c>
       <c r="K194" s="63" t="n">
         <f aca="false">J194+K193</f>
-        <v>1301199.82527384</v>
+        <v>1301213.48292071</v>
       </c>
       <c r="L194" s="63" t="n">
         <f aca="false">K194+L193</f>
-        <v>1468083.99623008</v>
+        <v>1468099.40552576</v>
       </c>
       <c r="M194" s="63" t="n">
         <f aca="false">L194+M193</f>
-        <v>1634968.16718633</v>
+        <v>1634985.3281308</v>
       </c>
       <c r="N194" s="63" t="n">
         <f aca="false">M194+N193</f>
-        <v>1801852.33814258</v>
+        <v>1802495.96633663</v>
       </c>
       <c r="O194" s="63" t="n">
         <f aca="false">N194+O193</f>
-        <v>1968938.409252</v>
+        <v>1969583.791214</v>
       </c>
       <c r="P194" s="63" t="n">
         <f aca="false">O194+P193</f>
-        <v>2136024.48036142</v>
+        <v>2136671.61609137</v>
       </c>
       <c r="Q194" s="63" t="n">
         <f aca="false">P194+Q193</f>
-        <v>2309830.3214263</v>
+        <v>2310479.28145622</v>
       </c>
       <c r="R194" s="63" t="n">
         <f aca="false">Q194+R193</f>
-        <v>2483636.16249118</v>
+        <v>2484286.94682106</v>
       </c>
       <c r="S194" s="63" t="n">
         <f aca="false">R194+S193</f>
-        <v>2657442.00355606</v>
+        <v>2658094.6121859</v>
       </c>
       <c r="T194" s="63" t="n">
         <f aca="false">S194+T193</f>
-        <v>2831247.84462094</v>
+        <v>2831902.27755074</v>
       </c>
       <c r="U194" s="63" t="n">
         <f aca="false">T194+U193</f>
-        <v>3005053.68568582</v>
+        <v>3005709.94291559</v>
       </c>
       <c r="V194" s="63" t="n">
         <f aca="false">U194+V193</f>
-        <v>3178859.5267507</v>
+        <v>3179517.60828043</v>
       </c>
       <c r="W194" s="63" t="n">
         <f aca="false">V194+W193</f>
-        <v>3309127.93568803</v>
+        <v>3309621.49683532</v>
       </c>
       <c r="X194" s="63" t="n">
         <f aca="false">W194+X193</f>
-        <v>3439396.34462535</v>
+        <v>3439725.38539022</v>
       </c>
       <c r="Y194" s="63" t="n">
         <f aca="false">X194+Y193</f>
-        <v>3569664.75356268</v>
+        <v>3569829.27394511</v>
       </c>
       <c r="Z194" s="63" t="n">
         <f aca="false">Y194+Z193</f>
@@ -42094,15 +42094,15 @@
       </c>
       <c r="E13" s="71" t="n">
         <f aca="false">SUM(E14:E23)</f>
-        <v>1009907.33</v>
+        <v>1010682.33</v>
       </c>
       <c r="F13" s="71" t="n">
         <f aca="false">SUM(F14:F23)</f>
-        <v>1009907.33</v>
+        <v>1010537.41</v>
       </c>
       <c r="G13" s="71" t="n">
         <f aca="false">SUM(G14:G23)</f>
-        <v>807925.85</v>
+        <v>808429.91</v>
       </c>
       <c r="H13" s="63"/>
       <c r="I13" s="71" t="n">
@@ -42119,15 +42119,15 @@
       </c>
       <c r="L13" s="71" t="n">
         <f aca="false">E13-I13</f>
-        <v>-217028.38</v>
+        <v>-216253.38</v>
       </c>
       <c r="M13" s="71" t="n">
         <f aca="false">F13-J13</f>
-        <v>-194028.38</v>
+        <v>-193398.3</v>
       </c>
       <c r="N13" s="71" t="n">
         <f aca="false">G13-K13</f>
-        <v>-155222.71</v>
+        <v>-154718.65</v>
       </c>
       <c r="O13" s="40"/>
       <c r="P13" s="70" t="str">
@@ -42566,15 +42566,15 @@
       </c>
       <c r="E21" s="74" t="n">
         <f aca="false">ROUND(F21*założenia!$C$8,2)</f>
-        <v>0</v>
+        <v>775</v>
       </c>
       <c r="F21" s="74" t="n">
         <f aca="false">założenia!$C$14</f>
-        <v>0</v>
+        <v>630.08</v>
       </c>
       <c r="G21" s="74" t="n">
         <f aca="false">założenia!$C$9</f>
-        <v>0</v>
+        <v>504.06</v>
       </c>
       <c r="H21" s="49"/>
       <c r="I21" s="73" t="n">
@@ -42591,15 +42591,15 @@
       </c>
       <c r="L21" s="73" t="n">
         <f aca="false">E21-I21</f>
-        <v>-123000</v>
+        <v>-122225</v>
       </c>
       <c r="M21" s="73" t="n">
         <f aca="false">F21-J21</f>
-        <v>-100000</v>
+        <v>-99369.92</v>
       </c>
       <c r="N21" s="73" t="n">
         <f aca="false">G21-K21</f>
-        <v>-80000</v>
+        <v>-79495.94</v>
       </c>
       <c r="O21" s="41"/>
       <c r="P21" s="72" t="str">
@@ -43333,15 +43333,15 @@
       </c>
       <c r="E34" s="71" t="n">
         <f aca="false">SUM(E35:E43)</f>
-        <v>658351.76</v>
+        <v>657511.66</v>
       </c>
       <c r="F34" s="71" t="n">
         <f aca="false">SUM(F35:F43)</f>
-        <v>658351.76</v>
+        <v>657511.66</v>
       </c>
       <c r="G34" s="71" t="n">
         <f aca="false">SUM(G35:G43)</f>
-        <v>395011.06</v>
+        <v>394507</v>
       </c>
       <c r="H34" s="63"/>
       <c r="I34" s="71" t="n">
@@ -43358,15 +43358,15 @@
       </c>
       <c r="L34" s="71" t="n">
         <f aca="false">E34-I34</f>
-        <v>-39885.38</v>
+        <v>-40725.4800000001</v>
       </c>
       <c r="M34" s="71" t="n">
         <f aca="false">F34-J34</f>
-        <v>-39885.38</v>
+        <v>-40725.4800000001</v>
       </c>
       <c r="N34" s="71" t="n">
         <f aca="false">G34-K34</f>
-        <v>-23931.22</v>
+        <v>-24435.28</v>
       </c>
       <c r="O34" s="40"/>
       <c r="P34" s="70" t="str">
@@ -43392,15 +43392,15 @@
       </c>
       <c r="E35" s="74" t="n">
         <f aca="false">F35</f>
-        <v>219882.59</v>
+        <v>221600</v>
       </c>
       <c r="F35" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$84,2)</f>
-        <v>219882.59</v>
+        <v>221600</v>
       </c>
       <c r="G35" s="74" t="n">
-        <f aca="false">ROUND(założenia!$C$13-(G4+G5+G6+G7+G8+G9+G10+G11+G12+G14+G15+G16+G17+G18+G19+G20+G21+G22+G23+G25+G26+G27+G28+G29+G30+G31+G32+G33+G36+G37+G38+G39+G40+G41+G42+G43),2)</f>
-        <v>131929.56</v>
+        <f aca="false">ROUND('budżet po miesiącach'!$C$178,2)</f>
+        <v>132960</v>
       </c>
       <c r="H35" s="49"/>
       <c r="I35" s="73" t="n">
@@ -43417,24 +43417,21 @@
       </c>
       <c r="L35" s="73" t="n">
         <f aca="false">E35-I35</f>
-        <v>-1717.41</v>
+        <v>0</v>
       </c>
       <c r="M35" s="73" t="n">
         <f aca="false">F35-J35</f>
-        <v>-1717.41</v>
+        <v>0</v>
       </c>
       <c r="N35" s="73" t="n">
         <f aca="false">G35-K35</f>
-        <v>-1030.44</v>
+        <v>0</v>
       </c>
       <c r="O35" s="41"/>
       <c r="P35" s="72" t="str">
         <f aca="false">IF(AND(E35&gt;=B35-0.005,F35&gt;=C35-0.005,G35&gt;=D35-0.005),"OK","&lt; narastająco")</f>
         <v>OK</v>
       </c>
-      <c r="Q35" s="55" t="s">
-        <v>248</v>
-      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="72" t="s">
@@ -43454,15 +43451,15 @@
       </c>
       <c r="E36" s="74" t="n">
         <f aca="false">F36</f>
-        <v>37427.67</v>
+        <v>37720</v>
       </c>
       <c r="F36" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$85,2)</f>
-        <v>37427.67</v>
+        <v>37720</v>
       </c>
       <c r="G36" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$179,2)</f>
-        <v>22456.6</v>
+        <v>22632</v>
       </c>
       <c r="H36" s="49"/>
       <c r="I36" s="73" t="n">
@@ -43479,15 +43476,15 @@
       </c>
       <c r="L36" s="73" t="n">
         <f aca="false">E36-I36</f>
-        <v>-292.330000000002</v>
+        <v>0</v>
       </c>
       <c r="M36" s="73" t="n">
         <f aca="false">F36-J36</f>
-        <v>-292.330000000002</v>
+        <v>0</v>
       </c>
       <c r="N36" s="73" t="n">
         <f aca="false">G36-K36</f>
-        <v>-175.400000000001</v>
+        <v>0</v>
       </c>
       <c r="O36" s="41"/>
       <c r="P36" s="72" t="str">
@@ -43513,15 +43510,15 @@
       </c>
       <c r="E37" s="74" t="n">
         <f aca="false">F37</f>
-        <v>107599.59</v>
+        <v>108440</v>
       </c>
       <c r="F37" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$86,2)</f>
-        <v>107599.59</v>
+        <v>108440</v>
       </c>
       <c r="G37" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$180,2)</f>
-        <v>64559.75</v>
+        <v>65064</v>
       </c>
       <c r="H37" s="49"/>
       <c r="I37" s="73" t="n">
@@ -43538,15 +43535,15 @@
       </c>
       <c r="L37" s="73" t="n">
         <f aca="false">E37-I37</f>
-        <v>-840.410000000004</v>
+        <v>0</v>
       </c>
       <c r="M37" s="73" t="n">
         <f aca="false">F37-J37</f>
-        <v>-840.410000000004</v>
+        <v>0</v>
       </c>
       <c r="N37" s="73" t="n">
         <f aca="false">G37-K37</f>
-        <v>-504.25</v>
+        <v>0</v>
       </c>
       <c r="O37" s="41"/>
       <c r="P37" s="72" t="str">
@@ -43572,15 +43569,15 @@
       </c>
       <c r="E38" s="74" t="n">
         <f aca="false">F38</f>
-        <v>81860.62</v>
+        <v>82500</v>
       </c>
       <c r="F38" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$87,2)</f>
-        <v>81860.62</v>
+        <v>82500</v>
       </c>
       <c r="G38" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$181,2)</f>
-        <v>49116.37</v>
+        <v>49500</v>
       </c>
       <c r="H38" s="49"/>
       <c r="I38" s="73" t="n">
@@ -43597,15 +43594,15 @@
       </c>
       <c r="L38" s="73" t="n">
         <f aca="false">E38-I38</f>
-        <v>-639.380000000005</v>
+        <v>0</v>
       </c>
       <c r="M38" s="73" t="n">
         <f aca="false">F38-J38</f>
-        <v>-639.380000000005</v>
+        <v>0</v>
       </c>
       <c r="N38" s="73" t="n">
         <f aca="false">G38-K38</f>
-        <v>-383.629999999997</v>
+        <v>0</v>
       </c>
       <c r="O38" s="41"/>
       <c r="P38" s="72" t="str">
@@ -43631,15 +43628,15 @@
       </c>
       <c r="E39" s="74" t="n">
         <f aca="false">F39</f>
-        <v>29529.36</v>
+        <v>29760</v>
       </c>
       <c r="F39" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$88,2)</f>
-        <v>29529.36</v>
+        <v>29760</v>
       </c>
       <c r="G39" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$182,2)</f>
-        <v>17717.62</v>
+        <v>17856</v>
       </c>
       <c r="H39" s="49"/>
       <c r="I39" s="73" t="n">
@@ -43656,15 +43653,15 @@
       </c>
       <c r="L39" s="73" t="n">
         <f aca="false">E39-I39</f>
-        <v>-230.639999999999</v>
+        <v>0</v>
       </c>
       <c r="M39" s="73" t="n">
         <f aca="false">F39-J39</f>
-        <v>-230.639999999999</v>
+        <v>0</v>
       </c>
       <c r="N39" s="73" t="n">
         <f aca="false">G39-K39</f>
-        <v>-138.380000000001</v>
+        <v>0</v>
       </c>
       <c r="O39" s="41"/>
       <c r="P39" s="72" t="str">
@@ -43690,15 +43687,15 @@
       </c>
       <c r="E40" s="74" t="n">
         <f aca="false">F40</f>
-        <v>81860.62</v>
+        <v>82500</v>
       </c>
       <c r="F40" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$89,2)</f>
-        <v>81860.62</v>
+        <v>82500</v>
       </c>
       <c r="G40" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$183,2)</f>
-        <v>49116.37</v>
+        <v>49500</v>
       </c>
       <c r="H40" s="49"/>
       <c r="I40" s="73" t="n">
@@ -43715,15 +43712,15 @@
       </c>
       <c r="L40" s="73" t="n">
         <f aca="false">E40-I40</f>
-        <v>-639.380000000005</v>
+        <v>0</v>
       </c>
       <c r="M40" s="73" t="n">
         <f aca="false">F40-J40</f>
-        <v>-639.380000000005</v>
+        <v>0</v>
       </c>
       <c r="N40" s="73" t="n">
         <f aca="false">G40-K40</f>
-        <v>-383.629999999997</v>
+        <v>0</v>
       </c>
       <c r="O40" s="41"/>
       <c r="P40" s="72" t="str">
@@ -43808,15 +43805,15 @@
       </c>
       <c r="E42" s="74" t="n">
         <f aca="false">F42</f>
-        <v>78387.75</v>
+        <v>79000</v>
       </c>
       <c r="F42" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$91,2)</f>
-        <v>78387.75</v>
+        <v>79000</v>
       </c>
       <c r="G42" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$185,2)</f>
-        <v>47032.65</v>
+        <v>47400</v>
       </c>
       <c r="H42" s="49"/>
       <c r="I42" s="73" t="n">
@@ -43833,15 +43830,15 @@
       </c>
       <c r="L42" s="73" t="n">
         <f aca="false">E42-I42</f>
-        <v>-612.25</v>
+        <v>0</v>
       </c>
       <c r="M42" s="73" t="n">
         <f aca="false">F42-J42</f>
-        <v>-612.25</v>
+        <v>0</v>
       </c>
       <c r="N42" s="73" t="n">
         <f aca="false">G42-K42</f>
-        <v>-367.349999999999</v>
+        <v>0</v>
       </c>
       <c r="O42" s="41"/>
       <c r="P42" s="72" t="str">
@@ -43867,15 +43864,15 @@
       </c>
       <c r="E43" s="74" t="n">
         <f aca="false">F43</f>
-        <v>19527.48</v>
+        <v>13715.58</v>
       </c>
       <c r="F43" s="74" t="n">
         <f aca="false">ROUND('budżet po miesiącach'!$C$92,2)</f>
-        <v>19527.48</v>
+        <v>13715.58</v>
       </c>
       <c r="G43" s="74" t="n">
-        <f aca="false">ROUND('budżet po miesiącach'!$C$186,2)</f>
-        <v>11716.49</v>
+        <f aca="false">ROUND(założenia!$C$13-(G4+G5+G6+G7+G8+G9+G10+G11+G12+G14+G15+G16+G17+G18+G19+G20+G21+G22+G23+G25+G26+G27+G28+G29+G30+G31+G32+G33+G35+G36+G37+G38+G39+G40+G41+G42),2)</f>
+        <v>8229.35</v>
       </c>
       <c r="H43" s="49"/>
       <c r="I43" s="73" t="n">
@@ -43892,21 +43889,24 @@
       </c>
       <c r="L43" s="73" t="n">
         <f aca="false">E43-I43</f>
-        <v>-34332.52</v>
+        <v>-40144.42</v>
       </c>
       <c r="M43" s="73" t="n">
         <f aca="false">F43-J43</f>
-        <v>-34332.52</v>
+        <v>-40144.42</v>
       </c>
       <c r="N43" s="73" t="n">
         <f aca="false">G43-K43</f>
-        <v>-20599.51</v>
+        <v>-24086.65</v>
       </c>
       <c r="O43" s="41"/>
       <c r="P43" s="72" t="str">
         <f aca="false">IF(AND(E43&gt;=B43-0.005,F43&gt;=C43-0.005,G43&gt;=D43-0.005),"OK","&lt; narastająco")</f>
         <v>OK</v>
       </c>
+      <c r="Q43" s="55" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="75" t="s">
@@ -43973,11 +43973,11 @@
       </c>
       <c r="E48" s="73" t="n">
         <f aca="false">E3+E13+E24+E34</f>
-        <v>3864521.12</v>
+        <v>3864456.02</v>
       </c>
       <c r="F48" s="73" t="n">
         <f aca="false">F3+F13+F24+F34</f>
-        <v>3864521.12</v>
+        <v>3864311.1</v>
       </c>
       <c r="G48" s="73" t="n">
         <f aca="false">G3+G13+G24+G34</f>
@@ -43998,11 +43998,11 @@
       </c>
       <c r="L48" s="73" t="n">
         <f aca="false">E48-I48</f>
-        <v>-32971.3700000001</v>
+        <v>-33036.4700000007</v>
       </c>
       <c r="M48" s="73" t="n">
         <f aca="false">F48-J48</f>
-        <v>-9971.37000000011</v>
+        <v>-10181.3900000006</v>
       </c>
       <c r="N48" s="73" t="n">
         <f aca="false">G48-K48</f>
@@ -44027,11 +44027,11 @@
       </c>
       <c r="E49" s="73" t="n">
         <f aca="false">F49</f>
-        <v>966130.28</v>
+        <v>966077.78</v>
       </c>
       <c r="F49" s="73" t="n">
         <f aca="false">ROUND(0.25*F48,2)</f>
-        <v>966130.28</v>
+        <v>966077.78</v>
       </c>
       <c r="G49" s="73" t="n">
         <f aca="false">ROUNDDOWN(F49*G48/F48,2)</f>
@@ -44052,11 +44052,11 @@
       </c>
       <c r="L49" s="73" t="n">
         <f aca="false">E49-I49</f>
-        <v>-2492.83999999997</v>
+        <v>-2545.33999999997</v>
       </c>
       <c r="M49" s="73" t="n">
         <f aca="false">F49-J49</f>
-        <v>-2492.83999999997</v>
+        <v>-2545.33999999997</v>
       </c>
       <c r="N49" s="73" t="n">
         <f aca="false">G49-K49</f>
@@ -44081,11 +44081,11 @@
       </c>
       <c r="E50" s="77" t="n">
         <f aca="false">E48+E49</f>
-        <v>4830651.4</v>
+        <v>4830533.8</v>
       </c>
       <c r="F50" s="77" t="n">
         <f aca="false">F48+F49</f>
-        <v>4830651.4</v>
+        <v>4830388.88</v>
       </c>
       <c r="G50" s="77" t="n">
         <f aca="false">G48+G49</f>
@@ -44106,11 +44106,11 @@
       </c>
       <c r="L50" s="77" t="n">
         <f aca="false">E50-I50</f>
-        <v>-35464.21</v>
+        <v>-35581.8100000005</v>
       </c>
       <c r="M50" s="77" t="n">
         <f aca="false">F50-J50</f>
-        <v>-12464.21</v>
+        <v>-12726.7300000004</v>
       </c>
       <c r="N50" s="77" t="n">
         <f aca="false">G50-K50</f>
@@ -44151,7 +44151,7 @@
       <c r="E52" s="73"/>
       <c r="F52" s="73" t="n">
         <f aca="false">ROUND(F50-F51,2)</f>
-        <v>-12464.21</v>
+        <v>-12726.73</v>
       </c>
       <c r="G52" s="73" t="n">
         <f aca="false">ROUND(G50-G51,2)</f>

</xml_diff>